<commit_message>
Move Common Box #1
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -35223,7 +35223,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -35270,7 +35270,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -35317,7 +35317,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -35364,7 +35364,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -35505,7 +35505,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -35975,7 +35975,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -36022,7 +36022,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -36069,7 +36069,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -36116,7 +36116,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -36163,7 +36163,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -36210,7 +36210,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -36257,7 +36257,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -36304,7 +36304,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -36351,7 +36351,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -36398,7 +36398,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -36445,7 +36445,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -36492,7 +36492,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -36539,7 +36539,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -36586,7 +36586,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -36633,7 +36633,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -36680,7 +36680,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -36727,7 +36727,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -36774,7 +36774,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -36821,7 +36821,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -36868,7 +36868,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -37149,7 +37149,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">

</xml_diff>

<commit_message>
Edit HEK ATF3 KO rep2 from unknown device
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -20861,7 +20861,7 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="F252" t="inlineStr">
@@ -33694,7 +33694,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -33704,7 +33704,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -33725,7 +33725,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CASPEX Single</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -33735,7 +33735,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -33747,7 +33747,7 @@
         <v>2</v>
       </c>
       <c r="F45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G45">
         <v>1</v>
@@ -33756,7 +33756,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX</t>
+          <t xml:space="preserve">HEK CASPEX Single</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -33766,12 +33766,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E46">
@@ -33787,7 +33787,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK E2F1 sh1</t>
+          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -33797,12 +33797,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E47">
@@ -33818,7 +33818,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK E2F1 sh2</t>
+          <t xml:space="preserve">HEK E2F1 sh1</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -33849,7 +33849,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK FOXA1 KO g1</t>
+          <t xml:space="preserve">HEK E2F1 sh2</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -33859,12 +33859,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E49">
@@ -33880,7 +33880,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK FOXA1 KO g2</t>
+          <t xml:space="preserve">HEK FOXA1 KO g1</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -33895,7 +33895,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E50">
@@ -33911,7 +33911,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 OX</t>
+          <t xml:space="preserve">HEK FOXA1 KO g2</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -33926,7 +33926,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E51">
@@ -33942,7 +33942,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g1</t>
+          <t xml:space="preserve">HEK HOXB6 OX</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -33952,12 +33952,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E52">
@@ -33967,13 +33967,13 @@
         <v>0</v>
       </c>
       <c r="G52">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g2</t>
+          <t xml:space="preserve">HEK POU3F3 KO g1</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -33988,7 +33988,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E53">
@@ -33998,13 +33998,13 @@
         <v>0</v>
       </c>
       <c r="G53">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK STAT1 KO g2</t>
+          <t xml:space="preserve">HEK POU3F3 KO g2</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -34035,7 +34035,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT(20)</t>
+          <t xml:space="preserve">HEK STAT1 KO g2</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -34045,12 +34045,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E55">
@@ -34060,44 +34060,44 @@
         <v>0</v>
       </c>
       <c r="G55">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">HEK gNT(20)</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E56">
         <v>2</v>
       </c>
       <c r="F56">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G56">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -34107,7 +34107,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -34128,7 +34128,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATP7B KO #24</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -34138,7 +34138,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -34150,7 +34150,7 @@
         <v>2</v>
       </c>
       <c r="F58">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G58">
         <v>1</v>
@@ -34159,17 +34159,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-V</t>
+          <t xml:space="preserve">Huh7 ATP7B KO #24</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -34184,13 +34184,13 @@
         <v>0</v>
       </c>
       <c r="G59">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-V 99.17%</t>
+          <t xml:space="preserve">LCC-V</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -34221,7 +34221,22 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gC1</t>
+          <t xml:space="preserve">LCC-V 99.17%</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E61">
@@ -34231,13 +34246,13 @@
         <v>0</v>
       </c>
       <c r="G61">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gC2</t>
+          <t xml:space="preserve">LNCX gC1</t>
         </is>
       </c>
       <c r="E62">
@@ -34253,22 +34268,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gC3</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gC3</t>
+          <t xml:space="preserve">LNCX gC2</t>
         </is>
       </c>
       <c r="E63">
@@ -34284,7 +34284,22 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gC4</t>
+          <t xml:space="preserve">LNCX gC3</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gC3</t>
         </is>
       </c>
       <c r="E64">
@@ -34300,22 +34315,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gP3</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gP3</t>
+          <t xml:space="preserve">LNCX gC4</t>
         </is>
       </c>
       <c r="E65">
@@ -34331,22 +34331,22 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX gP2</t>
+          <t xml:space="preserve">LNCX gP3</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t xml:space="preserve">gP2</t>
+          <t xml:space="preserve">gP3</t>
         </is>
       </c>
       <c r="E66">
@@ -34362,12 +34362,12 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap (m3) (sortER)</t>
+          <t xml:space="preserve">LUCX gP2</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -34377,7 +34377,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gP2</t>
         </is>
       </c>
       <c r="E67">
@@ -34393,7 +34393,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada CASPEX mCherry 1 (no use)</t>
+          <t xml:space="preserve">LnCap (m3) (sortER)</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -34403,7 +34403,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -34424,7 +34424,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canadaa V1G1</t>
+          <t xml:space="preserve">LnCap Canada CASPEX mCherry 1 (no use)</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -34434,7 +34434,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -34455,7 +34455,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select +P+D #1</t>
+          <t xml:space="preserve">LnCap Canadaa V1G1</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -34465,7 +34465,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -34480,13 +34480,13 @@
         <v>0</v>
       </c>
       <c r="G70">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select +P+D #2</t>
+          <t xml:space="preserve">LnCapCASPEX no select +P+D #1</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -34511,13 +34511,13 @@
         <v>0</v>
       </c>
       <c r="G71">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select E</t>
+          <t xml:space="preserve">LnCapCASPEX no select +P+D #2</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -34542,13 +34542,13 @@
         <v>0</v>
       </c>
       <c r="G72">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select H</t>
+          <t xml:space="preserve">LnCapCASPEX no select E</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -34573,23 +34573,23 @@
         <v>0</v>
       </c>
       <c r="G73">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145 ATF3 KO rep2</t>
+          <t xml:space="preserve">LnCapCASPEX no select H</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -34598,7 +34598,7 @@
         </is>
       </c>
       <c r="E74">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F74">
         <v>0</v>
@@ -34610,7 +34610,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145 ATF3 OX rep2</t>
+          <t xml:space="preserve">Du145 ATF3 KO rep2</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -34620,7 +34620,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -34641,7 +34641,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEXe g3</t>
+          <t xml:space="preserve">Du145 ATF3 OX rep2</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -34651,12 +34651,12 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t xml:space="preserve">g3</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E76">
@@ -34672,22 +34672,22 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK APEX1 KO g2</t>
+          <t xml:space="preserve">DuDtxR CASPEXe g3</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g3</t>
         </is>
       </c>
       <c r="E77">
@@ -34703,7 +34703,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK APEX1 OX</t>
+          <t xml:space="preserve">HEK APEX1 KO g2</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -34713,12 +34713,12 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E78">
@@ -34734,7 +34734,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK APEX1 g1</t>
+          <t xml:space="preserve">HEK APEX1 OX</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -34744,12 +34744,12 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E79">
@@ -34765,7 +34765,22 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO</t>
+          <t xml:space="preserve">HEK APEX1 g1</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E80">
@@ -34812,7 +34827,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">HEK ATF3 KO10</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -34834,7 +34849,7 @@
         <v>1</v>
       </c>
       <c r="F82">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G82">
         <v>1</v>
@@ -34843,7 +34858,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO10</t>
+          <t xml:space="preserve">HEK ATF3 OX</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -34853,7 +34868,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -34874,7 +34889,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX</t>
+          <t xml:space="preserve">HEK ATF3 OX rep2</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -34905,7 +34920,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep2</t>
+          <t xml:space="preserve">HEK ATF3 OX10r1</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -34936,7 +34951,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX10r1</t>
+          <t xml:space="preserve">HEK ATF3 OX20r1</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -34967,7 +34982,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX20r1</t>
+          <t xml:space="preserve">HEK ATF3OX10r1</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -34998,7 +35013,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3OX10r1</t>
+          <t xml:space="preserve">HEK ATP7B KO-1</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -35008,7 +35023,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -35029,7 +35044,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B KO-1</t>
+          <t xml:space="preserve">HEK ATP7B KO-2</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -35060,7 +35075,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B KO-2</t>
+          <t xml:space="preserve">HEK ATP7B KO-3</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -35091,7 +35106,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B KO-3</t>
+          <t xml:space="preserve">HEK CASPEX gNT</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -35101,12 +35116,12 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E91">
@@ -35122,7 +35137,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CASPEX gNT</t>
+          <t xml:space="preserve">HEK CBX3 KO g1 plv-GFP</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -35132,12 +35147,12 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E92">
@@ -35153,7 +35168,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO g1 plv-GFP</t>
+          <t xml:space="preserve">HEK CBX3 OX</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -35163,12 +35178,12 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E93">
@@ -35184,7 +35199,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 OX</t>
+          <t xml:space="preserve">HEK GATA6 KO g1</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -35194,12 +35209,12 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E94">
@@ -35215,7 +35230,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK GATA6 KO g1</t>
+          <t xml:space="preserve">HEK GATA6 KO g2</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -35230,7 +35245,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E95">
@@ -35246,7 +35261,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK GATA6 KO g2</t>
+          <t xml:space="preserve">HEK HOXB6 KO g2</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -35256,7 +35271,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -35277,7 +35292,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 KO g2</t>
+          <t xml:space="preserve">HEK JUN KO g1</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -35287,12 +35302,12 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E97">
@@ -35308,7 +35323,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK JUN KO g1</t>
+          <t xml:space="preserve">HEK JUN KO g2</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -35323,7 +35338,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E98">
@@ -35339,7 +35354,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK JUN KO g2</t>
+          <t xml:space="preserve">HEK JUN1 KO g2</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -35370,7 +35385,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK JUN1 KO g2</t>
+          <t xml:space="preserve">HEK NRF2 KO g1</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -35385,7 +35400,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E100">
@@ -35401,7 +35416,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK NRF2 KO g1</t>
+          <t xml:space="preserve">HEK NRF2 KO g2</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -35416,7 +35431,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E101">
@@ -35432,7 +35447,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK NRF2 KO g2</t>
+          <t xml:space="preserve">HEK RFX KO g1</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -35447,7 +35462,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E102">
@@ -35463,7 +35478,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK RFX KO g1</t>
+          <t xml:space="preserve">HEK RFX KO g2</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -35478,7 +35493,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E103">
@@ -35494,7 +35509,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK RFX KO g2</t>
+          <t xml:space="preserve">HEK SMARCE1 KO g1</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -35509,7 +35524,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E104">
@@ -35525,7 +35540,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK SMARCE1 KO g1</t>
+          <t xml:space="preserve">HEK SMARCE1 KO g2</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -35540,7 +35555,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E105">
@@ -35556,7 +35571,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK SMARCE1 KO g2</t>
+          <t xml:space="preserve">HEK SPEN KO g2</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -35587,7 +35602,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK SPEN KO g2</t>
+          <t xml:space="preserve">HEK STAT1 KO g1</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -35602,7 +35617,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E107">
@@ -35618,7 +35633,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK STAT1 KO g1</t>
+          <t xml:space="preserve">HEK TOX4 OX 3xFLAG</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -35628,12 +35643,12 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E108">
@@ -35649,7 +35664,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK TOX4 OX 3xFLAG</t>
+          <t xml:space="preserve">HEK gNT (10)</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -35659,12 +35674,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E109">
@@ -35680,7 +35695,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT (10)</t>
+          <t xml:space="preserve">HEK lef1 OX</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -35690,12 +35705,12 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E110">
@@ -35711,17 +35726,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK lef1 OX</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep2</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -35742,7 +35757,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep2</t>
+          <t xml:space="preserve">Huh7 ATF3 KO20</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -35773,7 +35788,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO20</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep2</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -35783,7 +35798,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -35804,7 +35819,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep2</t>
+          <t xml:space="preserve">Huh7 ATF3 OX20r1</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -35835,7 +35850,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX20r1</t>
+          <t xml:space="preserve">Huh7 ATF3KO10</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -35845,7 +35860,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -35866,7 +35881,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3KO10</t>
+          <t xml:space="preserve">Huh7 ATP7B KO</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -35897,7 +35912,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATP7B KO</t>
+          <t xml:space="preserve">Huh7 CASPEX gNT</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -35907,12 +35922,12 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E117">
@@ -35928,7 +35943,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 CASPEX gNT</t>
+          <t xml:space="preserve">Huh7 CBX3 KO g1</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -35938,12 +35953,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E118">
@@ -35959,7 +35974,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 CBX3 KO g1</t>
+          <t xml:space="preserve">Huh7 CBX3 KO g2</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -35974,7 +35989,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E119">
@@ -35990,7 +36005,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 CBX3 KO g2</t>
+          <t xml:space="preserve">Huh7 CBX3 OX</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -36000,12 +36015,12 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E120">
@@ -36021,7 +36036,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 CBX3 OX</t>
+          <t xml:space="preserve">Huh7 HOXB6 KO g1</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -36036,7 +36051,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E121">
@@ -36052,7 +36067,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 HOXB6 KO g1</t>
+          <t xml:space="preserve">Huh7 HOXB6 OX</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -36067,7 +36082,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E122">
@@ -36083,7 +36098,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 HOXB6 OX</t>
+          <t xml:space="preserve">Huh7 POU3F2 KO g1</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -36093,12 +36108,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E123">
@@ -36114,7 +36129,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 POU3F2 KO g1</t>
+          <t xml:space="preserve">Huh7 POU3F3 KO g1</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -36145,7 +36160,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 POU3F3 KO g1</t>
+          <t xml:space="preserve">Huh7 POU3F3 KO g2</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -36160,7 +36175,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E125">
@@ -36176,7 +36191,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 POU3F3 KO g2</t>
+          <t xml:space="preserve">Huh7 TOX4 KO g1</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -36186,12 +36201,12 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E126">
@@ -36207,7 +36222,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 TOX4 KO g1</t>
+          <t xml:space="preserve">Huh7 TOX4 OX</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -36222,7 +36237,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E127">
@@ -36238,7 +36253,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 TOX4 OX</t>
+          <t xml:space="preserve">Huh7 lef1 OX</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -36269,17 +36284,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 lef1 OX</t>
+          <t xml:space="preserve">LCC-C*</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -36300,7 +36315,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-C*</t>
+          <t xml:space="preserve">LCC-E</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -36331,7 +36346,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-E</t>
+          <t xml:space="preserve">LCC-H</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -36362,7 +36377,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-H</t>
+          <t xml:space="preserve">LNC478 #1</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -36393,7 +36408,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNC478 #1</t>
+          <t xml:space="preserve">LNC478 #2 98%</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -36424,7 +36439,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNC478 #2 98%</t>
+          <t xml:space="preserve">LNC478 #3</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -36455,7 +36470,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNC478 #3</t>
+          <t xml:space="preserve">LNCAP BMK</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -36486,7 +36501,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCAP BMK</t>
+          <t xml:space="preserve">LnCap (m3) no sort</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -36517,7 +36532,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap (m3) no sort</t>
+          <t xml:space="preserve">LnCap Canada V1G2</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -36548,7 +36563,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G2</t>
+          <t xml:space="preserve">LnCap Canada V1G3</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -36579,7 +36594,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G3</t>
+          <t xml:space="preserve">LnCap Canada V1G4</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -36610,7 +36625,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G4</t>
+          <t xml:space="preserve">LnCap ER</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -36641,7 +36656,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap ER</t>
+          <t xml:space="preserve">LnCap V1G1</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -36672,7 +36687,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap V1G1</t>
+          <t xml:space="preserve">LnCap478 #2 98%</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -36703,7 +36718,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap478 #2 98%</t>
+          <t xml:space="preserve">LnCapCASPEX no select</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -36713,7 +36728,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -36734,7 +36749,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select</t>
+          <t xml:space="preserve">LnCapCASPEX no select C</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -36765,17 +36780,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select C</t>
+          <t xml:space="preserve">LuCap (m1) no sort</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -36796,12 +36811,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap (m1) no sort</t>
-        </is>
-      </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">MDA-MB g1.1 p10</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -36811,7 +36821,7 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1.1</t>
         </is>
       </c>
       <c r="E146">
@@ -36827,7 +36837,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t xml:space="preserve">MDA-MB g1.1 p10</t>
+          <t xml:space="preserve">MDA-MB gNT</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -36837,7 +36847,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1.1</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E147">
@@ -36853,33 +36863,23 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t xml:space="preserve">MDA-MB gNT</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="D148" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">Hek caspex</t>
         </is>
       </c>
       <c r="E148">
+        <v>0</v>
+      </c>
+      <c r="F148">
         <v>1</v>
       </c>
-      <c r="F148">
+      <c r="G148">
         <v>0</v>
-      </c>
-      <c r="G148">
-        <v>1</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">deneme</t>
         </is>
       </c>
       <c r="E149">
@@ -36895,14 +36895,14 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="E150">
         <v>0</v>
       </c>
       <c r="F150">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G150">
         <v>0</v>
@@ -36911,14 +36911,14 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">khk</t>
         </is>
       </c>
       <c r="E151">
         <v>0</v>
       </c>
       <c r="F151">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G151">
         <v>0</v>
@@ -36927,14 +36927,24 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E152">
         <v>0</v>
       </c>
       <c r="F152">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G152">
         <v>0</v>
@@ -36943,42 +36953,16 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="D153" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="E153">
         <v>0</v>
       </c>
       <c r="F153">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G153">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t xml:space="preserve">klm ox</t>
-        </is>
-      </c>
-      <c r="E154">
-        <v>0</v>
-      </c>
-      <c r="F154">
-        <v>1</v>
-      </c>
-      <c r="G154">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Edit LNCX from Umut
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -12330,12 +12330,12 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t xml:space="preserve">p12</t>
+          <t xml:space="preserve">p+12</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">

</xml_diff>

<commit_message>
Add 5 × Huh7 from Umut
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -31161,34 +31161,54 @@
       </c>
     </row>
     <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A1</t>
+        </is>
+      </c>
       <c r="E378" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="F378" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+21</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G378" t="inlineStr">
         <is>
-          <t xml:space="preserve">relative</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H378" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-05-15</t>
+          <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
       <c r="I378" t="inlineStr">
         <is>
-          <t xml:space="preserve">15-05-26</t>
+          <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
       <c r="K378" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L378" t="inlineStr">
@@ -31203,7 +31223,7 @@
       </c>
       <c r="N378" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">No Casp</t>
         </is>
       </c>
       <c r="O378" t="inlineStr">
@@ -31213,24 +31233,44 @@
       </c>
       <c r="R378" t="inlineStr">
         <is>
-          <t xml:space="preserve">withdrawn</t>
+          <t xml:space="preserve">stored</t>
         </is>
       </c>
       <c r="S378" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-199</t>
+          <t xml:space="preserve">v-mupot2zh-0</t>
         </is>
       </c>
     </row>
     <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A2</t>
+        </is>
+      </c>
       <c r="E379" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="F379" t="inlineStr">
         <is>
-          <t xml:space="preserve">p19</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G379" t="inlineStr">
@@ -31240,17 +31280,17 @@
       </c>
       <c r="H379" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-07-31</t>
+          <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
       <c r="I379" t="inlineStr">
         <is>
-          <t xml:space="preserve">31-07-26</t>
+          <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
       <c r="K379" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L379" t="inlineStr">
@@ -31260,12 +31300,12 @@
       </c>
       <c r="M379" t="inlineStr">
         <is>
-          <t xml:space="preserve">CR</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N379" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">No Casp</t>
         </is>
       </c>
       <c r="O379" t="inlineStr">
@@ -31273,56 +31313,66 @@
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
-      <c r="P379" t="inlineStr">
-        <is>
-          <t xml:space="preserve">to-do</t>
-        </is>
-      </c>
-      <c r="Q379" t="inlineStr">
-        <is>
-          <t xml:space="preserve">to-do box / thaw</t>
-        </is>
-      </c>
       <c r="R379" t="inlineStr">
         <is>
-          <t xml:space="preserve">withdrawn</t>
+          <t xml:space="preserve">stored</t>
         </is>
       </c>
       <c r="S379" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-233</t>
+          <t xml:space="preserve">v-mupot2zh-1</t>
         </is>
       </c>
     </row>
     <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A3</t>
+        </is>
+      </c>
       <c r="E380" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="F380" t="inlineStr">
         <is>
-          <t xml:space="preserve">p?</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G380" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H380" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-06-30</t>
+          <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
       <c r="I380" t="inlineStr">
         <is>
-          <t xml:space="preserve">30-06-25</t>
+          <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
       <c r="K380" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L380" t="inlineStr">
@@ -31347,24 +31397,44 @@
       </c>
       <c r="R380" t="inlineStr">
         <is>
-          <t xml:space="preserve">withdrawn</t>
+          <t xml:space="preserve">stored</t>
         </is>
       </c>
       <c r="S380" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-295</t>
+          <t xml:space="preserve">v-mupot2zh-2</t>
         </is>
       </c>
     </row>
     <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A4</t>
+        </is>
+      </c>
       <c r="E381" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="F381" t="inlineStr">
         <is>
-          <t xml:space="preserve">p11</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G381" t="inlineStr">
@@ -31374,17 +31444,17 @@
       </c>
       <c r="H381" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-06-12</t>
+          <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
       <c r="I381" t="inlineStr">
         <is>
-          <t xml:space="preserve">12/6/2026</t>
+          <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
       <c r="K381" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L381" t="inlineStr">
@@ -31394,7 +31464,7 @@
       </c>
       <c r="M381" t="inlineStr">
         <is>
-          <t xml:space="preserve">CR</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N381" t="inlineStr">
@@ -31409,44 +31479,64 @@
       </c>
       <c r="R381" t="inlineStr">
         <is>
-          <t xml:space="preserve">withdrawn</t>
+          <t xml:space="preserve">stored</t>
         </is>
       </c>
       <c r="S381" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-311</t>
+          <t xml:space="preserve">v-mupot2zh-3</t>
         </is>
       </c>
     </row>
     <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A5</t>
+        </is>
+      </c>
       <c r="E382" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="F382" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+17</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G382" t="inlineStr">
         <is>
-          <t xml:space="preserve">relative</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H382" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-03-30</t>
+          <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
       <c r="I382" t="inlineStr">
         <is>
-          <t xml:space="preserve">30-03-26</t>
+          <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
       <c r="K382" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L382" t="inlineStr">
@@ -31461,7 +31551,7 @@
       </c>
       <c r="N382" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">No Casp</t>
         </is>
       </c>
       <c r="O382" t="inlineStr">
@@ -31471,24 +31561,24 @@
       </c>
       <c r="R382" t="inlineStr">
         <is>
-          <t xml:space="preserve">withdrawn</t>
+          <t xml:space="preserve">stored</t>
         </is>
       </c>
       <c r="S382" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-320</t>
+          <t xml:space="preserve">v-mupot2zh-4</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="E383" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F383" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+14</t>
+          <t xml:space="preserve">p+21</t>
         </is>
       </c>
       <c r="G383" t="inlineStr">
@@ -31498,12 +31588,12 @@
       </c>
       <c r="H383" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-03-23</t>
+          <t xml:space="preserve">2026-05-15</t>
         </is>
       </c>
       <c r="I383" t="inlineStr">
         <is>
-          <t xml:space="preserve">23-03-26</t>
+          <t xml:space="preserve">15-05-26</t>
         </is>
       </c>
       <c r="K383" t="inlineStr">
@@ -31523,7 +31613,7 @@
       </c>
       <c r="N383" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O383" t="inlineStr">
@@ -31538,19 +31628,19 @@
       </c>
       <c r="S383" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-321</t>
+          <t xml:space="preserve">v-199</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="E384" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LUCX</t>
         </is>
       </c>
       <c r="F384" t="inlineStr">
         <is>
-          <t xml:space="preserve">p16</t>
+          <t xml:space="preserve">p19</t>
         </is>
       </c>
       <c r="G384" t="inlineStr">
@@ -31560,17 +31650,17 @@
       </c>
       <c r="H384" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-11-06</t>
+          <t xml:space="preserve">2026-07-31</t>
         </is>
       </c>
       <c r="I384" t="inlineStr">
         <is>
-          <t xml:space="preserve">6/11/2025</t>
+          <t xml:space="preserve">31-07-26</t>
         </is>
       </c>
       <c r="K384" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L384" t="inlineStr">
@@ -31580,12 +31670,12 @@
       </c>
       <c r="M384" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N384" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O384" t="inlineStr">
@@ -31593,6 +31683,16 @@
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
+      <c r="P384" t="inlineStr">
+        <is>
+          <t xml:space="preserve">to-do</t>
+        </is>
+      </c>
+      <c r="Q384" t="inlineStr">
+        <is>
+          <t xml:space="preserve">to-do box / thaw</t>
+        </is>
+      </c>
       <c r="R384" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
@@ -31600,39 +31700,39 @@
       </c>
       <c r="S384" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-338</t>
+          <t xml:space="preserve">v-233</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="E385" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="F385" t="inlineStr">
         <is>
-          <t xml:space="preserve">p15</t>
+          <t xml:space="preserve">p?</t>
         </is>
       </c>
       <c r="G385" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H385" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-10</t>
+          <t xml:space="preserve">2025-06-30</t>
         </is>
       </c>
       <c r="I385" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/8/2026</t>
+          <t xml:space="preserve">30-06-25</t>
         </is>
       </c>
       <c r="K385" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="L385" t="inlineStr">
@@ -31662,19 +31762,19 @@
       </c>
       <c r="S385" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-354</t>
+          <t xml:space="preserve">v-295</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="E386" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="F386" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p11</t>
         </is>
       </c>
       <c r="G386" t="inlineStr">
@@ -31684,17 +31784,17 @@
       </c>
       <c r="H386" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-06-12</t>
         </is>
       </c>
       <c r="I386" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">12/6/2026</t>
         </is>
       </c>
       <c r="K386" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L386" t="inlineStr">
@@ -31704,7 +31804,7 @@
       </c>
       <c r="M386" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N386" t="inlineStr">
@@ -31714,7 +31814,7 @@
       </c>
       <c r="O386" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R386" t="inlineStr">
@@ -31724,44 +31824,44 @@
       </c>
       <c r="S386" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdx0po-0</t>
+          <t xml:space="preserve">v-311</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="E387" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F387" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p+17</t>
         </is>
       </c>
       <c r="G387" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H387" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-03-30</t>
         </is>
       </c>
       <c r="I387" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">30-03-26</t>
         </is>
       </c>
       <c r="K387" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L387" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M387" t="inlineStr">
@@ -31771,7 +31871,7 @@
       </c>
       <c r="N387" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O387" t="inlineStr">
@@ -31786,44 +31886,44 @@
       </c>
       <c r="S387" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdxsum-0</t>
+          <t xml:space="preserve">v-320</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="E388" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">LnCap Canada</t>
         </is>
       </c>
       <c r="F388" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p+14</t>
         </is>
       </c>
       <c r="G388" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H388" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-03-23</t>
         </is>
       </c>
       <c r="I388" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">23-03-26</t>
         </is>
       </c>
       <c r="K388" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L388" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M388" t="inlineStr">
@@ -31848,19 +31948,19 @@
       </c>
       <c r="S388" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-0</t>
+          <t xml:space="preserve">v-321</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="E389" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="F389" t="inlineStr">
         <is>
-          <t xml:space="preserve">p28</t>
+          <t xml:space="preserve">p16</t>
         </is>
       </c>
       <c r="G389" t="inlineStr">
@@ -31870,12 +31970,12 @@
       </c>
       <c r="H389" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2025-11-06</t>
         </is>
       </c>
       <c r="I389" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">6/11/2025</t>
         </is>
       </c>
       <c r="K389" t="inlineStr">
@@ -31885,7 +31985,7 @@
       </c>
       <c r="L389" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M389" t="inlineStr">
@@ -31910,19 +32010,19 @@
       </c>
       <c r="S389" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdz1vx-0</t>
+          <t xml:space="preserve">v-338</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="E390" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="F390" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p15</t>
         </is>
       </c>
       <c r="G390" t="inlineStr">
@@ -31932,12 +32032,12 @@
       </c>
       <c r="H390" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-08-10</t>
         </is>
       </c>
       <c r="I390" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">10/8/2026</t>
         </is>
       </c>
       <c r="K390" t="inlineStr">
@@ -31962,7 +32062,7 @@
       </c>
       <c r="O390" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R390" t="inlineStr">
@@ -31972,19 +32072,19 @@
       </c>
       <c r="S390" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdzpx7-0</t>
+          <t xml:space="preserve">v-354</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="E391" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G391" t="inlineStr">
@@ -32004,12 +32104,12 @@
       </c>
       <c r="K391" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L391" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M391" t="inlineStr">
@@ -32024,7 +32124,7 @@
       </c>
       <c r="O391" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R391" t="inlineStr">
@@ -32034,19 +32134,19 @@
       </c>
       <c r="S391" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0daw-0</t>
+          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="E392" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="F392" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G392" t="inlineStr">
@@ -32066,12 +32166,12 @@
       </c>
       <c r="K392" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L392" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M392" t="inlineStr">
@@ -32096,19 +32196,19 @@
       </c>
       <c r="S392" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0w3q-0</t>
+          <t xml:space="preserve">v-mtrdxsum-0</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="E393" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="F393" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G393" t="inlineStr">
@@ -32128,12 +32228,12 @@
       </c>
       <c r="K393" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L393" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M393" t="inlineStr">
@@ -32158,19 +32258,19 @@
       </c>
       <c r="S393" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre1ko0-0</t>
+          <t xml:space="preserve">v-mtrdyhss-0</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="E394" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="F394" t="inlineStr">
         <is>
-          <t xml:space="preserve">p6</t>
+          <t xml:space="preserve">p28</t>
         </is>
       </c>
       <c r="G394" t="inlineStr">
@@ -32180,12 +32280,12 @@
       </c>
       <c r="H394" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I394" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="K394" t="inlineStr">
@@ -32195,7 +32295,7 @@
       </c>
       <c r="L394" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M394" t="inlineStr">
@@ -32205,7 +32305,7 @@
       </c>
       <c r="N394" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">No Casp</t>
         </is>
       </c>
       <c r="O394" t="inlineStr">
@@ -32220,34 +32320,44 @@
       </c>
       <c r="S394" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtski3re-0</t>
+          <t xml:space="preserve">v-mtrdz1vx-0</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="E395" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">Huh7 gNT</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G395" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H395" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I395" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K395" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L395" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M395" t="inlineStr">
@@ -32262,7 +32372,7 @@
       </c>
       <c r="O395" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R395" t="inlineStr">
@@ -32272,34 +32382,44 @@
       </c>
       <c r="S395" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt0h140-0</t>
+          <t xml:space="preserve">v-mtrdzpx7-0</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="E396" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G396" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H396" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I396" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L396" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M396" t="inlineStr">
@@ -32324,34 +32444,44 @@
       </c>
       <c r="S396" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-0</t>
+          <t xml:space="preserve">v-mtre0daw-0</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="E397" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G397" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H397" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I397" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L397" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M397" t="inlineStr">
@@ -32376,34 +32506,44 @@
       </c>
       <c r="S397" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtre0w3q-0</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="E398" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G398" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H398" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I398" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K398" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L398" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M398" t="inlineStr">
@@ -32428,19 +32568,24 @@
       </c>
       <c r="S398" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-2</t>
+          <t xml:space="preserve">v-mtre1ko0-0</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="E399" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">Hek caspex</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p6</t>
         </is>
       </c>
       <c r="G399" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H399" t="inlineStr">
@@ -32453,6 +32598,11 @@
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
+      <c r="K399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
       <c r="L399" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -32465,7 +32615,7 @@
       </c>
       <c r="N399" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O399" t="inlineStr">
@@ -32480,14 +32630,14 @@
       </c>
       <c r="S399" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt5ckqo-0</t>
+          <t xml:space="preserve">v-mtski3re-0</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="E400" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="G400" t="inlineStr">
@@ -32497,17 +32647,17 @@
       </c>
       <c r="H400" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I400" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="L400" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M400" t="inlineStr">
@@ -32532,14 +32682,14 @@
       </c>
       <c r="S400" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmw7m-0</t>
+          <t xml:space="preserve">v-mtt0h140-0</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="E401" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="G401" t="inlineStr">
@@ -32549,12 +32699,12 @@
       </c>
       <c r="H401" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I401" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="L401" t="inlineStr">
@@ -32584,14 +32734,14 @@
       </c>
       <c r="S401" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmypa-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="E402" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="G402" t="inlineStr">
@@ -32601,12 +32751,12 @@
       </c>
       <c r="H402" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I402" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="L402" t="inlineStr">
@@ -32636,62 +32786,322 @@
       </c>
       <c r="S402" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmn045-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="E403" t="inlineStr">
         <is>
+          <t xml:space="preserve">jkl</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt3mo6u-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="E404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">khk</t>
+        </is>
+      </c>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt5ckqo-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="E405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mttmmw7m-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="E406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mttmmypa-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="E407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mttmn045-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="E408" t="inlineStr">
+        <is>
           <t xml:space="preserve">deneme</t>
         </is>
       </c>
-      <c r="G403" t="inlineStr">
+      <c r="G408" t="inlineStr">
         <is>
           <t xml:space="preserve">unknown</t>
         </is>
       </c>
-      <c r="H403" t="inlineStr">
+      <c r="H408" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
-      <c r="I403" t="inlineStr">
+      <c r="I408" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
-      <c r="K403" t="inlineStr">
+      <c r="K408" t="inlineStr">
         <is>
           <t xml:space="preserve">deneme</t>
         </is>
       </c>
-      <c r="L403" t="inlineStr">
+      <c r="L408" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
         </is>
       </c>
-      <c r="M403" t="inlineStr">
+      <c r="M408" t="inlineStr">
         <is>
           <t xml:space="preserve">Par</t>
         </is>
       </c>
-      <c r="N403" t="inlineStr">
+      <c r="N408" t="inlineStr">
         <is>
           <t xml:space="preserve">No Casp</t>
         </is>
       </c>
-      <c r="O403" t="inlineStr">
+      <c r="O408" t="inlineStr">
         <is>
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
-      <c r="R403" t="inlineStr">
+      <c r="R408" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
-      <c r="S403" t="inlineStr">
+      <c r="S408" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mtu5lgdc-0</t>
         </is>
@@ -32837,12 +33247,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -32856,24 +33266,24 @@
         </is>
       </c>
       <c r="E5">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -32887,7 +33297,7 @@
         </is>
       </c>
       <c r="E6">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F6">
         <v>1</v>
@@ -32899,12 +33309,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -32921,7 +33331,7 @@
         <v>10</v>
       </c>
       <c r="F7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G7">
         <v>3</v>
@@ -32930,12 +33340,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B-GFP</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -32949,38 +33359,38 @@
         </is>
       </c>
       <c r="E8">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G8">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g5.1</t>
+          <t xml:space="preserve">HEK ATP7B-GFP</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">g5.1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F9">
         <v>0</v>
@@ -32992,32 +33402,32 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">DuDtxR CASPEX g5.1</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g5.1</t>
         </is>
       </c>
       <c r="E10">
         <v>8</v>
       </c>
       <c r="F10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -40254,10 +40664,10 @@
         <v>81</v>
       </c>
       <c r="I18">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J18">
-        <v>81</v>
+        <v>76</v>
       </c>
     </row>
     <row r="19">

</xml_diff>

<commit_message>
Add 9 × LNCX gNT from Umut
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -31004,12 +31004,12 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D376" t="inlineStr">
@@ -31019,32 +31019,32 @@
       </c>
       <c r="E376" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LNCX gNT</t>
         </is>
       </c>
       <c r="F376" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p+27</t>
         </is>
       </c>
       <c r="G376" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H376" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="I376" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="K376" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L376" t="inlineStr">
@@ -31059,12 +31059,12 @@
       </c>
       <c r="N376" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O376" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R376" t="inlineStr">
@@ -31074,7 +31074,7 @@
       </c>
       <c r="S376" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-0</t>
+          <t xml:space="preserve">v-mv4yctrb-0</t>
         </is>
       </c>
     </row>
@@ -31086,12 +31086,12 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D377" t="inlineStr">
@@ -31101,32 +31101,32 @@
       </c>
       <c r="E377" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LNCX gNT</t>
         </is>
       </c>
       <c r="F377" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p+27</t>
         </is>
       </c>
       <c r="G377" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H377" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="I377" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="K377" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L377" t="inlineStr">
@@ -31141,12 +31141,12 @@
       </c>
       <c r="N377" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O377" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R377" t="inlineStr">
@@ -31156,7 +31156,7 @@
       </c>
       <c r="S377" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-1</t>
+          <t xml:space="preserve">v-mv4yctrb-1</t>
         </is>
       </c>
     </row>
@@ -31168,12 +31168,12 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D378" t="inlineStr">
@@ -31183,32 +31183,32 @@
       </c>
       <c r="E378" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LNCX gNT</t>
         </is>
       </c>
       <c r="F378" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p+27</t>
         </is>
       </c>
       <c r="G378" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H378" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="I378" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="K378" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L378" t="inlineStr">
@@ -31223,12 +31223,12 @@
       </c>
       <c r="N378" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O378" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R378" t="inlineStr">
@@ -31238,7 +31238,7 @@
       </c>
       <c r="S378" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-2</t>
+          <t xml:space="preserve">v-mv4yctrb-2</t>
         </is>
       </c>
     </row>
@@ -31250,12 +31250,12 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D379" t="inlineStr">
@@ -31265,32 +31265,32 @@
       </c>
       <c r="E379" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LNCX gNT</t>
         </is>
       </c>
       <c r="F379" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p+27</t>
         </is>
       </c>
       <c r="G379" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H379" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="I379" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="K379" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L379" t="inlineStr">
@@ -31305,12 +31305,12 @@
       </c>
       <c r="N379" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O379" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R379" t="inlineStr">
@@ -31320,7 +31320,7 @@
       </c>
       <c r="S379" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-3</t>
+          <t xml:space="preserve">v-mv4yctrb-3</t>
         </is>
       </c>
     </row>
@@ -31332,682 +31332,852 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A5</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LNCX gNT</t>
+        </is>
+      </c>
+      <c r="F380" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p+27</t>
+        </is>
+      </c>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t xml:space="preserve">relative</t>
+        </is>
+      </c>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="I380" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="K380" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="L380" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M380" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N380" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASPEX</t>
+        </is>
+      </c>
+      <c r="O380" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gNT</t>
+        </is>
+      </c>
+      <c r="R380" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S380" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv4yctrb-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A6</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LNCX gNT</t>
+        </is>
+      </c>
+      <c r="F381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p+27</t>
+        </is>
+      </c>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">relative</t>
+        </is>
+      </c>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="I381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="K381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="L381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASPEX</t>
+        </is>
+      </c>
+      <c r="O381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gNT</t>
+        </is>
+      </c>
+      <c r="R381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S381" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv4yctrb-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A7</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LNCX gNT</t>
+        </is>
+      </c>
+      <c r="F382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p+27</t>
+        </is>
+      </c>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">relative</t>
+        </is>
+      </c>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="I382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="K382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="L382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASPEX</t>
+        </is>
+      </c>
+      <c r="O382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gNT</t>
+        </is>
+      </c>
+      <c r="R382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S382" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv4yctrb-6</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A8</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LNCX gNT</t>
+        </is>
+      </c>
+      <c r="F383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p+27</t>
+        </is>
+      </c>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">relative</t>
+        </is>
+      </c>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="I383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="K383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="L383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASPEX</t>
+        </is>
+      </c>
+      <c r="O383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gNT</t>
+        </is>
+      </c>
+      <c r="R383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S383" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv4yctrb-7</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A9</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LNCX gNT</t>
+        </is>
+      </c>
+      <c r="F384" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p+27</t>
+        </is>
+      </c>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t xml:space="preserve">relative</t>
+        </is>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="I384" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="K384" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="L384" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M384" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N384" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASPEX</t>
+        </is>
+      </c>
+      <c r="O384" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gNT</t>
+        </is>
+      </c>
+      <c r="R384" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S384" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv4yctrb-8</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
           <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
-      <c r="C380" t="inlineStr">
+      <c r="C385" t="inlineStr">
         <is>
           <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
-      <c r="D380" t="inlineStr">
+      <c r="D385" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A1</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F385" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H385" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I385" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K385" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L385" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M385" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N385" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O385" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R385" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S385" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A2</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F386" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H386" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I386" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K386" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L386" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M386" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N386" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O386" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R386" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S386" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A3</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F387" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H387" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I387" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K387" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L387" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M387" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N387" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O387" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R387" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S387" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A4</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F388" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H388" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I388" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K388" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L388" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M388" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N388" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O388" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R388" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S388" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
         <is>
           <t xml:space="preserve">A5</t>
         </is>
       </c>
-      <c r="E380" t="inlineStr">
+      <c r="E389" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="F380" t="inlineStr">
+      <c r="F389" t="inlineStr">
         <is>
           <t xml:space="preserve">p18</t>
         </is>
       </c>
-      <c r="G380" t="inlineStr">
+      <c r="G389" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H380" t="inlineStr">
+      <c r="H389" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
-      <c r="I380" t="inlineStr">
+      <c r="I389" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
-      <c r="K380" t="inlineStr">
+      <c r="K389" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L380" t="inlineStr">
+      <c r="L389" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
         </is>
       </c>
-      <c r="M380" t="inlineStr">
+      <c r="M389" t="inlineStr">
         <is>
           <t xml:space="preserve">Par</t>
         </is>
       </c>
-      <c r="N380" t="inlineStr">
+      <c r="N389" t="inlineStr">
         <is>
           <t xml:space="preserve">No Casp</t>
         </is>
       </c>
-      <c r="O380" t="inlineStr">
+      <c r="O389" t="inlineStr">
         <is>
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
-      <c r="R380" t="inlineStr">
+      <c r="R389" t="inlineStr">
         <is>
           <t xml:space="preserve">stored</t>
         </is>
       </c>
-      <c r="S380" t="inlineStr">
+      <c r="S389" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mupot2zh-4</t>
-        </is>
-      </c>
-    </row>
-    <row r="381">
-      <c r="E381" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNCX</t>
-        </is>
-      </c>
-      <c r="F381" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p+21</t>
-        </is>
-      </c>
-      <c r="G381" t="inlineStr">
-        <is>
-          <t xml:space="preserve">relative</t>
-        </is>
-      </c>
-      <c r="H381" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-05-15</t>
-        </is>
-      </c>
-      <c r="I381" t="inlineStr">
-        <is>
-          <t xml:space="preserve">15-05-26</t>
-        </is>
-      </c>
-      <c r="K381" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="L381" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M381" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N381" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CASPEX</t>
-        </is>
-      </c>
-      <c r="O381" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R381" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S381" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-199</t>
-        </is>
-      </c>
-    </row>
-    <row r="382">
-      <c r="E382" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LUCX</t>
-        </is>
-      </c>
-      <c r="F382" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p19</t>
-        </is>
-      </c>
-      <c r="G382" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H382" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-07-31</t>
-        </is>
-      </c>
-      <c r="I382" t="inlineStr">
-        <is>
-          <t xml:space="preserve">31-07-26</t>
-        </is>
-      </c>
-      <c r="K382" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR</t>
-        </is>
-      </c>
-      <c r="L382" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M382" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CR</t>
-        </is>
-      </c>
-      <c r="N382" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CASPEX</t>
-        </is>
-      </c>
-      <c r="O382" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="P382" t="inlineStr">
-        <is>
-          <t xml:space="preserve">to-do</t>
-        </is>
-      </c>
-      <c r="Q382" t="inlineStr">
-        <is>
-          <t xml:space="preserve">to-do box / thaw</t>
-        </is>
-      </c>
-      <c r="R382" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S382" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-233</t>
-        </is>
-      </c>
-    </row>
-    <row r="383">
-      <c r="E383" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145</t>
-        </is>
-      </c>
-      <c r="F383" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p?</t>
-        </is>
-      </c>
-      <c r="G383" t="inlineStr">
-        <is>
-          <t xml:space="preserve">unknown</t>
-        </is>
-      </c>
-      <c r="H383" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-06-30</t>
-        </is>
-      </c>
-      <c r="I383" t="inlineStr">
-        <is>
-          <t xml:space="preserve">30-06-25</t>
-        </is>
-      </c>
-      <c r="K383" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145</t>
-        </is>
-      </c>
-      <c r="L383" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M383" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N383" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O383" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R383" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S383" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-295</t>
-        </is>
-      </c>
-    </row>
-    <row r="384">
-      <c r="E384" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR</t>
-        </is>
-      </c>
-      <c r="F384" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p11</t>
-        </is>
-      </c>
-      <c r="G384" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H384" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-12</t>
-        </is>
-      </c>
-      <c r="I384" t="inlineStr">
-        <is>
-          <t xml:space="preserve">12/6/2026</t>
-        </is>
-      </c>
-      <c r="K384" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR</t>
-        </is>
-      </c>
-      <c r="L384" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M384" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CR</t>
-        </is>
-      </c>
-      <c r="N384" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O384" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R384" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S384" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-311</t>
-        </is>
-      </c>
-    </row>
-    <row r="385">
-      <c r="E385" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNCX</t>
-        </is>
-      </c>
-      <c r="F385" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p+17</t>
-        </is>
-      </c>
-      <c r="G385" t="inlineStr">
-        <is>
-          <t xml:space="preserve">relative</t>
-        </is>
-      </c>
-      <c r="H385" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-03-30</t>
-        </is>
-      </c>
-      <c r="I385" t="inlineStr">
-        <is>
-          <t xml:space="preserve">30-03-26</t>
-        </is>
-      </c>
-      <c r="K385" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="L385" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M385" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N385" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CASPEX</t>
-        </is>
-      </c>
-      <c r="O385" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R385" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S385" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-320</t>
-        </is>
-      </c>
-    </row>
-    <row r="386">
-      <c r="E386" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap Canada</t>
-        </is>
-      </c>
-      <c r="F386" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p+14</t>
-        </is>
-      </c>
-      <c r="G386" t="inlineStr">
-        <is>
-          <t xml:space="preserve">relative</t>
-        </is>
-      </c>
-      <c r="H386" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-03-23</t>
-        </is>
-      </c>
-      <c r="I386" t="inlineStr">
-        <is>
-          <t xml:space="preserve">23-03-26</t>
-        </is>
-      </c>
-      <c r="K386" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="L386" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M386" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N386" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O386" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R386" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S386" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-321</t>
-        </is>
-      </c>
-    </row>
-    <row r="387">
-      <c r="E387" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
-      <c r="F387" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p16</t>
-        </is>
-      </c>
-      <c r="G387" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H387" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-11-06</t>
-        </is>
-      </c>
-      <c r="I387" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6/11/2025</t>
-        </is>
-      </c>
-      <c r="K387" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
-      <c r="L387" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M387" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N387" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O387" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R387" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S387" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-338</t>
-        </is>
-      </c>
-    </row>
-    <row r="388">
-      <c r="E388" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7</t>
-        </is>
-      </c>
-      <c r="F388" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p15</t>
-        </is>
-      </c>
-      <c r="G388" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H388" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-08-10</t>
-        </is>
-      </c>
-      <c r="I388" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10/8/2026</t>
-        </is>
-      </c>
-      <c r="K388" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7</t>
-        </is>
-      </c>
-      <c r="L388" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M388" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N388" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O388" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R388" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S388" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-354</t>
-        </is>
-      </c>
-    </row>
-    <row r="389">
-      <c r="E389" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK gNT</t>
-        </is>
-      </c>
-      <c r="F389" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p21</t>
-        </is>
-      </c>
-      <c r="G389" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H389" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-07</t>
-        </is>
-      </c>
-      <c r="I389" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-07</t>
-        </is>
-      </c>
-      <c r="K389" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
-      <c r="L389" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M389" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N389" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O389" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gNT</t>
-        </is>
-      </c>
-      <c r="R389" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S389" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="E390" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F390" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p+21</t>
         </is>
       </c>
       <c r="G390" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H390" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-05-15</t>
         </is>
       </c>
       <c r="I390" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">15-05-26</t>
         </is>
       </c>
       <c r="K390" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L390" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M390" t="inlineStr">
@@ -32017,7 +32187,7 @@
       </c>
       <c r="N390" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O390" t="inlineStr">
@@ -32032,19 +32202,19 @@
       </c>
       <c r="S390" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdxsum-0</t>
+          <t xml:space="preserve">v-199</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="E391" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">LUCX</t>
         </is>
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p19</t>
         </is>
       </c>
       <c r="G391" t="inlineStr">
@@ -32054,32 +32224,32 @@
       </c>
       <c r="H391" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-07-31</t>
         </is>
       </c>
       <c r="I391" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">31-07-26</t>
         </is>
       </c>
       <c r="K391" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L391" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M391" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N391" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O391" t="inlineStr">
@@ -32087,6 +32257,16 @@
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
+      <c r="P391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">to-do</t>
+        </is>
+      </c>
+      <c r="Q391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">to-do box / thaw</t>
+        </is>
+      </c>
       <c r="R391" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
@@ -32094,44 +32274,44 @@
       </c>
       <c r="S391" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-0</t>
+          <t xml:space="preserve">v-233</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="E392" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="F392" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p?</t>
         </is>
       </c>
       <c r="G392" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H392" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2025-06-30</t>
         </is>
       </c>
       <c r="I392" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">30-06-25</t>
         </is>
       </c>
       <c r="K392" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="L392" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M392" t="inlineStr">
@@ -32156,19 +32336,19 @@
       </c>
       <c r="S392" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-1</t>
+          <t xml:space="preserve">v-295</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="E393" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="F393" t="inlineStr">
         <is>
-          <t xml:space="preserve">p28</t>
+          <t xml:space="preserve">p11</t>
         </is>
       </c>
       <c r="G393" t="inlineStr">
@@ -32178,27 +32358,27 @@
       </c>
       <c r="H393" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-06-12</t>
         </is>
       </c>
       <c r="I393" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">12/6/2026</t>
         </is>
       </c>
       <c r="K393" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L393" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M393" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N393" t="inlineStr">
@@ -32218,39 +32398,39 @@
       </c>
       <c r="S393" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdz1vx-0</t>
+          <t xml:space="preserve">v-311</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="E394" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F394" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p+17</t>
         </is>
       </c>
       <c r="G394" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H394" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-03-30</t>
         </is>
       </c>
       <c r="I394" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">30-03-26</t>
         </is>
       </c>
       <c r="K394" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L394" t="inlineStr">
@@ -32265,12 +32445,12 @@
       </c>
       <c r="N394" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O394" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R394" t="inlineStr">
@@ -32280,44 +32460,44 @@
       </c>
       <c r="S394" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdzpx7-0</t>
+          <t xml:space="preserve">v-320</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="E395" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">LnCap Canada</t>
         </is>
       </c>
       <c r="F395" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p+14</t>
         </is>
       </c>
       <c r="G395" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H395" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-03-23</t>
         </is>
       </c>
       <c r="I395" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">23-03-26</t>
         </is>
       </c>
       <c r="K395" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L395" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M395" t="inlineStr">
@@ -32342,19 +32522,19 @@
       </c>
       <c r="S395" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0daw-0</t>
+          <t xml:space="preserve">v-321</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="E396" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="F396" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p16</t>
         </is>
       </c>
       <c r="G396" t="inlineStr">
@@ -32364,22 +32544,22 @@
       </c>
       <c r="H396" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2025-11-06</t>
         </is>
       </c>
       <c r="I396" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">6/11/2025</t>
         </is>
       </c>
       <c r="K396" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L396" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M396" t="inlineStr">
@@ -32404,19 +32584,19 @@
       </c>
       <c r="S396" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0w3q-0</t>
+          <t xml:space="preserve">v-338</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="E397" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="F397" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p15</t>
         </is>
       </c>
       <c r="G397" t="inlineStr">
@@ -32426,12 +32606,12 @@
       </c>
       <c r="H397" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-08-10</t>
         </is>
       </c>
       <c r="I397" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">10/8/2026</t>
         </is>
       </c>
       <c r="K397" t="inlineStr">
@@ -32441,7 +32621,7 @@
       </c>
       <c r="L397" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M397" t="inlineStr">
@@ -32466,19 +32646,19 @@
       </c>
       <c r="S397" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre1ko0-0</t>
+          <t xml:space="preserve">v-354</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="E398" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="F398" t="inlineStr">
         <is>
-          <t xml:space="preserve">p6</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G398" t="inlineStr">
@@ -32488,12 +32668,12 @@
       </c>
       <c r="H398" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I398" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="K398" t="inlineStr">
@@ -32513,12 +32693,12 @@
       </c>
       <c r="N398" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">No Casp</t>
         </is>
       </c>
       <c r="O398" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R398" t="inlineStr">
@@ -32528,34 +32708,44 @@
       </c>
       <c r="S398" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtski3re-0</t>
+          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="E399" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G399" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H399" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I399" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L399" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M399" t="inlineStr">
@@ -32580,34 +32770,44 @@
       </c>
       <c r="S399" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt0h140-0</t>
+          <t xml:space="preserve">v-mtrdxsum-0</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="E400" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G400" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H400" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I400" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K400" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L400" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M400" t="inlineStr">
@@ -32632,34 +32832,44 @@
       </c>
       <c r="S400" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-0</t>
+          <t xml:space="preserve">v-mtrdyhss-0</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="E401" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G401" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H401" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I401" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L401" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M401" t="inlineStr">
@@ -32684,34 +32894,44 @@
       </c>
       <c r="S401" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtrdyhss-1</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="E402" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p28</t>
         </is>
       </c>
       <c r="G402" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H402" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I402" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L402" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M402" t="inlineStr">
@@ -32736,29 +32956,39 @@
       </c>
       <c r="S402" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-2</t>
+          <t xml:space="preserve">v-mtrdz1vx-0</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="E403" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">Huh7 gNT</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G403" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H403" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I403" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L403" t="inlineStr">
@@ -32778,7 +33008,7 @@
       </c>
       <c r="O403" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R403" t="inlineStr">
@@ -32788,34 +33018,44 @@
       </c>
       <c r="S403" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt5ckqo-0</t>
+          <t xml:space="preserve">v-mtrdzpx7-0</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="E404" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G404" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H404" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I404" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L404" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M404" t="inlineStr">
@@ -32840,34 +33080,44 @@
       </c>
       <c r="S404" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmw7m-0</t>
+          <t xml:space="preserve">v-mtre0daw-0</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="E405" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G405" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H405" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I405" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L405" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M405" t="inlineStr">
@@ -32892,34 +33142,44 @@
       </c>
       <c r="S405" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmypa-0</t>
+          <t xml:space="preserve">v-mtre0w3q-0</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="E406" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G406" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H406" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I406" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L406" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M406" t="inlineStr">
@@ -32944,34 +33204,39 @@
       </c>
       <c r="S406" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmn045-0</t>
+          <t xml:space="preserve">v-mtre1ko0-0</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="E407" t="inlineStr">
         <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">Hek caspex</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p6</t>
         </is>
       </c>
       <c r="G407" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H407" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I407" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="K407" t="inlineStr">
         <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L407" t="inlineStr">
@@ -32986,7 +33251,7 @@
       </c>
       <c r="N407" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O407" t="inlineStr">
@@ -33001,67 +33266,540 @@
       </c>
       <c r="S407" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtu5lgdc-0</t>
+          <t xml:space="preserve">v-mtski3re-0</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="E408" t="inlineStr">
         <is>
+          <t xml:space="preserve">klm ox</t>
+        </is>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OX</t>
+        </is>
+      </c>
+      <c r="M408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt0h140-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="E409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jkl</t>
+        </is>
+      </c>
+      <c r="G409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="E410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jkl</t>
+        </is>
+      </c>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="E411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jkl</t>
+        </is>
+      </c>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt3mo6u-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="E412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">khk</t>
+        </is>
+      </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt5ckqo-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="E413" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H413" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I413" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L413" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M413" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N413" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O413" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R413" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S413" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mttmmw7m-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="E414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mttmmypa-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="E415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="G415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mttmn045-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="E416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deneme</t>
+        </is>
+      </c>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="K416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deneme</t>
+        </is>
+      </c>
+      <c r="L416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtu5lgdc-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="E417" t="inlineStr">
+        <is>
           <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
-      <c r="F408" t="inlineStr">
+      <c r="F417" t="inlineStr">
         <is>
           <t xml:space="preserve">p19</t>
         </is>
       </c>
-      <c r="G408" t="inlineStr">
+      <c r="G417" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H408" t="inlineStr">
+      <c r="H417" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-17</t>
         </is>
       </c>
-      <c r="I408" t="inlineStr">
+      <c r="I417" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-17</t>
         </is>
       </c>
-      <c r="K408" t="inlineStr">
+      <c r="K417" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L408" t="inlineStr">
+      <c r="L417" t="inlineStr">
         <is>
           <t xml:space="preserve">FLAG</t>
         </is>
       </c>
-      <c r="M408" t="inlineStr">
+      <c r="M417" t="inlineStr">
         <is>
           <t xml:space="preserve">Par</t>
         </is>
       </c>
-      <c r="N408" t="inlineStr">
+      <c r="N417" t="inlineStr">
         <is>
           <t xml:space="preserve">No Casp</t>
         </is>
       </c>
-      <c r="O408" t="inlineStr">
+      <c r="O417" t="inlineStr">
         <is>
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
-      <c r="R408" t="inlineStr">
+      <c r="R417" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
-      <c r="S408" t="inlineStr">
+      <c r="S417" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mu5anec8-0</t>
         </is>
@@ -33238,12 +33976,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LNCX gNT</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -33253,28 +33991,28 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E6">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -33288,7 +34026,7 @@
         </is>
       </c>
       <c r="E7">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F7">
         <v>1</v>
@@ -33300,12 +34038,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -33322,7 +34060,7 @@
         <v>10</v>
       </c>
       <c r="F8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G8">
         <v>3</v>
@@ -33331,12 +34069,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B-GFP</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -33350,38 +34088,38 @@
         </is>
       </c>
       <c r="E9">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F9">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G9">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g5.1</t>
+          <t xml:space="preserve">HEK ATP7B-GFP</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">g5.1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E10">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F10">
         <v>0</v>
@@ -33393,84 +34131,84 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX</t>
+          <t xml:space="preserve">DuDtxR CASPEX g5.1</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g5.1</t>
         </is>
       </c>
       <c r="E11">
         <v>8</v>
       </c>
       <c r="F11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX DSg1.2</t>
+          <t xml:space="preserve">LUCX</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">DSg1.2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E12">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B KO g3</t>
+          <t xml:space="preserve">DuDtxR CASPEX DSg1.2</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">g3</t>
+          <t xml:space="preserve">DSg1.2</t>
         </is>
       </c>
       <c r="E13">
@@ -33480,13 +34218,13 @@
         <v>0</v>
       </c>
       <c r="G13">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 KO g1</t>
+          <t xml:space="preserve">HEK ATP7B KO g3</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -33496,12 +34234,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">g3</t>
         </is>
       </c>
       <c r="E14">
@@ -33511,28 +34249,28 @@
         <v>0</v>
       </c>
       <c r="G14">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gP2</t>
+          <t xml:space="preserve">HEK HOXB6 KO g1</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">gP2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E15">
@@ -33542,44 +34280,44 @@
         <v>0</v>
       </c>
       <c r="G15">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g3</t>
+          <t xml:space="preserve">LNCX gP2</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">g3</t>
+          <t xml:space="preserve">gP2</t>
         </is>
       </c>
       <c r="E16">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F16">
         <v>0</v>
       </c>
       <c r="G16">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX gNT</t>
+          <t xml:space="preserve">DuDtxR CASPEX g3</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -33594,7 +34332,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">g3</t>
         </is>
       </c>
       <c r="E17">
@@ -33610,22 +34348,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G1</t>
+          <t xml:space="preserve">DuDtxR CASPEX gNT</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E18">
@@ -33635,23 +34373,23 @@
         <v>0</v>
       </c>
       <c r="G18">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO G1</t>
+          <t xml:space="preserve">LnCap Canada V1G1</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -33660,19 +34398,19 @@
         </is>
       </c>
       <c r="E19">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F19">
         <v>0</v>
       </c>
       <c r="G19">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK TOX4 OX</t>
+          <t xml:space="preserve">HEK CBX3 KO G1</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -33682,7 +34420,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -33697,13 +34435,13 @@
         <v>0</v>
       </c>
       <c r="G20">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
+          <t xml:space="preserve">HEK TOX4 OX</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -33713,33 +34451,33 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E21">
         <v>5</v>
       </c>
       <c r="F21">
+        <v>0</v>
+      </c>
+      <c r="G21">
         <v>1</v>
-      </c>
-      <c r="G21">
-        <v>3</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gP1</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -33749,28 +34487,28 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">gP1</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E22">
         <v>5</v>
       </c>
       <c r="F22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G22">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX gP1</t>
+          <t xml:space="preserve">LNCX gP1</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -33790,18 +34528,18 @@
         <v>0</v>
       </c>
       <c r="G23">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR+1</t>
+          <t xml:space="preserve">LUCX gP1</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -33811,28 +34549,28 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gP1</t>
         </is>
       </c>
       <c r="E24">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F24">
         <v>0</v>
       </c>
       <c r="G24">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">HepG2</t>
+          <t xml:space="preserve">DuPar50CR+1</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">HepG2</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -33852,18 +34590,18 @@
         <v>0</v>
       </c>
       <c r="G25">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gNT</t>
+          <t xml:space="preserve">HepG2</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">HepG2</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -33873,7 +34611,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E26">
@@ -33883,7 +34621,7 @@
         <v>0</v>
       </c>
       <c r="G26">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -40718,10 +41456,10 @@
         <v>81</v>
       </c>
       <c r="I18">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J18">
-        <v>81</v>
+        <v>72</v>
       </c>
     </row>
     <row r="19">

</xml_diff>

<commit_message>
Add 1 × Huh7 from Umut
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -31742,17 +31742,17 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D385" t="inlineStr">
         <is>
-          <t xml:space="preserve">A1</t>
+          <t xml:space="preserve">B1</t>
         </is>
       </c>
       <c r="E385" t="inlineStr">
@@ -31762,7 +31762,7 @@
       </c>
       <c r="F385" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">24</t>
         </is>
       </c>
       <c r="G385" t="inlineStr">
@@ -31772,12 +31772,12 @@
       </c>
       <c r="H385" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="I385" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="K385" t="inlineStr">
@@ -31812,7 +31812,7 @@
       </c>
       <c r="S385" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-0</t>
+          <t xml:space="preserve">v-mv4ydq8o-0</t>
         </is>
       </c>
     </row>
@@ -31834,7 +31834,7 @@
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t xml:space="preserve">A2</t>
+          <t xml:space="preserve">A1</t>
         </is>
       </c>
       <c r="E386" t="inlineStr">
@@ -31894,7 +31894,7 @@
       </c>
       <c r="S386" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-1</t>
+          <t xml:space="preserve">v-mupot2zh-0</t>
         </is>
       </c>
     </row>
@@ -31916,7 +31916,7 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t xml:space="preserve">A3</t>
+          <t xml:space="preserve">A2</t>
         </is>
       </c>
       <c r="E387" t="inlineStr">
@@ -31976,7 +31976,7 @@
       </c>
       <c r="S387" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-2</t>
+          <t xml:space="preserve">v-mupot2zh-1</t>
         </is>
       </c>
     </row>
@@ -31998,7 +31998,7 @@
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t xml:space="preserve">A4</t>
+          <t xml:space="preserve">A3</t>
         </is>
       </c>
       <c r="E388" t="inlineStr">
@@ -32058,7 +32058,7 @@
       </c>
       <c r="S388" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-3</t>
+          <t xml:space="preserve">v-mupot2zh-2</t>
         </is>
       </c>
     </row>
@@ -32080,161 +32080,181 @@
       </c>
       <c r="D389" t="inlineStr">
         <is>
+          <t xml:space="preserve">A4</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F389" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H389" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I389" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K389" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L389" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M389" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N389" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O389" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R389" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S389" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
           <t xml:space="preserve">A5</t>
         </is>
       </c>
-      <c r="E389" t="inlineStr">
+      <c r="E390" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="F389" t="inlineStr">
+      <c r="F390" t="inlineStr">
         <is>
           <t xml:space="preserve">p18</t>
         </is>
       </c>
-      <c r="G389" t="inlineStr">
+      <c r="G390" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H389" t="inlineStr">
+      <c r="H390" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
-      <c r="I389" t="inlineStr">
+      <c r="I390" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
-      <c r="K389" t="inlineStr">
+      <c r="K390" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L389" t="inlineStr">
+      <c r="L390" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
         </is>
       </c>
-      <c r="M389" t="inlineStr">
+      <c r="M390" t="inlineStr">
         <is>
           <t xml:space="preserve">Par</t>
         </is>
       </c>
-      <c r="N389" t="inlineStr">
+      <c r="N390" t="inlineStr">
         <is>
           <t xml:space="preserve">No Casp</t>
         </is>
       </c>
-      <c r="O389" t="inlineStr">
+      <c r="O390" t="inlineStr">
         <is>
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
-      <c r="R389" t="inlineStr">
+      <c r="R390" t="inlineStr">
         <is>
           <t xml:space="preserve">stored</t>
         </is>
       </c>
-      <c r="S389" t="inlineStr">
+      <c r="S390" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mupot2zh-4</t>
-        </is>
-      </c>
-    </row>
-    <row r="390">
-      <c r="E390" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNCX</t>
-        </is>
-      </c>
-      <c r="F390" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p+21</t>
-        </is>
-      </c>
-      <c r="G390" t="inlineStr">
-        <is>
-          <t xml:space="preserve">relative</t>
-        </is>
-      </c>
-      <c r="H390" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-05-15</t>
-        </is>
-      </c>
-      <c r="I390" t="inlineStr">
-        <is>
-          <t xml:space="preserve">15-05-26</t>
-        </is>
-      </c>
-      <c r="K390" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="L390" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M390" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N390" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CASPEX</t>
-        </is>
-      </c>
-      <c r="O390" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R390" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S390" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-199</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="E391" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t xml:space="preserve">p19</t>
+          <t xml:space="preserve">p+21</t>
         </is>
       </c>
       <c r="G391" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H391" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-07-31</t>
+          <t xml:space="preserve">2026-05-15</t>
         </is>
       </c>
       <c r="I391" t="inlineStr">
         <is>
-          <t xml:space="preserve">31-07-26</t>
+          <t xml:space="preserve">15-05-26</t>
         </is>
       </c>
       <c r="K391" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L391" t="inlineStr">
@@ -32244,7 +32264,7 @@
       </c>
       <c r="M391" t="inlineStr">
         <is>
-          <t xml:space="preserve">CR</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N391" t="inlineStr">
@@ -32257,16 +32277,6 @@
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
-      <c r="P391" t="inlineStr">
-        <is>
-          <t xml:space="preserve">to-do</t>
-        </is>
-      </c>
-      <c r="Q391" t="inlineStr">
-        <is>
-          <t xml:space="preserve">to-do box / thaw</t>
-        </is>
-      </c>
       <c r="R391" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
@@ -32274,39 +32284,39 @@
       </c>
       <c r="S391" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-233</t>
+          <t xml:space="preserve">v-199</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="E392" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">LUCX</t>
         </is>
       </c>
       <c r="F392" t="inlineStr">
         <is>
-          <t xml:space="preserve">p?</t>
+          <t xml:space="preserve">p19</t>
         </is>
       </c>
       <c r="G392" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H392" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-06-30</t>
+          <t xml:space="preserve">2026-07-31</t>
         </is>
       </c>
       <c r="I392" t="inlineStr">
         <is>
-          <t xml:space="preserve">30-06-25</t>
+          <t xml:space="preserve">31-07-26</t>
         </is>
       </c>
       <c r="K392" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L392" t="inlineStr">
@@ -32316,12 +32326,12 @@
       </c>
       <c r="M392" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N392" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O392" t="inlineStr">
@@ -32329,6 +32339,16 @@
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
+      <c r="P392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">to-do</t>
+        </is>
+      </c>
+      <c r="Q392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">to-do box / thaw</t>
+        </is>
+      </c>
       <c r="R392" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
@@ -32336,39 +32356,39 @@
       </c>
       <c r="S392" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-295</t>
+          <t xml:space="preserve">v-233</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="E393" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="F393" t="inlineStr">
         <is>
-          <t xml:space="preserve">p11</t>
+          <t xml:space="preserve">p?</t>
         </is>
       </c>
       <c r="G393" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H393" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-06-12</t>
+          <t xml:space="preserve">2025-06-30</t>
         </is>
       </c>
       <c r="I393" t="inlineStr">
         <is>
-          <t xml:space="preserve">12/6/2026</t>
+          <t xml:space="preserve">30-06-25</t>
         </is>
       </c>
       <c r="K393" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="L393" t="inlineStr">
@@ -32378,7 +32398,7 @@
       </c>
       <c r="M393" t="inlineStr">
         <is>
-          <t xml:space="preserve">CR</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N393" t="inlineStr">
@@ -32398,39 +32418,39 @@
       </c>
       <c r="S393" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-311</t>
+          <t xml:space="preserve">v-295</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="E394" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="F394" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+17</t>
+          <t xml:space="preserve">p11</t>
         </is>
       </c>
       <c r="G394" t="inlineStr">
         <is>
-          <t xml:space="preserve">relative</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H394" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-03-30</t>
+          <t xml:space="preserve">2026-06-12</t>
         </is>
       </c>
       <c r="I394" t="inlineStr">
         <is>
-          <t xml:space="preserve">30-03-26</t>
+          <t xml:space="preserve">12/6/2026</t>
         </is>
       </c>
       <c r="K394" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L394" t="inlineStr">
@@ -32440,12 +32460,12 @@
       </c>
       <c r="M394" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N394" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">No Casp</t>
         </is>
       </c>
       <c r="O394" t="inlineStr">
@@ -32460,19 +32480,19 @@
       </c>
       <c r="S394" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-320</t>
+          <t xml:space="preserve">v-311</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="E395" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F395" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+14</t>
+          <t xml:space="preserve">p+17</t>
         </is>
       </c>
       <c r="G395" t="inlineStr">
@@ -32482,12 +32502,12 @@
       </c>
       <c r="H395" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-03-23</t>
+          <t xml:space="preserve">2026-03-30</t>
         </is>
       </c>
       <c r="I395" t="inlineStr">
         <is>
-          <t xml:space="preserve">23-03-26</t>
+          <t xml:space="preserve">30-03-26</t>
         </is>
       </c>
       <c r="K395" t="inlineStr">
@@ -32507,7 +32527,7 @@
       </c>
       <c r="N395" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O395" t="inlineStr">
@@ -32522,39 +32542,39 @@
       </c>
       <c r="S395" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-321</t>
+          <t xml:space="preserve">v-320</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="E396" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap Canada</t>
         </is>
       </c>
       <c r="F396" t="inlineStr">
         <is>
-          <t xml:space="preserve">p16</t>
+          <t xml:space="preserve">p+14</t>
         </is>
       </c>
       <c r="G396" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H396" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-11-06</t>
+          <t xml:space="preserve">2026-03-23</t>
         </is>
       </c>
       <c r="I396" t="inlineStr">
         <is>
-          <t xml:space="preserve">6/11/2025</t>
+          <t xml:space="preserve">23-03-26</t>
         </is>
       </c>
       <c r="K396" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L396" t="inlineStr">
@@ -32584,19 +32604,19 @@
       </c>
       <c r="S396" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-338</t>
+          <t xml:space="preserve">v-321</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="E397" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="F397" t="inlineStr">
         <is>
-          <t xml:space="preserve">p15</t>
+          <t xml:space="preserve">p16</t>
         </is>
       </c>
       <c r="G397" t="inlineStr">
@@ -32606,17 +32626,17 @@
       </c>
       <c r="H397" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-10</t>
+          <t xml:space="preserve">2025-11-06</t>
         </is>
       </c>
       <c r="I397" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/8/2026</t>
+          <t xml:space="preserve">6/11/2025</t>
         </is>
       </c>
       <c r="K397" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L397" t="inlineStr">
@@ -32646,19 +32666,19 @@
       </c>
       <c r="S397" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-354</t>
+          <t xml:space="preserve">v-338</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="E398" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="F398" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p15</t>
         </is>
       </c>
       <c r="G398" t="inlineStr">
@@ -32668,17 +32688,17 @@
       </c>
       <c r="H398" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-08-10</t>
         </is>
       </c>
       <c r="I398" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">10/8/2026</t>
         </is>
       </c>
       <c r="K398" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L398" t="inlineStr">
@@ -32698,7 +32718,7 @@
       </c>
       <c r="O398" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R398" t="inlineStr">
@@ -32708,14 +32728,14 @@
       </c>
       <c r="S398" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdx0po-0</t>
+          <t xml:space="preserve">v-354</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="E399" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="F399" t="inlineStr">
@@ -32745,7 +32765,7 @@
       </c>
       <c r="L399" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M399" t="inlineStr">
@@ -32760,7 +32780,7 @@
       </c>
       <c r="O399" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R399" t="inlineStr">
@@ -32770,14 +32790,14 @@
       </c>
       <c r="S399" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdxsum-0</t>
+          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="E400" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="F400" t="inlineStr">
@@ -32807,7 +32827,7 @@
       </c>
       <c r="L400" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M400" t="inlineStr">
@@ -32832,7 +32852,7 @@
       </c>
       <c r="S400" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-0</t>
+          <t xml:space="preserve">v-mtrdxsum-0</t>
         </is>
       </c>
     </row>
@@ -32894,19 +32914,19 @@
       </c>
       <c r="S401" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-1</t>
+          <t xml:space="preserve">v-mtrdyhss-0</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="E402" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="F402" t="inlineStr">
         <is>
-          <t xml:space="preserve">p28</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G402" t="inlineStr">
@@ -32931,7 +32951,7 @@
       </c>
       <c r="L402" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M402" t="inlineStr">
@@ -32956,19 +32976,19 @@
       </c>
       <c r="S402" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdz1vx-0</t>
+          <t xml:space="preserve">v-mtrdyhss-1</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="E403" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="F403" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p28</t>
         </is>
       </c>
       <c r="G403" t="inlineStr">
@@ -32988,12 +33008,12 @@
       </c>
       <c r="K403" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L403" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M403" t="inlineStr">
@@ -33008,7 +33028,7 @@
       </c>
       <c r="O403" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R403" t="inlineStr">
@@ -33018,19 +33038,19 @@
       </c>
       <c r="S403" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdzpx7-0</t>
+          <t xml:space="preserve">v-mtrdz1vx-0</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="E404" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">Huh7 gNT</t>
         </is>
       </c>
       <c r="F404" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G404" t="inlineStr">
@@ -33055,7 +33075,7 @@
       </c>
       <c r="L404" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M404" t="inlineStr">
@@ -33070,7 +33090,7 @@
       </c>
       <c r="O404" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R404" t="inlineStr">
@@ -33080,19 +33100,19 @@
       </c>
       <c r="S404" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0daw-0</t>
+          <t xml:space="preserve">v-mtrdzpx7-0</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="E405" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="F405" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G405" t="inlineStr">
@@ -33117,7 +33137,7 @@
       </c>
       <c r="L405" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M405" t="inlineStr">
@@ -33142,19 +33162,19 @@
       </c>
       <c r="S405" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0w3q-0</t>
+          <t xml:space="preserve">v-mtre0daw-0</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="E406" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="F406" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G406" t="inlineStr">
@@ -33179,7 +33199,7 @@
       </c>
       <c r="L406" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M406" t="inlineStr">
@@ -33204,19 +33224,19 @@
       </c>
       <c r="S406" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre1ko0-0</t>
+          <t xml:space="preserve">v-mtre0w3q-0</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="E407" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="F407" t="inlineStr">
         <is>
-          <t xml:space="preserve">p6</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G407" t="inlineStr">
@@ -33226,22 +33246,22 @@
       </c>
       <c r="H407" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I407" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="K407" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L407" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M407" t="inlineStr">
@@ -33251,7 +33271,7 @@
       </c>
       <c r="N407" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">No Casp</t>
         </is>
       </c>
       <c r="O407" t="inlineStr">
@@ -33266,19 +33286,24 @@
       </c>
       <c r="S407" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtski3re-0</t>
+          <t xml:space="preserve">v-mtre1ko0-0</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="E408" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">Hek caspex</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p6</t>
         </is>
       </c>
       <c r="G408" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H408" t="inlineStr">
@@ -33291,9 +33316,14 @@
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
+      <c r="K408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
       <c r="L408" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M408" t="inlineStr">
@@ -33303,7 +33333,7 @@
       </c>
       <c r="N408" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O408" t="inlineStr">
@@ -33318,14 +33348,14 @@
       </c>
       <c r="S408" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt0h140-0</t>
+          <t xml:space="preserve">v-mtski3re-0</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="E409" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="G409" t="inlineStr">
@@ -33345,7 +33375,7 @@
       </c>
       <c r="L409" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M409" t="inlineStr">
@@ -33370,7 +33400,7 @@
       </c>
       <c r="S409" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-0</t>
+          <t xml:space="preserve">v-mtt0h140-0</t>
         </is>
       </c>
     </row>
@@ -33422,7 +33452,7 @@
       </c>
       <c r="S410" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
         </is>
       </c>
     </row>
@@ -33474,14 +33504,14 @@
       </c>
       <c r="S411" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-2</t>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="E412" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="G412" t="inlineStr">
@@ -33526,14 +33556,14 @@
       </c>
       <c r="S412" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt5ckqo-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-2</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="E413" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">khk</t>
         </is>
       </c>
       <c r="G413" t="inlineStr">
@@ -33543,12 +33573,12 @@
       </c>
       <c r="H413" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I413" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="L413" t="inlineStr">
@@ -33578,7 +33608,7 @@
       </c>
       <c r="S413" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmw7m-0</t>
+          <t xml:space="preserve">v-mtt5ckqo-0</t>
         </is>
       </c>
     </row>
@@ -33630,7 +33660,7 @@
       </c>
       <c r="S414" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmypa-0</t>
+          <t xml:space="preserve">v-mttmmw7m-0</t>
         </is>
       </c>
     </row>
@@ -33682,14 +33712,14 @@
       </c>
       <c r="S415" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmn045-0</t>
+          <t xml:space="preserve">v-mttmmypa-0</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="E416" t="inlineStr">
         <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">kkk</t>
         </is>
       </c>
       <c r="G416" t="inlineStr">
@@ -33707,11 +33737,6 @@
           <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
-      <c r="K416" t="inlineStr">
-        <is>
-          <t xml:space="preserve">deneme</t>
-        </is>
-      </c>
       <c r="L416" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -33739,67 +33764,124 @@
       </c>
       <c r="S416" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtu5lgdc-0</t>
+          <t xml:space="preserve">v-mttmn045-0</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="E417" t="inlineStr">
         <is>
+          <t xml:space="preserve">deneme</t>
+        </is>
+      </c>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="K417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deneme</t>
+        </is>
+      </c>
+      <c r="L417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtu5lgdc-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="E418" t="inlineStr">
+        <is>
           <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
-      <c r="F417" t="inlineStr">
+      <c r="F418" t="inlineStr">
         <is>
           <t xml:space="preserve">p19</t>
         </is>
       </c>
-      <c r="G417" t="inlineStr">
+      <c r="G418" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H417" t="inlineStr">
+      <c r="H418" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-17</t>
         </is>
       </c>
-      <c r="I417" t="inlineStr">
+      <c r="I418" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-17</t>
         </is>
       </c>
-      <c r="K417" t="inlineStr">
+      <c r="K418" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L417" t="inlineStr">
+      <c r="L418" t="inlineStr">
         <is>
           <t xml:space="preserve">FLAG</t>
         </is>
       </c>
-      <c r="M417" t="inlineStr">
+      <c r="M418" t="inlineStr">
         <is>
           <t xml:space="preserve">Par</t>
         </is>
       </c>
-      <c r="N417" t="inlineStr">
+      <c r="N418" t="inlineStr">
         <is>
           <t xml:space="preserve">No Casp</t>
         </is>
       </c>
-      <c r="O417" t="inlineStr">
+      <c r="O418" t="inlineStr">
         <is>
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
-      <c r="R417" t="inlineStr">
+      <c r="R418" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
-      <c r="S417" t="inlineStr">
+      <c r="S418" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mu5anec8-0</t>
         </is>
@@ -33914,63 +33996,63 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g1.1</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1.1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E4">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">DuDtxR CASPEX g1.1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1.1</t>
         </is>
       </c>
       <c r="E5">
         <v>13</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G5">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -41456,10 +41538,10 @@
         <v>81</v>
       </c>
       <c r="I18">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J18">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="19">

</xml_diff>

<commit_message>
Add 1 × HEK from Umut
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -31824,27 +31824,27 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t xml:space="preserve">A1</t>
+          <t xml:space="preserve">C1</t>
         </is>
       </c>
       <c r="E386" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK</t>
         </is>
       </c>
       <c r="F386" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="G386" t="inlineStr">
@@ -31854,17 +31854,17 @@
       </c>
       <c r="H386" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="I386" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="K386" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L386" t="inlineStr">
@@ -31894,7 +31894,7 @@
       </c>
       <c r="S386" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-0</t>
+          <t xml:space="preserve">v-mv4ye7g5-0</t>
         </is>
       </c>
     </row>
@@ -31916,7 +31916,7 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t xml:space="preserve">A2</t>
+          <t xml:space="preserve">A1</t>
         </is>
       </c>
       <c r="E387" t="inlineStr">
@@ -31976,7 +31976,7 @@
       </c>
       <c r="S387" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-1</t>
+          <t xml:space="preserve">v-mupot2zh-0</t>
         </is>
       </c>
     </row>
@@ -31998,7 +31998,7 @@
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t xml:space="preserve">A3</t>
+          <t xml:space="preserve">A2</t>
         </is>
       </c>
       <c r="E388" t="inlineStr">
@@ -32058,7 +32058,7 @@
       </c>
       <c r="S388" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-2</t>
+          <t xml:space="preserve">v-mupot2zh-1</t>
         </is>
       </c>
     </row>
@@ -32080,7 +32080,7 @@
       </c>
       <c r="D389" t="inlineStr">
         <is>
-          <t xml:space="preserve">A4</t>
+          <t xml:space="preserve">A3</t>
         </is>
       </c>
       <c r="E389" t="inlineStr">
@@ -32140,7 +32140,7 @@
       </c>
       <c r="S389" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-3</t>
+          <t xml:space="preserve">v-mupot2zh-2</t>
         </is>
       </c>
     </row>
@@ -32162,161 +32162,181 @@
       </c>
       <c r="D390" t="inlineStr">
         <is>
+          <t xml:space="preserve">A4</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S390" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
           <t xml:space="preserve">A5</t>
         </is>
       </c>
-      <c r="E390" t="inlineStr">
+      <c r="E391" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="F390" t="inlineStr">
+      <c r="F391" t="inlineStr">
         <is>
           <t xml:space="preserve">p18</t>
         </is>
       </c>
-      <c r="G390" t="inlineStr">
+      <c r="G391" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H390" t="inlineStr">
+      <c r="H391" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
-      <c r="I390" t="inlineStr">
+      <c r="I391" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
-      <c r="K390" t="inlineStr">
+      <c r="K391" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L390" t="inlineStr">
+      <c r="L391" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
         </is>
       </c>
-      <c r="M390" t="inlineStr">
+      <c r="M391" t="inlineStr">
         <is>
           <t xml:space="preserve">Par</t>
         </is>
       </c>
-      <c r="N390" t="inlineStr">
+      <c r="N391" t="inlineStr">
         <is>
           <t xml:space="preserve">No Casp</t>
         </is>
       </c>
-      <c r="O390" t="inlineStr">
+      <c r="O391" t="inlineStr">
         <is>
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
-      <c r="R390" t="inlineStr">
+      <c r="R391" t="inlineStr">
         <is>
           <t xml:space="preserve">stored</t>
         </is>
       </c>
-      <c r="S390" t="inlineStr">
+      <c r="S391" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mupot2zh-4</t>
-        </is>
-      </c>
-    </row>
-    <row r="391">
-      <c r="E391" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNCX</t>
-        </is>
-      </c>
-      <c r="F391" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p+21</t>
-        </is>
-      </c>
-      <c r="G391" t="inlineStr">
-        <is>
-          <t xml:space="preserve">relative</t>
-        </is>
-      </c>
-      <c r="H391" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-05-15</t>
-        </is>
-      </c>
-      <c r="I391" t="inlineStr">
-        <is>
-          <t xml:space="preserve">15-05-26</t>
-        </is>
-      </c>
-      <c r="K391" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="L391" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M391" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N391" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CASPEX</t>
-        </is>
-      </c>
-      <c r="O391" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R391" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S391" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-199</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="E392" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F392" t="inlineStr">
         <is>
-          <t xml:space="preserve">p19</t>
+          <t xml:space="preserve">p+21</t>
         </is>
       </c>
       <c r="G392" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H392" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-07-31</t>
+          <t xml:space="preserve">2026-05-15</t>
         </is>
       </c>
       <c r="I392" t="inlineStr">
         <is>
-          <t xml:space="preserve">31-07-26</t>
+          <t xml:space="preserve">15-05-26</t>
         </is>
       </c>
       <c r="K392" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L392" t="inlineStr">
@@ -32326,7 +32346,7 @@
       </c>
       <c r="M392" t="inlineStr">
         <is>
-          <t xml:space="preserve">CR</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N392" t="inlineStr">
@@ -32339,16 +32359,6 @@
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
-      <c r="P392" t="inlineStr">
-        <is>
-          <t xml:space="preserve">to-do</t>
-        </is>
-      </c>
-      <c r="Q392" t="inlineStr">
-        <is>
-          <t xml:space="preserve">to-do box / thaw</t>
-        </is>
-      </c>
       <c r="R392" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
@@ -32356,39 +32366,39 @@
       </c>
       <c r="S392" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-233</t>
+          <t xml:space="preserve">v-199</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="E393" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">LUCX</t>
         </is>
       </c>
       <c r="F393" t="inlineStr">
         <is>
-          <t xml:space="preserve">p?</t>
+          <t xml:space="preserve">p19</t>
         </is>
       </c>
       <c r="G393" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H393" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-06-30</t>
+          <t xml:space="preserve">2026-07-31</t>
         </is>
       </c>
       <c r="I393" t="inlineStr">
         <is>
-          <t xml:space="preserve">30-06-25</t>
+          <t xml:space="preserve">31-07-26</t>
         </is>
       </c>
       <c r="K393" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L393" t="inlineStr">
@@ -32398,12 +32408,12 @@
       </c>
       <c r="M393" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N393" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O393" t="inlineStr">
@@ -32411,6 +32421,16 @@
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
+      <c r="P393" t="inlineStr">
+        <is>
+          <t xml:space="preserve">to-do</t>
+        </is>
+      </c>
+      <c r="Q393" t="inlineStr">
+        <is>
+          <t xml:space="preserve">to-do box / thaw</t>
+        </is>
+      </c>
       <c r="R393" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
@@ -32418,39 +32438,39 @@
       </c>
       <c r="S393" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-295</t>
+          <t xml:space="preserve">v-233</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="E394" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="F394" t="inlineStr">
         <is>
-          <t xml:space="preserve">p11</t>
+          <t xml:space="preserve">p?</t>
         </is>
       </c>
       <c r="G394" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H394" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-06-12</t>
+          <t xml:space="preserve">2025-06-30</t>
         </is>
       </c>
       <c r="I394" t="inlineStr">
         <is>
-          <t xml:space="preserve">12/6/2026</t>
+          <t xml:space="preserve">30-06-25</t>
         </is>
       </c>
       <c r="K394" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="L394" t="inlineStr">
@@ -32460,7 +32480,7 @@
       </c>
       <c r="M394" t="inlineStr">
         <is>
-          <t xml:space="preserve">CR</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N394" t="inlineStr">
@@ -32480,39 +32500,39 @@
       </c>
       <c r="S394" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-311</t>
+          <t xml:space="preserve">v-295</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="E395" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="F395" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+17</t>
+          <t xml:space="preserve">p11</t>
         </is>
       </c>
       <c r="G395" t="inlineStr">
         <is>
-          <t xml:space="preserve">relative</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H395" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-03-30</t>
+          <t xml:space="preserve">2026-06-12</t>
         </is>
       </c>
       <c r="I395" t="inlineStr">
         <is>
-          <t xml:space="preserve">30-03-26</t>
+          <t xml:space="preserve">12/6/2026</t>
         </is>
       </c>
       <c r="K395" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L395" t="inlineStr">
@@ -32522,12 +32542,12 @@
       </c>
       <c r="M395" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N395" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">No Casp</t>
         </is>
       </c>
       <c r="O395" t="inlineStr">
@@ -32542,19 +32562,19 @@
       </c>
       <c r="S395" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-320</t>
+          <t xml:space="preserve">v-311</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="E396" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F396" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+14</t>
+          <t xml:space="preserve">p+17</t>
         </is>
       </c>
       <c r="G396" t="inlineStr">
@@ -32564,12 +32584,12 @@
       </c>
       <c r="H396" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-03-23</t>
+          <t xml:space="preserve">2026-03-30</t>
         </is>
       </c>
       <c r="I396" t="inlineStr">
         <is>
-          <t xml:space="preserve">23-03-26</t>
+          <t xml:space="preserve">30-03-26</t>
         </is>
       </c>
       <c r="K396" t="inlineStr">
@@ -32589,7 +32609,7 @@
       </c>
       <c r="N396" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O396" t="inlineStr">
@@ -32604,39 +32624,39 @@
       </c>
       <c r="S396" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-321</t>
+          <t xml:space="preserve">v-320</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="E397" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap Canada</t>
         </is>
       </c>
       <c r="F397" t="inlineStr">
         <is>
-          <t xml:space="preserve">p16</t>
+          <t xml:space="preserve">p+14</t>
         </is>
       </c>
       <c r="G397" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H397" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-11-06</t>
+          <t xml:space="preserve">2026-03-23</t>
         </is>
       </c>
       <c r="I397" t="inlineStr">
         <is>
-          <t xml:space="preserve">6/11/2025</t>
+          <t xml:space="preserve">23-03-26</t>
         </is>
       </c>
       <c r="K397" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L397" t="inlineStr">
@@ -32666,19 +32686,19 @@
       </c>
       <c r="S397" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-338</t>
+          <t xml:space="preserve">v-321</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="E398" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="F398" t="inlineStr">
         <is>
-          <t xml:space="preserve">p15</t>
+          <t xml:space="preserve">p16</t>
         </is>
       </c>
       <c r="G398" t="inlineStr">
@@ -32688,17 +32708,17 @@
       </c>
       <c r="H398" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-10</t>
+          <t xml:space="preserve">2025-11-06</t>
         </is>
       </c>
       <c r="I398" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/8/2026</t>
+          <t xml:space="preserve">6/11/2025</t>
         </is>
       </c>
       <c r="K398" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L398" t="inlineStr">
@@ -32728,19 +32748,19 @@
       </c>
       <c r="S398" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-354</t>
+          <t xml:space="preserve">v-338</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="E399" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="F399" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p15</t>
         </is>
       </c>
       <c r="G399" t="inlineStr">
@@ -32750,17 +32770,17 @@
       </c>
       <c r="H399" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-08-10</t>
         </is>
       </c>
       <c r="I399" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">10/8/2026</t>
         </is>
       </c>
       <c r="K399" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L399" t="inlineStr">
@@ -32780,7 +32800,7 @@
       </c>
       <c r="O399" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R399" t="inlineStr">
@@ -32790,14 +32810,14 @@
       </c>
       <c r="S399" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdx0po-0</t>
+          <t xml:space="preserve">v-354</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="E400" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="F400" t="inlineStr">
@@ -32827,7 +32847,7 @@
       </c>
       <c r="L400" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M400" t="inlineStr">
@@ -32842,7 +32862,7 @@
       </c>
       <c r="O400" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R400" t="inlineStr">
@@ -32852,14 +32872,14 @@
       </c>
       <c r="S400" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdxsum-0</t>
+          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="E401" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="F401" t="inlineStr">
@@ -32889,7 +32909,7 @@
       </c>
       <c r="L401" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M401" t="inlineStr">
@@ -32914,7 +32934,7 @@
       </c>
       <c r="S401" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-0</t>
+          <t xml:space="preserve">v-mtrdxsum-0</t>
         </is>
       </c>
     </row>
@@ -32976,19 +32996,19 @@
       </c>
       <c r="S402" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-1</t>
+          <t xml:space="preserve">v-mtrdyhss-0</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="E403" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="F403" t="inlineStr">
         <is>
-          <t xml:space="preserve">p28</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G403" t="inlineStr">
@@ -33013,7 +33033,7 @@
       </c>
       <c r="L403" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M403" t="inlineStr">
@@ -33038,19 +33058,19 @@
       </c>
       <c r="S403" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdz1vx-0</t>
+          <t xml:space="preserve">v-mtrdyhss-1</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="E404" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="F404" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p28</t>
         </is>
       </c>
       <c r="G404" t="inlineStr">
@@ -33070,12 +33090,12 @@
       </c>
       <c r="K404" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L404" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M404" t="inlineStr">
@@ -33090,7 +33110,7 @@
       </c>
       <c r="O404" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R404" t="inlineStr">
@@ -33100,19 +33120,19 @@
       </c>
       <c r="S404" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdzpx7-0</t>
+          <t xml:space="preserve">v-mtrdz1vx-0</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="E405" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">Huh7 gNT</t>
         </is>
       </c>
       <c r="F405" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G405" t="inlineStr">
@@ -33137,7 +33157,7 @@
       </c>
       <c r="L405" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M405" t="inlineStr">
@@ -33152,7 +33172,7 @@
       </c>
       <c r="O405" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R405" t="inlineStr">
@@ -33162,19 +33182,19 @@
       </c>
       <c r="S405" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0daw-0</t>
+          <t xml:space="preserve">v-mtrdzpx7-0</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="E406" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="F406" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G406" t="inlineStr">
@@ -33199,7 +33219,7 @@
       </c>
       <c r="L406" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M406" t="inlineStr">
@@ -33224,19 +33244,19 @@
       </c>
       <c r="S406" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0w3q-0</t>
+          <t xml:space="preserve">v-mtre0daw-0</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="E407" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="F407" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G407" t="inlineStr">
@@ -33261,7 +33281,7 @@
       </c>
       <c r="L407" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M407" t="inlineStr">
@@ -33286,19 +33306,19 @@
       </c>
       <c r="S407" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre1ko0-0</t>
+          <t xml:space="preserve">v-mtre0w3q-0</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="E408" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="F408" t="inlineStr">
         <is>
-          <t xml:space="preserve">p6</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G408" t="inlineStr">
@@ -33308,22 +33328,22 @@
       </c>
       <c r="H408" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I408" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="K408" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L408" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M408" t="inlineStr">
@@ -33333,7 +33353,7 @@
       </c>
       <c r="N408" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">No Casp</t>
         </is>
       </c>
       <c r="O408" t="inlineStr">
@@ -33348,19 +33368,24 @@
       </c>
       <c r="S408" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtski3re-0</t>
+          <t xml:space="preserve">v-mtre1ko0-0</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="E409" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">Hek caspex</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p6</t>
         </is>
       </c>
       <c r="G409" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H409" t="inlineStr">
@@ -33373,9 +33398,14 @@
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
+      <c r="K409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
       <c r="L409" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M409" t="inlineStr">
@@ -33385,7 +33415,7 @@
       </c>
       <c r="N409" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O409" t="inlineStr">
@@ -33400,14 +33430,14 @@
       </c>
       <c r="S409" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt0h140-0</t>
+          <t xml:space="preserve">v-mtski3re-0</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="E410" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="G410" t="inlineStr">
@@ -33427,7 +33457,7 @@
       </c>
       <c r="L410" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M410" t="inlineStr">
@@ -33452,7 +33482,7 @@
       </c>
       <c r="S410" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-0</t>
+          <t xml:space="preserve">v-mtt0h140-0</t>
         </is>
       </c>
     </row>
@@ -33504,7 +33534,7 @@
       </c>
       <c r="S411" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
         </is>
       </c>
     </row>
@@ -33556,14 +33586,14 @@
       </c>
       <c r="S412" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-2</t>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="E413" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="G413" t="inlineStr">
@@ -33608,14 +33638,14 @@
       </c>
       <c r="S413" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt5ckqo-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-2</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="E414" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">khk</t>
         </is>
       </c>
       <c r="G414" t="inlineStr">
@@ -33625,12 +33655,12 @@
       </c>
       <c r="H414" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I414" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="L414" t="inlineStr">
@@ -33660,7 +33690,7 @@
       </c>
       <c r="S414" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmw7m-0</t>
+          <t xml:space="preserve">v-mtt5ckqo-0</t>
         </is>
       </c>
     </row>
@@ -33712,7 +33742,7 @@
       </c>
       <c r="S415" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmypa-0</t>
+          <t xml:space="preserve">v-mttmmw7m-0</t>
         </is>
       </c>
     </row>
@@ -33764,14 +33794,14 @@
       </c>
       <c r="S416" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmn045-0</t>
+          <t xml:space="preserve">v-mttmmypa-0</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="E417" t="inlineStr">
         <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">kkk</t>
         </is>
       </c>
       <c r="G417" t="inlineStr">
@@ -33789,11 +33819,6 @@
           <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
-      <c r="K417" t="inlineStr">
-        <is>
-          <t xml:space="preserve">deneme</t>
-        </is>
-      </c>
       <c r="L417" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -33821,67 +33846,124 @@
       </c>
       <c r="S417" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtu5lgdc-0</t>
+          <t xml:space="preserve">v-mttmn045-0</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="E418" t="inlineStr">
         <is>
+          <t xml:space="preserve">deneme</t>
+        </is>
+      </c>
+      <c r="G418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="K418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deneme</t>
+        </is>
+      </c>
+      <c r="L418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtu5lgdc-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="E419" t="inlineStr">
+        <is>
           <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
-      <c r="F418" t="inlineStr">
+      <c r="F419" t="inlineStr">
         <is>
           <t xml:space="preserve">p19</t>
         </is>
       </c>
-      <c r="G418" t="inlineStr">
+      <c r="G419" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H418" t="inlineStr">
+      <c r="H419" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-17</t>
         </is>
       </c>
-      <c r="I418" t="inlineStr">
+      <c r="I419" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-17</t>
         </is>
       </c>
-      <c r="K418" t="inlineStr">
+      <c r="K419" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L418" t="inlineStr">
+      <c r="L419" t="inlineStr">
         <is>
           <t xml:space="preserve">FLAG</t>
         </is>
       </c>
-      <c r="M418" t="inlineStr">
+      <c r="M419" t="inlineStr">
         <is>
           <t xml:space="preserve">Par</t>
         </is>
       </c>
-      <c r="N418" t="inlineStr">
+      <c r="N419" t="inlineStr">
         <is>
           <t xml:space="preserve">No Casp</t>
         </is>
       </c>
-      <c r="O418" t="inlineStr">
+      <c r="O419" t="inlineStr">
         <is>
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
-      <c r="R418" t="inlineStr">
+      <c r="R419" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
-      <c r="S418" t="inlineStr">
+      <c r="S419" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mu5anec8-0</t>
         </is>
@@ -36245,22 +36327,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK APEX1 KO g2</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t xml:space="preserve">KO</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">HEK</t>
         </is>
       </c>
       <c r="E78">
@@ -36276,7 +36343,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK APEX1 OX</t>
+          <t xml:space="preserve">HEK APEX1 KO g2</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -36286,12 +36353,12 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E79">
@@ -36307,7 +36374,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK APEX1 g1</t>
+          <t xml:space="preserve">HEK APEX1 OX</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -36317,12 +36384,12 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E80">
@@ -36338,7 +36405,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO 20</t>
+          <t xml:space="preserve">HEK APEX1 g1</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -36348,12 +36415,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E81">
@@ -36369,7 +36436,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO10</t>
+          <t xml:space="preserve">HEK ATF3 KO 20</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -36400,7 +36467,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX</t>
+          <t xml:space="preserve">HEK ATF3 KO10</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -36410,7 +36477,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -36431,7 +36498,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep2</t>
+          <t xml:space="preserve">HEK ATF3 OX</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -36462,7 +36529,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX10r1</t>
+          <t xml:space="preserve">HEK ATF3 OX rep2</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -36493,7 +36560,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX20r1</t>
+          <t xml:space="preserve">HEK ATF3 OX10r1</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -36524,7 +36591,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3OX10r1</t>
+          <t xml:space="preserve">HEK ATF3 OX20r1</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -36555,7 +36622,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B KO-1</t>
+          <t xml:space="preserve">HEK ATF3OX10r1</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -36565,7 +36632,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -36586,7 +36653,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B KO-2</t>
+          <t xml:space="preserve">HEK ATP7B KO-1</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -36617,7 +36684,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B KO-3</t>
+          <t xml:space="preserve">HEK ATP7B KO-2</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -36648,7 +36715,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CASPEX gNT</t>
+          <t xml:space="preserve">HEK ATP7B KO-3</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -36658,12 +36725,12 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E91">
@@ -36679,7 +36746,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO g1 plv-GFP</t>
+          <t xml:space="preserve">HEK CASPEX gNT</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -36689,12 +36756,12 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E92">
@@ -36710,7 +36777,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 OX</t>
+          <t xml:space="preserve">HEK CBX3 KO g1 plv-GFP</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -36720,12 +36787,12 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E93">
@@ -36741,7 +36808,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK GATA6 KO g1</t>
+          <t xml:space="preserve">HEK CBX3 OX</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -36751,12 +36818,12 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E94">
@@ -36772,7 +36839,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK GATA6 KO g2</t>
+          <t xml:space="preserve">HEK GATA6 KO g1</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -36787,7 +36854,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E95">
@@ -36803,7 +36870,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 KO g2</t>
+          <t xml:space="preserve">HEK GATA6 KO g2</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -36813,7 +36880,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -36834,7 +36901,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK JUN KO g1</t>
+          <t xml:space="preserve">HEK HOXB6 KO g2</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -36844,12 +36911,12 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E97">
@@ -36865,7 +36932,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK JUN KO g2</t>
+          <t xml:space="preserve">HEK JUN KO g1</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -36880,7 +36947,7 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E98">
@@ -36896,7 +36963,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK JUN1 KO g2</t>
+          <t xml:space="preserve">HEK JUN KO g2</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -36927,7 +36994,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK NRF2 KO g1</t>
+          <t xml:space="preserve">HEK JUN1 KO g2</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -36942,7 +37009,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E100">
@@ -36958,7 +37025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK NRF2 KO g2</t>
+          <t xml:space="preserve">HEK NRF2 KO g1</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -36973,7 +37040,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E101">
@@ -36989,7 +37056,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK RFX KO g1</t>
+          <t xml:space="preserve">HEK NRF2 KO g2</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -37004,7 +37071,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E102">
@@ -37020,7 +37087,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK RFX KO g2</t>
+          <t xml:space="preserve">HEK RFX KO g1</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -37035,7 +37102,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E103">
@@ -37051,7 +37118,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK SMARCE1 KO g1</t>
+          <t xml:space="preserve">HEK RFX KO g2</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -37066,7 +37133,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E104">
@@ -37082,7 +37149,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK SMARCE1 KO g2</t>
+          <t xml:space="preserve">HEK SMARCE1 KO g1</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -37097,7 +37164,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E105">
@@ -37113,7 +37180,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK SPEN KO g2</t>
+          <t xml:space="preserve">HEK SMARCE1 KO g2</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -37144,7 +37211,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK STAT1 KO g1</t>
+          <t xml:space="preserve">HEK SPEN KO g2</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -37159,7 +37226,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E107">
@@ -37175,7 +37242,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK TOX4 OX 3xFLAG</t>
+          <t xml:space="preserve">HEK STAT1 KO g1</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -37185,12 +37252,12 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E108">
@@ -37206,7 +37273,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT (10)</t>
+          <t xml:space="preserve">HEK TOX4 OX 3xFLAG</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -37216,12 +37283,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E109">
@@ -37237,7 +37304,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK lef1 OX</t>
+          <t xml:space="preserve">HEK gNT (10)</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -37247,12 +37314,12 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E110">
@@ -37268,17 +37335,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep2</t>
+          <t xml:space="preserve">HEK lef1 OX</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -37299,7 +37366,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO20</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep2</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -37330,7 +37397,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep2</t>
+          <t xml:space="preserve">Huh7 ATF3 KO20</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -37340,7 +37407,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -37361,7 +37428,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX20r1</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep2</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -37392,7 +37459,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3KO10</t>
+          <t xml:space="preserve">Huh7 ATF3 OX20r1</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -37402,7 +37469,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -37423,7 +37490,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATP7B KO</t>
+          <t xml:space="preserve">Huh7 ATF3KO10</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -37454,7 +37521,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 CASPEX gNT</t>
+          <t xml:space="preserve">Huh7 ATP7B KO</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -37464,12 +37531,12 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E117">
@@ -37485,7 +37552,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 CBX3 KO g1</t>
+          <t xml:space="preserve">Huh7 CASPEX gNT</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -37495,12 +37562,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E118">
@@ -37516,7 +37583,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 CBX3 KO g2</t>
+          <t xml:space="preserve">Huh7 CBX3 KO g1</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -37531,7 +37598,7 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E119">
@@ -37547,7 +37614,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 CBX3 OX</t>
+          <t xml:space="preserve">Huh7 CBX3 KO g2</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -37557,12 +37624,12 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E120">
@@ -37578,7 +37645,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 HOXB6 KO g1</t>
+          <t xml:space="preserve">Huh7 CBX3 OX</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -37593,7 +37660,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E121">
@@ -37609,7 +37676,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 HOXB6 OX</t>
+          <t xml:space="preserve">Huh7 HOXB6 KO g1</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -37624,7 +37691,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E122">
@@ -37640,7 +37707,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 POU3F2 KO g1</t>
+          <t xml:space="preserve">Huh7 HOXB6 OX</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -37650,12 +37717,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E123">
@@ -37671,7 +37738,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 POU3F3 KO g1</t>
+          <t xml:space="preserve">Huh7 POU3F2 KO g1</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -37702,7 +37769,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 POU3F3 KO g2</t>
+          <t xml:space="preserve">Huh7 POU3F3 KO g1</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -37717,7 +37784,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E125">
@@ -37733,7 +37800,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 TOX4 KO g1</t>
+          <t xml:space="preserve">Huh7 POU3F3 KO g2</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -37743,12 +37810,12 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E126">
@@ -37764,7 +37831,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 TOX4 OX</t>
+          <t xml:space="preserve">Huh7 TOX4 KO g1</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -37779,7 +37846,7 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E127">
@@ -37795,7 +37862,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 lef1 OX</t>
+          <t xml:space="preserve">Huh7 TOX4 OX</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -37826,17 +37893,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-C*</t>
+          <t xml:space="preserve">Huh7 lef1 OX</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -37857,7 +37924,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-E</t>
+          <t xml:space="preserve">LCC-C*</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -37888,7 +37955,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-H</t>
+          <t xml:space="preserve">LCC-E</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -37919,7 +37986,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNC478 #1</t>
+          <t xml:space="preserve">LCC-H</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -37950,7 +38017,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNC478 #2 98%</t>
+          <t xml:space="preserve">LNC478 #1</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -37981,7 +38048,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNC478 #3</t>
+          <t xml:space="preserve">LNC478 #2 98%</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -38012,7 +38079,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCAP BMK</t>
+          <t xml:space="preserve">LNC478 #3</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -38043,7 +38110,22 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX gC1</t>
+          <t xml:space="preserve">LNCAP BMK</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E136">
@@ -38059,7 +38141,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX gC2</t>
+          <t xml:space="preserve">LUCX gC1</t>
         </is>
       </c>
       <c r="E137">
@@ -38075,7 +38157,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX gC3</t>
+          <t xml:space="preserve">LUCX gC2</t>
         </is>
       </c>
       <c r="E138">
@@ -38091,7 +38173,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX gC4</t>
+          <t xml:space="preserve">LUCX gC3</t>
         </is>
       </c>
       <c r="E139">
@@ -38107,7 +38189,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX gP3</t>
+          <t xml:space="preserve">LUCX gC4</t>
         </is>
       </c>
       <c r="E140">
@@ -38123,22 +38205,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap (m3) no sort</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="D141" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">LUCX gP3</t>
         </is>
       </c>
       <c r="E141">
@@ -38154,7 +38221,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G2</t>
+          <t xml:space="preserve">LnCap (m3) no sort</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -38185,7 +38252,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G3</t>
+          <t xml:space="preserve">LnCap Canada V1G2</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -38216,7 +38283,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G4</t>
+          <t xml:space="preserve">LnCap Canada V1G3</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -38247,7 +38314,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap ER</t>
+          <t xml:space="preserve">LnCap Canada V1G4</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -38278,7 +38345,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap V1G1</t>
+          <t xml:space="preserve">LnCap ER</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -38309,7 +38376,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap478 #2 98%</t>
+          <t xml:space="preserve">LnCap V1G1</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -38340,7 +38407,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select</t>
+          <t xml:space="preserve">LnCap478 #2 98%</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -38350,7 +38417,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -38371,7 +38438,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select C</t>
+          <t xml:space="preserve">LnCapCASPEX no select</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -38402,17 +38469,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap (m1) no sort</t>
+          <t xml:space="preserve">LnCapCASPEX no select C</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -38433,7 +38500,12 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t xml:space="preserve">MDA-MB g1.1 p10</t>
+          <t xml:space="preserve">LuCap (m1) no sort</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -38443,7 +38515,7 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1.1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E151">
@@ -38459,7 +38531,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t xml:space="preserve">MDA-MB gNT</t>
+          <t xml:space="preserve">MDA-MB g1.1 p10</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -38469,7 +38541,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">g1.1</t>
         </is>
       </c>
       <c r="E152">
@@ -38485,23 +38557,33 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">MDA-MB gNT</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E153">
+        <v>1</v>
+      </c>
+      <c r="F153">
         <v>0</v>
       </c>
-      <c r="F153">
+      <c r="G153">
         <v>1</v>
-      </c>
-      <c r="G153">
-        <v>0</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">Hek caspex</t>
         </is>
       </c>
       <c r="E154">
@@ -38517,14 +38599,14 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">deneme</t>
         </is>
       </c>
       <c r="E155">
         <v>0</v>
       </c>
       <c r="F155">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G155">
         <v>0</v>
@@ -38533,14 +38615,14 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="E156">
         <v>0</v>
       </c>
       <c r="F156">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G156">
         <v>0</v>
@@ -38549,24 +38631,14 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
-        </is>
-      </c>
-      <c r="C157" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="D157" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">khk</t>
         </is>
       </c>
       <c r="E157">
         <v>0</v>
       </c>
       <c r="F157">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G157">
         <v>0</v>
@@ -38575,16 +38647,42 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E158">
         <v>0</v>
       </c>
       <c r="F158">
+        <v>3</v>
+      </c>
+      <c r="G158">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t xml:space="preserve">klm ox</t>
+        </is>
+      </c>
+      <c r="E159">
+        <v>0</v>
+      </c>
+      <c r="F159">
         <v>1</v>
       </c>
-      <c r="G158">
+      <c r="G159">
         <v>0</v>
       </c>
     </row>
@@ -41538,10 +41636,10 @@
         <v>81</v>
       </c>
       <c r="I18">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J18">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="19">

</xml_diff>

<commit_message>
Add 6 × Huh7 from Umut
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -31834,17 +31834,17 @@
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t xml:space="preserve">C1</t>
+          <t xml:space="preserve">B2</t>
         </is>
       </c>
       <c r="E386" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="F386" t="inlineStr">
         <is>
-          <t xml:space="preserve">7</t>
+          <t xml:space="preserve">18</t>
         </is>
       </c>
       <c r="G386" t="inlineStr">
@@ -31864,7 +31864,7 @@
       </c>
       <c r="K386" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L386" t="inlineStr">
@@ -31894,7 +31894,7 @@
       </c>
       <c r="S386" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv4ye7g5-0</t>
+          <t xml:space="preserve">v-mv4yequa-0</t>
         </is>
       </c>
     </row>
@@ -31906,17 +31906,17 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t xml:space="preserve">A1</t>
+          <t xml:space="preserve">B3</t>
         </is>
       </c>
       <c r="E387" t="inlineStr">
@@ -31926,7 +31926,7 @@
       </c>
       <c r="F387" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">18</t>
         </is>
       </c>
       <c r="G387" t="inlineStr">
@@ -31936,12 +31936,12 @@
       </c>
       <c r="H387" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="I387" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="K387" t="inlineStr">
@@ -31976,7 +31976,7 @@
       </c>
       <c r="S387" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-0</t>
+          <t xml:space="preserve">v-mv4yequa-1</t>
         </is>
       </c>
     </row>
@@ -31988,17 +31988,17 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t xml:space="preserve">A2</t>
+          <t xml:space="preserve">B4</t>
         </is>
       </c>
       <c r="E388" t="inlineStr">
@@ -32008,7 +32008,7 @@
       </c>
       <c r="F388" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">18</t>
         </is>
       </c>
       <c r="G388" t="inlineStr">
@@ -32018,12 +32018,12 @@
       </c>
       <c r="H388" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="I388" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="K388" t="inlineStr">
@@ -32058,7 +32058,7 @@
       </c>
       <c r="S388" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-1</t>
+          <t xml:space="preserve">v-mv4yequa-2</t>
         </is>
       </c>
     </row>
@@ -32070,17 +32070,17 @@
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D389" t="inlineStr">
         <is>
-          <t xml:space="preserve">A3</t>
+          <t xml:space="preserve">B5</t>
         </is>
       </c>
       <c r="E389" t="inlineStr">
@@ -32090,7 +32090,7 @@
       </c>
       <c r="F389" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">18</t>
         </is>
       </c>
       <c r="G389" t="inlineStr">
@@ -32100,12 +32100,12 @@
       </c>
       <c r="H389" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="I389" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="K389" t="inlineStr">
@@ -32140,7 +32140,7 @@
       </c>
       <c r="S389" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-2</t>
+          <t xml:space="preserve">v-mv4yequa-3</t>
         </is>
       </c>
     </row>
@@ -32152,17 +32152,17 @@
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D390" t="inlineStr">
         <is>
-          <t xml:space="preserve">A4</t>
+          <t xml:space="preserve">B6</t>
         </is>
       </c>
       <c r="E390" t="inlineStr">
@@ -32172,7 +32172,7 @@
       </c>
       <c r="F390" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">18</t>
         </is>
       </c>
       <c r="G390" t="inlineStr">
@@ -32182,12 +32182,12 @@
       </c>
       <c r="H390" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="I390" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="K390" t="inlineStr">
@@ -32222,7 +32222,7 @@
       </c>
       <c r="S390" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-3</t>
+          <t xml:space="preserve">v-mv4yequa-4</t>
         </is>
       </c>
     </row>
@@ -32234,491 +32234,601 @@
       </c>
       <c r="B391" t="inlineStr">
         <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B7</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">18</t>
+        </is>
+      </c>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="I391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="K391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S391" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv4yequa-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C1</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7</t>
+        </is>
+      </c>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="I392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="K392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
+      <c r="L392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S392" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv4ye7g5-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
           <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
-      <c r="C391" t="inlineStr">
+      <c r="C393" t="inlineStr">
         <is>
           <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
-      <c r="D391" t="inlineStr">
+      <c r="D393" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A1</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H393" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I393" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K393" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L393" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M393" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N393" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O393" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R393" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S393" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A2</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I394" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K394" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L394" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M394" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N394" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O394" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R394" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S394" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A3</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I395" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K395" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L395" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M395" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N395" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O395" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R395" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S395" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A4</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
         <is>
           <t xml:space="preserve">A5</t>
         </is>
       </c>
-      <c r="E391" t="inlineStr">
+      <c r="E397" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="F391" t="inlineStr">
+      <c r="F397" t="inlineStr">
         <is>
           <t xml:space="preserve">p18</t>
         </is>
       </c>
-      <c r="G391" t="inlineStr">
+      <c r="G397" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H391" t="inlineStr">
+      <c r="H397" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
-      <c r="I391" t="inlineStr">
+      <c r="I397" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
-      <c r="K391" t="inlineStr">
+      <c r="K397" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L391" t="inlineStr">
+      <c r="L397" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
         </is>
       </c>
-      <c r="M391" t="inlineStr">
+      <c r="M397" t="inlineStr">
         <is>
           <t xml:space="preserve">Par</t>
         </is>
       </c>
-      <c r="N391" t="inlineStr">
+      <c r="N397" t="inlineStr">
         <is>
           <t xml:space="preserve">No Casp</t>
         </is>
       </c>
-      <c r="O391" t="inlineStr">
+      <c r="O397" t="inlineStr">
         <is>
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
-      <c r="R391" t="inlineStr">
+      <c r="R397" t="inlineStr">
         <is>
           <t xml:space="preserve">stored</t>
         </is>
       </c>
-      <c r="S391" t="inlineStr">
+      <c r="S397" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mupot2zh-4</t>
-        </is>
-      </c>
-    </row>
-    <row r="392">
-      <c r="E392" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNCX</t>
-        </is>
-      </c>
-      <c r="F392" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p+21</t>
-        </is>
-      </c>
-      <c r="G392" t="inlineStr">
-        <is>
-          <t xml:space="preserve">relative</t>
-        </is>
-      </c>
-      <c r="H392" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-05-15</t>
-        </is>
-      </c>
-      <c r="I392" t="inlineStr">
-        <is>
-          <t xml:space="preserve">15-05-26</t>
-        </is>
-      </c>
-      <c r="K392" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="L392" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M392" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N392" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CASPEX</t>
-        </is>
-      </c>
-      <c r="O392" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R392" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S392" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-199</t>
-        </is>
-      </c>
-    </row>
-    <row r="393">
-      <c r="E393" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LUCX</t>
-        </is>
-      </c>
-      <c r="F393" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p19</t>
-        </is>
-      </c>
-      <c r="G393" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H393" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-07-31</t>
-        </is>
-      </c>
-      <c r="I393" t="inlineStr">
-        <is>
-          <t xml:space="preserve">31-07-26</t>
-        </is>
-      </c>
-      <c r="K393" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR</t>
-        </is>
-      </c>
-      <c r="L393" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M393" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CR</t>
-        </is>
-      </c>
-      <c r="N393" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CASPEX</t>
-        </is>
-      </c>
-      <c r="O393" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="P393" t="inlineStr">
-        <is>
-          <t xml:space="preserve">to-do</t>
-        </is>
-      </c>
-      <c r="Q393" t="inlineStr">
-        <is>
-          <t xml:space="preserve">to-do box / thaw</t>
-        </is>
-      </c>
-      <c r="R393" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S393" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-233</t>
-        </is>
-      </c>
-    </row>
-    <row r="394">
-      <c r="E394" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145</t>
-        </is>
-      </c>
-      <c r="F394" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p?</t>
-        </is>
-      </c>
-      <c r="G394" t="inlineStr">
-        <is>
-          <t xml:space="preserve">unknown</t>
-        </is>
-      </c>
-      <c r="H394" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-06-30</t>
-        </is>
-      </c>
-      <c r="I394" t="inlineStr">
-        <is>
-          <t xml:space="preserve">30-06-25</t>
-        </is>
-      </c>
-      <c r="K394" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145</t>
-        </is>
-      </c>
-      <c r="L394" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M394" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N394" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O394" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R394" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S394" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-295</t>
-        </is>
-      </c>
-    </row>
-    <row r="395">
-      <c r="E395" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR</t>
-        </is>
-      </c>
-      <c r="F395" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p11</t>
-        </is>
-      </c>
-      <c r="G395" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H395" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-12</t>
-        </is>
-      </c>
-      <c r="I395" t="inlineStr">
-        <is>
-          <t xml:space="preserve">12/6/2026</t>
-        </is>
-      </c>
-      <c r="K395" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR</t>
-        </is>
-      </c>
-      <c r="L395" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M395" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CR</t>
-        </is>
-      </c>
-      <c r="N395" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O395" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R395" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S395" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-311</t>
-        </is>
-      </c>
-    </row>
-    <row r="396">
-      <c r="E396" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNCX</t>
-        </is>
-      </c>
-      <c r="F396" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p+17</t>
-        </is>
-      </c>
-      <c r="G396" t="inlineStr">
-        <is>
-          <t xml:space="preserve">relative</t>
-        </is>
-      </c>
-      <c r="H396" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-03-30</t>
-        </is>
-      </c>
-      <c r="I396" t="inlineStr">
-        <is>
-          <t xml:space="preserve">30-03-26</t>
-        </is>
-      </c>
-      <c r="K396" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="L396" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M396" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N396" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CASPEX</t>
-        </is>
-      </c>
-      <c r="O396" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R396" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S396" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-320</t>
-        </is>
-      </c>
-    </row>
-    <row r="397">
-      <c r="E397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap Canada</t>
-        </is>
-      </c>
-      <c r="F397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p+14</t>
-        </is>
-      </c>
-      <c r="G397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">relative</t>
-        </is>
-      </c>
-      <c r="H397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-03-23</t>
-        </is>
-      </c>
-      <c r="I397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">23-03-26</t>
-        </is>
-      </c>
-      <c r="K397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="L397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-321</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="E398" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F398" t="inlineStr">
         <is>
-          <t xml:space="preserve">p16</t>
+          <t xml:space="preserve">p+21</t>
         </is>
       </c>
       <c r="G398" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H398" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-11-06</t>
+          <t xml:space="preserve">2026-05-15</t>
         </is>
       </c>
       <c r="I398" t="inlineStr">
         <is>
-          <t xml:space="preserve">6/11/2025</t>
+          <t xml:space="preserve">15-05-26</t>
         </is>
       </c>
       <c r="K398" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L398" t="inlineStr">
@@ -32733,7 +32843,7 @@
       </c>
       <c r="N398" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O398" t="inlineStr">
@@ -32748,19 +32858,19 @@
       </c>
       <c r="S398" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-338</t>
+          <t xml:space="preserve">v-199</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="E399" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LUCX</t>
         </is>
       </c>
       <c r="F399" t="inlineStr">
         <is>
-          <t xml:space="preserve">p15</t>
+          <t xml:space="preserve">p19</t>
         </is>
       </c>
       <c r="G399" t="inlineStr">
@@ -32770,17 +32880,17 @@
       </c>
       <c r="H399" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-10</t>
+          <t xml:space="preserve">2026-07-31</t>
         </is>
       </c>
       <c r="I399" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/8/2026</t>
+          <t xml:space="preserve">31-07-26</t>
         </is>
       </c>
       <c r="K399" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L399" t="inlineStr">
@@ -32790,12 +32900,12 @@
       </c>
       <c r="M399" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N399" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O399" t="inlineStr">
@@ -32803,6 +32913,16 @@
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
+      <c r="P399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">to-do</t>
+        </is>
+      </c>
+      <c r="Q399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">to-do box / thaw</t>
+        </is>
+      </c>
       <c r="R399" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
@@ -32810,39 +32930,39 @@
       </c>
       <c r="S399" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-354</t>
+          <t xml:space="preserve">v-233</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="E400" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="F400" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p?</t>
         </is>
       </c>
       <c r="G400" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H400" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2025-06-30</t>
         </is>
       </c>
       <c r="I400" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">30-06-25</t>
         </is>
       </c>
       <c r="K400" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="L400" t="inlineStr">
@@ -32862,7 +32982,7 @@
       </c>
       <c r="O400" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R400" t="inlineStr">
@@ -32872,19 +32992,19 @@
       </c>
       <c r="S400" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdx0po-0</t>
+          <t xml:space="preserve">v-295</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="E401" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="F401" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p11</t>
         </is>
       </c>
       <c r="G401" t="inlineStr">
@@ -32894,27 +33014,27 @@
       </c>
       <c r="H401" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-06-12</t>
         </is>
       </c>
       <c r="I401" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">12/6/2026</t>
         </is>
       </c>
       <c r="K401" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L401" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M401" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N401" t="inlineStr">
@@ -32934,44 +33054,44 @@
       </c>
       <c r="S401" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdxsum-0</t>
+          <t xml:space="preserve">v-311</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="E402" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F402" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p+17</t>
         </is>
       </c>
       <c r="G402" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H402" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-03-30</t>
         </is>
       </c>
       <c r="I402" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">30-03-26</t>
         </is>
       </c>
       <c r="K402" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L402" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M402" t="inlineStr">
@@ -32981,7 +33101,7 @@
       </c>
       <c r="N402" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O402" t="inlineStr">
@@ -32996,44 +33116,44 @@
       </c>
       <c r="S402" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-0</t>
+          <t xml:space="preserve">v-320</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="E403" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">LnCap Canada</t>
         </is>
       </c>
       <c r="F403" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p+14</t>
         </is>
       </c>
       <c r="G403" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H403" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-03-23</t>
         </is>
       </c>
       <c r="I403" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">23-03-26</t>
         </is>
       </c>
       <c r="K403" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L403" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M403" t="inlineStr">
@@ -33058,19 +33178,19 @@
       </c>
       <c r="S403" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-1</t>
+          <t xml:space="preserve">v-321</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="E404" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="F404" t="inlineStr">
         <is>
-          <t xml:space="preserve">p28</t>
+          <t xml:space="preserve">p16</t>
         </is>
       </c>
       <c r="G404" t="inlineStr">
@@ -33080,12 +33200,12 @@
       </c>
       <c r="H404" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2025-11-06</t>
         </is>
       </c>
       <c r="I404" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">6/11/2025</t>
         </is>
       </c>
       <c r="K404" t="inlineStr">
@@ -33095,7 +33215,7 @@
       </c>
       <c r="L404" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M404" t="inlineStr">
@@ -33120,19 +33240,19 @@
       </c>
       <c r="S404" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdz1vx-0</t>
+          <t xml:space="preserve">v-338</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="E405" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="F405" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p15</t>
         </is>
       </c>
       <c r="G405" t="inlineStr">
@@ -33142,12 +33262,12 @@
       </c>
       <c r="H405" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-08-10</t>
         </is>
       </c>
       <c r="I405" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">10/8/2026</t>
         </is>
       </c>
       <c r="K405" t="inlineStr">
@@ -33172,7 +33292,7 @@
       </c>
       <c r="O405" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R405" t="inlineStr">
@@ -33182,19 +33302,19 @@
       </c>
       <c r="S405" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdzpx7-0</t>
+          <t xml:space="preserve">v-354</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="E406" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="F406" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G406" t="inlineStr">
@@ -33214,12 +33334,12 @@
       </c>
       <c r="K406" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L406" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M406" t="inlineStr">
@@ -33234,7 +33354,7 @@
       </c>
       <c r="O406" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R406" t="inlineStr">
@@ -33244,19 +33364,19 @@
       </c>
       <c r="S406" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0daw-0</t>
+          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="E407" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="F407" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G407" t="inlineStr">
@@ -33276,12 +33396,12 @@
       </c>
       <c r="K407" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L407" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M407" t="inlineStr">
@@ -33306,19 +33426,19 @@
       </c>
       <c r="S407" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0w3q-0</t>
+          <t xml:space="preserve">v-mtrdxsum-0</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="E408" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="F408" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G408" t="inlineStr">
@@ -33338,12 +33458,12 @@
       </c>
       <c r="K408" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L408" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M408" t="inlineStr">
@@ -33368,19 +33488,19 @@
       </c>
       <c r="S408" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre1ko0-0</t>
+          <t xml:space="preserve">v-mtrdyhss-0</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="E409" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="F409" t="inlineStr">
         <is>
-          <t xml:space="preserve">p6</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G409" t="inlineStr">
@@ -33390,12 +33510,12 @@
       </c>
       <c r="H409" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I409" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="K409" t="inlineStr">
@@ -33405,7 +33525,7 @@
       </c>
       <c r="L409" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M409" t="inlineStr">
@@ -33415,7 +33535,7 @@
       </c>
       <c r="N409" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">No Casp</t>
         </is>
       </c>
       <c r="O409" t="inlineStr">
@@ -33430,29 +33550,39 @@
       </c>
       <c r="S409" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtski3re-0</t>
+          <t xml:space="preserve">v-mtrdyhss-1</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="E410" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p28</t>
         </is>
       </c>
       <c r="G410" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H410" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I410" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L410" t="inlineStr">
@@ -33482,29 +33612,39 @@
       </c>
       <c r="S410" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt0h140-0</t>
+          <t xml:space="preserve">v-mtrdz1vx-0</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="E411" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">Huh7 gNT</t>
+        </is>
+      </c>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G411" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H411" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I411" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L411" t="inlineStr">
@@ -33524,7 +33664,7 @@
       </c>
       <c r="O411" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R411" t="inlineStr">
@@ -33534,34 +33674,44 @@
       </c>
       <c r="S411" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-0</t>
+          <t xml:space="preserve">v-mtrdzpx7-0</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="E412" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G412" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H412" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I412" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L412" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M412" t="inlineStr">
@@ -33586,34 +33736,44 @@
       </c>
       <c r="S412" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtre0daw-0</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="E413" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G413" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H413" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I413" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K413" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L413" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M413" t="inlineStr">
@@ -33638,34 +33798,44 @@
       </c>
       <c r="S413" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-2</t>
+          <t xml:space="preserve">v-mtre0w3q-0</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="E414" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G414" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H414" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I414" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L414" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M414" t="inlineStr">
@@ -33690,29 +33860,39 @@
       </c>
       <c r="S414" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt5ckqo-0</t>
+          <t xml:space="preserve">v-mtre1ko0-0</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="E415" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">Hek caspex</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p6</t>
         </is>
       </c>
       <c r="G415" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H415" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I415" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="K415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L415" t="inlineStr">
@@ -33727,7 +33907,7 @@
       </c>
       <c r="N415" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O415" t="inlineStr">
@@ -33742,14 +33922,14 @@
       </c>
       <c r="S415" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmw7m-0</t>
+          <t xml:space="preserve">v-mtski3re-0</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="E416" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="G416" t="inlineStr">
@@ -33759,17 +33939,17 @@
       </c>
       <c r="H416" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I416" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="L416" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M416" t="inlineStr">
@@ -33794,14 +33974,14 @@
       </c>
       <c r="S416" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmypa-0</t>
+          <t xml:space="preserve">v-mtt0h140-0</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="E417" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="G417" t="inlineStr">
@@ -33811,12 +33991,12 @@
       </c>
       <c r="H417" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I417" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="L417" t="inlineStr">
@@ -33846,14 +34026,14 @@
       </c>
       <c r="S417" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmn045-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="E418" t="inlineStr">
         <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="G418" t="inlineStr">
@@ -33863,17 +34043,12 @@
       </c>
       <c r="H418" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I418" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
-        </is>
-      </c>
-      <c r="K418" t="inlineStr">
-        <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="L418" t="inlineStr">
@@ -33903,67 +34078,384 @@
       </c>
       <c r="S418" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtu5lgdc-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="E419" t="inlineStr">
         <is>
+          <t xml:space="preserve">jkl</t>
+        </is>
+      </c>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt3mo6u-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="E420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">khk</t>
+        </is>
+      </c>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt5ckqo-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="E421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="G421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mttmmw7m-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="E422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="G422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mttmmypa-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="E423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="G423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mttmn045-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="E424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deneme</t>
+        </is>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="K424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deneme</t>
+        </is>
+      </c>
+      <c r="L424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtu5lgdc-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="E425" t="inlineStr">
+        <is>
           <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
-      <c r="F419" t="inlineStr">
+      <c r="F425" t="inlineStr">
         <is>
           <t xml:space="preserve">p19</t>
         </is>
       </c>
-      <c r="G419" t="inlineStr">
+      <c r="G425" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H419" t="inlineStr">
+      <c r="H425" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-17</t>
         </is>
       </c>
-      <c r="I419" t="inlineStr">
+      <c r="I425" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-09-17</t>
         </is>
       </c>
-      <c r="K419" t="inlineStr">
+      <c r="K425" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L419" t="inlineStr">
+      <c r="L425" t="inlineStr">
         <is>
           <t xml:space="preserve">FLAG</t>
         </is>
       </c>
-      <c r="M419" t="inlineStr">
+      <c r="M425" t="inlineStr">
         <is>
           <t xml:space="preserve">Par</t>
         </is>
       </c>
-      <c r="N419" t="inlineStr">
+      <c r="N425" t="inlineStr">
         <is>
           <t xml:space="preserve">No Casp</t>
         </is>
       </c>
-      <c r="O419" t="inlineStr">
+      <c r="O425" t="inlineStr">
         <is>
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
-      <c r="R419" t="inlineStr">
+      <c r="R425" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
-      <c r="S419" t="inlineStr">
+      <c r="S425" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mu5anec8-0</t>
         </is>
@@ -34016,12 +34508,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -34035,24 +34527,24 @@
         </is>
       </c>
       <c r="E2">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F2">
         <v>1</v>
       </c>
       <c r="G2">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">LnCap Canada</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -34066,24 +34558,24 @@
         </is>
       </c>
       <c r="E3">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F3">
         <v>1</v>
       </c>
       <c r="G3">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -34097,13 +34589,13 @@
         </is>
       </c>
       <c r="E4">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F4">
         <v>1</v>
       </c>
       <c r="G4">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -41636,10 +42128,10 @@
         <v>81</v>
       </c>
       <c r="I18">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="J18">
-        <v>70</v>
+        <v>64</v>
       </c>
     </row>
     <row r="19">

</xml_diff>

<commit_message>
Take out Huh7 from Umut
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -32244,17 +32244,17 @@
       </c>
       <c r="D391" t="inlineStr">
         <is>
-          <t xml:space="preserve">B7</t>
+          <t xml:space="preserve">C1</t>
         </is>
       </c>
       <c r="E391" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK</t>
         </is>
       </c>
       <c r="F391" t="inlineStr">
         <is>
-          <t xml:space="preserve">18</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="G391" t="inlineStr">
@@ -32274,7 +32274,7 @@
       </c>
       <c r="K391" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L391" t="inlineStr">
@@ -32304,7 +32304,7 @@
       </c>
       <c r="S391" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv4yequa-5</t>
+          <t xml:space="preserve">v-mv4ye7g5-0</t>
         </is>
       </c>
     </row>
@@ -32316,27 +32316,27 @@
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t xml:space="preserve">Umut Cell Box -5-</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="D392" t="inlineStr">
         <is>
-          <t xml:space="preserve">C1</t>
+          <t xml:space="preserve">A1</t>
         </is>
       </c>
       <c r="E392" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="F392" t="inlineStr">
         <is>
-          <t xml:space="preserve">7</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G392" t="inlineStr">
@@ -32346,17 +32346,17 @@
       </c>
       <c r="H392" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-09</t>
+          <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
       <c r="I392" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-09</t>
+          <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
       <c r="K392" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L392" t="inlineStr">
@@ -32386,7 +32386,7 @@
       </c>
       <c r="S392" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv4ye7g5-0</t>
+          <t xml:space="preserve">v-mupot2zh-0</t>
         </is>
       </c>
     </row>
@@ -32408,7 +32408,7 @@
       </c>
       <c r="D393" t="inlineStr">
         <is>
-          <t xml:space="preserve">A1</t>
+          <t xml:space="preserve">A2</t>
         </is>
       </c>
       <c r="E393" t="inlineStr">
@@ -32468,7 +32468,7 @@
       </c>
       <c r="S393" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-0</t>
+          <t xml:space="preserve">v-mupot2zh-1</t>
         </is>
       </c>
     </row>
@@ -32490,7 +32490,7 @@
       </c>
       <c r="D394" t="inlineStr">
         <is>
-          <t xml:space="preserve">A2</t>
+          <t xml:space="preserve">A3</t>
         </is>
       </c>
       <c r="E394" t="inlineStr">
@@ -32550,7 +32550,7 @@
       </c>
       <c r="S394" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-1</t>
+          <t xml:space="preserve">v-mupot2zh-2</t>
         </is>
       </c>
     </row>
@@ -32572,7 +32572,7 @@
       </c>
       <c r="D395" t="inlineStr">
         <is>
-          <t xml:space="preserve">A3</t>
+          <t xml:space="preserve">A4</t>
         </is>
       </c>
       <c r="E395" t="inlineStr">
@@ -32632,7 +32632,7 @@
       </c>
       <c r="S395" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-2</t>
+          <t xml:space="preserve">v-mupot2zh-3</t>
         </is>
       </c>
     </row>
@@ -32654,7 +32654,7 @@
       </c>
       <c r="D396" t="inlineStr">
         <is>
-          <t xml:space="preserve">A4</t>
+          <t xml:space="preserve">A5</t>
         </is>
       </c>
       <c r="E396" t="inlineStr">
@@ -32714,59 +32714,39 @@
       </c>
       <c r="S396" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-3</t>
+          <t xml:space="preserve">v-mupot2zh-4</t>
         </is>
       </c>
     </row>
     <row r="397">
-      <c r="A397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Freezer 1</t>
-        </is>
-      </c>
-      <c r="B397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rack 2</t>
-        </is>
-      </c>
-      <c r="C397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Common Box #1</t>
-        </is>
-      </c>
-      <c r="D397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A5</t>
-        </is>
-      </c>
       <c r="E397" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F397" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p+21</t>
         </is>
       </c>
       <c r="G397" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H397" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-05-15</t>
         </is>
       </c>
       <c r="I397" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">15-05-26</t>
         </is>
       </c>
       <c r="K397" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L397" t="inlineStr">
@@ -32781,7 +32761,7 @@
       </c>
       <c r="N397" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O397" t="inlineStr">
@@ -32791,44 +32771,44 @@
       </c>
       <c r="R397" t="inlineStr">
         <is>
-          <t xml:space="preserve">stored</t>
+          <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
       <c r="S397" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-4</t>
+          <t xml:space="preserve">v-199</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="E398" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX</t>
+          <t xml:space="preserve">LUCX</t>
         </is>
       </c>
       <c r="F398" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+21</t>
+          <t xml:space="preserve">p19</t>
         </is>
       </c>
       <c r="G398" t="inlineStr">
         <is>
-          <t xml:space="preserve">relative</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H398" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-05-15</t>
+          <t xml:space="preserve">2026-07-31</t>
         </is>
       </c>
       <c r="I398" t="inlineStr">
         <is>
-          <t xml:space="preserve">15-05-26</t>
+          <t xml:space="preserve">31-07-26</t>
         </is>
       </c>
       <c r="K398" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L398" t="inlineStr">
@@ -32838,7 +32818,7 @@
       </c>
       <c r="M398" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N398" t="inlineStr">
@@ -32851,6 +32831,16 @@
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
+      <c r="P398" t="inlineStr">
+        <is>
+          <t xml:space="preserve">to-do</t>
+        </is>
+      </c>
+      <c r="Q398" t="inlineStr">
+        <is>
+          <t xml:space="preserve">to-do box / thaw</t>
+        </is>
+      </c>
       <c r="R398" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
@@ -32858,39 +32848,39 @@
       </c>
       <c r="S398" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-199</t>
+          <t xml:space="preserve">v-233</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="E399" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="F399" t="inlineStr">
         <is>
-          <t xml:space="preserve">p19</t>
+          <t xml:space="preserve">p?</t>
         </is>
       </c>
       <c r="G399" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H399" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-07-31</t>
+          <t xml:space="preserve">2025-06-30</t>
         </is>
       </c>
       <c r="I399" t="inlineStr">
         <is>
-          <t xml:space="preserve">31-07-26</t>
+          <t xml:space="preserve">30-06-25</t>
         </is>
       </c>
       <c r="K399" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="L399" t="inlineStr">
@@ -32900,12 +32890,12 @@
       </c>
       <c r="M399" t="inlineStr">
         <is>
-          <t xml:space="preserve">CR</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N399" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">No Casp</t>
         </is>
       </c>
       <c r="O399" t="inlineStr">
@@ -32913,16 +32903,6 @@
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
-      <c r="P399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">to-do</t>
-        </is>
-      </c>
-      <c r="Q399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">to-do box / thaw</t>
-        </is>
-      </c>
       <c r="R399" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
@@ -32930,39 +32910,39 @@
       </c>
       <c r="S399" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-233</t>
+          <t xml:space="preserve">v-295</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="E400" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="F400" t="inlineStr">
         <is>
-          <t xml:space="preserve">p?</t>
+          <t xml:space="preserve">p11</t>
         </is>
       </c>
       <c r="G400" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H400" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-06-30</t>
+          <t xml:space="preserve">2026-06-12</t>
         </is>
       </c>
       <c r="I400" t="inlineStr">
         <is>
-          <t xml:space="preserve">30-06-25</t>
+          <t xml:space="preserve">12/6/2026</t>
         </is>
       </c>
       <c r="K400" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L400" t="inlineStr">
@@ -32972,7 +32952,7 @@
       </c>
       <c r="M400" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N400" t="inlineStr">
@@ -32992,39 +32972,39 @@
       </c>
       <c r="S400" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-295</t>
+          <t xml:space="preserve">v-311</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="E401" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F401" t="inlineStr">
         <is>
-          <t xml:space="preserve">p11</t>
+          <t xml:space="preserve">p+17</t>
         </is>
       </c>
       <c r="G401" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H401" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-06-12</t>
+          <t xml:space="preserve">2026-03-30</t>
         </is>
       </c>
       <c r="I401" t="inlineStr">
         <is>
-          <t xml:space="preserve">12/6/2026</t>
+          <t xml:space="preserve">30-03-26</t>
         </is>
       </c>
       <c r="K401" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L401" t="inlineStr">
@@ -33034,12 +33014,12 @@
       </c>
       <c r="M401" t="inlineStr">
         <is>
-          <t xml:space="preserve">CR</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N401" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O401" t="inlineStr">
@@ -33054,19 +33034,19 @@
       </c>
       <c r="S401" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-311</t>
+          <t xml:space="preserve">v-320</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="E402" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX</t>
+          <t xml:space="preserve">LnCap Canada</t>
         </is>
       </c>
       <c r="F402" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+17</t>
+          <t xml:space="preserve">p+14</t>
         </is>
       </c>
       <c r="G402" t="inlineStr">
@@ -33076,12 +33056,12 @@
       </c>
       <c r="H402" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-03-30</t>
+          <t xml:space="preserve">2026-03-23</t>
         </is>
       </c>
       <c r="I402" t="inlineStr">
         <is>
-          <t xml:space="preserve">30-03-26</t>
+          <t xml:space="preserve">23-03-26</t>
         </is>
       </c>
       <c r="K402" t="inlineStr">
@@ -33101,7 +33081,7 @@
       </c>
       <c r="N402" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">No Casp</t>
         </is>
       </c>
       <c r="O402" t="inlineStr">
@@ -33116,39 +33096,39 @@
       </c>
       <c r="S402" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-320</t>
+          <t xml:space="preserve">v-321</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="E403" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="F403" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+14</t>
+          <t xml:space="preserve">p16</t>
         </is>
       </c>
       <c r="G403" t="inlineStr">
         <is>
-          <t xml:space="preserve">relative</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H403" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-03-23</t>
+          <t xml:space="preserve">2025-11-06</t>
         </is>
       </c>
       <c r="I403" t="inlineStr">
         <is>
-          <t xml:space="preserve">23-03-26</t>
+          <t xml:space="preserve">6/11/2025</t>
         </is>
       </c>
       <c r="K403" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L403" t="inlineStr">
@@ -33178,19 +33158,19 @@
       </c>
       <c r="S403" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-321</t>
+          <t xml:space="preserve">v-338</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="E404" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="F404" t="inlineStr">
         <is>
-          <t xml:space="preserve">p16</t>
+          <t xml:space="preserve">p15</t>
         </is>
       </c>
       <c r="G404" t="inlineStr">
@@ -33200,17 +33180,17 @@
       </c>
       <c r="H404" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-11-06</t>
+          <t xml:space="preserve">2026-08-10</t>
         </is>
       </c>
       <c r="I404" t="inlineStr">
         <is>
-          <t xml:space="preserve">6/11/2025</t>
+          <t xml:space="preserve">10/8/2026</t>
         </is>
       </c>
       <c r="K404" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L404" t="inlineStr">
@@ -33240,19 +33220,19 @@
       </c>
       <c r="S404" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-338</t>
+          <t xml:space="preserve">v-354</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="E405" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="F405" t="inlineStr">
         <is>
-          <t xml:space="preserve">p15</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G405" t="inlineStr">
@@ -33262,17 +33242,17 @@
       </c>
       <c r="H405" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-10</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I405" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/8/2026</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="K405" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L405" t="inlineStr">
@@ -33292,7 +33272,7 @@
       </c>
       <c r="O405" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R405" t="inlineStr">
@@ -33302,14 +33282,14 @@
       </c>
       <c r="S405" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-354</t>
+          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="E406" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="F406" t="inlineStr">
@@ -33339,7 +33319,7 @@
       </c>
       <c r="L406" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M406" t="inlineStr">
@@ -33354,7 +33334,7 @@
       </c>
       <c r="O406" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R406" t="inlineStr">
@@ -33364,14 +33344,14 @@
       </c>
       <c r="S406" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdx0po-0</t>
+          <t xml:space="preserve">v-mtrdxsum-0</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="E407" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="F407" t="inlineStr">
@@ -33401,7 +33381,7 @@
       </c>
       <c r="L407" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M407" t="inlineStr">
@@ -33426,7 +33406,7 @@
       </c>
       <c r="S407" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdxsum-0</t>
+          <t xml:space="preserve">v-mtrdyhss-0</t>
         </is>
       </c>
     </row>
@@ -33488,19 +33468,19 @@
       </c>
       <c r="S408" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-0</t>
+          <t xml:space="preserve">v-mtrdyhss-1</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="E409" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="F409" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p28</t>
         </is>
       </c>
       <c r="G409" t="inlineStr">
@@ -33525,7 +33505,7 @@
       </c>
       <c r="L409" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M409" t="inlineStr">
@@ -33550,19 +33530,19 @@
       </c>
       <c r="S409" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-1</t>
+          <t xml:space="preserve">v-mtrdz1vx-0</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="E410" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7 gNT</t>
         </is>
       </c>
       <c r="F410" t="inlineStr">
         <is>
-          <t xml:space="preserve">p28</t>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G410" t="inlineStr">
@@ -33582,12 +33562,12 @@
       </c>
       <c r="K410" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L410" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M410" t="inlineStr">
@@ -33602,7 +33582,7 @@
       </c>
       <c r="O410" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R410" t="inlineStr">
@@ -33612,19 +33592,19 @@
       </c>
       <c r="S410" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdz1vx-0</t>
+          <t xml:space="preserve">v-mtrdzpx7-0</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="E411" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="F411" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G411" t="inlineStr">
@@ -33649,7 +33629,7 @@
       </c>
       <c r="L411" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M411" t="inlineStr">
@@ -33664,7 +33644,7 @@
       </c>
       <c r="O411" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R411" t="inlineStr">
@@ -33674,19 +33654,19 @@
       </c>
       <c r="S411" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdzpx7-0</t>
+          <t xml:space="preserve">v-mtre0daw-0</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="E412" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="F412" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G412" t="inlineStr">
@@ -33711,7 +33691,7 @@
       </c>
       <c r="L412" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M412" t="inlineStr">
@@ -33736,19 +33716,19 @@
       </c>
       <c r="S412" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0daw-0</t>
+          <t xml:space="preserve">v-mtre0w3q-0</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="E413" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="F413" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G413" t="inlineStr">
@@ -33773,7 +33753,7 @@
       </c>
       <c r="L413" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M413" t="inlineStr">
@@ -33798,19 +33778,19 @@
       </c>
       <c r="S413" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0w3q-0</t>
+          <t xml:space="preserve">v-mtre1ko0-0</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="E414" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Hek caspex</t>
         </is>
       </c>
       <c r="F414" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p6</t>
         </is>
       </c>
       <c r="G414" t="inlineStr">
@@ -33820,22 +33800,22 @@
       </c>
       <c r="H414" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I414" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="K414" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L414" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M414" t="inlineStr">
@@ -33845,7 +33825,7 @@
       </c>
       <c r="N414" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O414" t="inlineStr">
@@ -33860,24 +33840,19 @@
       </c>
       <c r="S414" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre1ko0-0</t>
+          <t xml:space="preserve">v-mtski3re-0</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="E415" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
-        </is>
-      </c>
-      <c r="F415" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p6</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="G415" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H415" t="inlineStr">
@@ -33890,14 +33865,9 @@
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
-      <c r="K415" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
       <c r="L415" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M415" t="inlineStr">
@@ -33907,7 +33877,7 @@
       </c>
       <c r="N415" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">No Casp</t>
         </is>
       </c>
       <c r="O415" t="inlineStr">
@@ -33922,14 +33892,14 @@
       </c>
       <c r="S415" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtski3re-0</t>
+          <t xml:space="preserve">v-mtt0h140-0</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="E416" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="G416" t="inlineStr">
@@ -33949,7 +33919,7 @@
       </c>
       <c r="L416" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M416" t="inlineStr">
@@ -33974,7 +33944,7 @@
       </c>
       <c r="S416" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt0h140-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
         </is>
       </c>
     </row>
@@ -34026,7 +33996,7 @@
       </c>
       <c r="S417" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
         </is>
       </c>
     </row>
@@ -34078,14 +34048,14 @@
       </c>
       <c r="S418" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtt3mo6u-2</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="E419" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">khk</t>
         </is>
       </c>
       <c r="G419" t="inlineStr">
@@ -34130,14 +34100,14 @@
       </c>
       <c r="S419" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-2</t>
+          <t xml:space="preserve">v-mtt5ckqo-0</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="E420" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">kkk</t>
         </is>
       </c>
       <c r="G420" t="inlineStr">
@@ -34147,12 +34117,12 @@
       </c>
       <c r="H420" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
       <c r="I420" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
       <c r="L420" t="inlineStr">
@@ -34182,7 +34152,7 @@
       </c>
       <c r="S420" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt5ckqo-0</t>
+          <t xml:space="preserve">v-mttmmw7m-0</t>
         </is>
       </c>
     </row>
@@ -34234,7 +34204,7 @@
       </c>
       <c r="S421" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmw7m-0</t>
+          <t xml:space="preserve">v-mttmmypa-0</t>
         </is>
       </c>
     </row>
@@ -34286,14 +34256,14 @@
       </c>
       <c r="S422" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmypa-0</t>
+          <t xml:space="preserve">v-mttmn045-0</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="E423" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">deneme</t>
         </is>
       </c>
       <c r="G423" t="inlineStr">
@@ -34311,6 +34281,11 @@
           <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
+      <c r="K423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deneme</t>
+        </is>
+      </c>
       <c r="L423" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -34338,39 +34313,44 @@
       </c>
       <c r="S423" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmn045-0</t>
+          <t xml:space="preserve">v-mtu5lgdc-0</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="E424" t="inlineStr">
         <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p19</t>
         </is>
       </c>
       <c r="G424" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H424" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-17</t>
         </is>
       </c>
       <c r="I424" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-17</t>
         </is>
       </c>
       <c r="K424" t="inlineStr">
         <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L424" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M424" t="inlineStr">
@@ -34395,19 +34375,19 @@
       </c>
       <c r="S424" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtu5lgdc-0</t>
+          <t xml:space="preserve">v-mu5anec8-0</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="E425" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="F425" t="inlineStr">
         <is>
-          <t xml:space="preserve">p19</t>
+          <t xml:space="preserve">18</t>
         </is>
       </c>
       <c r="G425" t="inlineStr">
@@ -34417,12 +34397,12 @@
       </c>
       <c r="H425" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-17</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="I425" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-17</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="K425" t="inlineStr">
@@ -34432,7 +34412,7 @@
       </c>
       <c r="L425" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M425" t="inlineStr">
@@ -34457,7 +34437,7 @@
       </c>
       <c r="S425" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mu5anec8-0</t>
+          <t xml:space="preserve">v-mv4yequa-5</t>
         </is>
       </c>
     </row>
@@ -34527,10 +34507,10 @@
         </is>
       </c>
       <c r="E2">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G2">
         <v>5</v>
@@ -39240,12 +39220,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-09</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -39260,12 +39240,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">UMUT CELLS -4-</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve">A7</t>
+          <t xml:space="preserve">B7</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -39280,7 +39260,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-1</t>
+          <t xml:space="preserve">v-mv4yequa-5</t>
         </is>
       </c>
     </row>
@@ -39292,7 +39272,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -39312,7 +39292,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve">D3</t>
+          <t xml:space="preserve">A7</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -39327,19 +39307,19 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mu5anec8-0</t>
+          <t xml:space="preserve">v-mtrdyhss-1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -39354,12 +39334,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ONGOING</t>
+          <t xml:space="preserve">UMUT CELLS -4-</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve">I4</t>
+          <t xml:space="preserve">D3</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -39374,7 +39354,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-320</t>
+          <t xml:space="preserve">v-mu5anec8-0</t>
         </is>
       </c>
     </row>
@@ -39401,12 +39381,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">DUZENLE</t>
+          <t xml:space="preserve">ONGOING</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve">D9</t>
+          <t xml:space="preserve">I4</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -39421,19 +39401,19 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-199</t>
+          <t xml:space="preserve">v-320</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-29</t>
+          <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -39448,12 +39428,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">UMUT CELLS -4-</t>
+          <t xml:space="preserve">DUZENLE</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">D2</t>
+          <t xml:space="preserve">D9</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -39468,7 +39448,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-354</t>
+          <t xml:space="preserve">v-199</t>
         </is>
       </c>
     </row>
@@ -39480,7 +39460,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -39495,12 +39475,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">DUZENLE</t>
+          <t xml:space="preserve">UMUT CELLS -4-</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve">H7</t>
+          <t xml:space="preserve">D2</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -39515,19 +39495,19 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-233</t>
+          <t xml:space="preserve">v-354</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-24</t>
+          <t xml:space="preserve">2026-09-29</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LUCX</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -39542,17 +39522,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ONGOING</t>
+          <t xml:space="preserve">DUZENLE</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">H4</t>
+          <t xml:space="preserve">H7</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown device</t>
+          <t xml:space="preserve">Umut</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -39562,7 +39542,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-311</t>
+          <t xml:space="preserve">v-233</t>
         </is>
       </c>
     </row>
@@ -39574,7 +39554,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -39594,7 +39574,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve">I5</t>
+          <t xml:space="preserve">H4</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -39609,7 +39589,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-321</t>
+          <t xml:space="preserve">v-311</t>
         </is>
       </c>
     </row>
@@ -39621,7 +39601,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap Canada</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -39636,12 +39616,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">UMUT CELLS -4-</t>
+          <t xml:space="preserve">ONGOING</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve">B4</t>
+          <t xml:space="preserve">I5</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -39656,19 +39636,19 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-338</t>
+          <t xml:space="preserve">v-321</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-11</t>
+          <t xml:space="preserve">2026-09-24</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -39688,7 +39668,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve">H1</t>
+          <t xml:space="preserve">B4</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -39703,19 +39683,19 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmw7m-0</t>
+          <t xml:space="preserve">v-338</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-10</t>
+          <t xml:space="preserve">2026-09-11</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">kkk</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -39730,12 +39710,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">ONGOING</t>
+          <t xml:space="preserve">UMUT CELLS -4-</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t xml:space="preserve">F6</t>
+          <t xml:space="preserve">H1</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -39750,19 +39730,19 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-295</t>
+          <t xml:space="preserve">v-mttmmw7m-0</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -39772,17 +39752,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">ONGOING</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t xml:space="preserve">A4</t>
+          <t xml:space="preserve">F6</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -39797,7 +39777,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-2</t>
+          <t xml:space="preserve">v-295</t>
         </is>
       </c>
     </row>
@@ -39829,7 +39809,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t xml:space="preserve">A3</t>
+          <t xml:space="preserve">A4</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -39844,7 +39824,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtt3mo6u-2</t>
         </is>
       </c>
     </row>
@@ -39876,7 +39856,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t xml:space="preserve">A2</t>
+          <t xml:space="preserve">A3</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -39891,7 +39871,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
         </is>
       </c>
     </row>
@@ -39903,7 +39883,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -39923,7 +39903,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t xml:space="preserve">A1</t>
+          <t xml:space="preserve">A2</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -39938,7 +39918,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt0h140-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
         </is>
       </c>
     </row>
@@ -39950,7 +39930,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -39960,17 +39940,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">UMUT CELLS -4-</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t xml:space="preserve">H3</t>
+          <t xml:space="preserve">A1</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -39985,7 +39965,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmn045-0</t>
+          <t xml:space="preserve">v-mtt0h140-0</t>
         </is>
       </c>
     </row>
@@ -40017,7 +39997,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t xml:space="preserve">H2</t>
+          <t xml:space="preserve">H3</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -40032,7 +40012,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmypa-0</t>
+          <t xml:space="preserve">v-mttmn045-0</t>
         </is>
       </c>
     </row>
@@ -40044,7 +40024,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">kkk</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -40054,17 +40034,17 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">UMUT CELLS -4-</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t xml:space="preserve">B3</t>
+          <t xml:space="preserve">H2</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -40079,19 +40059,19 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtu5lgdc-0</t>
+          <t xml:space="preserve">v-mttmmypa-0</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">deneme</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -40101,17 +40081,17 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 1</t>
+          <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t xml:space="preserve">DUZENLE</t>
+          <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t xml:space="preserve">I8</t>
+          <t xml:space="preserve">B3</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -40126,7 +40106,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtski3re-0</t>
+          <t xml:space="preserve">v-mtu5lgdc-0</t>
         </is>
       </c>
     </row>
@@ -40138,7 +40118,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">Hek caspex</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -40153,12 +40133,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t xml:space="preserve">UMUT CELLS -4-</t>
+          <t xml:space="preserve">DUZENLE</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t xml:space="preserve">A4</t>
+          <t xml:space="preserve">I8</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -40173,7 +40153,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdxsum-0</t>
+          <t xml:space="preserve">v-mtski3re-0</t>
         </is>
       </c>
     </row>
@@ -40185,7 +40165,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -40205,7 +40185,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t xml:space="preserve">A6</t>
+          <t xml:space="preserve">A4</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -40220,7 +40200,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-0</t>
+          <t xml:space="preserve">v-mtrdxsum-0</t>
         </is>
       </c>
     </row>
@@ -40232,7 +40212,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -40252,7 +40232,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t xml:space="preserve">A8</t>
+          <t xml:space="preserve">A6</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -40267,7 +40247,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdz1vx-0</t>
+          <t xml:space="preserve">v-mtrdyhss-0</t>
         </is>
       </c>
     </row>
@@ -40279,7 +40259,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -40294,12 +40274,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t xml:space="preserve">DUZENLE</t>
+          <t xml:space="preserve">UMUT CELLS -4-</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t xml:space="preserve">E6</t>
+          <t xml:space="preserve">A8</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -40314,7 +40294,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdzpx7-0</t>
+          <t xml:space="preserve">v-mtrdz1vx-0</t>
         </is>
       </c>
     </row>
@@ -40326,7 +40306,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">Huh7 gNT</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -40346,7 +40326,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t xml:space="preserve">E8</t>
+          <t xml:space="preserve">E6</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -40361,7 +40341,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0daw-0</t>
+          <t xml:space="preserve">v-mtrdzpx7-0</t>
         </is>
       </c>
     </row>
@@ -40373,7 +40353,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -40388,12 +40368,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">UMUT CELLS -4-</t>
+          <t xml:space="preserve">DUZENLE</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t xml:space="preserve">B8</t>
+          <t xml:space="preserve">E8</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -40408,7 +40388,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdx0po-0</t>
+          <t xml:space="preserve">v-mtre0daw-0</t>
         </is>
       </c>
     </row>
@@ -40420,7 +40400,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -40440,7 +40420,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t xml:space="preserve">D5</t>
+          <t xml:space="preserve">B8</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -40455,7 +40435,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre1ko0-0</t>
+          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
@@ -40467,7 +40447,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -40487,7 +40467,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t xml:space="preserve">D3</t>
+          <t xml:space="preserve">D5</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -40502,7 +40482,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0w3q-0</t>
+          <t xml:space="preserve">v-mtre1ko0-0</t>
         </is>
       </c>
     </row>
@@ -40514,7 +40494,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -40524,17 +40504,17 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">UMUT CELLS -4-</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t xml:space="preserve">D4</t>
+          <t xml:space="preserve">D3</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -40549,7 +40529,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt5ckqo-0</t>
+          <t xml:space="preserve">v-mtre0w3q-0</t>
         </is>
       </c>
     </row>
@@ -40561,7 +40541,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">khk</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -40581,7 +40561,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t xml:space="preserve">A1</t>
+          <t xml:space="preserve">D4</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -40596,7 +40576,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt0h140-0</t>
+          <t xml:space="preserve">v-mtt5ckqo-0</t>
         </is>
       </c>
     </row>
@@ -40608,7 +40588,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -40628,7 +40608,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t xml:space="preserve">A2</t>
+          <t xml:space="preserve">A1</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -40643,7 +40623,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-0</t>
+          <t xml:space="preserve">v-mtt0h140-0</t>
         </is>
       </c>
     </row>
@@ -40675,7 +40655,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t xml:space="preserve">A3</t>
+          <t xml:space="preserve">A2</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -40690,7 +40670,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
         </is>
       </c>
     </row>
@@ -40722,7 +40702,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t xml:space="preserve">A4</t>
+          <t xml:space="preserve">A3</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -40737,7 +40717,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-2</t>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
         </is>
       </c>
     </row>
@@ -40749,7 +40729,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -40769,7 +40749,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t xml:space="preserve">A1</t>
+          <t xml:space="preserve">A4</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -40784,7 +40764,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt0h140-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-2</t>
         </is>
       </c>
     </row>
@@ -40796,7 +40776,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -40816,7 +40796,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t xml:space="preserve">A2</t>
+          <t xml:space="preserve">A1</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -40831,7 +40811,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-0</t>
+          <t xml:space="preserve">v-mtt0h140-0</t>
         </is>
       </c>
     </row>
@@ -40843,7 +40823,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -40863,7 +40843,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t xml:space="preserve">A1</t>
+          <t xml:space="preserve">A2</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -40878,7 +40858,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt0h140-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
         </is>
       </c>
     </row>
@@ -40890,7 +40870,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -40910,7 +40890,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t xml:space="preserve">A2</t>
+          <t xml:space="preserve">A1</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -40925,7 +40905,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-0</t>
+          <t xml:space="preserve">v-mtt0h140-0</t>
         </is>
       </c>
     </row>
@@ -40957,7 +40937,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t xml:space="preserve">A3</t>
+          <t xml:space="preserve">A2</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -40972,7 +40952,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
         </is>
       </c>
     </row>
@@ -41004,7 +40984,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t xml:space="preserve">A4</t>
+          <t xml:space="preserve">A3</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -41019,7 +40999,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-2</t>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
         </is>
       </c>
     </row>
@@ -41098,7 +41078,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t xml:space="preserve">A3</t>
+          <t xml:space="preserve">A4</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -41113,7 +41093,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtt3mo6u-2</t>
         </is>
       </c>
     </row>
@@ -41145,7 +41125,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t xml:space="preserve">A2</t>
+          <t xml:space="preserve">A3</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -41160,7 +41140,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
         </is>
       </c>
     </row>
@@ -41172,7 +41152,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -41192,7 +41172,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t xml:space="preserve">A1</t>
+          <t xml:space="preserve">A2</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -41207,7 +41187,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt0h140-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
         </is>
       </c>
     </row>
@@ -41219,7 +41199,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -41239,7 +41219,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t xml:space="preserve">A4</t>
+          <t xml:space="preserve">A1</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -41254,7 +41234,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-2</t>
+          <t xml:space="preserve">v-mtt0h140-0</t>
         </is>
       </c>
     </row>
@@ -41286,7 +41266,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t xml:space="preserve">A3</t>
+          <t xml:space="preserve">A4</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -41301,7 +41281,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtt3mo6u-2</t>
         </is>
       </c>
     </row>
@@ -41333,7 +41313,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t xml:space="preserve">A4</t>
+          <t xml:space="preserve">A3</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -41348,7 +41328,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-2</t>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
         </is>
       </c>
     </row>
@@ -41380,7 +41360,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t xml:space="preserve">A3</t>
+          <t xml:space="preserve">A4</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -41395,7 +41375,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtt3mo6u-2</t>
         </is>
       </c>
     </row>
@@ -41427,20 +41407,67 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
+          <t xml:space="preserve">A3</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown device</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">thaw</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jkl</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
           <t xml:space="preserve">A4</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr">
+      <c r="G49" t="inlineStr">
         <is>
           <t xml:space="preserve">unknown device</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
+      <c r="H49" t="inlineStr">
         <is>
           <t xml:space="preserve">thaw</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr">
+      <c r="J49" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mtt3mo6u-2</t>
         </is>
@@ -42128,10 +42155,10 @@
         <v>81</v>
       </c>
       <c r="I18">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="J18">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="19">

</xml_diff>

<commit_message>
Add 6 × HEK from Umut
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -32316,27 +32316,27 @@
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D392" t="inlineStr">
         <is>
-          <t xml:space="preserve">A1</t>
+          <t xml:space="preserve">C2</t>
         </is>
       </c>
       <c r="E392" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK</t>
         </is>
       </c>
       <c r="F392" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">28</t>
         </is>
       </c>
       <c r="G392" t="inlineStr">
@@ -32346,17 +32346,17 @@
       </c>
       <c r="H392" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="I392" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="K392" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L392" t="inlineStr">
@@ -32386,7 +32386,7 @@
       </c>
       <c r="S392" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-0</t>
+          <t xml:space="preserve">v-mv4yfgcs-0</t>
         </is>
       </c>
     </row>
@@ -32398,27 +32398,27 @@
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D393" t="inlineStr">
         <is>
-          <t xml:space="preserve">A2</t>
+          <t xml:space="preserve">C3</t>
         </is>
       </c>
       <c r="E393" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK</t>
         </is>
       </c>
       <c r="F393" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">28</t>
         </is>
       </c>
       <c r="G393" t="inlineStr">
@@ -32428,17 +32428,17 @@
       </c>
       <c r="H393" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="I393" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="K393" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L393" t="inlineStr">
@@ -32468,7 +32468,7 @@
       </c>
       <c r="S393" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-1</t>
+          <t xml:space="preserve">v-mv4yfgcs-1</t>
         </is>
       </c>
     </row>
@@ -32480,27 +32480,27 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D394" t="inlineStr">
         <is>
-          <t xml:space="preserve">A3</t>
+          <t xml:space="preserve">C4</t>
         </is>
       </c>
       <c r="E394" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK</t>
         </is>
       </c>
       <c r="F394" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">28</t>
         </is>
       </c>
       <c r="G394" t="inlineStr">
@@ -32510,17 +32510,17 @@
       </c>
       <c r="H394" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="I394" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="K394" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L394" t="inlineStr">
@@ -32550,7 +32550,7 @@
       </c>
       <c r="S394" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-2</t>
+          <t xml:space="preserve">v-mv4yfgcs-2</t>
         </is>
       </c>
     </row>
@@ -32562,27 +32562,27 @@
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D395" t="inlineStr">
         <is>
-          <t xml:space="preserve">A4</t>
+          <t xml:space="preserve">C5</t>
         </is>
       </c>
       <c r="E395" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK</t>
         </is>
       </c>
       <c r="F395" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">28</t>
         </is>
       </c>
       <c r="G395" t="inlineStr">
@@ -32592,17 +32592,17 @@
       </c>
       <c r="H395" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="I395" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="K395" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L395" t="inlineStr">
@@ -32632,7 +32632,7 @@
       </c>
       <c r="S395" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-3</t>
+          <t xml:space="preserve">v-mv4yfgcs-3</t>
         </is>
       </c>
     </row>
@@ -32644,491 +32644,601 @@
       </c>
       <c r="B396" t="inlineStr">
         <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C6</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">28</t>
+        </is>
+      </c>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="I396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="K396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
+      <c r="L396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S396" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv4yfgcs-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C7</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">28</t>
+        </is>
+      </c>
+      <c r="G397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="I397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="K397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
+      <c r="L397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S397" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv4yfgcs-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
           <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
-      <c r="C396" t="inlineStr">
+      <c r="C398" t="inlineStr">
         <is>
           <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
-      <c r="D396" t="inlineStr">
+      <c r="D398" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A1</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H398" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I398" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K398" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L398" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M398" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N398" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O398" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R398" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S398" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A2</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S399" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A3</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G400" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H400" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I400" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K400" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L400" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M400" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N400" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O400" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R400" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S400" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A4</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S401" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
         <is>
           <t xml:space="preserve">A5</t>
         </is>
       </c>
-      <c r="E396" t="inlineStr">
+      <c r="E402" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="F396" t="inlineStr">
+      <c r="F402" t="inlineStr">
         <is>
           <t xml:space="preserve">p18</t>
         </is>
       </c>
-      <c r="G396" t="inlineStr">
+      <c r="G402" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H396" t="inlineStr">
+      <c r="H402" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
-      <c r="I396" t="inlineStr">
+      <c r="I402" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
-      <c r="K396" t="inlineStr">
+      <c r="K402" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L396" t="inlineStr">
+      <c r="L402" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
         </is>
       </c>
-      <c r="M396" t="inlineStr">
+      <c r="M402" t="inlineStr">
         <is>
           <t xml:space="preserve">Par</t>
         </is>
       </c>
-      <c r="N396" t="inlineStr">
+      <c r="N402" t="inlineStr">
         <is>
           <t xml:space="preserve">No Casp</t>
         </is>
       </c>
-      <c r="O396" t="inlineStr">
+      <c r="O402" t="inlineStr">
         <is>
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
-      <c r="R396" t="inlineStr">
+      <c r="R402" t="inlineStr">
         <is>
           <t xml:space="preserve">stored</t>
         </is>
       </c>
-      <c r="S396" t="inlineStr">
+      <c r="S402" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mupot2zh-4</t>
-        </is>
-      </c>
-    </row>
-    <row r="397">
-      <c r="E397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNCX</t>
-        </is>
-      </c>
-      <c r="F397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p+21</t>
-        </is>
-      </c>
-      <c r="G397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">relative</t>
-        </is>
-      </c>
-      <c r="H397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-05-15</t>
-        </is>
-      </c>
-      <c r="I397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">15-05-26</t>
-        </is>
-      </c>
-      <c r="K397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="L397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CASPEX</t>
-        </is>
-      </c>
-      <c r="O397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S397" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-199</t>
-        </is>
-      </c>
-    </row>
-    <row r="398">
-      <c r="E398" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LUCX</t>
-        </is>
-      </c>
-      <c r="F398" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p19</t>
-        </is>
-      </c>
-      <c r="G398" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H398" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-07-31</t>
-        </is>
-      </c>
-      <c r="I398" t="inlineStr">
-        <is>
-          <t xml:space="preserve">31-07-26</t>
-        </is>
-      </c>
-      <c r="K398" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR</t>
-        </is>
-      </c>
-      <c r="L398" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M398" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CR</t>
-        </is>
-      </c>
-      <c r="N398" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CASPEX</t>
-        </is>
-      </c>
-      <c r="O398" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="P398" t="inlineStr">
-        <is>
-          <t xml:space="preserve">to-do</t>
-        </is>
-      </c>
-      <c r="Q398" t="inlineStr">
-        <is>
-          <t xml:space="preserve">to-do box / thaw</t>
-        </is>
-      </c>
-      <c r="R398" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S398" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-233</t>
-        </is>
-      </c>
-    </row>
-    <row r="399">
-      <c r="E399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145</t>
-        </is>
-      </c>
-      <c r="F399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p?</t>
-        </is>
-      </c>
-      <c r="G399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">unknown</t>
-        </is>
-      </c>
-      <c r="H399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-06-30</t>
-        </is>
-      </c>
-      <c r="I399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">30-06-25</t>
-        </is>
-      </c>
-      <c r="K399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145</t>
-        </is>
-      </c>
-      <c r="L399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S399" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-295</t>
-        </is>
-      </c>
-    </row>
-    <row r="400">
-      <c r="E400" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR</t>
-        </is>
-      </c>
-      <c r="F400" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p11</t>
-        </is>
-      </c>
-      <c r="G400" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H400" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-12</t>
-        </is>
-      </c>
-      <c r="I400" t="inlineStr">
-        <is>
-          <t xml:space="preserve">12/6/2026</t>
-        </is>
-      </c>
-      <c r="K400" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR</t>
-        </is>
-      </c>
-      <c r="L400" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M400" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CR</t>
-        </is>
-      </c>
-      <c r="N400" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O400" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R400" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S400" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-311</t>
-        </is>
-      </c>
-    </row>
-    <row r="401">
-      <c r="E401" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNCX</t>
-        </is>
-      </c>
-      <c r="F401" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p+17</t>
-        </is>
-      </c>
-      <c r="G401" t="inlineStr">
-        <is>
-          <t xml:space="preserve">relative</t>
-        </is>
-      </c>
-      <c r="H401" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-03-30</t>
-        </is>
-      </c>
-      <c r="I401" t="inlineStr">
-        <is>
-          <t xml:space="preserve">30-03-26</t>
-        </is>
-      </c>
-      <c r="K401" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="L401" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M401" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N401" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CASPEX</t>
-        </is>
-      </c>
-      <c r="O401" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R401" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S401" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-320</t>
-        </is>
-      </c>
-    </row>
-    <row r="402">
-      <c r="E402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap Canada</t>
-        </is>
-      </c>
-      <c r="F402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p+14</t>
-        </is>
-      </c>
-      <c r="G402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">relative</t>
-        </is>
-      </c>
-      <c r="H402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-03-23</t>
-        </is>
-      </c>
-      <c r="I402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">23-03-26</t>
-        </is>
-      </c>
-      <c r="K402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="L402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S402" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-321</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="E403" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F403" t="inlineStr">
         <is>
-          <t xml:space="preserve">p16</t>
+          <t xml:space="preserve">p+21</t>
         </is>
       </c>
       <c r="G403" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H403" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-11-06</t>
+          <t xml:space="preserve">2026-05-15</t>
         </is>
       </c>
       <c r="I403" t="inlineStr">
         <is>
-          <t xml:space="preserve">6/11/2025</t>
+          <t xml:space="preserve">15-05-26</t>
         </is>
       </c>
       <c r="K403" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L403" t="inlineStr">
@@ -33143,7 +33253,7 @@
       </c>
       <c r="N403" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O403" t="inlineStr">
@@ -33158,19 +33268,19 @@
       </c>
       <c r="S403" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-338</t>
+          <t xml:space="preserve">v-199</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="E404" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LUCX</t>
         </is>
       </c>
       <c r="F404" t="inlineStr">
         <is>
-          <t xml:space="preserve">p15</t>
+          <t xml:space="preserve">p19</t>
         </is>
       </c>
       <c r="G404" t="inlineStr">
@@ -33180,17 +33290,17 @@
       </c>
       <c r="H404" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-10</t>
+          <t xml:space="preserve">2026-07-31</t>
         </is>
       </c>
       <c r="I404" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/8/2026</t>
+          <t xml:space="preserve">31-07-26</t>
         </is>
       </c>
       <c r="K404" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L404" t="inlineStr">
@@ -33200,12 +33310,12 @@
       </c>
       <c r="M404" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N404" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O404" t="inlineStr">
@@ -33213,6 +33323,16 @@
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
+      <c r="P404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">to-do</t>
+        </is>
+      </c>
+      <c r="Q404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">to-do box / thaw</t>
+        </is>
+      </c>
       <c r="R404" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
@@ -33220,39 +33340,39 @@
       </c>
       <c r="S404" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-354</t>
+          <t xml:space="preserve">v-233</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="E405" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="F405" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p?</t>
         </is>
       </c>
       <c r="G405" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H405" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2025-06-30</t>
         </is>
       </c>
       <c r="I405" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">30-06-25</t>
         </is>
       </c>
       <c r="K405" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="L405" t="inlineStr">
@@ -33272,7 +33392,7 @@
       </c>
       <c r="O405" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R405" t="inlineStr">
@@ -33282,19 +33402,19 @@
       </c>
       <c r="S405" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdx0po-0</t>
+          <t xml:space="preserve">v-295</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="E406" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="F406" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p11</t>
         </is>
       </c>
       <c r="G406" t="inlineStr">
@@ -33304,27 +33424,27 @@
       </c>
       <c r="H406" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-06-12</t>
         </is>
       </c>
       <c r="I406" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">12/6/2026</t>
         </is>
       </c>
       <c r="K406" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L406" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M406" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N406" t="inlineStr">
@@ -33344,44 +33464,44 @@
       </c>
       <c r="S406" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdxsum-0</t>
+          <t xml:space="preserve">v-311</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="E407" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F407" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p+17</t>
         </is>
       </c>
       <c r="G407" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H407" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-03-30</t>
         </is>
       </c>
       <c r="I407" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">30-03-26</t>
         </is>
       </c>
       <c r="K407" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L407" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M407" t="inlineStr">
@@ -33391,7 +33511,7 @@
       </c>
       <c r="N407" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O407" t="inlineStr">
@@ -33406,44 +33526,44 @@
       </c>
       <c r="S407" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-0</t>
+          <t xml:space="preserve">v-320</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="E408" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">LnCap Canada</t>
         </is>
       </c>
       <c r="F408" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p+14</t>
         </is>
       </c>
       <c r="G408" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H408" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-03-23</t>
         </is>
       </c>
       <c r="I408" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">23-03-26</t>
         </is>
       </c>
       <c r="K408" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L408" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M408" t="inlineStr">
@@ -33468,19 +33588,19 @@
       </c>
       <c r="S408" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-1</t>
+          <t xml:space="preserve">v-321</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="E409" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="F409" t="inlineStr">
         <is>
-          <t xml:space="preserve">p28</t>
+          <t xml:space="preserve">p16</t>
         </is>
       </c>
       <c r="G409" t="inlineStr">
@@ -33490,12 +33610,12 @@
       </c>
       <c r="H409" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2025-11-06</t>
         </is>
       </c>
       <c r="I409" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">6/11/2025</t>
         </is>
       </c>
       <c r="K409" t="inlineStr">
@@ -33505,7 +33625,7 @@
       </c>
       <c r="L409" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M409" t="inlineStr">
@@ -33530,19 +33650,19 @@
       </c>
       <c r="S409" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdz1vx-0</t>
+          <t xml:space="preserve">v-338</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="E410" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="F410" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p15</t>
         </is>
       </c>
       <c r="G410" t="inlineStr">
@@ -33552,12 +33672,12 @@
       </c>
       <c r="H410" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-08-10</t>
         </is>
       </c>
       <c r="I410" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">10/8/2026</t>
         </is>
       </c>
       <c r="K410" t="inlineStr">
@@ -33582,7 +33702,7 @@
       </c>
       <c r="O410" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R410" t="inlineStr">
@@ -33592,19 +33712,19 @@
       </c>
       <c r="S410" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdzpx7-0</t>
+          <t xml:space="preserve">v-354</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="E411" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="F411" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G411" t="inlineStr">
@@ -33624,12 +33744,12 @@
       </c>
       <c r="K411" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L411" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M411" t="inlineStr">
@@ -33644,7 +33764,7 @@
       </c>
       <c r="O411" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R411" t="inlineStr">
@@ -33654,19 +33774,19 @@
       </c>
       <c r="S411" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0daw-0</t>
+          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="E412" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="F412" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G412" t="inlineStr">
@@ -33686,12 +33806,12 @@
       </c>
       <c r="K412" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L412" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M412" t="inlineStr">
@@ -33716,19 +33836,19 @@
       </c>
       <c r="S412" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0w3q-0</t>
+          <t xml:space="preserve">v-mtrdxsum-0</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="E413" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="F413" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G413" t="inlineStr">
@@ -33748,12 +33868,12 @@
       </c>
       <c r="K413" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L413" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M413" t="inlineStr">
@@ -33778,19 +33898,19 @@
       </c>
       <c r="S413" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre1ko0-0</t>
+          <t xml:space="preserve">v-mtrdyhss-0</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="E414" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="F414" t="inlineStr">
         <is>
-          <t xml:space="preserve">p6</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G414" t="inlineStr">
@@ -33800,12 +33920,12 @@
       </c>
       <c r="H414" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I414" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="K414" t="inlineStr">
@@ -33815,7 +33935,7 @@
       </c>
       <c r="L414" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M414" t="inlineStr">
@@ -33825,7 +33945,7 @@
       </c>
       <c r="N414" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">No Casp</t>
         </is>
       </c>
       <c r="O414" t="inlineStr">
@@ -33840,29 +33960,39 @@
       </c>
       <c r="S414" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtski3re-0</t>
+          <t xml:space="preserve">v-mtrdyhss-1</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="E415" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p28</t>
         </is>
       </c>
       <c r="G415" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H415" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I415" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L415" t="inlineStr">
@@ -33892,29 +34022,39 @@
       </c>
       <c r="S415" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt0h140-0</t>
+          <t xml:space="preserve">v-mtrdz1vx-0</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="E416" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">Huh7 gNT</t>
+        </is>
+      </c>
+      <c r="F416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G416" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H416" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I416" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L416" t="inlineStr">
@@ -33934,7 +34074,7 @@
       </c>
       <c r="O416" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R416" t="inlineStr">
@@ -33944,34 +34084,44 @@
       </c>
       <c r="S416" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-0</t>
+          <t xml:space="preserve">v-mtrdzpx7-0</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="E417" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+        </is>
+      </c>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G417" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H417" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I417" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L417" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M417" t="inlineStr">
@@ -33996,34 +34146,44 @@
       </c>
       <c r="S417" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtre0daw-0</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="E418" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G418" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H418" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I418" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L418" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M418" t="inlineStr">
@@ -34048,34 +34208,44 @@
       </c>
       <c r="S418" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-2</t>
+          <t xml:space="preserve">v-mtre0w3q-0</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="E419" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+        </is>
+      </c>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G419" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H419" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I419" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L419" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M419" t="inlineStr">
@@ -34100,29 +34270,39 @@
       </c>
       <c r="S419" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt5ckqo-0</t>
+          <t xml:space="preserve">v-mtre1ko0-0</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="E420" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">Hek caspex</t>
+        </is>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p6</t>
         </is>
       </c>
       <c r="G420" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H420" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I420" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="K420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L420" t="inlineStr">
@@ -34137,7 +34317,7 @@
       </c>
       <c r="N420" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O420" t="inlineStr">
@@ -34152,14 +34332,14 @@
       </c>
       <c r="S420" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmw7m-0</t>
+          <t xml:space="preserve">v-mtski3re-0</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="E421" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="G421" t="inlineStr">
@@ -34169,17 +34349,17 @@
       </c>
       <c r="H421" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I421" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="L421" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M421" t="inlineStr">
@@ -34204,14 +34384,14 @@
       </c>
       <c r="S421" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmypa-0</t>
+          <t xml:space="preserve">v-mtt0h140-0</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="E422" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="G422" t="inlineStr">
@@ -34221,12 +34401,12 @@
       </c>
       <c r="H422" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I422" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="L422" t="inlineStr">
@@ -34256,14 +34436,14 @@
       </c>
       <c r="S422" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmn045-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="E423" t="inlineStr">
         <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="G423" t="inlineStr">
@@ -34273,17 +34453,12 @@
       </c>
       <c r="H423" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I423" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
-        </is>
-      </c>
-      <c r="K423" t="inlineStr">
-        <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="L423" t="inlineStr">
@@ -34313,44 +34488,34 @@
       </c>
       <c r="S423" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtu5lgdc-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="E424" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
-        </is>
-      </c>
-      <c r="F424" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p19</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="G424" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H424" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-17</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I424" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-17</t>
-        </is>
-      </c>
-      <c r="K424" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="L424" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M424" t="inlineStr">
@@ -34375,67 +34540,394 @@
       </c>
       <c r="S424" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mu5anec8-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-2</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="E425" t="inlineStr">
         <is>
+          <t xml:space="preserve">khk</t>
+        </is>
+      </c>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt5ckqo-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="E426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="G426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mttmmw7m-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="E427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="G427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mttmmypa-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="E428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mttmn045-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="E429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deneme</t>
+        </is>
+      </c>
+      <c r="G429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="K429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deneme</t>
+        </is>
+      </c>
+      <c r="L429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtu5lgdc-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="E430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p19</t>
+        </is>
+      </c>
+      <c r="G430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-17</t>
+        </is>
+      </c>
+      <c r="I430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-17</t>
+        </is>
+      </c>
+      <c r="K430" t="inlineStr">
+        <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="F425" t="inlineStr">
+      <c r="L430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FLAG</t>
+        </is>
+      </c>
+      <c r="M430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mu5anec8-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="E431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
         <is>
           <t xml:space="preserve">18</t>
         </is>
       </c>
-      <c r="G425" t="inlineStr">
+      <c r="G431" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H425" t="inlineStr">
+      <c r="H431" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
-      <c r="I425" t="inlineStr">
+      <c r="I431" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
-      <c r="K425" t="inlineStr">
+      <c r="K431" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L425" t="inlineStr">
+      <c r="L431" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
         </is>
       </c>
-      <c r="M425" t="inlineStr">
+      <c r="M431" t="inlineStr">
         <is>
           <t xml:space="preserve">Par</t>
         </is>
       </c>
-      <c r="N425" t="inlineStr">
+      <c r="N431" t="inlineStr">
         <is>
           <t xml:space="preserve">No Casp</t>
         </is>
       </c>
-      <c r="O425" t="inlineStr">
+      <c r="O431" t="inlineStr">
         <is>
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
-      <c r="R425" t="inlineStr">
+      <c r="R431" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
-      <c r="S425" t="inlineStr">
+      <c r="S431" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mv4yequa-5</t>
         </is>
@@ -34860,22 +35352,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B KO g3</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">KO</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">g3</t>
+          <t xml:space="preserve">HEK</t>
         </is>
       </c>
       <c r="E14">
@@ -34885,13 +35362,13 @@
         <v>0</v>
       </c>
       <c r="G14">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 KO g1</t>
+          <t xml:space="preserve">HEK ATP7B KO g3</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -34901,12 +35378,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">g3</t>
         </is>
       </c>
       <c r="E15">
@@ -34916,28 +35393,28 @@
         <v>0</v>
       </c>
       <c r="G15">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gP2</t>
+          <t xml:space="preserve">HEK HOXB6 KO g1</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">gP2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E16">
@@ -34947,44 +35424,44 @@
         <v>0</v>
       </c>
       <c r="G16">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g3</t>
+          <t xml:space="preserve">LNCX gP2</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">g3</t>
+          <t xml:space="preserve">gP2</t>
         </is>
       </c>
       <c r="E17">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F17">
         <v>0</v>
       </c>
       <c r="G17">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX gNT</t>
+          <t xml:space="preserve">DuDtxR CASPEX g3</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -34999,7 +35476,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">g3</t>
         </is>
       </c>
       <c r="E18">
@@ -35015,22 +35492,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G1</t>
+          <t xml:space="preserve">DuDtxR CASPEX gNT</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E19">
@@ -35040,23 +35517,23 @@
         <v>0</v>
       </c>
       <c r="G19">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO G1</t>
+          <t xml:space="preserve">LnCap Canada V1G1</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -35065,19 +35542,19 @@
         </is>
       </c>
       <c r="E20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F20">
         <v>0</v>
       </c>
       <c r="G20">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK TOX4 OX</t>
+          <t xml:space="preserve">HEK CBX3 KO G1</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -35087,7 +35564,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -35102,13 +35579,13 @@
         <v>0</v>
       </c>
       <c r="G21">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
+          <t xml:space="preserve">HEK TOX4 OX</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -35118,33 +35595,33 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E22">
         <v>5</v>
       </c>
       <c r="F22">
+        <v>0</v>
+      </c>
+      <c r="G22">
         <v>1</v>
-      </c>
-      <c r="G22">
-        <v>3</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gP1</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -35154,28 +35631,28 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">gP1</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E23">
         <v>5</v>
       </c>
       <c r="F23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G23">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX gP1</t>
+          <t xml:space="preserve">LNCX gP1</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -35195,18 +35672,18 @@
         <v>0</v>
       </c>
       <c r="G24">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR+1</t>
+          <t xml:space="preserve">LUCX gP1</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -35216,28 +35693,28 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gP1</t>
         </is>
       </c>
       <c r="E25">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F25">
         <v>0</v>
       </c>
       <c r="G25">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">HepG2</t>
+          <t xml:space="preserve">DuPar50CR+1</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">HepG2</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -35257,23 +35734,23 @@
         <v>0</v>
       </c>
       <c r="G26">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">HepG2</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">HepG2</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -35282,19 +35759,19 @@
         </is>
       </c>
       <c r="E27">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F27">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G27">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK TOX4 KO g2</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -35304,33 +35781,33 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E28">
         <v>3</v>
       </c>
       <c r="F28">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G28">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 TOX4 KO</t>
+          <t xml:space="preserve">HEK TOX4 KO g2</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -35340,7 +35817,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E29">
@@ -35356,7 +35833,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">Huh7 TOX4 KO</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -35366,19 +35843,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E30">
         <v>3</v>
       </c>
       <c r="F30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G30">
         <v>2</v>
@@ -35387,12 +35864,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-I no sort</t>
+          <t xml:space="preserve">Huh7 gNT</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -35402,23 +35879,23 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E31">
         <v>3</v>
       </c>
       <c r="F31">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G31">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-K no sort</t>
+          <t xml:space="preserve">LCC-I no sort</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -35449,7 +35926,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-R no sort</t>
+          <t xml:space="preserve">LCC-K no sort</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -35480,7 +35957,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada CASPEX (no sort)</t>
+          <t xml:space="preserve">LCC-R no sort</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -35490,7 +35967,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -35511,26 +35988,26 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145 TOX4 KO g2.2</t>
+          <t xml:space="preserve">LnCap Canada CASPEX (no sort)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2.2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E35">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F35">
         <v>0</v>
@@ -35542,7 +36019,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR</t>
+          <t xml:space="preserve">Du145 TOX4 KO g2.2</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -35552,12 +36029,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2.2</t>
         </is>
       </c>
       <c r="E36">
@@ -35573,7 +36050,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR ATF3 KO</t>
+          <t xml:space="preserve">DuDtxR</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -35583,7 +36060,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -35604,7 +36081,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR ATP7B KO</t>
+          <t xml:space="preserve">DuPar50CR ATF3 KO</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -35635,7 +36112,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR MTF1 KO</t>
+          <t xml:space="preserve">DuPar50CR ATP7B KO</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -35666,7 +36143,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR NT KO</t>
+          <t xml:space="preserve">DuPar50CR MTF1 KO</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -35697,7 +36174,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR TOX4 KO g1.2</t>
+          <t xml:space="preserve">DuPar50CR NT KO</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -35707,12 +36184,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1.2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E41">
@@ -35728,7 +36205,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR TOX4 KO g2.2</t>
+          <t xml:space="preserve">DuPar50CR TOX4 KO g1.2</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -35743,7 +36220,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2.2</t>
+          <t xml:space="preserve">g1.2</t>
         </is>
       </c>
       <c r="E42">
@@ -35759,29 +36236,29 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">DuPar50CR TOX4 KO g2.2</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2.2</t>
         </is>
       </c>
       <c r="E43">
         <v>2</v>
       </c>
       <c r="F43">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G43">
         <v>1</v>
@@ -35790,7 +36267,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -35800,7 +36277,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -35821,7 +36298,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CASPEX Single</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -35831,7 +36308,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -35843,7 +36320,7 @@
         <v>2</v>
       </c>
       <c r="F45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G45">
         <v>1</v>
@@ -35852,7 +36329,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX</t>
+          <t xml:space="preserve">HEK CASPEX Single</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -35862,12 +36339,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E46">
@@ -35883,7 +36360,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK E2F1 sh1</t>
+          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -35893,12 +36370,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E47">
@@ -35914,7 +36391,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK E2F1 sh2</t>
+          <t xml:space="preserve">HEK E2F1 sh1</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -35945,7 +36422,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK FOXA1 KO g1</t>
+          <t xml:space="preserve">HEK E2F1 sh2</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -35955,12 +36432,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E49">
@@ -35976,7 +36453,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK FOXA1 KO g2</t>
+          <t xml:space="preserve">HEK FOXA1 KO g1</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -35991,7 +36468,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E50">
@@ -36007,7 +36484,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 OX</t>
+          <t xml:space="preserve">HEK FOXA1 KO g2</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -36022,7 +36499,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E51">
@@ -36038,7 +36515,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g1</t>
+          <t xml:space="preserve">HEK HOXB6 OX</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -36048,12 +36525,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E52">
@@ -36063,13 +36540,13 @@
         <v>0</v>
       </c>
       <c r="G52">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g2</t>
+          <t xml:space="preserve">HEK POU3F3 KO g1</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -36084,7 +36561,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E53">
@@ -36094,13 +36571,13 @@
         <v>0</v>
       </c>
       <c r="G53">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK STAT1 KO g2</t>
+          <t xml:space="preserve">HEK POU3F3 KO g2</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -36131,7 +36608,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT(20)</t>
+          <t xml:space="preserve">HEK STAT1 KO g2</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -36141,12 +36618,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E55">
@@ -36156,35 +36633,35 @@
         <v>0</v>
       </c>
       <c r="G55">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">HEK gNT(20)</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E56">
         <v>2</v>
       </c>
       <c r="F56">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G56">
         <v>2</v>
@@ -36193,7 +36670,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -36203,7 +36680,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -36215,16 +36692,16 @@
         <v>2</v>
       </c>
       <c r="F57">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G57">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -36234,7 +36711,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -36255,7 +36732,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATP7B KO #24</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -36265,7 +36742,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -36277,7 +36754,7 @@
         <v>2</v>
       </c>
       <c r="F59">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G59">
         <v>1</v>
@@ -36286,17 +36763,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-V</t>
+          <t xml:space="preserve">Huh7 ATP7B KO #24</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -36311,13 +36788,13 @@
         <v>0</v>
       </c>
       <c r="G60">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-V 99.17%</t>
+          <t xml:space="preserve">LCC-V</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -36348,7 +36825,22 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gC1</t>
+          <t xml:space="preserve">LCC-V 99.17%</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E62">
@@ -36358,13 +36850,13 @@
         <v>0</v>
       </c>
       <c r="G62">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gC2</t>
+          <t xml:space="preserve">LNCX gC1</t>
         </is>
       </c>
       <c r="E63">
@@ -36380,22 +36872,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gC3</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gC3</t>
+          <t xml:space="preserve">LNCX gC2</t>
         </is>
       </c>
       <c r="E64">
@@ -36411,7 +36888,22 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gC4</t>
+          <t xml:space="preserve">LNCX gC3</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gC3</t>
         </is>
       </c>
       <c r="E65">
@@ -36427,22 +36919,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gP3</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gP3</t>
+          <t xml:space="preserve">LNCX gC4</t>
         </is>
       </c>
       <c r="E66">
@@ -36458,22 +36935,22 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX gP2</t>
+          <t xml:space="preserve">LNCX gP3</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t xml:space="preserve">gP2</t>
+          <t xml:space="preserve">gP3</t>
         </is>
       </c>
       <c r="E67">
@@ -36489,12 +36966,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap (m3) (sortER)</t>
+          <t xml:space="preserve">LUCX gP2</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -36504,7 +36981,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gP2</t>
         </is>
       </c>
       <c r="E68">
@@ -36520,7 +36997,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada CASPEX mCherry 1 (no use)</t>
+          <t xml:space="preserve">LnCap (m3) (sortER)</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -36530,7 +37007,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -36551,7 +37028,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canadaa V1G1</t>
+          <t xml:space="preserve">LnCap Canada CASPEX mCherry 1 (no use)</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -36561,7 +37038,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -36582,7 +37059,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select +P+D #1</t>
+          <t xml:space="preserve">LnCap Canadaa V1G1</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -36592,7 +37069,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -36607,13 +37084,13 @@
         <v>0</v>
       </c>
       <c r="G71">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select +P+D #2</t>
+          <t xml:space="preserve">LnCapCASPEX no select +P+D #1</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -36638,13 +37115,13 @@
         <v>0</v>
       </c>
       <c r="G72">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select E</t>
+          <t xml:space="preserve">LnCapCASPEX no select +P+D #2</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -36669,13 +37146,13 @@
         <v>0</v>
       </c>
       <c r="G73">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select H</t>
+          <t xml:space="preserve">LnCapCASPEX no select E</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -36700,23 +37177,23 @@
         <v>0</v>
       </c>
       <c r="G74">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145 ATF3 KO rep2</t>
+          <t xml:space="preserve">LnCapCASPEX no select H</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -36725,7 +37202,7 @@
         </is>
       </c>
       <c r="E75">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F75">
         <v>0</v>
@@ -36737,7 +37214,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145 ATF3 OX rep2</t>
+          <t xml:space="preserve">Du145 ATF3 KO rep2</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -36747,7 +37224,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -36768,7 +37245,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEXe g3</t>
+          <t xml:space="preserve">Du145 ATF3 OX rep2</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -36778,12 +37255,12 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t xml:space="preserve">g3</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E77">
@@ -36799,7 +37276,22 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK</t>
+          <t xml:space="preserve">DuDtxR CASPEXe g3</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Du145</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASPEX</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">g3</t>
         </is>
       </c>
       <c r="E78">
@@ -42155,10 +42647,10 @@
         <v>81</v>
       </c>
       <c r="I18">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="J18">
-        <v>65</v>
+        <v>59</v>
       </c>
     </row>
     <row r="19">

</xml_diff>

<commit_message>
Add 6 × LnCap Canada from Umut
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -32808,47 +32808,47 @@
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D398" t="inlineStr">
         <is>
-          <t xml:space="preserve">A1</t>
+          <t xml:space="preserve">D1</t>
         </is>
       </c>
       <c r="E398" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap Canada</t>
         </is>
       </c>
       <c r="F398" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">+16</t>
         </is>
       </c>
       <c r="G398" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H398" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="I398" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="K398" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L398" t="inlineStr">
@@ -32878,7 +32878,7 @@
       </c>
       <c r="S398" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-0</t>
+          <t xml:space="preserve">v-mv4yfyco-0</t>
         </is>
       </c>
     </row>
@@ -32890,47 +32890,47 @@
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t xml:space="preserve">A2</t>
+          <t xml:space="preserve">D2</t>
         </is>
       </c>
       <c r="E399" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap Canada</t>
         </is>
       </c>
       <c r="F399" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">+16</t>
         </is>
       </c>
       <c r="G399" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H399" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="I399" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="K399" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L399" t="inlineStr">
@@ -32960,7 +32960,7 @@
       </c>
       <c r="S399" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-1</t>
+          <t xml:space="preserve">v-mv4yfyco-1</t>
         </is>
       </c>
     </row>
@@ -32972,47 +32972,47 @@
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t xml:space="preserve">A3</t>
+          <t xml:space="preserve">D3</t>
         </is>
       </c>
       <c r="E400" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap Canada</t>
         </is>
       </c>
       <c r="F400" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">+16</t>
         </is>
       </c>
       <c r="G400" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H400" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="I400" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="K400" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L400" t="inlineStr">
@@ -33042,7 +33042,7 @@
       </c>
       <c r="S400" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-2</t>
+          <t xml:space="preserve">v-mv4yfyco-2</t>
         </is>
       </c>
     </row>
@@ -33054,47 +33054,47 @@
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t xml:space="preserve">A4</t>
+          <t xml:space="preserve">D4</t>
         </is>
       </c>
       <c r="E401" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap Canada</t>
         </is>
       </c>
       <c r="F401" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">+16</t>
         </is>
       </c>
       <c r="G401" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H401" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="I401" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="K401" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L401" t="inlineStr">
@@ -33124,7 +33124,7 @@
       </c>
       <c r="S401" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-3</t>
+          <t xml:space="preserve">v-mv4yfyco-3</t>
         </is>
       </c>
     </row>
@@ -33136,491 +33136,601 @@
       </c>
       <c r="B402" t="inlineStr">
         <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D5</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap Canada</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+16</t>
+        </is>
+      </c>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">relative</t>
+        </is>
+      </c>
+      <c r="H402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="K402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="L402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S402" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv4yfyco-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">D6</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap Canada</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">+16</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">relative</t>
+        </is>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="K403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="L403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S403" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv4yfyco-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
           <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
-      <c r="C402" t="inlineStr">
+      <c r="C404" t="inlineStr">
         <is>
           <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
-      <c r="D402" t="inlineStr">
+      <c r="D404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A1</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S404" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A2</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S405" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A3</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S406" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A4</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S407" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
         <is>
           <t xml:space="preserve">A5</t>
         </is>
       </c>
-      <c r="E402" t="inlineStr">
+      <c r="E408" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="F402" t="inlineStr">
+      <c r="F408" t="inlineStr">
         <is>
           <t xml:space="preserve">p18</t>
         </is>
       </c>
-      <c r="G402" t="inlineStr">
+      <c r="G408" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H402" t="inlineStr">
+      <c r="H408" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
-      <c r="I402" t="inlineStr">
+      <c r="I408" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
-      <c r="K402" t="inlineStr">
+      <c r="K408" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L402" t="inlineStr">
+      <c r="L408" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
         </is>
       </c>
-      <c r="M402" t="inlineStr">
+      <c r="M408" t="inlineStr">
         <is>
           <t xml:space="preserve">Par</t>
         </is>
       </c>
-      <c r="N402" t="inlineStr">
+      <c r="N408" t="inlineStr">
         <is>
           <t xml:space="preserve">No Casp</t>
         </is>
       </c>
-      <c r="O402" t="inlineStr">
+      <c r="O408" t="inlineStr">
         <is>
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
-      <c r="R402" t="inlineStr">
+      <c r="R408" t="inlineStr">
         <is>
           <t xml:space="preserve">stored</t>
         </is>
       </c>
-      <c r="S402" t="inlineStr">
+      <c r="S408" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mupot2zh-4</t>
-        </is>
-      </c>
-    </row>
-    <row r="403">
-      <c r="E403" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNCX</t>
-        </is>
-      </c>
-      <c r="F403" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p+21</t>
-        </is>
-      </c>
-      <c r="G403" t="inlineStr">
-        <is>
-          <t xml:space="preserve">relative</t>
-        </is>
-      </c>
-      <c r="H403" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-05-15</t>
-        </is>
-      </c>
-      <c r="I403" t="inlineStr">
-        <is>
-          <t xml:space="preserve">15-05-26</t>
-        </is>
-      </c>
-      <c r="K403" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="L403" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M403" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N403" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CASPEX</t>
-        </is>
-      </c>
-      <c r="O403" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R403" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S403" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-199</t>
-        </is>
-      </c>
-    </row>
-    <row r="404">
-      <c r="E404" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LUCX</t>
-        </is>
-      </c>
-      <c r="F404" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p19</t>
-        </is>
-      </c>
-      <c r="G404" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H404" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-07-31</t>
-        </is>
-      </c>
-      <c r="I404" t="inlineStr">
-        <is>
-          <t xml:space="preserve">31-07-26</t>
-        </is>
-      </c>
-      <c r="K404" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR</t>
-        </is>
-      </c>
-      <c r="L404" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M404" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CR</t>
-        </is>
-      </c>
-      <c r="N404" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CASPEX</t>
-        </is>
-      </c>
-      <c r="O404" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="P404" t="inlineStr">
-        <is>
-          <t xml:space="preserve">to-do</t>
-        </is>
-      </c>
-      <c r="Q404" t="inlineStr">
-        <is>
-          <t xml:space="preserve">to-do box / thaw</t>
-        </is>
-      </c>
-      <c r="R404" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S404" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-233</t>
-        </is>
-      </c>
-    </row>
-    <row r="405">
-      <c r="E405" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145</t>
-        </is>
-      </c>
-      <c r="F405" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p?</t>
-        </is>
-      </c>
-      <c r="G405" t="inlineStr">
-        <is>
-          <t xml:space="preserve">unknown</t>
-        </is>
-      </c>
-      <c r="H405" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-06-30</t>
-        </is>
-      </c>
-      <c r="I405" t="inlineStr">
-        <is>
-          <t xml:space="preserve">30-06-25</t>
-        </is>
-      </c>
-      <c r="K405" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145</t>
-        </is>
-      </c>
-      <c r="L405" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M405" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N405" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O405" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R405" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S405" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-295</t>
-        </is>
-      </c>
-    </row>
-    <row r="406">
-      <c r="E406" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR</t>
-        </is>
-      </c>
-      <c r="F406" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p11</t>
-        </is>
-      </c>
-      <c r="G406" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H406" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-12</t>
-        </is>
-      </c>
-      <c r="I406" t="inlineStr">
-        <is>
-          <t xml:space="preserve">12/6/2026</t>
-        </is>
-      </c>
-      <c r="K406" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR</t>
-        </is>
-      </c>
-      <c r="L406" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M406" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CR</t>
-        </is>
-      </c>
-      <c r="N406" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O406" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R406" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S406" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-311</t>
-        </is>
-      </c>
-    </row>
-    <row r="407">
-      <c r="E407" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNCX</t>
-        </is>
-      </c>
-      <c r="F407" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p+17</t>
-        </is>
-      </c>
-      <c r="G407" t="inlineStr">
-        <is>
-          <t xml:space="preserve">relative</t>
-        </is>
-      </c>
-      <c r="H407" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-03-30</t>
-        </is>
-      </c>
-      <c r="I407" t="inlineStr">
-        <is>
-          <t xml:space="preserve">30-03-26</t>
-        </is>
-      </c>
-      <c r="K407" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="L407" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M407" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N407" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CASPEX</t>
-        </is>
-      </c>
-      <c r="O407" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R407" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S407" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-320</t>
-        </is>
-      </c>
-    </row>
-    <row r="408">
-      <c r="E408" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap Canada</t>
-        </is>
-      </c>
-      <c r="F408" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p+14</t>
-        </is>
-      </c>
-      <c r="G408" t="inlineStr">
-        <is>
-          <t xml:space="preserve">relative</t>
-        </is>
-      </c>
-      <c r="H408" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-03-23</t>
-        </is>
-      </c>
-      <c r="I408" t="inlineStr">
-        <is>
-          <t xml:space="preserve">23-03-26</t>
-        </is>
-      </c>
-      <c r="K408" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="L408" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M408" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N408" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O408" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R408" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S408" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-321</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="E409" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F409" t="inlineStr">
         <is>
-          <t xml:space="preserve">p16</t>
+          <t xml:space="preserve">p+21</t>
         </is>
       </c>
       <c r="G409" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H409" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-11-06</t>
+          <t xml:space="preserve">2026-05-15</t>
         </is>
       </c>
       <c r="I409" t="inlineStr">
         <is>
-          <t xml:space="preserve">6/11/2025</t>
+          <t xml:space="preserve">15-05-26</t>
         </is>
       </c>
       <c r="K409" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L409" t="inlineStr">
@@ -33635,7 +33745,7 @@
       </c>
       <c r="N409" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O409" t="inlineStr">
@@ -33650,19 +33760,19 @@
       </c>
       <c r="S409" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-338</t>
+          <t xml:space="preserve">v-199</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="E410" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LUCX</t>
         </is>
       </c>
       <c r="F410" t="inlineStr">
         <is>
-          <t xml:space="preserve">p15</t>
+          <t xml:space="preserve">p19</t>
         </is>
       </c>
       <c r="G410" t="inlineStr">
@@ -33672,17 +33782,17 @@
       </c>
       <c r="H410" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-10</t>
+          <t xml:space="preserve">2026-07-31</t>
         </is>
       </c>
       <c r="I410" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/8/2026</t>
+          <t xml:space="preserve">31-07-26</t>
         </is>
       </c>
       <c r="K410" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L410" t="inlineStr">
@@ -33692,12 +33802,12 @@
       </c>
       <c r="M410" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N410" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O410" t="inlineStr">
@@ -33705,6 +33815,16 @@
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
+      <c r="P410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">to-do</t>
+        </is>
+      </c>
+      <c r="Q410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">to-do box / thaw</t>
+        </is>
+      </c>
       <c r="R410" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
@@ -33712,39 +33832,39 @@
       </c>
       <c r="S410" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-354</t>
+          <t xml:space="preserve">v-233</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="E411" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="F411" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p?</t>
         </is>
       </c>
       <c r="G411" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H411" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2025-06-30</t>
         </is>
       </c>
       <c r="I411" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">30-06-25</t>
         </is>
       </c>
       <c r="K411" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="L411" t="inlineStr">
@@ -33764,7 +33884,7 @@
       </c>
       <c r="O411" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R411" t="inlineStr">
@@ -33774,19 +33894,19 @@
       </c>
       <c r="S411" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdx0po-0</t>
+          <t xml:space="preserve">v-295</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="E412" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="F412" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p11</t>
         </is>
       </c>
       <c r="G412" t="inlineStr">
@@ -33796,27 +33916,27 @@
       </c>
       <c r="H412" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-06-12</t>
         </is>
       </c>
       <c r="I412" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">12/6/2026</t>
         </is>
       </c>
       <c r="K412" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L412" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M412" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N412" t="inlineStr">
@@ -33836,44 +33956,44 @@
       </c>
       <c r="S412" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdxsum-0</t>
+          <t xml:space="preserve">v-311</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="E413" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F413" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p+17</t>
         </is>
       </c>
       <c r="G413" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H413" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-03-30</t>
         </is>
       </c>
       <c r="I413" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">30-03-26</t>
         </is>
       </c>
       <c r="K413" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L413" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M413" t="inlineStr">
@@ -33883,7 +34003,7 @@
       </c>
       <c r="N413" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O413" t="inlineStr">
@@ -33898,44 +34018,44 @@
       </c>
       <c r="S413" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-0</t>
+          <t xml:space="preserve">v-320</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="E414" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">LnCap Canada</t>
         </is>
       </c>
       <c r="F414" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p+14</t>
         </is>
       </c>
       <c r="G414" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H414" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-03-23</t>
         </is>
       </c>
       <c r="I414" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">23-03-26</t>
         </is>
       </c>
       <c r="K414" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L414" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M414" t="inlineStr">
@@ -33960,19 +34080,19 @@
       </c>
       <c r="S414" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-1</t>
+          <t xml:space="preserve">v-321</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="E415" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="F415" t="inlineStr">
         <is>
-          <t xml:space="preserve">p28</t>
+          <t xml:space="preserve">p16</t>
         </is>
       </c>
       <c r="G415" t="inlineStr">
@@ -33982,12 +34102,12 @@
       </c>
       <c r="H415" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2025-11-06</t>
         </is>
       </c>
       <c r="I415" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">6/11/2025</t>
         </is>
       </c>
       <c r="K415" t="inlineStr">
@@ -33997,7 +34117,7 @@
       </c>
       <c r="L415" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M415" t="inlineStr">
@@ -34022,19 +34142,19 @@
       </c>
       <c r="S415" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdz1vx-0</t>
+          <t xml:space="preserve">v-338</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="E416" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="F416" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p15</t>
         </is>
       </c>
       <c r="G416" t="inlineStr">
@@ -34044,12 +34164,12 @@
       </c>
       <c r="H416" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-08-10</t>
         </is>
       </c>
       <c r="I416" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">10/8/2026</t>
         </is>
       </c>
       <c r="K416" t="inlineStr">
@@ -34074,7 +34194,7 @@
       </c>
       <c r="O416" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R416" t="inlineStr">
@@ -34084,19 +34204,19 @@
       </c>
       <c r="S416" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdzpx7-0</t>
+          <t xml:space="preserve">v-354</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="E417" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="F417" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G417" t="inlineStr">
@@ -34116,12 +34236,12 @@
       </c>
       <c r="K417" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L417" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M417" t="inlineStr">
@@ -34136,7 +34256,7 @@
       </c>
       <c r="O417" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R417" t="inlineStr">
@@ -34146,19 +34266,19 @@
       </c>
       <c r="S417" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0daw-0</t>
+          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="E418" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="F418" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G418" t="inlineStr">
@@ -34178,12 +34298,12 @@
       </c>
       <c r="K418" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L418" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M418" t="inlineStr">
@@ -34208,19 +34328,19 @@
       </c>
       <c r="S418" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0w3q-0</t>
+          <t xml:space="preserve">v-mtrdxsum-0</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="E419" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="F419" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G419" t="inlineStr">
@@ -34240,12 +34360,12 @@
       </c>
       <c r="K419" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L419" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M419" t="inlineStr">
@@ -34270,19 +34390,19 @@
       </c>
       <c r="S419" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre1ko0-0</t>
+          <t xml:space="preserve">v-mtrdyhss-0</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="E420" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="F420" t="inlineStr">
         <is>
-          <t xml:space="preserve">p6</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G420" t="inlineStr">
@@ -34292,12 +34412,12 @@
       </c>
       <c r="H420" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I420" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="K420" t="inlineStr">
@@ -34307,7 +34427,7 @@
       </c>
       <c r="L420" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M420" t="inlineStr">
@@ -34317,7 +34437,7 @@
       </c>
       <c r="N420" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">No Casp</t>
         </is>
       </c>
       <c r="O420" t="inlineStr">
@@ -34332,29 +34452,39 @@
       </c>
       <c r="S420" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtski3re-0</t>
+          <t xml:space="preserve">v-mtrdyhss-1</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="E421" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+        </is>
+      </c>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p28</t>
         </is>
       </c>
       <c r="G421" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H421" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I421" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L421" t="inlineStr">
@@ -34384,29 +34514,39 @@
       </c>
       <c r="S421" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt0h140-0</t>
+          <t xml:space="preserve">v-mtrdz1vx-0</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="E422" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">Huh7 gNT</t>
+        </is>
+      </c>
+      <c r="F422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G422" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H422" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I422" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L422" t="inlineStr">
@@ -34426,7 +34566,7 @@
       </c>
       <c r="O422" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R422" t="inlineStr">
@@ -34436,34 +34576,44 @@
       </c>
       <c r="S422" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-0</t>
+          <t xml:space="preserve">v-mtrdzpx7-0</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="E423" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+        </is>
+      </c>
+      <c r="F423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G423" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H423" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I423" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L423" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M423" t="inlineStr">
@@ -34488,34 +34638,44 @@
       </c>
       <c r="S423" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtre0daw-0</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="E424" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G424" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H424" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I424" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L424" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M424" t="inlineStr">
@@ -34540,34 +34700,44 @@
       </c>
       <c r="S424" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-2</t>
+          <t xml:space="preserve">v-mtre0w3q-0</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="E425" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+        </is>
+      </c>
+      <c r="F425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G425" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H425" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I425" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L425" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M425" t="inlineStr">
@@ -34592,29 +34762,39 @@
       </c>
       <c r="S425" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt5ckqo-0</t>
+          <t xml:space="preserve">v-mtre1ko0-0</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="E426" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">Hek caspex</t>
+        </is>
+      </c>
+      <c r="F426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p6</t>
         </is>
       </c>
       <c r="G426" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H426" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I426" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="K426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L426" t="inlineStr">
@@ -34629,7 +34809,7 @@
       </c>
       <c r="N426" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O426" t="inlineStr">
@@ -34644,14 +34824,14 @@
       </c>
       <c r="S426" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmw7m-0</t>
+          <t xml:space="preserve">v-mtski3re-0</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="E427" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="G427" t="inlineStr">
@@ -34661,17 +34841,17 @@
       </c>
       <c r="H427" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I427" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="L427" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M427" t="inlineStr">
@@ -34696,14 +34876,14 @@
       </c>
       <c r="S427" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmypa-0</t>
+          <t xml:space="preserve">v-mtt0h140-0</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="E428" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="G428" t="inlineStr">
@@ -34713,12 +34893,12 @@
       </c>
       <c r="H428" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I428" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="L428" t="inlineStr">
@@ -34748,14 +34928,14 @@
       </c>
       <c r="S428" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmn045-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="E429" t="inlineStr">
         <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="G429" t="inlineStr">
@@ -34765,17 +34945,12 @@
       </c>
       <c r="H429" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I429" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
-        </is>
-      </c>
-      <c r="K429" t="inlineStr">
-        <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="L429" t="inlineStr">
@@ -34805,44 +34980,34 @@
       </c>
       <c r="S429" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtu5lgdc-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="E430" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
-        </is>
-      </c>
-      <c r="F430" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p19</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="G430" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H430" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-17</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I430" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-17</t>
-        </is>
-      </c>
-      <c r="K430" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="L430" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M430" t="inlineStr">
@@ -34867,67 +35032,394 @@
       </c>
       <c r="S430" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mu5anec8-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-2</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="E431" t="inlineStr">
         <is>
+          <t xml:space="preserve">khk</t>
+        </is>
+      </c>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt5ckqo-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="E432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="G432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mttmmw7m-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="E433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="G433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mttmmypa-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="E434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="G434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mttmn045-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="E435" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deneme</t>
+        </is>
+      </c>
+      <c r="G435" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H435" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I435" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="K435" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deneme</t>
+        </is>
+      </c>
+      <c r="L435" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M435" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N435" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O435" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R435" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S435" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtu5lgdc-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="E436" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p19</t>
+        </is>
+      </c>
+      <c r="G436" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H436" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-17</t>
+        </is>
+      </c>
+      <c r="I436" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-17</t>
+        </is>
+      </c>
+      <c r="K436" t="inlineStr">
+        <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="F431" t="inlineStr">
+      <c r="L436" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FLAG</t>
+        </is>
+      </c>
+      <c r="M436" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N436" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O436" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R436" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S436" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mu5anec8-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="E437" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F437" t="inlineStr">
         <is>
           <t xml:space="preserve">18</t>
         </is>
       </c>
-      <c r="G431" t="inlineStr">
+      <c r="G437" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H431" t="inlineStr">
+      <c r="H437" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
-      <c r="I431" t="inlineStr">
+      <c r="I437" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
-      <c r="K431" t="inlineStr">
+      <c r="K437" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L431" t="inlineStr">
+      <c r="L437" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
         </is>
       </c>
-      <c r="M431" t="inlineStr">
+      <c r="M437" t="inlineStr">
         <is>
           <t xml:space="preserve">Par</t>
         </is>
       </c>
-      <c r="N431" t="inlineStr">
+      <c r="N437" t="inlineStr">
         <is>
           <t xml:space="preserve">No Casp</t>
         </is>
       </c>
-      <c r="O431" t="inlineStr">
+      <c r="O437" t="inlineStr">
         <is>
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
-      <c r="R431" t="inlineStr">
+      <c r="R437" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
-      <c r="S431" t="inlineStr">
+      <c r="S437" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mv4yequa-5</t>
         </is>
@@ -34980,12 +35472,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap Canada</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -34999,24 +35491,24 @@
         </is>
       </c>
       <c r="E2">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="F2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -35030,13 +35522,13 @@
         </is>
       </c>
       <c r="E3">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -42647,10 +43139,10 @@
         <v>81</v>
       </c>
       <c r="I18">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="J18">
-        <v>59</v>
+        <v>53</v>
       </c>
     </row>
     <row r="19">

</xml_diff>

<commit_message>
Add 9 × HEK from Umut
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -33300,27 +33300,27 @@
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D404" t="inlineStr">
         <is>
-          <t xml:space="preserve">A1</t>
+          <t xml:space="preserve">E1</t>
         </is>
       </c>
       <c r="E404" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK</t>
         </is>
       </c>
       <c r="F404" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">30</t>
         </is>
       </c>
       <c r="G404" t="inlineStr">
@@ -33330,17 +33330,17 @@
       </c>
       <c r="H404" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="I404" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="K404" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L404" t="inlineStr">
@@ -33370,7 +33370,7 @@
       </c>
       <c r="S404" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-0</t>
+          <t xml:space="preserve">v-mv4yhtbo-0</t>
         </is>
       </c>
     </row>
@@ -33382,27 +33382,27 @@
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t xml:space="preserve">A2</t>
+          <t xml:space="preserve">E2</t>
         </is>
       </c>
       <c r="E405" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK</t>
         </is>
       </c>
       <c r="F405" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">30</t>
         </is>
       </c>
       <c r="G405" t="inlineStr">
@@ -33412,17 +33412,17 @@
       </c>
       <c r="H405" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="I405" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="K405" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L405" t="inlineStr">
@@ -33452,7 +33452,7 @@
       </c>
       <c r="S405" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-1</t>
+          <t xml:space="preserve">v-mv4yhtbo-1</t>
         </is>
       </c>
     </row>
@@ -33464,27 +33464,27 @@
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t xml:space="preserve">A3</t>
+          <t xml:space="preserve">E3</t>
         </is>
       </c>
       <c r="E406" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK</t>
         </is>
       </c>
       <c r="F406" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">30</t>
         </is>
       </c>
       <c r="G406" t="inlineStr">
@@ -33494,17 +33494,17 @@
       </c>
       <c r="H406" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="I406" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="K406" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L406" t="inlineStr">
@@ -33534,7 +33534,7 @@
       </c>
       <c r="S406" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-2</t>
+          <t xml:space="preserve">v-mv4yhtbo-2</t>
         </is>
       </c>
     </row>
@@ -33546,27 +33546,27 @@
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D407" t="inlineStr">
         <is>
-          <t xml:space="preserve">A4</t>
+          <t xml:space="preserve">E4</t>
         </is>
       </c>
       <c r="E407" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK</t>
         </is>
       </c>
       <c r="F407" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">30</t>
         </is>
       </c>
       <c r="G407" t="inlineStr">
@@ -33576,17 +33576,17 @@
       </c>
       <c r="H407" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="I407" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="K407" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L407" t="inlineStr">
@@ -33616,7 +33616,7 @@
       </c>
       <c r="S407" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-3</t>
+          <t xml:space="preserve">v-mv4yhtbo-3</t>
         </is>
       </c>
     </row>
@@ -33628,682 +33628,852 @@
       </c>
       <c r="B408" t="inlineStr">
         <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">E5</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30</t>
+        </is>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="I408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="K408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
+      <c r="L408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S408" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv4yhtbo-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">E6</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30</t>
+        </is>
+      </c>
+      <c r="G409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="K409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
+      <c r="L409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S409" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv4yhtbo-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">E7</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30</t>
+        </is>
+      </c>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="I410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="K410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
+      <c r="L410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S410" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv4yhtbo-6</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">E8</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK</t>
+        </is>
+      </c>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30</t>
+        </is>
+      </c>
+      <c r="G411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="I411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="K411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
+      <c r="L411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S411" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv4yhtbo-7</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">E9</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">30</t>
+        </is>
+      </c>
+      <c r="G412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="I412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-09</t>
+        </is>
+      </c>
+      <c r="K412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
+      <c r="L412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S412" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv4yhtbo-8</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
           <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
-      <c r="C408" t="inlineStr">
+      <c r="C413" t="inlineStr">
         <is>
           <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
-      <c r="D408" t="inlineStr">
+      <c r="D413" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A1</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G413" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H413" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I413" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K413" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L413" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M413" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N413" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O413" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R413" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S413" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A2</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S414" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A3</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S415" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A4</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S416" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
         <is>
           <t xml:space="preserve">A5</t>
         </is>
       </c>
-      <c r="E408" t="inlineStr">
+      <c r="E417" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="F408" t="inlineStr">
+      <c r="F417" t="inlineStr">
         <is>
           <t xml:space="preserve">p18</t>
         </is>
       </c>
-      <c r="G408" t="inlineStr">
+      <c r="G417" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H408" t="inlineStr">
+      <c r="H417" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
-      <c r="I408" t="inlineStr">
+      <c r="I417" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
-      <c r="K408" t="inlineStr">
+      <c r="K417" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L408" t="inlineStr">
+      <c r="L417" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
         </is>
       </c>
-      <c r="M408" t="inlineStr">
+      <c r="M417" t="inlineStr">
         <is>
           <t xml:space="preserve">Par</t>
         </is>
       </c>
-      <c r="N408" t="inlineStr">
+      <c r="N417" t="inlineStr">
         <is>
           <t xml:space="preserve">No Casp</t>
         </is>
       </c>
-      <c r="O408" t="inlineStr">
+      <c r="O417" t="inlineStr">
         <is>
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
-      <c r="R408" t="inlineStr">
+      <c r="R417" t="inlineStr">
         <is>
           <t xml:space="preserve">stored</t>
         </is>
       </c>
-      <c r="S408" t="inlineStr">
+      <c r="S417" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mupot2zh-4</t>
-        </is>
-      </c>
-    </row>
-    <row r="409">
-      <c r="E409" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNCX</t>
-        </is>
-      </c>
-      <c r="F409" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p+21</t>
-        </is>
-      </c>
-      <c r="G409" t="inlineStr">
-        <is>
-          <t xml:space="preserve">relative</t>
-        </is>
-      </c>
-      <c r="H409" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-05-15</t>
-        </is>
-      </c>
-      <c r="I409" t="inlineStr">
-        <is>
-          <t xml:space="preserve">15-05-26</t>
-        </is>
-      </c>
-      <c r="K409" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="L409" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M409" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N409" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CASPEX</t>
-        </is>
-      </c>
-      <c r="O409" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R409" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S409" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-199</t>
-        </is>
-      </c>
-    </row>
-    <row r="410">
-      <c r="E410" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LUCX</t>
-        </is>
-      </c>
-      <c r="F410" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p19</t>
-        </is>
-      </c>
-      <c r="G410" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H410" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-07-31</t>
-        </is>
-      </c>
-      <c r="I410" t="inlineStr">
-        <is>
-          <t xml:space="preserve">31-07-26</t>
-        </is>
-      </c>
-      <c r="K410" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR</t>
-        </is>
-      </c>
-      <c r="L410" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M410" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CR</t>
-        </is>
-      </c>
-      <c r="N410" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CASPEX</t>
-        </is>
-      </c>
-      <c r="O410" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="P410" t="inlineStr">
-        <is>
-          <t xml:space="preserve">to-do</t>
-        </is>
-      </c>
-      <c r="Q410" t="inlineStr">
-        <is>
-          <t xml:space="preserve">to-do box / thaw</t>
-        </is>
-      </c>
-      <c r="R410" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S410" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-233</t>
-        </is>
-      </c>
-    </row>
-    <row r="411">
-      <c r="E411" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145</t>
-        </is>
-      </c>
-      <c r="F411" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p?</t>
-        </is>
-      </c>
-      <c r="G411" t="inlineStr">
-        <is>
-          <t xml:space="preserve">unknown</t>
-        </is>
-      </c>
-      <c r="H411" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-06-30</t>
-        </is>
-      </c>
-      <c r="I411" t="inlineStr">
-        <is>
-          <t xml:space="preserve">30-06-25</t>
-        </is>
-      </c>
-      <c r="K411" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145</t>
-        </is>
-      </c>
-      <c r="L411" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M411" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N411" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O411" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R411" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S411" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-295</t>
-        </is>
-      </c>
-    </row>
-    <row r="412">
-      <c r="E412" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR</t>
-        </is>
-      </c>
-      <c r="F412" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p11</t>
-        </is>
-      </c>
-      <c r="G412" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H412" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-12</t>
-        </is>
-      </c>
-      <c r="I412" t="inlineStr">
-        <is>
-          <t xml:space="preserve">12/6/2026</t>
-        </is>
-      </c>
-      <c r="K412" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR</t>
-        </is>
-      </c>
-      <c r="L412" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M412" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CR</t>
-        </is>
-      </c>
-      <c r="N412" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O412" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R412" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S412" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-311</t>
-        </is>
-      </c>
-    </row>
-    <row r="413">
-      <c r="E413" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNCX</t>
-        </is>
-      </c>
-      <c r="F413" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p+17</t>
-        </is>
-      </c>
-      <c r="G413" t="inlineStr">
-        <is>
-          <t xml:space="preserve">relative</t>
-        </is>
-      </c>
-      <c r="H413" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-03-30</t>
-        </is>
-      </c>
-      <c r="I413" t="inlineStr">
-        <is>
-          <t xml:space="preserve">30-03-26</t>
-        </is>
-      </c>
-      <c r="K413" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="L413" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M413" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N413" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CASPEX</t>
-        </is>
-      </c>
-      <c r="O413" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R413" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S413" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-320</t>
-        </is>
-      </c>
-    </row>
-    <row r="414">
-      <c r="E414" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap Canada</t>
-        </is>
-      </c>
-      <c r="F414" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p+14</t>
-        </is>
-      </c>
-      <c r="G414" t="inlineStr">
-        <is>
-          <t xml:space="preserve">relative</t>
-        </is>
-      </c>
-      <c r="H414" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-03-23</t>
-        </is>
-      </c>
-      <c r="I414" t="inlineStr">
-        <is>
-          <t xml:space="preserve">23-03-26</t>
-        </is>
-      </c>
-      <c r="K414" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="L414" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M414" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N414" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O414" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R414" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S414" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-321</t>
-        </is>
-      </c>
-    </row>
-    <row r="415">
-      <c r="E415" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
-      <c r="F415" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p16</t>
-        </is>
-      </c>
-      <c r="G415" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H415" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-11-06</t>
-        </is>
-      </c>
-      <c r="I415" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6/11/2025</t>
-        </is>
-      </c>
-      <c r="K415" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
-      <c r="L415" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M415" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N415" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O415" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R415" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S415" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-338</t>
-        </is>
-      </c>
-    </row>
-    <row r="416">
-      <c r="E416" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7</t>
-        </is>
-      </c>
-      <c r="F416" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p15</t>
-        </is>
-      </c>
-      <c r="G416" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H416" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-08-10</t>
-        </is>
-      </c>
-      <c r="I416" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10/8/2026</t>
-        </is>
-      </c>
-      <c r="K416" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7</t>
-        </is>
-      </c>
-      <c r="L416" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M416" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N416" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O416" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R416" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S416" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-354</t>
-        </is>
-      </c>
-    </row>
-    <row r="417">
-      <c r="E417" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK gNT</t>
-        </is>
-      </c>
-      <c r="F417" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p21</t>
-        </is>
-      </c>
-      <c r="G417" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H417" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-07</t>
-        </is>
-      </c>
-      <c r="I417" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-07</t>
-        </is>
-      </c>
-      <c r="K417" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
-      <c r="L417" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M417" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N417" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O417" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gNT</t>
-        </is>
-      </c>
-      <c r="R417" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S417" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="E418" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F418" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p+21</t>
         </is>
       </c>
       <c r="G418" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H418" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-05-15</t>
         </is>
       </c>
       <c r="I418" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">15-05-26</t>
         </is>
       </c>
       <c r="K418" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L418" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M418" t="inlineStr">
@@ -34313,7 +34483,7 @@
       </c>
       <c r="N418" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O418" t="inlineStr">
@@ -34328,19 +34498,19 @@
       </c>
       <c r="S418" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdxsum-0</t>
+          <t xml:space="preserve">v-199</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="E419" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">LUCX</t>
         </is>
       </c>
       <c r="F419" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p19</t>
         </is>
       </c>
       <c r="G419" t="inlineStr">
@@ -34350,32 +34520,32 @@
       </c>
       <c r="H419" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-07-31</t>
         </is>
       </c>
       <c r="I419" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">31-07-26</t>
         </is>
       </c>
       <c r="K419" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L419" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M419" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N419" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O419" t="inlineStr">
@@ -34383,6 +34553,16 @@
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
+      <c r="P419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">to-do</t>
+        </is>
+      </c>
+      <c r="Q419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">to-do box / thaw</t>
+        </is>
+      </c>
       <c r="R419" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
@@ -34390,44 +34570,44 @@
       </c>
       <c r="S419" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-0</t>
+          <t xml:space="preserve">v-233</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="E420" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="F420" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p?</t>
         </is>
       </c>
       <c r="G420" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H420" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2025-06-30</t>
         </is>
       </c>
       <c r="I420" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">30-06-25</t>
         </is>
       </c>
       <c r="K420" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="L420" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M420" t="inlineStr">
@@ -34452,19 +34632,19 @@
       </c>
       <c r="S420" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-1</t>
+          <t xml:space="preserve">v-295</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="E421" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="F421" t="inlineStr">
         <is>
-          <t xml:space="preserve">p28</t>
+          <t xml:space="preserve">p11</t>
         </is>
       </c>
       <c r="G421" t="inlineStr">
@@ -34474,27 +34654,27 @@
       </c>
       <c r="H421" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-06-12</t>
         </is>
       </c>
       <c r="I421" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">12/6/2026</t>
         </is>
       </c>
       <c r="K421" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L421" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M421" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N421" t="inlineStr">
@@ -34514,39 +34694,39 @@
       </c>
       <c r="S421" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdz1vx-0</t>
+          <t xml:space="preserve">v-311</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="E422" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F422" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p+17</t>
         </is>
       </c>
       <c r="G422" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H422" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-03-30</t>
         </is>
       </c>
       <c r="I422" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">30-03-26</t>
         </is>
       </c>
       <c r="K422" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L422" t="inlineStr">
@@ -34561,12 +34741,12 @@
       </c>
       <c r="N422" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O422" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R422" t="inlineStr">
@@ -34576,44 +34756,44 @@
       </c>
       <c r="S422" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdzpx7-0</t>
+          <t xml:space="preserve">v-320</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="E423" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">LnCap Canada</t>
         </is>
       </c>
       <c r="F423" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p+14</t>
         </is>
       </c>
       <c r="G423" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H423" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-03-23</t>
         </is>
       </c>
       <c r="I423" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">23-03-26</t>
         </is>
       </c>
       <c r="K423" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L423" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M423" t="inlineStr">
@@ -34638,19 +34818,19 @@
       </c>
       <c r="S423" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0daw-0</t>
+          <t xml:space="preserve">v-321</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="E424" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="F424" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p16</t>
         </is>
       </c>
       <c r="G424" t="inlineStr">
@@ -34660,22 +34840,22 @@
       </c>
       <c r="H424" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2025-11-06</t>
         </is>
       </c>
       <c r="I424" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">6/11/2025</t>
         </is>
       </c>
       <c r="K424" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L424" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M424" t="inlineStr">
@@ -34700,19 +34880,19 @@
       </c>
       <c r="S424" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0w3q-0</t>
+          <t xml:space="preserve">v-338</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="E425" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="F425" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p15</t>
         </is>
       </c>
       <c r="G425" t="inlineStr">
@@ -34722,12 +34902,12 @@
       </c>
       <c r="H425" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-08-10</t>
         </is>
       </c>
       <c r="I425" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">10/8/2026</t>
         </is>
       </c>
       <c r="K425" t="inlineStr">
@@ -34737,7 +34917,7 @@
       </c>
       <c r="L425" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M425" t="inlineStr">
@@ -34762,19 +34942,19 @@
       </c>
       <c r="S425" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre1ko0-0</t>
+          <t xml:space="preserve">v-354</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="E426" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="F426" t="inlineStr">
         <is>
-          <t xml:space="preserve">p6</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G426" t="inlineStr">
@@ -34784,12 +34964,12 @@
       </c>
       <c r="H426" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I426" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="K426" t="inlineStr">
@@ -34809,12 +34989,12 @@
       </c>
       <c r="N426" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">No Casp</t>
         </is>
       </c>
       <c r="O426" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R426" t="inlineStr">
@@ -34824,34 +35004,44 @@
       </c>
       <c r="S426" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtski3re-0</t>
+          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="E427" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+        </is>
+      </c>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G427" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H427" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I427" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L427" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M427" t="inlineStr">
@@ -34876,34 +35066,44 @@
       </c>
       <c r="S427" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt0h140-0</t>
+          <t xml:space="preserve">v-mtrdxsum-0</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="E428" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G428" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H428" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I428" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L428" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M428" t="inlineStr">
@@ -34928,34 +35128,44 @@
       </c>
       <c r="S428" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-0</t>
+          <t xml:space="preserve">v-mtrdyhss-0</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="E429" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G429" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H429" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I429" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L429" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M429" t="inlineStr">
@@ -34980,34 +35190,44 @@
       </c>
       <c r="S429" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtrdyhss-1</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="E430" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p28</t>
         </is>
       </c>
       <c r="G430" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H430" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I430" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L430" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M430" t="inlineStr">
@@ -35032,29 +35252,39 @@
       </c>
       <c r="S430" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-2</t>
+          <t xml:space="preserve">v-mtrdz1vx-0</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="E431" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">Huh7 gNT</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G431" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H431" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I431" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L431" t="inlineStr">
@@ -35074,7 +35304,7 @@
       </c>
       <c r="O431" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R431" t="inlineStr">
@@ -35084,34 +35314,44 @@
       </c>
       <c r="S431" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt5ckqo-0</t>
+          <t xml:space="preserve">v-mtrdzpx7-0</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="E432" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G432" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H432" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I432" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L432" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M432" t="inlineStr">
@@ -35136,34 +35376,44 @@
       </c>
       <c r="S432" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmw7m-0</t>
+          <t xml:space="preserve">v-mtre0daw-0</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="E433" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G433" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H433" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I433" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L433" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M433" t="inlineStr">
@@ -35188,34 +35438,44 @@
       </c>
       <c r="S433" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmypa-0</t>
+          <t xml:space="preserve">v-mtre0w3q-0</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="E434" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+        </is>
+      </c>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G434" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H434" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I434" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L434" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M434" t="inlineStr">
@@ -35240,34 +35500,39 @@
       </c>
       <c r="S434" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmn045-0</t>
+          <t xml:space="preserve">v-mtre1ko0-0</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="E435" t="inlineStr">
         <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">Hek caspex</t>
+        </is>
+      </c>
+      <c r="F435" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p6</t>
         </is>
       </c>
       <c r="G435" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H435" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I435" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="K435" t="inlineStr">
         <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L435" t="inlineStr">
@@ -35282,7 +35547,7 @@
       </c>
       <c r="N435" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O435" t="inlineStr">
@@ -35297,44 +35562,34 @@
       </c>
       <c r="S435" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtu5lgdc-0</t>
+          <t xml:space="preserve">v-mtski3re-0</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="E436" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
-        </is>
-      </c>
-      <c r="F436" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p19</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="G436" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H436" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-17</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I436" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-17</t>
-        </is>
-      </c>
-      <c r="K436" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="L436" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M436" t="inlineStr">
@@ -35359,67 +35614,550 @@
       </c>
       <c r="S436" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mu5anec8-0</t>
+          <t xml:space="preserve">v-mtt0h140-0</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="E437" t="inlineStr">
         <is>
+          <t xml:space="preserve">jkl</t>
+        </is>
+      </c>
+      <c r="G437" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H437" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I437" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L437" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M437" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N437" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O437" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R437" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S437" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="E438" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jkl</t>
+        </is>
+      </c>
+      <c r="G438" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H438" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L438" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M438" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N438" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O438" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R438" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S438" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="E439" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jkl</t>
+        </is>
+      </c>
+      <c r="G439" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H439" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I439" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L439" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M439" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N439" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O439" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R439" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S439" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt3mo6u-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="E440" t="inlineStr">
+        <is>
+          <t xml:space="preserve">khk</t>
+        </is>
+      </c>
+      <c r="G440" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H440" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I440" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L440" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M440" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N440" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O440" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R440" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S440" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt5ckqo-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="E441" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="G441" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H441" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I441" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L441" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M441" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N441" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O441" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R441" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S441" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mttmmw7m-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="E442" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="G442" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H442" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I442" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L442" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M442" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N442" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O442" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R442" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S442" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mttmmypa-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="E443" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="G443" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H443" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I443" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L443" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M443" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N443" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O443" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R443" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S443" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mttmn045-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="E444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deneme</t>
+        </is>
+      </c>
+      <c r="G444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="K444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deneme</t>
+        </is>
+      </c>
+      <c r="L444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtu5lgdc-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="E445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p19</t>
+        </is>
+      </c>
+      <c r="G445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-17</t>
+        </is>
+      </c>
+      <c r="I445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-17</t>
+        </is>
+      </c>
+      <c r="K445" t="inlineStr">
+        <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="F437" t="inlineStr">
+      <c r="L445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FLAG</t>
+        </is>
+      </c>
+      <c r="M445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mu5anec8-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="E446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F446" t="inlineStr">
         <is>
           <t xml:space="preserve">18</t>
         </is>
       </c>
-      <c r="G437" t="inlineStr">
+      <c r="G446" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H437" t="inlineStr">
+      <c r="H446" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
-      <c r="I437" t="inlineStr">
+      <c r="I446" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
-      <c r="K437" t="inlineStr">
+      <c r="K446" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L437" t="inlineStr">
+      <c r="L446" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
         </is>
       </c>
-      <c r="M437" t="inlineStr">
+      <c r="M446" t="inlineStr">
         <is>
           <t xml:space="preserve">Par</t>
         </is>
       </c>
-      <c r="N437" t="inlineStr">
+      <c r="N446" t="inlineStr">
         <is>
           <t xml:space="preserve">No Casp</t>
         </is>
       </c>
-      <c r="O437" t="inlineStr">
+      <c r="O446" t="inlineStr">
         <is>
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
-      <c r="R437" t="inlineStr">
+      <c r="R446" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
-      <c r="S437" t="inlineStr">
+      <c r="S446" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mv4yequa-5</t>
         </is>
@@ -35534,38 +36272,23 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">HEK</t>
         </is>
       </c>
       <c r="E4">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
         <v>1</v>
-      </c>
-      <c r="G4">
-        <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g1.1</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -35575,43 +36298,43 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1.1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E5">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gNT</t>
+          <t xml:space="preserve">DuDtxR CASPEX g1.1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">g1.1</t>
         </is>
       </c>
       <c r="E6">
@@ -35621,18 +36344,18 @@
         <v>0</v>
       </c>
       <c r="G6">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LNCX gNT</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -35642,28 +36365,28 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E7">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -35677,7 +36400,7 @@
         </is>
       </c>
       <c r="E8">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F8">
         <v>1</v>
@@ -35689,12 +36412,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -35711,7 +36434,7 @@
         <v>10</v>
       </c>
       <c r="F9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G9">
         <v>3</v>
@@ -35720,12 +36443,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B-GFP</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -35739,38 +36462,38 @@
         </is>
       </c>
       <c r="E10">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G10">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g5.1</t>
+          <t xml:space="preserve">HEK ATP7B-GFP</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">g5.1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E11">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F11">
         <v>0</v>
@@ -35782,69 +36505,84 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX</t>
+          <t xml:space="preserve">DuDtxR CASPEX g5.1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g5.1</t>
         </is>
       </c>
       <c r="E12">
         <v>8</v>
       </c>
       <c r="F12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX DSg1.2</t>
+          <t xml:space="preserve">LUCX</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">DSg1.2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E13">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G13">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK</t>
+          <t xml:space="preserve">DuDtxR CASPEX DSg1.2</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Du145</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASPEX</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DSg1.2</t>
         </is>
       </c>
       <c r="E14">
@@ -35854,7 +36592,7 @@
         <v>0</v>
       </c>
       <c r="G14">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
@@ -43139,10 +43877,10 @@
         <v>81</v>
       </c>
       <c r="I18">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="J18">
-        <v>53</v>
+        <v>44</v>
       </c>
     </row>
     <row r="19">

</xml_diff>

<commit_message>
Add 9 × LnCap Canada from Umut
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -34038,47 +34038,47 @@
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t xml:space="preserve">A1</t>
+          <t xml:space="preserve">F1</t>
         </is>
       </c>
       <c r="E413" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap Canada</t>
         </is>
       </c>
       <c r="F413" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p+18</t>
         </is>
       </c>
       <c r="G413" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H413" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="I413" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="K413" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L413" t="inlineStr">
@@ -34108,7 +34108,7 @@
       </c>
       <c r="S413" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-0</t>
+          <t xml:space="preserve">v-mv5d2kfh-0</t>
         </is>
       </c>
     </row>
@@ -34120,47 +34120,47 @@
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D414" t="inlineStr">
         <is>
-          <t xml:space="preserve">A2</t>
+          <t xml:space="preserve">F2</t>
         </is>
       </c>
       <c r="E414" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap Canada</t>
         </is>
       </c>
       <c r="F414" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p+18</t>
         </is>
       </c>
       <c r="G414" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H414" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="I414" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="K414" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L414" t="inlineStr">
@@ -34190,7 +34190,7 @@
       </c>
       <c r="S414" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-1</t>
+          <t xml:space="preserve">v-mv5d2kfh-1</t>
         </is>
       </c>
     </row>
@@ -34202,47 +34202,47 @@
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t xml:space="preserve">A3</t>
+          <t xml:space="preserve">F3</t>
         </is>
       </c>
       <c r="E415" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap Canada</t>
         </is>
       </c>
       <c r="F415" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p+18</t>
         </is>
       </c>
       <c r="G415" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H415" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="I415" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="K415" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L415" t="inlineStr">
@@ -34272,7 +34272,7 @@
       </c>
       <c r="S415" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-2</t>
+          <t xml:space="preserve">v-mv5d2kfh-2</t>
         </is>
       </c>
     </row>
@@ -34284,47 +34284,47 @@
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D416" t="inlineStr">
         <is>
-          <t xml:space="preserve">A4</t>
+          <t xml:space="preserve">F4</t>
         </is>
       </c>
       <c r="E416" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap Canada</t>
         </is>
       </c>
       <c r="F416" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p+18</t>
         </is>
       </c>
       <c r="G416" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H416" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="I416" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="K416" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L416" t="inlineStr">
@@ -34354,7 +34354,7 @@
       </c>
       <c r="S416" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-3</t>
+          <t xml:space="preserve">v-mv5d2kfh-3</t>
         </is>
       </c>
     </row>
@@ -34366,682 +34366,852 @@
       </c>
       <c r="B417" t="inlineStr">
         <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F5</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap Canada</t>
+        </is>
+      </c>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p+18</t>
+        </is>
+      </c>
+      <c r="G417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">relative</t>
+        </is>
+      </c>
+      <c r="H417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="I417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="K417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="L417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S417" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv5d2kfh-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F6</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap Canada</t>
+        </is>
+      </c>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p+18</t>
+        </is>
+      </c>
+      <c r="G418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">relative</t>
+        </is>
+      </c>
+      <c r="H418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="I418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="K418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="L418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S418" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv5d2kfh-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F7</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap Canada</t>
+        </is>
+      </c>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p+18</t>
+        </is>
+      </c>
+      <c r="G419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">relative</t>
+        </is>
+      </c>
+      <c r="H419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="I419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="K419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="L419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S419" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv5d2kfh-6</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F8</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap Canada</t>
+        </is>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p+18</t>
+        </is>
+      </c>
+      <c r="G420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">relative</t>
+        </is>
+      </c>
+      <c r="H420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="I420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="K420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="L420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S420" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv5d2kfh-7</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F9</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap Canada</t>
+        </is>
+      </c>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p+18</t>
+        </is>
+      </c>
+      <c r="G421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">relative</t>
+        </is>
+      </c>
+      <c r="H421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="I421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="K421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="L421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S421" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv5d2kfh-8</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
           <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
-      <c r="C417" t="inlineStr">
+      <c r="C422" t="inlineStr">
         <is>
           <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
-      <c r="D417" t="inlineStr">
+      <c r="D422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A1</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S422" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A2</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S423" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A3</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S424" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A4</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S425" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
         <is>
           <t xml:space="preserve">A5</t>
         </is>
       </c>
-      <c r="E417" t="inlineStr">
+      <c r="E426" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="F417" t="inlineStr">
+      <c r="F426" t="inlineStr">
         <is>
           <t xml:space="preserve">p18</t>
         </is>
       </c>
-      <c r="G417" t="inlineStr">
+      <c r="G426" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H417" t="inlineStr">
+      <c r="H426" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
-      <c r="I417" t="inlineStr">
+      <c r="I426" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
-      <c r="K417" t="inlineStr">
+      <c r="K426" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L417" t="inlineStr">
+      <c r="L426" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
         </is>
       </c>
-      <c r="M417" t="inlineStr">
+      <c r="M426" t="inlineStr">
         <is>
           <t xml:space="preserve">Par</t>
         </is>
       </c>
-      <c r="N417" t="inlineStr">
+      <c r="N426" t="inlineStr">
         <is>
           <t xml:space="preserve">No Casp</t>
         </is>
       </c>
-      <c r="O417" t="inlineStr">
+      <c r="O426" t="inlineStr">
         <is>
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
-      <c r="R417" t="inlineStr">
+      <c r="R426" t="inlineStr">
         <is>
           <t xml:space="preserve">stored</t>
         </is>
       </c>
-      <c r="S417" t="inlineStr">
+      <c r="S426" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mupot2zh-4</t>
-        </is>
-      </c>
-    </row>
-    <row r="418">
-      <c r="E418" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNCX</t>
-        </is>
-      </c>
-      <c r="F418" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p+21</t>
-        </is>
-      </c>
-      <c r="G418" t="inlineStr">
-        <is>
-          <t xml:space="preserve">relative</t>
-        </is>
-      </c>
-      <c r="H418" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-05-15</t>
-        </is>
-      </c>
-      <c r="I418" t="inlineStr">
-        <is>
-          <t xml:space="preserve">15-05-26</t>
-        </is>
-      </c>
-      <c r="K418" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="L418" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M418" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N418" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CASPEX</t>
-        </is>
-      </c>
-      <c r="O418" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R418" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S418" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-199</t>
-        </is>
-      </c>
-    </row>
-    <row r="419">
-      <c r="E419" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LUCX</t>
-        </is>
-      </c>
-      <c r="F419" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p19</t>
-        </is>
-      </c>
-      <c r="G419" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H419" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-07-31</t>
-        </is>
-      </c>
-      <c r="I419" t="inlineStr">
-        <is>
-          <t xml:space="preserve">31-07-26</t>
-        </is>
-      </c>
-      <c r="K419" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR</t>
-        </is>
-      </c>
-      <c r="L419" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M419" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CR</t>
-        </is>
-      </c>
-      <c r="N419" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CASPEX</t>
-        </is>
-      </c>
-      <c r="O419" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="P419" t="inlineStr">
-        <is>
-          <t xml:space="preserve">to-do</t>
-        </is>
-      </c>
-      <c r="Q419" t="inlineStr">
-        <is>
-          <t xml:space="preserve">to-do box / thaw</t>
-        </is>
-      </c>
-      <c r="R419" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S419" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-233</t>
-        </is>
-      </c>
-    </row>
-    <row r="420">
-      <c r="E420" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145</t>
-        </is>
-      </c>
-      <c r="F420" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p?</t>
-        </is>
-      </c>
-      <c r="G420" t="inlineStr">
-        <is>
-          <t xml:space="preserve">unknown</t>
-        </is>
-      </c>
-      <c r="H420" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-06-30</t>
-        </is>
-      </c>
-      <c r="I420" t="inlineStr">
-        <is>
-          <t xml:space="preserve">30-06-25</t>
-        </is>
-      </c>
-      <c r="K420" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145</t>
-        </is>
-      </c>
-      <c r="L420" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M420" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N420" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O420" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R420" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S420" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-295</t>
-        </is>
-      </c>
-    </row>
-    <row r="421">
-      <c r="E421" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR</t>
-        </is>
-      </c>
-      <c r="F421" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p11</t>
-        </is>
-      </c>
-      <c r="G421" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H421" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-12</t>
-        </is>
-      </c>
-      <c r="I421" t="inlineStr">
-        <is>
-          <t xml:space="preserve">12/6/2026</t>
-        </is>
-      </c>
-      <c r="K421" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR</t>
-        </is>
-      </c>
-      <c r="L421" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M421" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CR</t>
-        </is>
-      </c>
-      <c r="N421" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O421" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R421" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S421" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-311</t>
-        </is>
-      </c>
-    </row>
-    <row r="422">
-      <c r="E422" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNCX</t>
-        </is>
-      </c>
-      <c r="F422" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p+17</t>
-        </is>
-      </c>
-      <c r="G422" t="inlineStr">
-        <is>
-          <t xml:space="preserve">relative</t>
-        </is>
-      </c>
-      <c r="H422" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-03-30</t>
-        </is>
-      </c>
-      <c r="I422" t="inlineStr">
-        <is>
-          <t xml:space="preserve">30-03-26</t>
-        </is>
-      </c>
-      <c r="K422" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="L422" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M422" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N422" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CASPEX</t>
-        </is>
-      </c>
-      <c r="O422" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R422" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S422" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-320</t>
-        </is>
-      </c>
-    </row>
-    <row r="423">
-      <c r="E423" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap Canada</t>
-        </is>
-      </c>
-      <c r="F423" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p+14</t>
-        </is>
-      </c>
-      <c r="G423" t="inlineStr">
-        <is>
-          <t xml:space="preserve">relative</t>
-        </is>
-      </c>
-      <c r="H423" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-03-23</t>
-        </is>
-      </c>
-      <c r="I423" t="inlineStr">
-        <is>
-          <t xml:space="preserve">23-03-26</t>
-        </is>
-      </c>
-      <c r="K423" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="L423" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M423" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N423" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O423" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R423" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S423" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-321</t>
-        </is>
-      </c>
-    </row>
-    <row r="424">
-      <c r="E424" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
-      <c r="F424" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p16</t>
-        </is>
-      </c>
-      <c r="G424" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H424" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-11-06</t>
-        </is>
-      </c>
-      <c r="I424" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6/11/2025</t>
-        </is>
-      </c>
-      <c r="K424" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
-      <c r="L424" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M424" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N424" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O424" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R424" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S424" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-338</t>
-        </is>
-      </c>
-    </row>
-    <row r="425">
-      <c r="E425" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7</t>
-        </is>
-      </c>
-      <c r="F425" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p15</t>
-        </is>
-      </c>
-      <c r="G425" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H425" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-08-10</t>
-        </is>
-      </c>
-      <c r="I425" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10/8/2026</t>
-        </is>
-      </c>
-      <c r="K425" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7</t>
-        </is>
-      </c>
-      <c r="L425" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M425" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N425" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O425" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R425" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S425" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-354</t>
-        </is>
-      </c>
-    </row>
-    <row r="426">
-      <c r="E426" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK gNT</t>
-        </is>
-      </c>
-      <c r="F426" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p21</t>
-        </is>
-      </c>
-      <c r="G426" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H426" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-07</t>
-        </is>
-      </c>
-      <c r="I426" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-07</t>
-        </is>
-      </c>
-      <c r="K426" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
-      <c r="L426" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M426" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N426" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O426" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gNT</t>
-        </is>
-      </c>
-      <c r="R426" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S426" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="E427" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F427" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p+21</t>
         </is>
       </c>
       <c r="G427" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H427" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-05-15</t>
         </is>
       </c>
       <c r="I427" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">15-05-26</t>
         </is>
       </c>
       <c r="K427" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L427" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M427" t="inlineStr">
@@ -35051,7 +35221,7 @@
       </c>
       <c r="N427" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O427" t="inlineStr">
@@ -35066,19 +35236,19 @@
       </c>
       <c r="S427" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdxsum-0</t>
+          <t xml:space="preserve">v-199</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="E428" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">LUCX</t>
         </is>
       </c>
       <c r="F428" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p19</t>
         </is>
       </c>
       <c r="G428" t="inlineStr">
@@ -35088,32 +35258,32 @@
       </c>
       <c r="H428" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-07-31</t>
         </is>
       </c>
       <c r="I428" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">31-07-26</t>
         </is>
       </c>
       <c r="K428" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L428" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M428" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N428" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O428" t="inlineStr">
@@ -35121,6 +35291,16 @@
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
+      <c r="P428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">to-do</t>
+        </is>
+      </c>
+      <c r="Q428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">to-do box / thaw</t>
+        </is>
+      </c>
       <c r="R428" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
@@ -35128,44 +35308,44 @@
       </c>
       <c r="S428" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-0</t>
+          <t xml:space="preserve">v-233</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="E429" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="F429" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p?</t>
         </is>
       </c>
       <c r="G429" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H429" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2025-06-30</t>
         </is>
       </c>
       <c r="I429" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">30-06-25</t>
         </is>
       </c>
       <c r="K429" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="L429" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M429" t="inlineStr">
@@ -35190,19 +35370,19 @@
       </c>
       <c r="S429" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-1</t>
+          <t xml:space="preserve">v-295</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="E430" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="F430" t="inlineStr">
         <is>
-          <t xml:space="preserve">p28</t>
+          <t xml:space="preserve">p11</t>
         </is>
       </c>
       <c r="G430" t="inlineStr">
@@ -35212,27 +35392,27 @@
       </c>
       <c r="H430" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-06-12</t>
         </is>
       </c>
       <c r="I430" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">12/6/2026</t>
         </is>
       </c>
       <c r="K430" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L430" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M430" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N430" t="inlineStr">
@@ -35252,39 +35432,39 @@
       </c>
       <c r="S430" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdz1vx-0</t>
+          <t xml:space="preserve">v-311</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="E431" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F431" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p+17</t>
         </is>
       </c>
       <c r="G431" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H431" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-03-30</t>
         </is>
       </c>
       <c r="I431" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">30-03-26</t>
         </is>
       </c>
       <c r="K431" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L431" t="inlineStr">
@@ -35299,12 +35479,12 @@
       </c>
       <c r="N431" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O431" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R431" t="inlineStr">
@@ -35314,44 +35494,44 @@
       </c>
       <c r="S431" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdzpx7-0</t>
+          <t xml:space="preserve">v-320</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="E432" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">LnCap Canada</t>
         </is>
       </c>
       <c r="F432" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p+14</t>
         </is>
       </c>
       <c r="G432" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H432" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-03-23</t>
         </is>
       </c>
       <c r="I432" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">23-03-26</t>
         </is>
       </c>
       <c r="K432" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L432" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M432" t="inlineStr">
@@ -35376,19 +35556,19 @@
       </c>
       <c r="S432" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0daw-0</t>
+          <t xml:space="preserve">v-321</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="E433" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="F433" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p16</t>
         </is>
       </c>
       <c r="G433" t="inlineStr">
@@ -35398,22 +35578,22 @@
       </c>
       <c r="H433" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2025-11-06</t>
         </is>
       </c>
       <c r="I433" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">6/11/2025</t>
         </is>
       </c>
       <c r="K433" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L433" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M433" t="inlineStr">
@@ -35438,19 +35618,19 @@
       </c>
       <c r="S433" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0w3q-0</t>
+          <t xml:space="preserve">v-338</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="E434" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="F434" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p15</t>
         </is>
       </c>
       <c r="G434" t="inlineStr">
@@ -35460,12 +35640,12 @@
       </c>
       <c r="H434" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-08-10</t>
         </is>
       </c>
       <c r="I434" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">10/8/2026</t>
         </is>
       </c>
       <c r="K434" t="inlineStr">
@@ -35475,7 +35655,7 @@
       </c>
       <c r="L434" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M434" t="inlineStr">
@@ -35500,19 +35680,19 @@
       </c>
       <c r="S434" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre1ko0-0</t>
+          <t xml:space="preserve">v-354</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="E435" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="F435" t="inlineStr">
         <is>
-          <t xml:space="preserve">p6</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G435" t="inlineStr">
@@ -35522,12 +35702,12 @@
       </c>
       <c r="H435" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I435" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="K435" t="inlineStr">
@@ -35547,12 +35727,12 @@
       </c>
       <c r="N435" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">No Casp</t>
         </is>
       </c>
       <c r="O435" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R435" t="inlineStr">
@@ -35562,34 +35742,44 @@
       </c>
       <c r="S435" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtski3re-0</t>
+          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="E436" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+        </is>
+      </c>
+      <c r="F436" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G436" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H436" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I436" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K436" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L436" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M436" t="inlineStr">
@@ -35614,34 +35804,44 @@
       </c>
       <c r="S436" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt0h140-0</t>
+          <t xml:space="preserve">v-mtrdxsum-0</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="E437" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F437" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G437" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H437" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I437" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K437" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L437" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M437" t="inlineStr">
@@ -35666,34 +35866,44 @@
       </c>
       <c r="S437" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-0</t>
+          <t xml:space="preserve">v-mtrdyhss-0</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="E438" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F438" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G438" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H438" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I438" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K438" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L438" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M438" t="inlineStr">
@@ -35718,34 +35928,44 @@
       </c>
       <c r="S438" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtrdyhss-1</t>
         </is>
       </c>
     </row>
     <row r="439">
       <c r="E439" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+        </is>
+      </c>
+      <c r="F439" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p28</t>
         </is>
       </c>
       <c r="G439" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H439" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I439" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K439" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L439" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M439" t="inlineStr">
@@ -35770,29 +35990,39 @@
       </c>
       <c r="S439" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-2</t>
+          <t xml:space="preserve">v-mtrdz1vx-0</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="E440" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">Huh7 gNT</t>
+        </is>
+      </c>
+      <c r="F440" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G440" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H440" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I440" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K440" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L440" t="inlineStr">
@@ -35812,7 +36042,7 @@
       </c>
       <c r="O440" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R440" t="inlineStr">
@@ -35822,34 +36052,44 @@
       </c>
       <c r="S440" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt5ckqo-0</t>
+          <t xml:space="preserve">v-mtrdzpx7-0</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="E441" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+        </is>
+      </c>
+      <c r="F441" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G441" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H441" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I441" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K441" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L441" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M441" t="inlineStr">
@@ -35874,34 +36114,44 @@
       </c>
       <c r="S441" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmw7m-0</t>
+          <t xml:space="preserve">v-mtre0daw-0</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="E442" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F442" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G442" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H442" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I442" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K442" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L442" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M442" t="inlineStr">
@@ -35926,34 +36176,44 @@
       </c>
       <c r="S442" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmypa-0</t>
+          <t xml:space="preserve">v-mtre0w3q-0</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="E443" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+        </is>
+      </c>
+      <c r="F443" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G443" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H443" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I443" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K443" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L443" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M443" t="inlineStr">
@@ -35978,34 +36238,39 @@
       </c>
       <c r="S443" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmn045-0</t>
+          <t xml:space="preserve">v-mtre1ko0-0</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="E444" t="inlineStr">
         <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">Hek caspex</t>
+        </is>
+      </c>
+      <c r="F444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p6</t>
         </is>
       </c>
       <c r="G444" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H444" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I444" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="K444" t="inlineStr">
         <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L444" t="inlineStr">
@@ -36020,7 +36285,7 @@
       </c>
       <c r="N444" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O444" t="inlineStr">
@@ -36035,44 +36300,34 @@
       </c>
       <c r="S444" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtu5lgdc-0</t>
+          <t xml:space="preserve">v-mtski3re-0</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="E445" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
-        </is>
-      </c>
-      <c r="F445" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p19</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="G445" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H445" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-17</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I445" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-17</t>
-        </is>
-      </c>
-      <c r="K445" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="L445" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M445" t="inlineStr">
@@ -36097,67 +36352,550 @@
       </c>
       <c r="S445" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mu5anec8-0</t>
+          <t xml:space="preserve">v-mtt0h140-0</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="E446" t="inlineStr">
         <is>
+          <t xml:space="preserve">jkl</t>
+        </is>
+      </c>
+      <c r="G446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="E447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jkl</t>
+        </is>
+      </c>
+      <c r="G447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="E448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jkl</t>
+        </is>
+      </c>
+      <c r="G448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt3mo6u-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="E449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">khk</t>
+        </is>
+      </c>
+      <c r="G449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt5ckqo-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="E450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="G450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mttmmw7m-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="E451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="G451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mttmmypa-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="E452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="G452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mttmn045-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="E453" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deneme</t>
+        </is>
+      </c>
+      <c r="G453" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H453" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I453" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="K453" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deneme</t>
+        </is>
+      </c>
+      <c r="L453" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M453" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N453" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O453" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R453" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S453" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtu5lgdc-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="E454" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F454" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p19</t>
+        </is>
+      </c>
+      <c r="G454" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H454" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-17</t>
+        </is>
+      </c>
+      <c r="I454" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-17</t>
+        </is>
+      </c>
+      <c r="K454" t="inlineStr">
+        <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="F446" t="inlineStr">
+      <c r="L454" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FLAG</t>
+        </is>
+      </c>
+      <c r="M454" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N454" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O454" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R454" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S454" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mu5anec8-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="E455" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F455" t="inlineStr">
         <is>
           <t xml:space="preserve">18</t>
         </is>
       </c>
-      <c r="G446" t="inlineStr">
+      <c r="G455" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H446" t="inlineStr">
+      <c r="H455" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
-      <c r="I446" t="inlineStr">
+      <c r="I455" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
-      <c r="K446" t="inlineStr">
+      <c r="K455" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L446" t="inlineStr">
+      <c r="L455" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
         </is>
       </c>
-      <c r="M446" t="inlineStr">
+      <c r="M455" t="inlineStr">
         <is>
           <t xml:space="preserve">Par</t>
         </is>
       </c>
-      <c r="N446" t="inlineStr">
+      <c r="N455" t="inlineStr">
         <is>
           <t xml:space="preserve">No Casp</t>
         </is>
       </c>
-      <c r="O446" t="inlineStr">
+      <c r="O455" t="inlineStr">
         <is>
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
-      <c r="R446" t="inlineStr">
+      <c r="R455" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
-      <c r="S446" t="inlineStr">
+      <c r="S455" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mv4yequa-5</t>
         </is>
@@ -36229,7 +36967,7 @@
         </is>
       </c>
       <c r="E2">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="F2">
         <v>1</v>
@@ -43877,10 +44615,10 @@
         <v>81</v>
       </c>
       <c r="I18">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="J18">
-        <v>44</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19">

</xml_diff>

<commit_message>
Add 9 × LNCX from Umut
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -34776,47 +34776,47 @@
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t xml:space="preserve">A1</t>
+          <t xml:space="preserve">G1</t>
         </is>
       </c>
       <c r="E422" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F422" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p+19</t>
         </is>
       </c>
       <c r="G422" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H422" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="I422" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="K422" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L422" t="inlineStr">
@@ -34831,7 +34831,7 @@
       </c>
       <c r="N422" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O422" t="inlineStr">
@@ -34846,7 +34846,7 @@
       </c>
       <c r="S422" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-0</t>
+          <t xml:space="preserve">v-mv5d4q3i-0</t>
         </is>
       </c>
     </row>
@@ -34858,47 +34858,47 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D423" t="inlineStr">
         <is>
-          <t xml:space="preserve">A2</t>
+          <t xml:space="preserve">G2</t>
         </is>
       </c>
       <c r="E423" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F423" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p+19</t>
         </is>
       </c>
       <c r="G423" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H423" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="I423" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="K423" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L423" t="inlineStr">
@@ -34913,7 +34913,7 @@
       </c>
       <c r="N423" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O423" t="inlineStr">
@@ -34928,7 +34928,7 @@
       </c>
       <c r="S423" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-1</t>
+          <t xml:space="preserve">v-mv5d4q3i-1</t>
         </is>
       </c>
     </row>
@@ -34940,47 +34940,47 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t xml:space="preserve">A3</t>
+          <t xml:space="preserve">G3</t>
         </is>
       </c>
       <c r="E424" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F424" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p+19</t>
         </is>
       </c>
       <c r="G424" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H424" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="I424" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="K424" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L424" t="inlineStr">
@@ -34995,7 +34995,7 @@
       </c>
       <c r="N424" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O424" t="inlineStr">
@@ -35010,7 +35010,7 @@
       </c>
       <c r="S424" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-2</t>
+          <t xml:space="preserve">v-mv5d4q3i-2</t>
         </is>
       </c>
     </row>
@@ -35022,47 +35022,47 @@
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D425" t="inlineStr">
         <is>
-          <t xml:space="preserve">A4</t>
+          <t xml:space="preserve">G4</t>
         </is>
       </c>
       <c r="E425" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F425" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p+19</t>
         </is>
       </c>
       <c r="G425" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H425" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="I425" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="K425" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L425" t="inlineStr">
@@ -35077,7 +35077,7 @@
       </c>
       <c r="N425" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O425" t="inlineStr">
@@ -35092,7 +35092,7 @@
       </c>
       <c r="S425" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-3</t>
+          <t xml:space="preserve">v-mv5d4q3i-3</t>
         </is>
       </c>
     </row>
@@ -35104,682 +35104,852 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">G5</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LNCX</t>
+        </is>
+      </c>
+      <c r="F426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p+19</t>
+        </is>
+      </c>
+      <c r="G426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">relative</t>
+        </is>
+      </c>
+      <c r="H426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="K426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="L426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASPEX</t>
+        </is>
+      </c>
+      <c r="O426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S426" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv5d4q3i-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">G6</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LNCX</t>
+        </is>
+      </c>
+      <c r="F427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p+19</t>
+        </is>
+      </c>
+      <c r="G427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">relative</t>
+        </is>
+      </c>
+      <c r="H427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="I427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="K427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="L427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASPEX</t>
+        </is>
+      </c>
+      <c r="O427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S427" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv5d4q3i-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">G7</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LNCX</t>
+        </is>
+      </c>
+      <c r="F428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p+19</t>
+        </is>
+      </c>
+      <c r="G428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">relative</t>
+        </is>
+      </c>
+      <c r="H428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="I428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="K428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="L428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASPEX</t>
+        </is>
+      </c>
+      <c r="O428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S428" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv5d4q3i-6</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">G8</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LNCX</t>
+        </is>
+      </c>
+      <c r="F429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p+19</t>
+        </is>
+      </c>
+      <c r="G429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">relative</t>
+        </is>
+      </c>
+      <c r="H429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="I429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="K429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="L429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASPEX</t>
+        </is>
+      </c>
+      <c r="O429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S429" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv5d4q3i-7</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">G9</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LNCX</t>
+        </is>
+      </c>
+      <c r="F430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p+19</t>
+        </is>
+      </c>
+      <c r="G430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">relative</t>
+        </is>
+      </c>
+      <c r="H430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="I430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="K430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="L430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASPEX</t>
+        </is>
+      </c>
+      <c r="O430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S430" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv5d4q3i-8</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
           <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
-      <c r="C426" t="inlineStr">
+      <c r="C431" t="inlineStr">
         <is>
           <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
-      <c r="D426" t="inlineStr">
+      <c r="D431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A1</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S431" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A2</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S432" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A3</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S433" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A4</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S434" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
         <is>
           <t xml:space="preserve">A5</t>
         </is>
       </c>
-      <c r="E426" t="inlineStr">
+      <c r="E435" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="F426" t="inlineStr">
+      <c r="F435" t="inlineStr">
         <is>
           <t xml:space="preserve">p18</t>
         </is>
       </c>
-      <c r="G426" t="inlineStr">
+      <c r="G435" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H426" t="inlineStr">
+      <c r="H435" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
-      <c r="I426" t="inlineStr">
+      <c r="I435" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
-      <c r="K426" t="inlineStr">
+      <c r="K435" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L426" t="inlineStr">
+      <c r="L435" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
         </is>
       </c>
-      <c r="M426" t="inlineStr">
+      <c r="M435" t="inlineStr">
         <is>
           <t xml:space="preserve">Par</t>
         </is>
       </c>
-      <c r="N426" t="inlineStr">
+      <c r="N435" t="inlineStr">
         <is>
           <t xml:space="preserve">No Casp</t>
         </is>
       </c>
-      <c r="O426" t="inlineStr">
+      <c r="O435" t="inlineStr">
         <is>
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
-      <c r="R426" t="inlineStr">
+      <c r="R435" t="inlineStr">
         <is>
           <t xml:space="preserve">stored</t>
         </is>
       </c>
-      <c r="S426" t="inlineStr">
+      <c r="S435" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mupot2zh-4</t>
-        </is>
-      </c>
-    </row>
-    <row r="427">
-      <c r="E427" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNCX</t>
-        </is>
-      </c>
-      <c r="F427" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p+21</t>
-        </is>
-      </c>
-      <c r="G427" t="inlineStr">
-        <is>
-          <t xml:space="preserve">relative</t>
-        </is>
-      </c>
-      <c r="H427" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-05-15</t>
-        </is>
-      </c>
-      <c r="I427" t="inlineStr">
-        <is>
-          <t xml:space="preserve">15-05-26</t>
-        </is>
-      </c>
-      <c r="K427" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="L427" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M427" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N427" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CASPEX</t>
-        </is>
-      </c>
-      <c r="O427" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R427" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S427" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-199</t>
-        </is>
-      </c>
-    </row>
-    <row r="428">
-      <c r="E428" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LUCX</t>
-        </is>
-      </c>
-      <c r="F428" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p19</t>
-        </is>
-      </c>
-      <c r="G428" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H428" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-07-31</t>
-        </is>
-      </c>
-      <c r="I428" t="inlineStr">
-        <is>
-          <t xml:space="preserve">31-07-26</t>
-        </is>
-      </c>
-      <c r="K428" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR</t>
-        </is>
-      </c>
-      <c r="L428" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M428" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CR</t>
-        </is>
-      </c>
-      <c r="N428" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CASPEX</t>
-        </is>
-      </c>
-      <c r="O428" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="P428" t="inlineStr">
-        <is>
-          <t xml:space="preserve">to-do</t>
-        </is>
-      </c>
-      <c r="Q428" t="inlineStr">
-        <is>
-          <t xml:space="preserve">to-do box / thaw</t>
-        </is>
-      </c>
-      <c r="R428" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S428" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-233</t>
-        </is>
-      </c>
-    </row>
-    <row r="429">
-      <c r="E429" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145</t>
-        </is>
-      </c>
-      <c r="F429" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p?</t>
-        </is>
-      </c>
-      <c r="G429" t="inlineStr">
-        <is>
-          <t xml:space="preserve">unknown</t>
-        </is>
-      </c>
-      <c r="H429" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-06-30</t>
-        </is>
-      </c>
-      <c r="I429" t="inlineStr">
-        <is>
-          <t xml:space="preserve">30-06-25</t>
-        </is>
-      </c>
-      <c r="K429" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145</t>
-        </is>
-      </c>
-      <c r="L429" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M429" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N429" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O429" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R429" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S429" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-295</t>
-        </is>
-      </c>
-    </row>
-    <row r="430">
-      <c r="E430" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR</t>
-        </is>
-      </c>
-      <c r="F430" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p11</t>
-        </is>
-      </c>
-      <c r="G430" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H430" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-12</t>
-        </is>
-      </c>
-      <c r="I430" t="inlineStr">
-        <is>
-          <t xml:space="preserve">12/6/2026</t>
-        </is>
-      </c>
-      <c r="K430" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR</t>
-        </is>
-      </c>
-      <c r="L430" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M430" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CR</t>
-        </is>
-      </c>
-      <c r="N430" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O430" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R430" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S430" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-311</t>
-        </is>
-      </c>
-    </row>
-    <row r="431">
-      <c r="E431" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNCX</t>
-        </is>
-      </c>
-      <c r="F431" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p+17</t>
-        </is>
-      </c>
-      <c r="G431" t="inlineStr">
-        <is>
-          <t xml:space="preserve">relative</t>
-        </is>
-      </c>
-      <c r="H431" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-03-30</t>
-        </is>
-      </c>
-      <c r="I431" t="inlineStr">
-        <is>
-          <t xml:space="preserve">30-03-26</t>
-        </is>
-      </c>
-      <c r="K431" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="L431" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M431" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N431" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CASPEX</t>
-        </is>
-      </c>
-      <c r="O431" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R431" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S431" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-320</t>
-        </is>
-      </c>
-    </row>
-    <row r="432">
-      <c r="E432" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap Canada</t>
-        </is>
-      </c>
-      <c r="F432" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p+14</t>
-        </is>
-      </c>
-      <c r="G432" t="inlineStr">
-        <is>
-          <t xml:space="preserve">relative</t>
-        </is>
-      </c>
-      <c r="H432" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-03-23</t>
-        </is>
-      </c>
-      <c r="I432" t="inlineStr">
-        <is>
-          <t xml:space="preserve">23-03-26</t>
-        </is>
-      </c>
-      <c r="K432" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="L432" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M432" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N432" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O432" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R432" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S432" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-321</t>
-        </is>
-      </c>
-    </row>
-    <row r="433">
-      <c r="E433" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
-      <c r="F433" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p16</t>
-        </is>
-      </c>
-      <c r="G433" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H433" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-11-06</t>
-        </is>
-      </c>
-      <c r="I433" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6/11/2025</t>
-        </is>
-      </c>
-      <c r="K433" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
-      <c r="L433" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M433" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N433" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O433" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R433" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S433" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-338</t>
-        </is>
-      </c>
-    </row>
-    <row r="434">
-      <c r="E434" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7</t>
-        </is>
-      </c>
-      <c r="F434" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p15</t>
-        </is>
-      </c>
-      <c r="G434" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H434" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-08-10</t>
-        </is>
-      </c>
-      <c r="I434" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10/8/2026</t>
-        </is>
-      </c>
-      <c r="K434" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7</t>
-        </is>
-      </c>
-      <c r="L434" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M434" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N434" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O434" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R434" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S434" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-354</t>
-        </is>
-      </c>
-    </row>
-    <row r="435">
-      <c r="E435" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK gNT</t>
-        </is>
-      </c>
-      <c r="F435" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p21</t>
-        </is>
-      </c>
-      <c r="G435" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H435" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-07</t>
-        </is>
-      </c>
-      <c r="I435" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-07</t>
-        </is>
-      </c>
-      <c r="K435" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
-      <c r="L435" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M435" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N435" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O435" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gNT</t>
-        </is>
-      </c>
-      <c r="R435" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S435" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="E436" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F436" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p+21</t>
         </is>
       </c>
       <c r="G436" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H436" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-05-15</t>
         </is>
       </c>
       <c r="I436" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">15-05-26</t>
         </is>
       </c>
       <c r="K436" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L436" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M436" t="inlineStr">
@@ -35789,7 +35959,7 @@
       </c>
       <c r="N436" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O436" t="inlineStr">
@@ -35804,19 +35974,19 @@
       </c>
       <c r="S436" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdxsum-0</t>
+          <t xml:space="preserve">v-199</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="E437" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">LUCX</t>
         </is>
       </c>
       <c r="F437" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p19</t>
         </is>
       </c>
       <c r="G437" t="inlineStr">
@@ -35826,32 +35996,32 @@
       </c>
       <c r="H437" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-07-31</t>
         </is>
       </c>
       <c r="I437" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">31-07-26</t>
         </is>
       </c>
       <c r="K437" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L437" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M437" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N437" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O437" t="inlineStr">
@@ -35859,6 +36029,16 @@
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
+      <c r="P437" t="inlineStr">
+        <is>
+          <t xml:space="preserve">to-do</t>
+        </is>
+      </c>
+      <c r="Q437" t="inlineStr">
+        <is>
+          <t xml:space="preserve">to-do box / thaw</t>
+        </is>
+      </c>
       <c r="R437" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
@@ -35866,44 +36046,44 @@
       </c>
       <c r="S437" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-0</t>
+          <t xml:space="preserve">v-233</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="E438" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="F438" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p?</t>
         </is>
       </c>
       <c r="G438" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H438" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2025-06-30</t>
         </is>
       </c>
       <c r="I438" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">30-06-25</t>
         </is>
       </c>
       <c r="K438" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="L438" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M438" t="inlineStr">
@@ -35928,19 +36108,19 @@
       </c>
       <c r="S438" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-1</t>
+          <t xml:space="preserve">v-295</t>
         </is>
       </c>
     </row>
     <row r="439">
       <c r="E439" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="F439" t="inlineStr">
         <is>
-          <t xml:space="preserve">p28</t>
+          <t xml:space="preserve">p11</t>
         </is>
       </c>
       <c r="G439" t="inlineStr">
@@ -35950,27 +36130,27 @@
       </c>
       <c r="H439" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-06-12</t>
         </is>
       </c>
       <c r="I439" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">12/6/2026</t>
         </is>
       </c>
       <c r="K439" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L439" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M439" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N439" t="inlineStr">
@@ -35990,39 +36170,39 @@
       </c>
       <c r="S439" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdz1vx-0</t>
+          <t xml:space="preserve">v-311</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="E440" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F440" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p+17</t>
         </is>
       </c>
       <c r="G440" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H440" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-03-30</t>
         </is>
       </c>
       <c r="I440" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">30-03-26</t>
         </is>
       </c>
       <c r="K440" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L440" t="inlineStr">
@@ -36037,12 +36217,12 @@
       </c>
       <c r="N440" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O440" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R440" t="inlineStr">
@@ -36052,44 +36232,44 @@
       </c>
       <c r="S440" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdzpx7-0</t>
+          <t xml:space="preserve">v-320</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="E441" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">LnCap Canada</t>
         </is>
       </c>
       <c r="F441" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p+14</t>
         </is>
       </c>
       <c r="G441" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H441" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-03-23</t>
         </is>
       </c>
       <c r="I441" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">23-03-26</t>
         </is>
       </c>
       <c r="K441" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L441" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M441" t="inlineStr">
@@ -36114,19 +36294,19 @@
       </c>
       <c r="S441" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0daw-0</t>
+          <t xml:space="preserve">v-321</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="E442" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="F442" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p16</t>
         </is>
       </c>
       <c r="G442" t="inlineStr">
@@ -36136,22 +36316,22 @@
       </c>
       <c r="H442" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2025-11-06</t>
         </is>
       </c>
       <c r="I442" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">6/11/2025</t>
         </is>
       </c>
       <c r="K442" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L442" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M442" t="inlineStr">
@@ -36176,19 +36356,19 @@
       </c>
       <c r="S442" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0w3q-0</t>
+          <t xml:space="preserve">v-338</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="E443" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="F443" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p15</t>
         </is>
       </c>
       <c r="G443" t="inlineStr">
@@ -36198,12 +36378,12 @@
       </c>
       <c r="H443" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-08-10</t>
         </is>
       </c>
       <c r="I443" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">10/8/2026</t>
         </is>
       </c>
       <c r="K443" t="inlineStr">
@@ -36213,7 +36393,7 @@
       </c>
       <c r="L443" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M443" t="inlineStr">
@@ -36238,19 +36418,19 @@
       </c>
       <c r="S443" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre1ko0-0</t>
+          <t xml:space="preserve">v-354</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="E444" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="F444" t="inlineStr">
         <is>
-          <t xml:space="preserve">p6</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G444" t="inlineStr">
@@ -36260,12 +36440,12 @@
       </c>
       <c r="H444" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I444" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="K444" t="inlineStr">
@@ -36285,12 +36465,12 @@
       </c>
       <c r="N444" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">No Casp</t>
         </is>
       </c>
       <c r="O444" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R444" t="inlineStr">
@@ -36300,34 +36480,44 @@
       </c>
       <c r="S444" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtski3re-0</t>
+          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="E445" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G445" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H445" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I445" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L445" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M445" t="inlineStr">
@@ -36352,34 +36542,44 @@
       </c>
       <c r="S445" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt0h140-0</t>
+          <t xml:space="preserve">v-mtrdxsum-0</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="E446" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G446" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H446" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I446" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L446" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M446" t="inlineStr">
@@ -36404,34 +36604,44 @@
       </c>
       <c r="S446" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-0</t>
+          <t xml:space="preserve">v-mtrdyhss-0</t>
         </is>
       </c>
     </row>
     <row r="447">
       <c r="E447" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G447" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H447" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I447" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L447" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M447" t="inlineStr">
@@ -36456,34 +36666,44 @@
       </c>
       <c r="S447" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtrdyhss-1</t>
         </is>
       </c>
     </row>
     <row r="448">
       <c r="E448" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+        </is>
+      </c>
+      <c r="F448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p28</t>
         </is>
       </c>
       <c r="G448" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H448" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I448" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L448" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M448" t="inlineStr">
@@ -36508,29 +36728,39 @@
       </c>
       <c r="S448" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-2</t>
+          <t xml:space="preserve">v-mtrdz1vx-0</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="E449" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">Huh7 gNT</t>
+        </is>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G449" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H449" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I449" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L449" t="inlineStr">
@@ -36550,7 +36780,7 @@
       </c>
       <c r="O449" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R449" t="inlineStr">
@@ -36560,34 +36790,44 @@
       </c>
       <c r="S449" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt5ckqo-0</t>
+          <t xml:space="preserve">v-mtrdzpx7-0</t>
         </is>
       </c>
     </row>
     <row r="450">
       <c r="E450" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+        </is>
+      </c>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G450" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H450" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I450" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L450" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M450" t="inlineStr">
@@ -36612,34 +36852,44 @@
       </c>
       <c r="S450" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmw7m-0</t>
+          <t xml:space="preserve">v-mtre0daw-0</t>
         </is>
       </c>
     </row>
     <row r="451">
       <c r="E451" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G451" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H451" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I451" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L451" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M451" t="inlineStr">
@@ -36664,34 +36914,44 @@
       </c>
       <c r="S451" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmypa-0</t>
+          <t xml:space="preserve">v-mtre0w3q-0</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="E452" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+        </is>
+      </c>
+      <c r="F452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G452" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H452" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I452" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L452" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M452" t="inlineStr">
@@ -36716,34 +36976,39 @@
       </c>
       <c r="S452" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmn045-0</t>
+          <t xml:space="preserve">v-mtre1ko0-0</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="E453" t="inlineStr">
         <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">Hek caspex</t>
+        </is>
+      </c>
+      <c r="F453" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p6</t>
         </is>
       </c>
       <c r="G453" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H453" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I453" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="K453" t="inlineStr">
         <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L453" t="inlineStr">
@@ -36758,7 +37023,7 @@
       </c>
       <c r="N453" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O453" t="inlineStr">
@@ -36773,44 +37038,34 @@
       </c>
       <c r="S453" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtu5lgdc-0</t>
+          <t xml:space="preserve">v-mtski3re-0</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="E454" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
-        </is>
-      </c>
-      <c r="F454" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p19</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="G454" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H454" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-17</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I454" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-17</t>
-        </is>
-      </c>
-      <c r="K454" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="L454" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M454" t="inlineStr">
@@ -36835,67 +37090,550 @@
       </c>
       <c r="S454" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mu5anec8-0</t>
+          <t xml:space="preserve">v-mtt0h140-0</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="E455" t="inlineStr">
         <is>
+          <t xml:space="preserve">jkl</t>
+        </is>
+      </c>
+      <c r="G455" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H455" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I455" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L455" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M455" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N455" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O455" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R455" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S455" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="E456" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jkl</t>
+        </is>
+      </c>
+      <c r="G456" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H456" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I456" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L456" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M456" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N456" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O456" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R456" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S456" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="E457" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jkl</t>
+        </is>
+      </c>
+      <c r="G457" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H457" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I457" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L457" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M457" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N457" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O457" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R457" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S457" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt3mo6u-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="E458" t="inlineStr">
+        <is>
+          <t xml:space="preserve">khk</t>
+        </is>
+      </c>
+      <c r="G458" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H458" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I458" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L458" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M458" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N458" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O458" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R458" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S458" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt5ckqo-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="E459" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="G459" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H459" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I459" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L459" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M459" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N459" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O459" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R459" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S459" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mttmmw7m-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="E460" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="G460" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H460" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I460" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L460" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M460" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N460" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O460" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R460" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S460" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mttmmypa-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="E461" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="G461" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H461" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I461" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L461" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M461" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N461" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O461" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R461" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S461" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mttmn045-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="E462" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deneme</t>
+        </is>
+      </c>
+      <c r="G462" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H462" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I462" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="K462" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deneme</t>
+        </is>
+      </c>
+      <c r="L462" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M462" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N462" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O462" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R462" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S462" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtu5lgdc-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="E463" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p19</t>
+        </is>
+      </c>
+      <c r="G463" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H463" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-17</t>
+        </is>
+      </c>
+      <c r="I463" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-17</t>
+        </is>
+      </c>
+      <c r="K463" t="inlineStr">
+        <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="F455" t="inlineStr">
+      <c r="L463" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FLAG</t>
+        </is>
+      </c>
+      <c r="M463" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N463" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O463" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R463" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S463" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mu5anec8-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="E464" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F464" t="inlineStr">
         <is>
           <t xml:space="preserve">18</t>
         </is>
       </c>
-      <c r="G455" t="inlineStr">
+      <c r="G464" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H455" t="inlineStr">
+      <c r="H464" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
-      <c r="I455" t="inlineStr">
+      <c r="I464" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
-      <c r="K455" t="inlineStr">
+      <c r="K464" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L455" t="inlineStr">
+      <c r="L464" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
         </is>
       </c>
-      <c r="M455" t="inlineStr">
+      <c r="M464" t="inlineStr">
         <is>
           <t xml:space="preserve">Par</t>
         </is>
       </c>
-      <c r="N455" t="inlineStr">
+      <c r="N464" t="inlineStr">
         <is>
           <t xml:space="preserve">No Casp</t>
         </is>
       </c>
-      <c r="O455" t="inlineStr">
+      <c r="O464" t="inlineStr">
         <is>
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
-      <c r="R455" t="inlineStr">
+      <c r="R464" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
-      <c r="S455" t="inlineStr">
+      <c r="S464" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mv4yequa-5</t>
         </is>
@@ -37010,54 +37748,54 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK</t>
+          <t xml:space="preserve">LNCX</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E4">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G4">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">HEK</t>
         </is>
       </c>
       <c r="E5">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
         <v>1</v>
-      </c>
-      <c r="G5">
-        <v>4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g1.1</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -37067,43 +37805,43 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1.1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E6">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gNT</t>
+          <t xml:space="preserve">DuDtxR CASPEX g1.1</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">g1.1</t>
         </is>
       </c>
       <c r="E7">
@@ -37113,18 +37851,18 @@
         <v>0</v>
       </c>
       <c r="G7">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LNCX gNT</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -37134,28 +37872,28 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E8">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G8">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -37169,7 +37907,7 @@
         </is>
       </c>
       <c r="E9">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F9">
         <v>1</v>
@@ -37181,12 +37919,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -37203,7 +37941,7 @@
         <v>10</v>
       </c>
       <c r="F10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G10">
         <v>3</v>
@@ -44615,10 +45353,10 @@
         <v>81</v>
       </c>
       <c r="I18">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="J18">
-        <v>35</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19">

</xml_diff>

<commit_message>
Add 9 × LuCap35CR from Umut
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -36252,27 +36252,27 @@
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D440" t="inlineStr">
         <is>
-          <t xml:space="preserve">A1</t>
+          <t xml:space="preserve">I1</t>
         </is>
       </c>
       <c r="E440" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="F440" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p13</t>
         </is>
       </c>
       <c r="G440" t="inlineStr">
@@ -36282,17 +36282,17 @@
       </c>
       <c r="H440" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="I440" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="K440" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L440" t="inlineStr">
@@ -36302,7 +36302,7 @@
       </c>
       <c r="M440" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N440" t="inlineStr">
@@ -36322,7 +36322,7 @@
       </c>
       <c r="S440" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-0</t>
+          <t xml:space="preserve">v-mv5d5bk8-0</t>
         </is>
       </c>
     </row>
@@ -36334,27 +36334,27 @@
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D441" t="inlineStr">
         <is>
-          <t xml:space="preserve">A2</t>
+          <t xml:space="preserve">I2</t>
         </is>
       </c>
       <c r="E441" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="F441" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p13</t>
         </is>
       </c>
       <c r="G441" t="inlineStr">
@@ -36364,17 +36364,17 @@
       </c>
       <c r="H441" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="I441" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="K441" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L441" t="inlineStr">
@@ -36384,7 +36384,7 @@
       </c>
       <c r="M441" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N441" t="inlineStr">
@@ -36404,7 +36404,7 @@
       </c>
       <c r="S441" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-1</t>
+          <t xml:space="preserve">v-mv5d5bk8-1</t>
         </is>
       </c>
     </row>
@@ -36416,27 +36416,27 @@
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D442" t="inlineStr">
         <is>
-          <t xml:space="preserve">A3</t>
+          <t xml:space="preserve">I3</t>
         </is>
       </c>
       <c r="E442" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="F442" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p13</t>
         </is>
       </c>
       <c r="G442" t="inlineStr">
@@ -36446,17 +36446,17 @@
       </c>
       <c r="H442" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="I442" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="K442" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L442" t="inlineStr">
@@ -36466,7 +36466,7 @@
       </c>
       <c r="M442" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N442" t="inlineStr">
@@ -36486,7 +36486,7 @@
       </c>
       <c r="S442" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-2</t>
+          <t xml:space="preserve">v-mv5d5bk8-2</t>
         </is>
       </c>
     </row>
@@ -36498,27 +36498,27 @@
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D443" t="inlineStr">
         <is>
-          <t xml:space="preserve">A4</t>
+          <t xml:space="preserve">I4</t>
         </is>
       </c>
       <c r="E443" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="F443" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p13</t>
         </is>
       </c>
       <c r="G443" t="inlineStr">
@@ -36528,17 +36528,17 @@
       </c>
       <c r="H443" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="I443" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="K443" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L443" t="inlineStr">
@@ -36548,7 +36548,7 @@
       </c>
       <c r="M443" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N443" t="inlineStr">
@@ -36568,7 +36568,7 @@
       </c>
       <c r="S443" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-3</t>
+          <t xml:space="preserve">v-mv5d5bk8-3</t>
         </is>
       </c>
     </row>
@@ -36580,682 +36580,852 @@
       </c>
       <c r="B444" t="inlineStr">
         <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I5</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LuCap35CR</t>
+        </is>
+      </c>
+      <c r="F444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p13</t>
+        </is>
+      </c>
+      <c r="G444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="I444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="K444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LuCap35CR</t>
+        </is>
+      </c>
+      <c r="L444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CR</t>
+        </is>
+      </c>
+      <c r="N444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S444" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv5d5bk8-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I6</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LuCap35CR</t>
+        </is>
+      </c>
+      <c r="F445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p13</t>
+        </is>
+      </c>
+      <c r="G445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="I445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="K445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LuCap35CR</t>
+        </is>
+      </c>
+      <c r="L445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CR</t>
+        </is>
+      </c>
+      <c r="N445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S445" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv5d5bk8-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I7</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LuCap35CR</t>
+        </is>
+      </c>
+      <c r="F446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p13</t>
+        </is>
+      </c>
+      <c r="G446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="I446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="K446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LuCap35CR</t>
+        </is>
+      </c>
+      <c r="L446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CR</t>
+        </is>
+      </c>
+      <c r="N446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S446" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv5d5bk8-6</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I8</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LuCap35CR</t>
+        </is>
+      </c>
+      <c r="F447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p13</t>
+        </is>
+      </c>
+      <c r="G447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="I447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="K447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LuCap35CR</t>
+        </is>
+      </c>
+      <c r="L447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CR</t>
+        </is>
+      </c>
+      <c r="N447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S447" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv5d5bk8-7</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 1</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">I9</t>
+        </is>
+      </c>
+      <c r="E448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LuCap35CR</t>
+        </is>
+      </c>
+      <c r="F448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p13</t>
+        </is>
+      </c>
+      <c r="G448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="I448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-12</t>
+        </is>
+      </c>
+      <c r="K448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LuCap35CR</t>
+        </is>
+      </c>
+      <c r="L448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CR</t>
+        </is>
+      </c>
+      <c r="N448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S448" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mv5d5bk8-8</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
           <t xml:space="preserve">Rack 2</t>
         </is>
       </c>
-      <c r="C444" t="inlineStr">
+      <c r="C449" t="inlineStr">
         <is>
           <t xml:space="preserve">Common Box #1</t>
         </is>
       </c>
-      <c r="D444" t="inlineStr">
+      <c r="D449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A1</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S449" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A2</t>
+        </is>
+      </c>
+      <c r="E450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S450" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A3</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S451" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A4</t>
+        </is>
+      </c>
+      <c r="E452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
+        </is>
+      </c>
+      <c r="G452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="I452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-01</t>
+        </is>
+      </c>
+      <c r="K452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="L452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S452" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mupot2zh-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
         <is>
           <t xml:space="preserve">A5</t>
         </is>
       </c>
-      <c r="E444" t="inlineStr">
+      <c r="E453" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="F444" t="inlineStr">
+      <c r="F453" t="inlineStr">
         <is>
           <t xml:space="preserve">p18</t>
         </is>
       </c>
-      <c r="G444" t="inlineStr">
+      <c r="G453" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H444" t="inlineStr">
+      <c r="H453" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
-      <c r="I444" t="inlineStr">
+      <c r="I453" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
-      <c r="K444" t="inlineStr">
+      <c r="K453" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L444" t="inlineStr">
+      <c r="L453" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
         </is>
       </c>
-      <c r="M444" t="inlineStr">
+      <c r="M453" t="inlineStr">
         <is>
           <t xml:space="preserve">Par</t>
         </is>
       </c>
-      <c r="N444" t="inlineStr">
+      <c r="N453" t="inlineStr">
         <is>
           <t xml:space="preserve">No Casp</t>
         </is>
       </c>
-      <c r="O444" t="inlineStr">
+      <c r="O453" t="inlineStr">
         <is>
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
-      <c r="R444" t="inlineStr">
+      <c r="R453" t="inlineStr">
         <is>
           <t xml:space="preserve">stored</t>
         </is>
       </c>
-      <c r="S444" t="inlineStr">
+      <c r="S453" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mupot2zh-4</t>
-        </is>
-      </c>
-    </row>
-    <row r="445">
-      <c r="E445" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNCX</t>
-        </is>
-      </c>
-      <c r="F445" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p+21</t>
-        </is>
-      </c>
-      <c r="G445" t="inlineStr">
-        <is>
-          <t xml:space="preserve">relative</t>
-        </is>
-      </c>
-      <c r="H445" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-05-15</t>
-        </is>
-      </c>
-      <c r="I445" t="inlineStr">
-        <is>
-          <t xml:space="preserve">15-05-26</t>
-        </is>
-      </c>
-      <c r="K445" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="L445" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M445" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N445" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CASPEX</t>
-        </is>
-      </c>
-      <c r="O445" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R445" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S445" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-199</t>
-        </is>
-      </c>
-    </row>
-    <row r="446">
-      <c r="E446" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LUCX</t>
-        </is>
-      </c>
-      <c r="F446" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p19</t>
-        </is>
-      </c>
-      <c r="G446" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H446" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-07-31</t>
-        </is>
-      </c>
-      <c r="I446" t="inlineStr">
-        <is>
-          <t xml:space="preserve">31-07-26</t>
-        </is>
-      </c>
-      <c r="K446" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR</t>
-        </is>
-      </c>
-      <c r="L446" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M446" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CR</t>
-        </is>
-      </c>
-      <c r="N446" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CASPEX</t>
-        </is>
-      </c>
-      <c r="O446" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="P446" t="inlineStr">
-        <is>
-          <t xml:space="preserve">to-do</t>
-        </is>
-      </c>
-      <c r="Q446" t="inlineStr">
-        <is>
-          <t xml:space="preserve">to-do box / thaw</t>
-        </is>
-      </c>
-      <c r="R446" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S446" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-233</t>
-        </is>
-      </c>
-    </row>
-    <row r="447">
-      <c r="E447" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145</t>
-        </is>
-      </c>
-      <c r="F447" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p?</t>
-        </is>
-      </c>
-      <c r="G447" t="inlineStr">
-        <is>
-          <t xml:space="preserve">unknown</t>
-        </is>
-      </c>
-      <c r="H447" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-06-30</t>
-        </is>
-      </c>
-      <c r="I447" t="inlineStr">
-        <is>
-          <t xml:space="preserve">30-06-25</t>
-        </is>
-      </c>
-      <c r="K447" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145</t>
-        </is>
-      </c>
-      <c r="L447" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M447" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N447" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O447" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R447" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S447" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-295</t>
-        </is>
-      </c>
-    </row>
-    <row r="448">
-      <c r="E448" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR</t>
-        </is>
-      </c>
-      <c r="F448" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p11</t>
-        </is>
-      </c>
-      <c r="G448" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H448" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-06-12</t>
-        </is>
-      </c>
-      <c r="I448" t="inlineStr">
-        <is>
-          <t xml:space="preserve">12/6/2026</t>
-        </is>
-      </c>
-      <c r="K448" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR</t>
-        </is>
-      </c>
-      <c r="L448" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M448" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CR</t>
-        </is>
-      </c>
-      <c r="N448" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O448" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R448" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S448" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-311</t>
-        </is>
-      </c>
-    </row>
-    <row r="449">
-      <c r="E449" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNCX</t>
-        </is>
-      </c>
-      <c r="F449" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p+17</t>
-        </is>
-      </c>
-      <c r="G449" t="inlineStr">
-        <is>
-          <t xml:space="preserve">relative</t>
-        </is>
-      </c>
-      <c r="H449" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-03-30</t>
-        </is>
-      </c>
-      <c r="I449" t="inlineStr">
-        <is>
-          <t xml:space="preserve">30-03-26</t>
-        </is>
-      </c>
-      <c r="K449" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="L449" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M449" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N449" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CASPEX</t>
-        </is>
-      </c>
-      <c r="O449" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R449" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S449" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-320</t>
-        </is>
-      </c>
-    </row>
-    <row r="450">
-      <c r="E450" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap Canada</t>
-        </is>
-      </c>
-      <c r="F450" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p+14</t>
-        </is>
-      </c>
-      <c r="G450" t="inlineStr">
-        <is>
-          <t xml:space="preserve">relative</t>
-        </is>
-      </c>
-      <c r="H450" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-03-23</t>
-        </is>
-      </c>
-      <c r="I450" t="inlineStr">
-        <is>
-          <t xml:space="preserve">23-03-26</t>
-        </is>
-      </c>
-      <c r="K450" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="L450" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M450" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N450" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O450" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R450" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S450" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-321</t>
-        </is>
-      </c>
-    </row>
-    <row r="451">
-      <c r="E451" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
-      <c r="F451" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p16</t>
-        </is>
-      </c>
-      <c r="G451" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H451" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-11-06</t>
-        </is>
-      </c>
-      <c r="I451" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6/11/2025</t>
-        </is>
-      </c>
-      <c r="K451" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
-      <c r="L451" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M451" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N451" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O451" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R451" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S451" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-338</t>
-        </is>
-      </c>
-    </row>
-    <row r="452">
-      <c r="E452" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7</t>
-        </is>
-      </c>
-      <c r="F452" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p15</t>
-        </is>
-      </c>
-      <c r="G452" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H452" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-08-10</t>
-        </is>
-      </c>
-      <c r="I452" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10/8/2026</t>
-        </is>
-      </c>
-      <c r="K452" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7</t>
-        </is>
-      </c>
-      <c r="L452" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M452" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N452" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O452" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R452" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S452" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-354</t>
-        </is>
-      </c>
-    </row>
-    <row r="453">
-      <c r="E453" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK gNT</t>
-        </is>
-      </c>
-      <c r="F453" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p21</t>
-        </is>
-      </c>
-      <c r="G453" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H453" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-07</t>
-        </is>
-      </c>
-      <c r="I453" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-09-07</t>
-        </is>
-      </c>
-      <c r="K453" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
-      <c r="L453" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M453" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N453" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No Casp</t>
-        </is>
-      </c>
-      <c r="O453" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gNT</t>
-        </is>
-      </c>
-      <c r="R453" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S453" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="E454" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F454" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p+21</t>
         </is>
       </c>
       <c r="G454" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H454" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-05-15</t>
         </is>
       </c>
       <c r="I454" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">15-05-26</t>
         </is>
       </c>
       <c r="K454" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L454" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M454" t="inlineStr">
@@ -37265,7 +37435,7 @@
       </c>
       <c r="N454" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O454" t="inlineStr">
@@ -37280,19 +37450,19 @@
       </c>
       <c r="S454" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdxsum-0</t>
+          <t xml:space="preserve">v-199</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="E455" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">LUCX</t>
         </is>
       </c>
       <c r="F455" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p19</t>
         </is>
       </c>
       <c r="G455" t="inlineStr">
@@ -37302,32 +37472,32 @@
       </c>
       <c r="H455" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-07-31</t>
         </is>
       </c>
       <c r="I455" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">31-07-26</t>
         </is>
       </c>
       <c r="K455" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L455" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M455" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N455" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O455" t="inlineStr">
@@ -37335,6 +37505,16 @@
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
+      <c r="P455" t="inlineStr">
+        <is>
+          <t xml:space="preserve">to-do</t>
+        </is>
+      </c>
+      <c r="Q455" t="inlineStr">
+        <is>
+          <t xml:space="preserve">to-do box / thaw</t>
+        </is>
+      </c>
       <c r="R455" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
@@ -37342,44 +37522,44 @@
       </c>
       <c r="S455" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-0</t>
+          <t xml:space="preserve">v-233</t>
         </is>
       </c>
     </row>
     <row r="456">
       <c r="E456" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="F456" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p?</t>
         </is>
       </c>
       <c r="G456" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H456" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2025-06-30</t>
         </is>
       </c>
       <c r="I456" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">30-06-25</t>
         </is>
       </c>
       <c r="K456" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="L456" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M456" t="inlineStr">
@@ -37404,19 +37584,19 @@
       </c>
       <c r="S456" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-1</t>
+          <t xml:space="preserve">v-295</t>
         </is>
       </c>
     </row>
     <row r="457">
       <c r="E457" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="F457" t="inlineStr">
         <is>
-          <t xml:space="preserve">p28</t>
+          <t xml:space="preserve">p11</t>
         </is>
       </c>
       <c r="G457" t="inlineStr">
@@ -37426,27 +37606,27 @@
       </c>
       <c r="H457" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-06-12</t>
         </is>
       </c>
       <c r="I457" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">12/6/2026</t>
         </is>
       </c>
       <c r="K457" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L457" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M457" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N457" t="inlineStr">
@@ -37466,39 +37646,39 @@
       </c>
       <c r="S457" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdz1vx-0</t>
+          <t xml:space="preserve">v-311</t>
         </is>
       </c>
     </row>
     <row r="458">
       <c r="E458" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F458" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p+17</t>
         </is>
       </c>
       <c r="G458" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H458" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-03-30</t>
         </is>
       </c>
       <c r="I458" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">30-03-26</t>
         </is>
       </c>
       <c r="K458" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L458" t="inlineStr">
@@ -37513,12 +37693,12 @@
       </c>
       <c r="N458" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O458" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R458" t="inlineStr">
@@ -37528,44 +37708,44 @@
       </c>
       <c r="S458" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdzpx7-0</t>
+          <t xml:space="preserve">v-320</t>
         </is>
       </c>
     </row>
     <row r="459">
       <c r="E459" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">LnCap Canada</t>
         </is>
       </c>
       <c r="F459" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p+14</t>
         </is>
       </c>
       <c r="G459" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H459" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-03-23</t>
         </is>
       </c>
       <c r="I459" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">23-03-26</t>
         </is>
       </c>
       <c r="K459" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L459" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M459" t="inlineStr">
@@ -37590,19 +37770,19 @@
       </c>
       <c r="S459" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0daw-0</t>
+          <t xml:space="preserve">v-321</t>
         </is>
       </c>
     </row>
     <row r="460">
       <c r="E460" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="F460" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p16</t>
         </is>
       </c>
       <c r="G460" t="inlineStr">
@@ -37612,22 +37792,22 @@
       </c>
       <c r="H460" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2025-11-06</t>
         </is>
       </c>
       <c r="I460" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">6/11/2025</t>
         </is>
       </c>
       <c r="K460" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L460" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M460" t="inlineStr">
@@ -37652,19 +37832,19 @@
       </c>
       <c r="S460" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0w3q-0</t>
+          <t xml:space="preserve">v-338</t>
         </is>
       </c>
     </row>
     <row r="461">
       <c r="E461" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="F461" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p15</t>
         </is>
       </c>
       <c r="G461" t="inlineStr">
@@ -37674,12 +37854,12 @@
       </c>
       <c r="H461" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-08-10</t>
         </is>
       </c>
       <c r="I461" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">10/8/2026</t>
         </is>
       </c>
       <c r="K461" t="inlineStr">
@@ -37689,7 +37869,7 @@
       </c>
       <c r="L461" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M461" t="inlineStr">
@@ -37714,19 +37894,19 @@
       </c>
       <c r="S461" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre1ko0-0</t>
+          <t xml:space="preserve">v-354</t>
         </is>
       </c>
     </row>
     <row r="462">
       <c r="E462" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="F462" t="inlineStr">
         <is>
-          <t xml:space="preserve">p6</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G462" t="inlineStr">
@@ -37736,12 +37916,12 @@
       </c>
       <c r="H462" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I462" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="K462" t="inlineStr">
@@ -37761,12 +37941,12 @@
       </c>
       <c r="N462" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">No Casp</t>
         </is>
       </c>
       <c r="O462" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R462" t="inlineStr">
@@ -37776,34 +37956,44 @@
       </c>
       <c r="S462" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtski3re-0</t>
+          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="463">
       <c r="E463" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+        </is>
+      </c>
+      <c r="F463" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G463" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H463" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I463" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K463" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L463" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M463" t="inlineStr">
@@ -37828,34 +38018,44 @@
       </c>
       <c r="S463" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt0h140-0</t>
+          <t xml:space="preserve">v-mtrdxsum-0</t>
         </is>
       </c>
     </row>
     <row r="464">
       <c r="E464" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F464" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G464" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H464" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I464" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K464" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L464" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M464" t="inlineStr">
@@ -37880,34 +38080,44 @@
       </c>
       <c r="S464" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-0</t>
+          <t xml:space="preserve">v-mtrdyhss-0</t>
         </is>
       </c>
     </row>
     <row r="465">
       <c r="E465" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F465" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G465" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H465" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I465" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K465" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L465" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M465" t="inlineStr">
@@ -37932,34 +38142,44 @@
       </c>
       <c r="S465" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtrdyhss-1</t>
         </is>
       </c>
     </row>
     <row r="466">
       <c r="E466" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+        </is>
+      </c>
+      <c r="F466" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p28</t>
         </is>
       </c>
       <c r="G466" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H466" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I466" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K466" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L466" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M466" t="inlineStr">
@@ -37984,29 +38204,39 @@
       </c>
       <c r="S466" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-2</t>
+          <t xml:space="preserve">v-mtrdz1vx-0</t>
         </is>
       </c>
     </row>
     <row r="467">
       <c r="E467" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">Huh7 gNT</t>
+        </is>
+      </c>
+      <c r="F467" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G467" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H467" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I467" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K467" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L467" t="inlineStr">
@@ -38026,7 +38256,7 @@
       </c>
       <c r="O467" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R467" t="inlineStr">
@@ -38036,34 +38266,44 @@
       </c>
       <c r="S467" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt5ckqo-0</t>
+          <t xml:space="preserve">v-mtrdzpx7-0</t>
         </is>
       </c>
     </row>
     <row r="468">
       <c r="E468" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G468" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H468" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I468" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K468" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L468" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M468" t="inlineStr">
@@ -38088,34 +38328,44 @@
       </c>
       <c r="S468" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmw7m-0</t>
+          <t xml:space="preserve">v-mtre0daw-0</t>
         </is>
       </c>
     </row>
     <row r="469">
       <c r="E469" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G469" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H469" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I469" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K469" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L469" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M469" t="inlineStr">
@@ -38140,34 +38390,44 @@
       </c>
       <c r="S469" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmypa-0</t>
+          <t xml:space="preserve">v-mtre0w3q-0</t>
         </is>
       </c>
     </row>
     <row r="470">
       <c r="E470" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G470" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H470" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I470" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K470" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L470" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M470" t="inlineStr">
@@ -38192,34 +38452,39 @@
       </c>
       <c r="S470" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmn045-0</t>
+          <t xml:space="preserve">v-mtre1ko0-0</t>
         </is>
       </c>
     </row>
     <row r="471">
       <c r="E471" t="inlineStr">
         <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">Hek caspex</t>
+        </is>
+      </c>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p6</t>
         </is>
       </c>
       <c r="G471" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H471" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I471" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="K471" t="inlineStr">
         <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L471" t="inlineStr">
@@ -38234,7 +38499,7 @@
       </c>
       <c r="N471" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O471" t="inlineStr">
@@ -38249,44 +38514,34 @@
       </c>
       <c r="S471" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtu5lgdc-0</t>
+          <t xml:space="preserve">v-mtski3re-0</t>
         </is>
       </c>
     </row>
     <row r="472">
       <c r="E472" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
-        </is>
-      </c>
-      <c r="F472" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p19</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="G472" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H472" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-17</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I472" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-17</t>
-        </is>
-      </c>
-      <c r="K472" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="L472" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M472" t="inlineStr">
@@ -38311,67 +38566,550 @@
       </c>
       <c r="S472" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mu5anec8-0</t>
+          <t xml:space="preserve">v-mtt0h140-0</t>
         </is>
       </c>
     </row>
     <row r="473">
       <c r="E473" t="inlineStr">
         <is>
+          <t xml:space="preserve">jkl</t>
+        </is>
+      </c>
+      <c r="G473" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H473" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I473" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L473" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M473" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N473" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O473" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R473" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S473" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="E474" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jkl</t>
+        </is>
+      </c>
+      <c r="G474" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H474" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I474" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L474" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M474" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N474" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O474" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R474" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S474" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="E475" t="inlineStr">
+        <is>
+          <t xml:space="preserve">jkl</t>
+        </is>
+      </c>
+      <c r="G475" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H475" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I475" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L475" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M475" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N475" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O475" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R475" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S475" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt3mo6u-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="E476" t="inlineStr">
+        <is>
+          <t xml:space="preserve">khk</t>
+        </is>
+      </c>
+      <c r="G476" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H476" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="I476" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-08</t>
+        </is>
+      </c>
+      <c r="L476" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M476" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N476" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O476" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R476" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S476" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtt5ckqo-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="E477" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="G477" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H477" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I477" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L477" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M477" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N477" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O477" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R477" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S477" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mttmmw7m-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="E478" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="G478" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H478" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I478" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L478" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M478" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N478" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O478" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R478" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S478" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mttmmypa-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="E479" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="G479" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H479" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I479" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="L479" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M479" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N479" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O479" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R479" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S479" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mttmn045-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="E480" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deneme</t>
+        </is>
+      </c>
+      <c r="G480" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H480" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I480" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="K480" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deneme</t>
+        </is>
+      </c>
+      <c r="L480" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M480" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N480" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O480" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R480" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S480" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtu5lgdc-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="E481" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F481" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p19</t>
+        </is>
+      </c>
+      <c r="G481" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H481" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-17</t>
+        </is>
+      </c>
+      <c r="I481" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-17</t>
+        </is>
+      </c>
+      <c r="K481" t="inlineStr">
+        <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="F473" t="inlineStr">
+      <c r="L481" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FLAG</t>
+        </is>
+      </c>
+      <c r="M481" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N481" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O481" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R481" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S481" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mu5anec8-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="E482" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F482" t="inlineStr">
         <is>
           <t xml:space="preserve">18</t>
         </is>
       </c>
-      <c r="G473" t="inlineStr">
+      <c r="G482" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H473" t="inlineStr">
+      <c r="H482" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
-      <c r="I473" t="inlineStr">
+      <c r="I482" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
-      <c r="K473" t="inlineStr">
+      <c r="K482" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L473" t="inlineStr">
+      <c r="L482" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
         </is>
       </c>
-      <c r="M473" t="inlineStr">
+      <c r="M482" t="inlineStr">
         <is>
           <t xml:space="preserve">Par</t>
         </is>
       </c>
-      <c r="N473" t="inlineStr">
+      <c r="N482" t="inlineStr">
         <is>
           <t xml:space="preserve">No Casp</t>
         </is>
       </c>
-      <c r="O473" t="inlineStr">
+      <c r="O482" t="inlineStr">
         <is>
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
-      <c r="R473" t="inlineStr">
+      <c r="R482" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
-      <c r="S473" t="inlineStr">
+      <c r="S482" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mv4yequa-5</t>
         </is>
@@ -38486,12 +39224,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -38505,66 +39243,66 @@
         </is>
       </c>
       <c r="E4">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G4">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK</t>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E5">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G5">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Du145</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">HEK</t>
         </is>
       </c>
       <c r="E6">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
         <v>1</v>
-      </c>
-      <c r="G6">
-        <v>4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g1.1</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -38574,43 +39312,43 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1.1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E7">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gNT</t>
+          <t xml:space="preserve">DuDtxR CASPEX g1.1</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">g1.1</t>
         </is>
       </c>
       <c r="E8">
@@ -38620,18 +39358,18 @@
         <v>0</v>
       </c>
       <c r="G8">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LNCX gNT</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -38641,17 +39379,17 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E9">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
@@ -46091,10 +46829,10 @@
         <v>81</v>
       </c>
       <c r="I18">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="J18">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19">

</xml_diff>

<commit_message>
Edit LNCX gP1 from Umut
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -31101,7 +31101,7 @@
       </c>
       <c r="E377" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gNT</t>
+          <t xml:space="preserve">LNCX gP1</t>
         </is>
       </c>
       <c r="F377" t="inlineStr">
@@ -31146,7 +31146,7 @@
       </c>
       <c r="O377" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">gP1</t>
         </is>
       </c>
       <c r="R377" t="inlineStr">
@@ -39473,7 +39473,7 @@
         </is>
       </c>
       <c r="E9">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F9">
         <v>0</v>
@@ -39795,7 +39795,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G1</t>
+          <t xml:space="preserve">LNCX gP1</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -39810,7 +39810,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gP1</t>
         </is>
       </c>
       <c r="E20">
@@ -39820,23 +39820,23 @@
         <v>0</v>
       </c>
       <c r="G20">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO G1</t>
+          <t xml:space="preserve">LnCap Canada V1G1</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -39845,19 +39845,19 @@
         </is>
       </c>
       <c r="E21">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F21">
         <v>0</v>
       </c>
       <c r="G21">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK TOX4 OX</t>
+          <t xml:space="preserve">HEK CBX3 KO G1</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -39867,7 +39867,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -39882,13 +39882,13 @@
         <v>0</v>
       </c>
       <c r="G22">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
+          <t xml:space="preserve">HEK TOX4 OX</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -39898,33 +39898,33 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E23">
         <v>5</v>
       </c>
       <c r="F23">
+        <v>0</v>
+      </c>
+      <c r="G23">
         <v>1</v>
-      </c>
-      <c r="G23">
-        <v>3</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gP1</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -39934,17 +39934,17 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">gP1</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E24">
         <v>5</v>
       </c>
       <c r="F24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G24">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">

</xml_diff>

<commit_message>
Edit LNCX gP2 from Umut
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -31183,7 +31183,7 @@
       </c>
       <c r="E378" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gNT</t>
+          <t xml:space="preserve">LNCX gP2</t>
         </is>
       </c>
       <c r="F378" t="inlineStr">
@@ -31228,7 +31228,7 @@
       </c>
       <c r="O378" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">gP2</t>
         </is>
       </c>
       <c r="R378" t="inlineStr">
@@ -39473,7 +39473,7 @@
         </is>
       </c>
       <c r="E9">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F9">
         <v>0</v>
@@ -39578,12 +39578,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX</t>
+          <t xml:space="preserve">LNCX gP2</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -39593,69 +39593,69 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gP2</t>
         </is>
       </c>
       <c r="E13">
         <v>8</v>
       </c>
       <c r="F13">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G13">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX DSg1.2</t>
+          <t xml:space="preserve">LUCX</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">DSg1.2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E14">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G14">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B KO g3</t>
+          <t xml:space="preserve">DuDtxR CASPEX DSg1.2</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">g3</t>
+          <t xml:space="preserve">DSg1.2</t>
         </is>
       </c>
       <c r="E15">
@@ -39665,13 +39665,13 @@
         <v>0</v>
       </c>
       <c r="G15">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 KO g1</t>
+          <t xml:space="preserve">HEK ATP7B KO g3</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -39681,12 +39681,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">g3</t>
         </is>
       </c>
       <c r="E16">
@@ -39696,28 +39696,28 @@
         <v>0</v>
       </c>
       <c r="G16">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gP2</t>
+          <t xml:space="preserve">HEK HOXB6 KO g1</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">gP2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E17">
@@ -39727,7 +39727,7 @@
         <v>0</v>
       </c>
       <c r="G17">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
Edit LNCX gP3 from Umut
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -31265,7 +31265,7 @@
       </c>
       <c r="E379" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gNT</t>
+          <t xml:space="preserve">LNCX gP3</t>
         </is>
       </c>
       <c r="F379" t="inlineStr">
@@ -31310,7 +31310,7 @@
       </c>
       <c r="O379" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">gP3</t>
         </is>
       </c>
       <c r="R379" t="inlineStr">
@@ -39454,12 +39454,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gNT</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -39469,28 +39469,28 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E9">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LNCX gNT</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -39500,17 +39500,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E10">
         <v>10</v>
       </c>
       <c r="F10">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -40260,7 +40260,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada CASPEX (no sort)</t>
+          <t xml:space="preserve">LNCX gP3</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -40270,12 +40270,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gP3</t>
         </is>
       </c>
       <c r="E35">
@@ -40285,32 +40285,32 @@
         <v>0</v>
       </c>
       <c r="G35">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145 TOX4 KO g2.2</t>
+          <t xml:space="preserve">LnCap Canada CASPEX (no sort)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2.2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E36">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F36">
         <v>0</v>
@@ -40322,7 +40322,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR</t>
+          <t xml:space="preserve">Du145 TOX4 KO g2.2</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -40332,12 +40332,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2.2</t>
         </is>
       </c>
       <c r="E37">
@@ -40353,7 +40353,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR ATF3 KO</t>
+          <t xml:space="preserve">DuDtxR</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -40363,7 +40363,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -40384,7 +40384,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR ATP7B KO</t>
+          <t xml:space="preserve">DuPar50CR ATF3 KO</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -40415,7 +40415,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR MTF1 KO</t>
+          <t xml:space="preserve">DuPar50CR ATP7B KO</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -40446,7 +40446,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR NT KO</t>
+          <t xml:space="preserve">DuPar50CR MTF1 KO</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -40477,7 +40477,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR TOX4 KO g1.2</t>
+          <t xml:space="preserve">DuPar50CR NT KO</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -40487,12 +40487,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1.2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E42">
@@ -40508,7 +40508,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR TOX4 KO g2.2</t>
+          <t xml:space="preserve">DuPar50CR TOX4 KO g1.2</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -40523,7 +40523,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2.2</t>
+          <t xml:space="preserve">g1.2</t>
         </is>
       </c>
       <c r="E43">
@@ -40539,29 +40539,29 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">DuPar50CR TOX4 KO g2.2</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2.2</t>
         </is>
       </c>
       <c r="E44">
         <v>2</v>
       </c>
       <c r="F44">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G44">
         <v>1</v>
@@ -40570,7 +40570,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -40580,7 +40580,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -40601,7 +40601,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CASPEX Single</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -40611,7 +40611,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -40623,7 +40623,7 @@
         <v>2</v>
       </c>
       <c r="F46">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G46">
         <v>1</v>
@@ -40632,7 +40632,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX</t>
+          <t xml:space="preserve">HEK CASPEX Single</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -40642,12 +40642,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E47">
@@ -40663,7 +40663,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK E2F1 sh1</t>
+          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -40673,12 +40673,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E48">
@@ -40694,7 +40694,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK E2F1 sh2</t>
+          <t xml:space="preserve">HEK E2F1 sh1</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -40725,7 +40725,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK FOXA1 KO g1</t>
+          <t xml:space="preserve">HEK E2F1 sh2</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -40735,12 +40735,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E50">
@@ -40756,7 +40756,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK FOXA1 KO g2</t>
+          <t xml:space="preserve">HEK FOXA1 KO g1</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -40771,7 +40771,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E51">
@@ -40787,7 +40787,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 OX</t>
+          <t xml:space="preserve">HEK FOXA1 KO g2</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -40802,7 +40802,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E52">
@@ -40818,7 +40818,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g1</t>
+          <t xml:space="preserve">HEK HOXB6 OX</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -40828,12 +40828,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E53">
@@ -40843,13 +40843,13 @@
         <v>0</v>
       </c>
       <c r="G53">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g2</t>
+          <t xml:space="preserve">HEK POU3F3 KO g1</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -40864,7 +40864,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E54">
@@ -40874,13 +40874,13 @@
         <v>0</v>
       </c>
       <c r="G54">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK STAT1 KO g2</t>
+          <t xml:space="preserve">HEK POU3F3 KO g2</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -40911,7 +40911,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT(20)</t>
+          <t xml:space="preserve">HEK STAT1 KO g2</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -40921,12 +40921,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E56">
@@ -40936,35 +40936,35 @@
         <v>0</v>
       </c>
       <c r="G56">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">HEK gNT(20)</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E57">
         <v>2</v>
       </c>
       <c r="F57">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G57">
         <v>2</v>
@@ -40973,7 +40973,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -40983,7 +40983,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -40995,16 +40995,16 @@
         <v>2</v>
       </c>
       <c r="F58">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G58">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -41014,7 +41014,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -41035,7 +41035,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATP7B KO #24</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -41045,7 +41045,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -41057,7 +41057,7 @@
         <v>2</v>
       </c>
       <c r="F60">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G60">
         <v>1</v>
@@ -41066,17 +41066,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-V</t>
+          <t xml:space="preserve">Huh7 ATP7B KO #24</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -41091,13 +41091,13 @@
         <v>0</v>
       </c>
       <c r="G61">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-V 99.17%</t>
+          <t xml:space="preserve">LCC-V</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -41128,7 +41128,22 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gC1</t>
+          <t xml:space="preserve">LCC-V 99.17%</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E63">
@@ -41138,13 +41153,13 @@
         <v>0</v>
       </c>
       <c r="G63">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gC2</t>
+          <t xml:space="preserve">LNCX gC1</t>
         </is>
       </c>
       <c r="E64">
@@ -41160,22 +41175,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gC3</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gC3</t>
+          <t xml:space="preserve">LNCX gC2</t>
         </is>
       </c>
       <c r="E65">
@@ -41191,7 +41191,22 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gC4</t>
+          <t xml:space="preserve">LNCX gC3</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gC3</t>
         </is>
       </c>
       <c r="E66">
@@ -41207,22 +41222,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gP3</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gP3</t>
+          <t xml:space="preserve">LNCX gC4</t>
         </is>
       </c>
       <c r="E67">

</xml_diff>

<commit_message>
Edit LNCX gP4 from Umut
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -31347,7 +31347,7 @@
       </c>
       <c r="E380" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gNT</t>
+          <t xml:space="preserve">LNCX gP4</t>
         </is>
       </c>
       <c r="F380" t="inlineStr">
@@ -31392,7 +31392,7 @@
       </c>
       <c r="O380" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">gP4</t>
         </is>
       </c>
       <c r="R380" t="inlineStr">
@@ -39485,12 +39485,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gNT</t>
+          <t xml:space="preserve">HEK ATP7B-GFP</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -39500,11 +39500,11 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E10">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F10">
         <v>0</v>
@@ -39516,12 +39516,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B-GFP</t>
+          <t xml:space="preserve">LNCX gNT</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -39531,7 +39531,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E11">
@@ -43377,7 +43377,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX gC1</t>
+          <t xml:space="preserve">LNCX gP4</t>
         </is>
       </c>
       <c r="E137">
@@ -43393,7 +43393,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX gC2</t>
+          <t xml:space="preserve">LUCX gC1</t>
         </is>
       </c>
       <c r="E138">
@@ -43409,7 +43409,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX gC3</t>
+          <t xml:space="preserve">LUCX gC2</t>
         </is>
       </c>
       <c r="E139">
@@ -43425,7 +43425,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX gC4</t>
+          <t xml:space="preserve">LUCX gC3</t>
         </is>
       </c>
       <c r="E140">
@@ -43441,7 +43441,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX gP3</t>
+          <t xml:space="preserve">LUCX gC4</t>
         </is>
       </c>
       <c r="E141">
@@ -43457,22 +43457,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap (m3) no sort</t>
-        </is>
-      </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="D142" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">LUCX gP3</t>
         </is>
       </c>
       <c r="E142">
@@ -43488,7 +43473,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G2</t>
+          <t xml:space="preserve">LnCap (m3) no sort</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -43519,7 +43504,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G3</t>
+          <t xml:space="preserve">LnCap Canada V1G2</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -43550,7 +43535,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G4</t>
+          <t xml:space="preserve">LnCap Canada V1G3</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -43581,7 +43566,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap ER</t>
+          <t xml:space="preserve">LnCap Canada V1G4</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -43612,7 +43597,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap V1G1</t>
+          <t xml:space="preserve">LnCap ER</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -43643,7 +43628,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap478 #2 98%</t>
+          <t xml:space="preserve">LnCap V1G1</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -43674,7 +43659,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select</t>
+          <t xml:space="preserve">LnCap478 #2 98%</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -43684,7 +43669,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -43705,7 +43690,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCapCASPEX no select C</t>
+          <t xml:space="preserve">LnCapCASPEX no select</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -43736,17 +43721,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap (m1) no sort</t>
+          <t xml:space="preserve">LnCapCASPEX no select C</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -43767,7 +43752,12 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t xml:space="preserve">MDA-MB g1.1 p10</t>
+          <t xml:space="preserve">LuCap (m1) no sort</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -43777,7 +43767,7 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1.1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E152">
@@ -43793,7 +43783,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t xml:space="preserve">MDA-MB gNT</t>
+          <t xml:space="preserve">MDA-MB g1.1 p10</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -43803,7 +43793,7 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">g1.1</t>
         </is>
       </c>
       <c r="E153">
@@ -43819,23 +43809,33 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">MDA-MB gNT</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E154">
+        <v>1</v>
+      </c>
+      <c r="F154">
         <v>0</v>
       </c>
-      <c r="F154">
+      <c r="G154">
         <v>1</v>
-      </c>
-      <c r="G154">
-        <v>0</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">Hek caspex</t>
         </is>
       </c>
       <c r="E155">
@@ -43851,14 +43851,14 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">deneme</t>
         </is>
       </c>
       <c r="E156">
         <v>0</v>
       </c>
       <c r="F156">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G156">
         <v>0</v>
@@ -43867,14 +43867,14 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="E157">
         <v>0</v>
       </c>
       <c r="F157">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G157">
         <v>0</v>
@@ -43883,24 +43883,14 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
-        </is>
-      </c>
-      <c r="C158" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="D158" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">khk</t>
         </is>
       </c>
       <c r="E158">
         <v>0</v>
       </c>
       <c r="F158">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G158">
         <v>0</v>
@@ -43909,16 +43899,42 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">kkk</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E159">
         <v>0</v>
       </c>
       <c r="F159">
+        <v>3</v>
+      </c>
+      <c r="G159">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t xml:space="preserve">klm ox</t>
+        </is>
+      </c>
+      <c r="E160">
+        <v>0</v>
+      </c>
+      <c r="F160">
         <v>1</v>
       </c>
-      <c r="G159">
+      <c r="G160">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Edit LNCX gC1 from Umut
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -31429,7 +31429,7 @@
       </c>
       <c r="E381" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gNT</t>
+          <t xml:space="preserve">LNCX gC1</t>
         </is>
       </c>
       <c r="F381" t="inlineStr">
@@ -31474,7 +31474,7 @@
       </c>
       <c r="O381" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">gC1</t>
         </is>
       </c>
       <c r="R381" t="inlineStr">
@@ -39516,26 +39516,26 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gNT</t>
+          <t xml:space="preserve">DuDtxR CASPEX g5.1</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">g5.1</t>
         </is>
       </c>
       <c r="E11">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F11">
         <v>0</v>
@@ -39547,22 +39547,22 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g5.1</t>
+          <t xml:space="preserve">LNCX gNT</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">g5.1</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E12">
@@ -40260,22 +40260,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gP3</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gP3</t>
+          <t xml:space="preserve">LNCX gC1</t>
         </is>
       </c>
       <c r="E35">
@@ -40291,7 +40276,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada CASPEX (no sort)</t>
+          <t xml:space="preserve">LNCX gP3</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -40301,12 +40286,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gP3</t>
         </is>
       </c>
       <c r="E36">
@@ -40316,32 +40301,32 @@
         <v>0</v>
       </c>
       <c r="G36">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145 TOX4 KO g2.2</t>
+          <t xml:space="preserve">LnCap Canada CASPEX (no sort)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2.2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E37">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F37">
         <v>0</v>
@@ -40353,7 +40338,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR</t>
+          <t xml:space="preserve">Du145 TOX4 KO g2.2</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -40363,12 +40348,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2.2</t>
         </is>
       </c>
       <c r="E38">
@@ -40384,7 +40369,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR ATF3 KO</t>
+          <t xml:space="preserve">DuDtxR</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -40394,7 +40379,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -40415,7 +40400,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR ATP7B KO</t>
+          <t xml:space="preserve">DuPar50CR ATF3 KO</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -40446,7 +40431,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR MTF1 KO</t>
+          <t xml:space="preserve">DuPar50CR ATP7B KO</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -40477,7 +40462,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR NT KO</t>
+          <t xml:space="preserve">DuPar50CR MTF1 KO</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -40508,7 +40493,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR TOX4 KO g1.2</t>
+          <t xml:space="preserve">DuPar50CR NT KO</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -40518,12 +40503,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1.2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E43">
@@ -40539,7 +40524,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR TOX4 KO g2.2</t>
+          <t xml:space="preserve">DuPar50CR TOX4 KO g1.2</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -40554,7 +40539,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2.2</t>
+          <t xml:space="preserve">g1.2</t>
         </is>
       </c>
       <c r="E44">
@@ -40570,29 +40555,29 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">DuPar50CR TOX4 KO g2.2</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2.2</t>
         </is>
       </c>
       <c r="E45">
         <v>2</v>
       </c>
       <c r="F45">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G45">
         <v>1</v>
@@ -40601,7 +40586,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -40611,7 +40596,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -40632,7 +40617,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CASPEX Single</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -40642,7 +40627,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -40654,7 +40639,7 @@
         <v>2</v>
       </c>
       <c r="F47">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G47">
         <v>1</v>
@@ -40663,7 +40648,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX</t>
+          <t xml:space="preserve">HEK CASPEX Single</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -40673,12 +40658,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E48">
@@ -40694,7 +40679,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK E2F1 sh1</t>
+          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -40704,12 +40689,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E49">
@@ -40725,7 +40710,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK E2F1 sh2</t>
+          <t xml:space="preserve">HEK E2F1 sh1</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -40756,7 +40741,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK FOXA1 KO g1</t>
+          <t xml:space="preserve">HEK E2F1 sh2</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -40766,12 +40751,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E51">
@@ -40787,7 +40772,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK FOXA1 KO g2</t>
+          <t xml:space="preserve">HEK FOXA1 KO g1</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -40802,7 +40787,7 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E52">
@@ -40818,7 +40803,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 OX</t>
+          <t xml:space="preserve">HEK FOXA1 KO g2</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -40833,7 +40818,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E53">
@@ -40849,7 +40834,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g1</t>
+          <t xml:space="preserve">HEK HOXB6 OX</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -40859,12 +40844,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E54">
@@ -40874,13 +40859,13 @@
         <v>0</v>
       </c>
       <c r="G54">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g2</t>
+          <t xml:space="preserve">HEK POU3F3 KO g1</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -40895,7 +40880,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E55">
@@ -40905,13 +40890,13 @@
         <v>0</v>
       </c>
       <c r="G55">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK STAT1 KO g2</t>
+          <t xml:space="preserve">HEK POU3F3 KO g2</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -40942,7 +40927,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT(20)</t>
+          <t xml:space="preserve">HEK STAT1 KO g2</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -40952,12 +40937,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E57">
@@ -40967,35 +40952,35 @@
         <v>0</v>
       </c>
       <c r="G57">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">HEK gNT(20)</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E58">
         <v>2</v>
       </c>
       <c r="F58">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G58">
         <v>2</v>
@@ -41004,7 +40989,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -41014,7 +40999,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -41026,16 +41011,16 @@
         <v>2</v>
       </c>
       <c r="F59">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G59">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -41045,7 +41030,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -41066,7 +41051,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATP7B KO #24</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -41076,7 +41061,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -41088,7 +41073,7 @@
         <v>2</v>
       </c>
       <c r="F61">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G61">
         <v>1</v>
@@ -41097,17 +41082,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-V</t>
+          <t xml:space="preserve">Huh7 ATP7B KO #24</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -41122,13 +41107,13 @@
         <v>0</v>
       </c>
       <c r="G62">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-V 99.17%</t>
+          <t xml:space="preserve">LCC-V</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -41159,7 +41144,22 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gC1</t>
+          <t xml:space="preserve">LCC-V 99.17%</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E64">
@@ -41169,7 +41169,7 @@
         <v>0</v>
       </c>
       <c r="G64">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="65">

</xml_diff>

<commit_message>
Edit LNCX gC2 from Umut
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -31511,7 +31511,7 @@
       </c>
       <c r="E382" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gNT</t>
+          <t xml:space="preserve">LNCX gC2</t>
         </is>
       </c>
       <c r="F382" t="inlineStr">
@@ -31556,7 +31556,7 @@
       </c>
       <c r="O382" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">gC2</t>
         </is>
       </c>
       <c r="R382" t="inlineStr">
@@ -39547,7 +39547,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gNT</t>
+          <t xml:space="preserve">LNCX gP2</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -39562,7 +39562,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">gP2</t>
         </is>
       </c>
       <c r="E12">
@@ -39572,18 +39572,18 @@
         <v>0</v>
       </c>
       <c r="G12">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gP2</t>
+          <t xml:space="preserve">LUCX</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -39593,69 +39593,69 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">gP2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E13">
         <v>8</v>
       </c>
       <c r="F13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G13">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX</t>
+          <t xml:space="preserve">DuDtxR CASPEX DSg1.2</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">DSg1.2</t>
         </is>
       </c>
       <c r="E14">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G14">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX DSg1.2</t>
+          <t xml:space="preserve">HEK ATP7B KO g3</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">DSg1.2</t>
+          <t xml:space="preserve">g3</t>
         </is>
       </c>
       <c r="E15">
@@ -39665,13 +39665,13 @@
         <v>0</v>
       </c>
       <c r="G15">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B KO g3</t>
+          <t xml:space="preserve">HEK HOXB6 KO g1</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -39681,12 +39681,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">g3</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E16">
@@ -39696,28 +39696,28 @@
         <v>0</v>
       </c>
       <c r="G16">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 KO g1</t>
+          <t xml:space="preserve">LNCX gNT</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E17">
@@ -39727,7 +39727,7 @@
         <v>0</v>
       </c>
       <c r="G17">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18">
@@ -40276,22 +40276,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gP3</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gP3</t>
+          <t xml:space="preserve">LNCX gC2</t>
         </is>
       </c>
       <c r="E36">
@@ -40307,7 +40292,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada CASPEX (no sort)</t>
+          <t xml:space="preserve">LNCX gP3</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -40317,12 +40302,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gP3</t>
         </is>
       </c>
       <c r="E37">
@@ -40332,32 +40317,32 @@
         <v>0</v>
       </c>
       <c r="G37">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145 TOX4 KO g2.2</t>
+          <t xml:space="preserve">LnCap Canada CASPEX (no sort)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2.2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E38">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F38">
         <v>0</v>
@@ -40369,7 +40354,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR</t>
+          <t xml:space="preserve">Du145 TOX4 KO g2.2</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -40379,12 +40364,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2.2</t>
         </is>
       </c>
       <c r="E39">
@@ -40400,7 +40385,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR ATF3 KO</t>
+          <t xml:space="preserve">DuDtxR</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -40410,7 +40395,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -40431,7 +40416,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR ATP7B KO</t>
+          <t xml:space="preserve">DuPar50CR ATF3 KO</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -40462,7 +40447,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR MTF1 KO</t>
+          <t xml:space="preserve">DuPar50CR ATP7B KO</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -40493,7 +40478,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR NT KO</t>
+          <t xml:space="preserve">DuPar50CR MTF1 KO</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -40524,7 +40509,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR TOX4 KO g1.2</t>
+          <t xml:space="preserve">DuPar50CR NT KO</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -40534,12 +40519,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1.2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E44">
@@ -40555,7 +40540,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR TOX4 KO g2.2</t>
+          <t xml:space="preserve">DuPar50CR TOX4 KO g1.2</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -40570,7 +40555,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2.2</t>
+          <t xml:space="preserve">g1.2</t>
         </is>
       </c>
       <c r="E45">
@@ -40586,29 +40571,29 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">DuPar50CR TOX4 KO g2.2</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2.2</t>
         </is>
       </c>
       <c r="E46">
         <v>2</v>
       </c>
       <c r="F46">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G46">
         <v>1</v>
@@ -40617,7 +40602,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -40627,7 +40612,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -40648,7 +40633,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CASPEX Single</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -40658,7 +40643,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -40670,7 +40655,7 @@
         <v>2</v>
       </c>
       <c r="F48">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G48">
         <v>1</v>
@@ -40679,7 +40664,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX</t>
+          <t xml:space="preserve">HEK CASPEX Single</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -40689,12 +40674,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E49">
@@ -40710,7 +40695,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK E2F1 sh1</t>
+          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -40720,12 +40705,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E50">
@@ -40741,7 +40726,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK E2F1 sh2</t>
+          <t xml:space="preserve">HEK E2F1 sh1</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -40772,7 +40757,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK FOXA1 KO g1</t>
+          <t xml:space="preserve">HEK E2F1 sh2</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -40782,12 +40767,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E52">
@@ -40803,7 +40788,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK FOXA1 KO g2</t>
+          <t xml:space="preserve">HEK FOXA1 KO g1</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -40818,7 +40803,7 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E53">
@@ -40834,7 +40819,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 OX</t>
+          <t xml:space="preserve">HEK FOXA1 KO g2</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -40849,7 +40834,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E54">
@@ -40865,7 +40850,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g1</t>
+          <t xml:space="preserve">HEK HOXB6 OX</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -40875,12 +40860,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E55">
@@ -40890,13 +40875,13 @@
         <v>0</v>
       </c>
       <c r="G55">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g2</t>
+          <t xml:space="preserve">HEK POU3F3 KO g1</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -40911,7 +40896,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E56">
@@ -40921,13 +40906,13 @@
         <v>0</v>
       </c>
       <c r="G56">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK STAT1 KO g2</t>
+          <t xml:space="preserve">HEK POU3F3 KO g2</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -40958,7 +40943,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT(20)</t>
+          <t xml:space="preserve">HEK STAT1 KO g2</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -40968,12 +40953,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E58">
@@ -40983,35 +40968,35 @@
         <v>0</v>
       </c>
       <c r="G58">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">HEK gNT(20)</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E59">
         <v>2</v>
       </c>
       <c r="F59">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G59">
         <v>2</v>
@@ -41020,7 +41005,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -41030,7 +41015,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -41042,16 +41027,16 @@
         <v>2</v>
       </c>
       <c r="F60">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G60">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -41061,7 +41046,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -41082,7 +41067,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATP7B KO #24</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -41092,7 +41077,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -41104,7 +41089,7 @@
         <v>2</v>
       </c>
       <c r="F62">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G62">
         <v>1</v>
@@ -41113,17 +41098,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-V</t>
+          <t xml:space="preserve">Huh7 ATP7B KO #24</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -41138,13 +41123,13 @@
         <v>0</v>
       </c>
       <c r="G63">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-V 99.17%</t>
+          <t xml:space="preserve">LCC-V</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -41175,7 +41160,22 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gC2</t>
+          <t xml:space="preserve">LCC-V 99.17%</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E65">
@@ -41185,7 +41185,7 @@
         <v>0</v>
       </c>
       <c r="G65">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="66">

</xml_diff>

<commit_message>
Edit LNCX gC3 from Umut
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -31593,7 +31593,7 @@
       </c>
       <c r="E383" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gNT</t>
+          <t xml:space="preserve">LNCX gC3</t>
         </is>
       </c>
       <c r="F383" t="inlineStr">
@@ -31638,7 +31638,7 @@
       </c>
       <c r="O383" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">gC3</t>
         </is>
       </c>
       <c r="R383" t="inlineStr">
@@ -39702,38 +39702,38 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gNT</t>
+          <t xml:space="preserve">DuDtxR CASPEX g3</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">g3</t>
         </is>
       </c>
       <c r="E17">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F17">
         <v>0</v>
       </c>
       <c r="G17">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX g3</t>
+          <t xml:space="preserve">DuDtxR CASPEX gNT</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -39748,7 +39748,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">g3</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E18">
@@ -39764,17 +39764,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR CASPEX gNT</t>
+          <t xml:space="preserve">LNCX gNT</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -39789,7 +39789,7 @@
         <v>0</v>
       </c>
       <c r="G19">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20">
@@ -40292,7 +40292,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gP3</t>
+          <t xml:space="preserve">LNCX gC3</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -40307,7 +40307,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">gP3</t>
+          <t xml:space="preserve">gC3</t>
         </is>
       </c>
       <c r="E37">
@@ -40323,7 +40323,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada CASPEX (no sort)</t>
+          <t xml:space="preserve">LNCX gP3</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -40333,12 +40333,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gP3</t>
         </is>
       </c>
       <c r="E38">
@@ -40348,32 +40348,32 @@
         <v>0</v>
       </c>
       <c r="G38">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145 TOX4 KO g2.2</t>
+          <t xml:space="preserve">LnCap Canada CASPEX (no sort)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2.2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E39">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F39">
         <v>0</v>
@@ -40385,7 +40385,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR</t>
+          <t xml:space="preserve">Du145 TOX4 KO g2.2</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -40395,12 +40395,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2.2</t>
         </is>
       </c>
       <c r="E40">
@@ -40416,7 +40416,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR ATF3 KO</t>
+          <t xml:space="preserve">DuDtxR</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -40426,7 +40426,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -40447,7 +40447,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR ATP7B KO</t>
+          <t xml:space="preserve">DuPar50CR ATF3 KO</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -40478,7 +40478,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR MTF1 KO</t>
+          <t xml:space="preserve">DuPar50CR ATP7B KO</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -40509,7 +40509,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR NT KO</t>
+          <t xml:space="preserve">DuPar50CR MTF1 KO</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -40540,7 +40540,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR TOX4 KO g1.2</t>
+          <t xml:space="preserve">DuPar50CR NT KO</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -40550,12 +40550,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1.2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E45">
@@ -40571,7 +40571,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR TOX4 KO g2.2</t>
+          <t xml:space="preserve">DuPar50CR TOX4 KO g1.2</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -40586,7 +40586,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2.2</t>
+          <t xml:space="preserve">g1.2</t>
         </is>
       </c>
       <c r="E46">
@@ -40602,29 +40602,29 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">DuPar50CR TOX4 KO g2.2</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2.2</t>
         </is>
       </c>
       <c r="E47">
         <v>2</v>
       </c>
       <c r="F47">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G47">
         <v>1</v>
@@ -40633,7 +40633,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -40643,7 +40643,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -40664,7 +40664,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CASPEX Single</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -40674,7 +40674,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -40686,7 +40686,7 @@
         <v>2</v>
       </c>
       <c r="F49">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G49">
         <v>1</v>
@@ -40695,7 +40695,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX</t>
+          <t xml:space="preserve">HEK CASPEX Single</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -40705,12 +40705,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E50">
@@ -40726,7 +40726,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK E2F1 sh1</t>
+          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -40736,12 +40736,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E51">
@@ -40757,7 +40757,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK E2F1 sh2</t>
+          <t xml:space="preserve">HEK E2F1 sh1</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -40788,7 +40788,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK FOXA1 KO g1</t>
+          <t xml:space="preserve">HEK E2F1 sh2</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -40798,12 +40798,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E53">
@@ -40819,7 +40819,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK FOXA1 KO g2</t>
+          <t xml:space="preserve">HEK FOXA1 KO g1</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -40834,7 +40834,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E54">
@@ -40850,7 +40850,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 OX</t>
+          <t xml:space="preserve">HEK FOXA1 KO g2</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -40865,7 +40865,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E55">
@@ -40881,7 +40881,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g1</t>
+          <t xml:space="preserve">HEK HOXB6 OX</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -40891,12 +40891,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E56">
@@ -40906,13 +40906,13 @@
         <v>0</v>
       </c>
       <c r="G56">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g2</t>
+          <t xml:space="preserve">HEK POU3F3 KO g1</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -40927,7 +40927,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E57">
@@ -40937,13 +40937,13 @@
         <v>0</v>
       </c>
       <c r="G57">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK STAT1 KO g2</t>
+          <t xml:space="preserve">HEK POU3F3 KO g2</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -40974,7 +40974,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT(20)</t>
+          <t xml:space="preserve">HEK STAT1 KO g2</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -40984,12 +40984,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E59">
@@ -40999,35 +40999,35 @@
         <v>0</v>
       </c>
       <c r="G59">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">HEK gNT(20)</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E60">
         <v>2</v>
       </c>
       <c r="F60">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G60">
         <v>2</v>
@@ -41036,7 +41036,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -41046,7 +41046,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -41058,16 +41058,16 @@
         <v>2</v>
       </c>
       <c r="F61">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G61">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -41077,7 +41077,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -41098,7 +41098,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATP7B KO #24</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -41108,7 +41108,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -41120,7 +41120,7 @@
         <v>2</v>
       </c>
       <c r="F63">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G63">
         <v>1</v>
@@ -41129,17 +41129,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-V</t>
+          <t xml:space="preserve">Huh7 ATP7B KO #24</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -41154,13 +41154,13 @@
         <v>0</v>
       </c>
       <c r="G64">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-V 99.17%</t>
+          <t xml:space="preserve">LCC-V</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -41191,7 +41191,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gC3</t>
+          <t xml:space="preserve">LCC-V 99.17%</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -41201,12 +41201,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
           <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gC3</t>
         </is>
       </c>
       <c r="E66">
@@ -41216,7 +41216,7 @@
         <v>0</v>
       </c>
       <c r="G66">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="67">

</xml_diff>

<commit_message>
Edit LNCX gC4 from Umut
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -31675,7 +31675,7 @@
       </c>
       <c r="E384" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gNT</t>
+          <t xml:space="preserve">LNCX gC4</t>
         </is>
       </c>
       <c r="F384" t="inlineStr">
@@ -31720,7 +31720,7 @@
       </c>
       <c r="O384" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">gC4</t>
         </is>
       </c>
       <c r="R384" t="inlineStr">
@@ -39764,7 +39764,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gNT</t>
+          <t xml:space="preserve">LNCX gP1</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -39779,7 +39779,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">gP1</t>
         </is>
       </c>
       <c r="E19">
@@ -39789,13 +39789,13 @@
         <v>0</v>
       </c>
       <c r="G19">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gP1</t>
+          <t xml:space="preserve">LnCap Canada V1G1</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -39810,7 +39810,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">gP1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E20">
@@ -39820,23 +39820,23 @@
         <v>0</v>
       </c>
       <c r="G20">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada V1G1</t>
+          <t xml:space="preserve">HEK CBX3 KO G1</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -39845,19 +39845,19 @@
         </is>
       </c>
       <c r="E21">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F21">
         <v>0</v>
       </c>
       <c r="G21">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO G1</t>
+          <t xml:space="preserve">HEK TOX4 OX</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -39867,7 +39867,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -39882,13 +39882,13 @@
         <v>0</v>
       </c>
       <c r="G22">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK TOX4 OX</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -39898,33 +39898,33 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E23">
         <v>5</v>
       </c>
       <c r="F23">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G23">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
+          <t xml:space="preserve">LNCX gNT</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -39941,10 +39941,10 @@
         <v>5</v>
       </c>
       <c r="F24">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G24">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25">
@@ -40323,22 +40323,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gP3</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gP3</t>
+          <t xml:space="preserve">LNCX gC4</t>
         </is>
       </c>
       <c r="E38">
@@ -40354,7 +40339,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada CASPEX (no sort)</t>
+          <t xml:space="preserve">LNCX gP3</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -40364,12 +40349,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gP3</t>
         </is>
       </c>
       <c r="E39">
@@ -40379,32 +40364,32 @@
         <v>0</v>
       </c>
       <c r="G39">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145 TOX4 KO g2.2</t>
+          <t xml:space="preserve">LnCap Canada CASPEX (no sort)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2.2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E40">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F40">
         <v>0</v>
@@ -40416,7 +40401,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR</t>
+          <t xml:space="preserve">Du145 TOX4 KO g2.2</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -40426,12 +40411,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2.2</t>
         </is>
       </c>
       <c r="E41">
@@ -40447,7 +40432,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR ATF3 KO</t>
+          <t xml:space="preserve">DuDtxR</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -40457,7 +40442,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -40478,7 +40463,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR ATP7B KO</t>
+          <t xml:space="preserve">DuPar50CR ATF3 KO</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -40509,7 +40494,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR MTF1 KO</t>
+          <t xml:space="preserve">DuPar50CR ATP7B KO</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -40540,7 +40525,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR NT KO</t>
+          <t xml:space="preserve">DuPar50CR MTF1 KO</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -40571,7 +40556,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR TOX4 KO g1.2</t>
+          <t xml:space="preserve">DuPar50CR NT KO</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -40581,12 +40566,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1.2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E46">
@@ -40602,7 +40587,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR TOX4 KO g2.2</t>
+          <t xml:space="preserve">DuPar50CR TOX4 KO g1.2</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -40617,7 +40602,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2.2</t>
+          <t xml:space="preserve">g1.2</t>
         </is>
       </c>
       <c r="E47">
@@ -40633,29 +40618,29 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">DuPar50CR TOX4 KO g2.2</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2.2</t>
         </is>
       </c>
       <c r="E48">
         <v>2</v>
       </c>
       <c r="F48">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G48">
         <v>1</v>
@@ -40664,7 +40649,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -40674,7 +40659,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -40695,7 +40680,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CASPEX Single</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -40705,7 +40690,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -40717,7 +40702,7 @@
         <v>2</v>
       </c>
       <c r="F50">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G50">
         <v>1</v>
@@ -40726,7 +40711,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX</t>
+          <t xml:space="preserve">HEK CASPEX Single</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -40736,12 +40721,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E51">
@@ -40757,7 +40742,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK E2F1 sh1</t>
+          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -40767,12 +40752,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E52">
@@ -40788,7 +40773,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK E2F1 sh2</t>
+          <t xml:space="preserve">HEK E2F1 sh1</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -40819,7 +40804,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK FOXA1 KO g1</t>
+          <t xml:space="preserve">HEK E2F1 sh2</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -40829,12 +40814,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E54">
@@ -40850,7 +40835,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK FOXA1 KO g2</t>
+          <t xml:space="preserve">HEK FOXA1 KO g1</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -40865,7 +40850,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E55">
@@ -40881,7 +40866,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 OX</t>
+          <t xml:space="preserve">HEK FOXA1 KO g2</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -40896,7 +40881,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E56">
@@ -40912,7 +40897,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g1</t>
+          <t xml:space="preserve">HEK HOXB6 OX</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -40922,12 +40907,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E57">
@@ -40937,13 +40922,13 @@
         <v>0</v>
       </c>
       <c r="G57">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g2</t>
+          <t xml:space="preserve">HEK POU3F3 KO g1</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -40958,7 +40943,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E58">
@@ -40968,13 +40953,13 @@
         <v>0</v>
       </c>
       <c r="G58">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK STAT1 KO g2</t>
+          <t xml:space="preserve">HEK POU3F3 KO g2</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -41005,7 +40990,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT(20)</t>
+          <t xml:space="preserve">HEK STAT1 KO g2</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -41015,12 +41000,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E60">
@@ -41030,35 +41015,35 @@
         <v>0</v>
       </c>
       <c r="G60">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">HEK gNT(20)</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E61">
         <v>2</v>
       </c>
       <c r="F61">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G61">
         <v>2</v>
@@ -41067,7 +41052,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -41077,7 +41062,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -41089,16 +41074,16 @@
         <v>2</v>
       </c>
       <c r="F62">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G62">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -41108,7 +41093,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -41129,7 +41114,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATP7B KO #24</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -41139,7 +41124,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -41151,7 +41136,7 @@
         <v>2</v>
       </c>
       <c r="F64">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G64">
         <v>1</v>
@@ -41160,17 +41145,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-V</t>
+          <t xml:space="preserve">Huh7 ATP7B KO #24</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -41185,13 +41170,13 @@
         <v>0</v>
       </c>
       <c r="G65">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-V 99.17%</t>
+          <t xml:space="preserve">LCC-V</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -41222,7 +41207,22 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gC4</t>
+          <t xml:space="preserve">LCC-V 99.17%</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E67">
@@ -41232,7 +41232,7 @@
         <v>0</v>
       </c>
       <c r="G67">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="68">

</xml_diff>

<commit_message>
Edit LUCX gNT from Umut
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -23550,9 +23550,14 @@
           <t xml:space="preserve">LUCX gNT</t>
         </is>
       </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t xml:space="preserve">26</t>
+        </is>
+      </c>
       <c r="G285" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H285" t="inlineStr">

</xml_diff>

<commit_message>
Edit LUCX gP2 from Umut
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -37590,9 +37590,14 @@
           <t xml:space="preserve">LUCX gP2</t>
         </is>
       </c>
+      <c r="F455" t="inlineStr">
+        <is>
+          <t xml:space="preserve">26</t>
+        </is>
+      </c>
       <c r="G455" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H455" t="inlineStr">

</xml_diff>

<commit_message>
Edit LUCX gP4 from Umut
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -37754,9 +37754,14 @@
           <t xml:space="preserve">LUCX gP4</t>
         </is>
       </c>
+      <c r="F457" t="inlineStr">
+        <is>
+          <t xml:space="preserve">26</t>
+        </is>
+      </c>
       <c r="G457" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H457" t="inlineStr">

</xml_diff>

<commit_message>
Add 2 × LNC478 #2 from Umut
</commit_message>
<xml_diff>
--- a/cellstocks/data/umut.xlsx
+++ b/cellstocks/data/umut.xlsx
@@ -34458,17 +34458,17 @@
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t xml:space="preserve">E1</t>
+          <t xml:space="preserve">D7</t>
         </is>
       </c>
       <c r="E418" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK</t>
+          <t xml:space="preserve">LNC478 #2</t>
         </is>
       </c>
       <c r="F418" t="inlineStr">
         <is>
-          <t xml:space="preserve">30</t>
+          <t xml:space="preserve">27</t>
         </is>
       </c>
       <c r="G418" t="inlineStr">
@@ -34478,17 +34478,17 @@
       </c>
       <c r="H418" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-09</t>
+          <t xml:space="preserve">2026-11-01</t>
         </is>
       </c>
       <c r="I418" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-09</t>
+          <t xml:space="preserve">2026-11-01</t>
         </is>
       </c>
       <c r="K418" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L418" t="inlineStr">
@@ -34518,7 +34518,7 @@
       </c>
       <c r="S418" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv4yhtbo-0</t>
+          <t xml:space="preserve">v-mvxuhltp-0</t>
         </is>
       </c>
     </row>
@@ -34540,17 +34540,17 @@
       </c>
       <c r="D419" t="inlineStr">
         <is>
-          <t xml:space="preserve">E2</t>
+          <t xml:space="preserve">D8</t>
         </is>
       </c>
       <c r="E419" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK</t>
+          <t xml:space="preserve">LNC478 #2</t>
         </is>
       </c>
       <c r="F419" t="inlineStr">
         <is>
-          <t xml:space="preserve">30</t>
+          <t xml:space="preserve">27</t>
         </is>
       </c>
       <c r="G419" t="inlineStr">
@@ -34560,17 +34560,17 @@
       </c>
       <c r="H419" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-09</t>
+          <t xml:space="preserve">2026-11-01</t>
         </is>
       </c>
       <c r="I419" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-09</t>
+          <t xml:space="preserve">2026-11-01</t>
         </is>
       </c>
       <c r="K419" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L419" t="inlineStr">
@@ -34600,7 +34600,7 @@
       </c>
       <c r="S419" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv4yhtbo-1</t>
+          <t xml:space="preserve">v-mvxuhltp-1</t>
         </is>
       </c>
     </row>
@@ -34622,7 +34622,7 @@
       </c>
       <c r="D420" t="inlineStr">
         <is>
-          <t xml:space="preserve">E3</t>
+          <t xml:space="preserve">E1</t>
         </is>
       </c>
       <c r="E420" t="inlineStr">
@@ -34682,7 +34682,7 @@
       </c>
       <c r="S420" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv4yhtbo-2</t>
+          <t xml:space="preserve">v-mv4yhtbo-0</t>
         </is>
       </c>
     </row>
@@ -34704,7 +34704,7 @@
       </c>
       <c r="D421" t="inlineStr">
         <is>
-          <t xml:space="preserve">E4</t>
+          <t xml:space="preserve">E2</t>
         </is>
       </c>
       <c r="E421" t="inlineStr">
@@ -34764,7 +34764,7 @@
       </c>
       <c r="S421" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv4yhtbo-3</t>
+          <t xml:space="preserve">v-mv4yhtbo-1</t>
         </is>
       </c>
     </row>
@@ -34786,7 +34786,7 @@
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t xml:space="preserve">E5</t>
+          <t xml:space="preserve">E3</t>
         </is>
       </c>
       <c r="E422" t="inlineStr">
@@ -34846,7 +34846,7 @@
       </c>
       <c r="S422" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv4yhtbo-4</t>
+          <t xml:space="preserve">v-mv4yhtbo-2</t>
         </is>
       </c>
     </row>
@@ -34868,7 +34868,7 @@
       </c>
       <c r="D423" t="inlineStr">
         <is>
-          <t xml:space="preserve">E6</t>
+          <t xml:space="preserve">E4</t>
         </is>
       </c>
       <c r="E423" t="inlineStr">
@@ -34928,7 +34928,7 @@
       </c>
       <c r="S423" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv4yhtbo-5</t>
+          <t xml:space="preserve">v-mv4yhtbo-3</t>
         </is>
       </c>
     </row>
@@ -34950,7 +34950,7 @@
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t xml:space="preserve">E7</t>
+          <t xml:space="preserve">E5</t>
         </is>
       </c>
       <c r="E424" t="inlineStr">
@@ -35010,7 +35010,7 @@
       </c>
       <c r="S424" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv4yhtbo-6</t>
+          <t xml:space="preserve">v-mv4yhtbo-4</t>
         </is>
       </c>
     </row>
@@ -35032,7 +35032,7 @@
       </c>
       <c r="D425" t="inlineStr">
         <is>
-          <t xml:space="preserve">E8</t>
+          <t xml:space="preserve">E6</t>
         </is>
       </c>
       <c r="E425" t="inlineStr">
@@ -35092,7 +35092,7 @@
       </c>
       <c r="S425" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv4yhtbo-7</t>
+          <t xml:space="preserve">v-mv4yhtbo-5</t>
         </is>
       </c>
     </row>
@@ -35114,7 +35114,7 @@
       </c>
       <c r="D426" t="inlineStr">
         <is>
-          <t xml:space="preserve">E9</t>
+          <t xml:space="preserve">E7</t>
         </is>
       </c>
       <c r="E426" t="inlineStr">
@@ -35174,7 +35174,7 @@
       </c>
       <c r="S426" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv4yhtbo-8</t>
+          <t xml:space="preserve">v-mv4yhtbo-6</t>
         </is>
       </c>
     </row>
@@ -35196,37 +35196,37 @@
       </c>
       <c r="D427" t="inlineStr">
         <is>
-          <t xml:space="preserve">F1</t>
+          <t xml:space="preserve">E8</t>
         </is>
       </c>
       <c r="E427" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada</t>
+          <t xml:space="preserve">HEK</t>
         </is>
       </c>
       <c r="F427" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+18</t>
+          <t xml:space="preserve">30</t>
         </is>
       </c>
       <c r="G427" t="inlineStr">
         <is>
-          <t xml:space="preserve">relative</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H427" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-12</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="I427" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-12</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="K427" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L427" t="inlineStr">
@@ -35256,7 +35256,7 @@
       </c>
       <c r="S427" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d2kfh-0</t>
+          <t xml:space="preserve">v-mv4yhtbo-7</t>
         </is>
       </c>
     </row>
@@ -35278,37 +35278,37 @@
       </c>
       <c r="D428" t="inlineStr">
         <is>
-          <t xml:space="preserve">F2</t>
+          <t xml:space="preserve">E9</t>
         </is>
       </c>
       <c r="E428" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada</t>
+          <t xml:space="preserve">HEK</t>
         </is>
       </c>
       <c r="F428" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+18</t>
+          <t xml:space="preserve">30</t>
         </is>
       </c>
       <c r="G428" t="inlineStr">
         <is>
-          <t xml:space="preserve">relative</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H428" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-12</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="I428" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-12</t>
+          <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
       <c r="K428" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L428" t="inlineStr">
@@ -35338,7 +35338,7 @@
       </c>
       <c r="S428" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d2kfh-1</t>
+          <t xml:space="preserve">v-mv4yhtbo-8</t>
         </is>
       </c>
     </row>
@@ -35360,7 +35360,7 @@
       </c>
       <c r="D429" t="inlineStr">
         <is>
-          <t xml:space="preserve">F3</t>
+          <t xml:space="preserve">F1</t>
         </is>
       </c>
       <c r="E429" t="inlineStr">
@@ -35420,7 +35420,7 @@
       </c>
       <c r="S429" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d2kfh-2</t>
+          <t xml:space="preserve">v-mv5d2kfh-0</t>
         </is>
       </c>
     </row>
@@ -35442,7 +35442,7 @@
       </c>
       <c r="D430" t="inlineStr">
         <is>
-          <t xml:space="preserve">F4</t>
+          <t xml:space="preserve">F2</t>
         </is>
       </c>
       <c r="E430" t="inlineStr">
@@ -35502,7 +35502,7 @@
       </c>
       <c r="S430" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d2kfh-3</t>
+          <t xml:space="preserve">v-mv5d2kfh-1</t>
         </is>
       </c>
     </row>
@@ -35524,7 +35524,7 @@
       </c>
       <c r="D431" t="inlineStr">
         <is>
-          <t xml:space="preserve">F5</t>
+          <t xml:space="preserve">F3</t>
         </is>
       </c>
       <c r="E431" t="inlineStr">
@@ -35584,7 +35584,7 @@
       </c>
       <c r="S431" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d2kfh-4</t>
+          <t xml:space="preserve">v-mv5d2kfh-2</t>
         </is>
       </c>
     </row>
@@ -35606,7 +35606,7 @@
       </c>
       <c r="D432" t="inlineStr">
         <is>
-          <t xml:space="preserve">F6</t>
+          <t xml:space="preserve">F4</t>
         </is>
       </c>
       <c r="E432" t="inlineStr">
@@ -35666,7 +35666,7 @@
       </c>
       <c r="S432" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d2kfh-5</t>
+          <t xml:space="preserve">v-mv5d2kfh-3</t>
         </is>
       </c>
     </row>
@@ -35688,7 +35688,7 @@
       </c>
       <c r="D433" t="inlineStr">
         <is>
-          <t xml:space="preserve">F7</t>
+          <t xml:space="preserve">F5</t>
         </is>
       </c>
       <c r="E433" t="inlineStr">
@@ -35748,7 +35748,7 @@
       </c>
       <c r="S433" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d2kfh-6</t>
+          <t xml:space="preserve">v-mv5d2kfh-4</t>
         </is>
       </c>
     </row>
@@ -35770,7 +35770,7 @@
       </c>
       <c r="D434" t="inlineStr">
         <is>
-          <t xml:space="preserve">F8</t>
+          <t xml:space="preserve">F6</t>
         </is>
       </c>
       <c r="E434" t="inlineStr">
@@ -35830,7 +35830,7 @@
       </c>
       <c r="S434" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d2kfh-7</t>
+          <t xml:space="preserve">v-mv5d2kfh-5</t>
         </is>
       </c>
     </row>
@@ -35852,7 +35852,7 @@
       </c>
       <c r="D435" t="inlineStr">
         <is>
-          <t xml:space="preserve">F9</t>
+          <t xml:space="preserve">F7</t>
         </is>
       </c>
       <c r="E435" t="inlineStr">
@@ -35912,7 +35912,7 @@
       </c>
       <c r="S435" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d2kfh-8</t>
+          <t xml:space="preserve">v-mv5d2kfh-6</t>
         </is>
       </c>
     </row>
@@ -35934,17 +35934,17 @@
       </c>
       <c r="D436" t="inlineStr">
         <is>
-          <t xml:space="preserve">G1</t>
+          <t xml:space="preserve">F8</t>
         </is>
       </c>
       <c r="E436" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX</t>
+          <t xml:space="preserve">LnCap Canada</t>
         </is>
       </c>
       <c r="F436" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+19</t>
+          <t xml:space="preserve">p+18</t>
         </is>
       </c>
       <c r="G436" t="inlineStr">
@@ -35979,7 +35979,7 @@
       </c>
       <c r="N436" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">No Casp</t>
         </is>
       </c>
       <c r="O436" t="inlineStr">
@@ -35987,11 +35987,6 @@
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
-      <c r="Q436" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mCherr</t>
-        </is>
-      </c>
       <c r="R436" t="inlineStr">
         <is>
           <t xml:space="preserve">stored</t>
@@ -35999,7 +35994,7 @@
       </c>
       <c r="S436" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d4q3i-0</t>
+          <t xml:space="preserve">v-mv5d2kfh-7</t>
         </is>
       </c>
     </row>
@@ -36021,17 +36016,17 @@
       </c>
       <c r="D437" t="inlineStr">
         <is>
-          <t xml:space="preserve">G2</t>
+          <t xml:space="preserve">F9</t>
         </is>
       </c>
       <c r="E437" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX</t>
+          <t xml:space="preserve">LnCap Canada</t>
         </is>
       </c>
       <c r="F437" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+19</t>
+          <t xml:space="preserve">p+18</t>
         </is>
       </c>
       <c r="G437" t="inlineStr">
@@ -36066,7 +36061,7 @@
       </c>
       <c r="N437" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">No Casp</t>
         </is>
       </c>
       <c r="O437" t="inlineStr">
@@ -36074,11 +36069,6 @@
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
-      <c r="Q437" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mCherr</t>
-        </is>
-      </c>
       <c r="R437" t="inlineStr">
         <is>
           <t xml:space="preserve">stored</t>
@@ -36086,7 +36076,7 @@
       </c>
       <c r="S437" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d4q3i-1</t>
+          <t xml:space="preserve">v-mv5d2kfh-8</t>
         </is>
       </c>
     </row>
@@ -36108,7 +36098,7 @@
       </c>
       <c r="D438" t="inlineStr">
         <is>
-          <t xml:space="preserve">G3</t>
+          <t xml:space="preserve">G1</t>
         </is>
       </c>
       <c r="E438" t="inlineStr">
@@ -36173,7 +36163,7 @@
       </c>
       <c r="S438" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d4q3i-2</t>
+          <t xml:space="preserve">v-mv5d4q3i-0</t>
         </is>
       </c>
     </row>
@@ -36195,7 +36185,7 @@
       </c>
       <c r="D439" t="inlineStr">
         <is>
-          <t xml:space="preserve">G4</t>
+          <t xml:space="preserve">G2</t>
         </is>
       </c>
       <c r="E439" t="inlineStr">
@@ -36260,7 +36250,7 @@
       </c>
       <c r="S439" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d4q3i-3</t>
+          <t xml:space="preserve">v-mv5d4q3i-1</t>
         </is>
       </c>
     </row>
@@ -36282,7 +36272,7 @@
       </c>
       <c r="D440" t="inlineStr">
         <is>
-          <t xml:space="preserve">G5</t>
+          <t xml:space="preserve">G3</t>
         </is>
       </c>
       <c r="E440" t="inlineStr">
@@ -36347,7 +36337,7 @@
       </c>
       <c r="S440" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d4q3i-4</t>
+          <t xml:space="preserve">v-mv5d4q3i-2</t>
         </is>
       </c>
     </row>
@@ -36369,7 +36359,7 @@
       </c>
       <c r="D441" t="inlineStr">
         <is>
-          <t xml:space="preserve">G6</t>
+          <t xml:space="preserve">G4</t>
         </is>
       </c>
       <c r="E441" t="inlineStr">
@@ -36434,7 +36424,7 @@
       </c>
       <c r="S441" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d4q3i-5</t>
+          <t xml:space="preserve">v-mv5d4q3i-3</t>
         </is>
       </c>
     </row>
@@ -36456,7 +36446,7 @@
       </c>
       <c r="D442" t="inlineStr">
         <is>
-          <t xml:space="preserve">G7</t>
+          <t xml:space="preserve">G5</t>
         </is>
       </c>
       <c r="E442" t="inlineStr">
@@ -36521,7 +36511,7 @@
       </c>
       <c r="S442" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d4q3i-6</t>
+          <t xml:space="preserve">v-mv5d4q3i-4</t>
         </is>
       </c>
     </row>
@@ -36543,7 +36533,7 @@
       </c>
       <c r="D443" t="inlineStr">
         <is>
-          <t xml:space="preserve">G8</t>
+          <t xml:space="preserve">G6</t>
         </is>
       </c>
       <c r="E443" t="inlineStr">
@@ -36608,7 +36598,7 @@
       </c>
       <c r="S443" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d4q3i-7</t>
+          <t xml:space="preserve">v-mv5d4q3i-5</t>
         </is>
       </c>
     </row>
@@ -36630,7 +36620,7 @@
       </c>
       <c r="D444" t="inlineStr">
         <is>
-          <t xml:space="preserve">G9</t>
+          <t xml:space="preserve">G7</t>
         </is>
       </c>
       <c r="E444" t="inlineStr">
@@ -36695,7 +36685,7 @@
       </c>
       <c r="S444" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d4q3i-8</t>
+          <t xml:space="preserve">v-mv5d4q3i-6</t>
         </is>
       </c>
     </row>
@@ -36717,7 +36707,7 @@
       </c>
       <c r="D445" t="inlineStr">
         <is>
-          <t xml:space="preserve">H1</t>
+          <t xml:space="preserve">G8</t>
         </is>
       </c>
       <c r="E445" t="inlineStr">
@@ -36727,7 +36717,7 @@
       </c>
       <c r="F445" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+23</t>
+          <t xml:space="preserve">p+19</t>
         </is>
       </c>
       <c r="G445" t="inlineStr">
@@ -36782,7 +36772,7 @@
       </c>
       <c r="S445" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d4t1e-0</t>
+          <t xml:space="preserve">v-mv5d4q3i-7</t>
         </is>
       </c>
     </row>
@@ -36804,7 +36794,7 @@
       </c>
       <c r="D446" t="inlineStr">
         <is>
-          <t xml:space="preserve">H2</t>
+          <t xml:space="preserve">G9</t>
         </is>
       </c>
       <c r="E446" t="inlineStr">
@@ -36814,7 +36804,7 @@
       </c>
       <c r="F446" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+23</t>
+          <t xml:space="preserve">p+19</t>
         </is>
       </c>
       <c r="G446" t="inlineStr">
@@ -36869,7 +36859,7 @@
       </c>
       <c r="S446" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d4t1e-1</t>
+          <t xml:space="preserve">v-mv5d4q3i-8</t>
         </is>
       </c>
     </row>
@@ -36891,7 +36881,7 @@
       </c>
       <c r="D447" t="inlineStr">
         <is>
-          <t xml:space="preserve">H3</t>
+          <t xml:space="preserve">H1</t>
         </is>
       </c>
       <c r="E447" t="inlineStr">
@@ -36956,7 +36946,7 @@
       </c>
       <c r="S447" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d4t1e-2</t>
+          <t xml:space="preserve">v-mv5d4t1e-0</t>
         </is>
       </c>
     </row>
@@ -36978,7 +36968,7 @@
       </c>
       <c r="D448" t="inlineStr">
         <is>
-          <t xml:space="preserve">H4</t>
+          <t xml:space="preserve">H2</t>
         </is>
       </c>
       <c r="E448" t="inlineStr">
@@ -37043,7 +37033,7 @@
       </c>
       <c r="S448" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d4t1e-3</t>
+          <t xml:space="preserve">v-mv5d4t1e-1</t>
         </is>
       </c>
     </row>
@@ -37065,7 +37055,7 @@
       </c>
       <c r="D449" t="inlineStr">
         <is>
-          <t xml:space="preserve">H5</t>
+          <t xml:space="preserve">H3</t>
         </is>
       </c>
       <c r="E449" t="inlineStr">
@@ -37130,7 +37120,7 @@
       </c>
       <c r="S449" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d4t1e-4</t>
+          <t xml:space="preserve">v-mv5d4t1e-2</t>
         </is>
       </c>
     </row>
@@ -37152,7 +37142,7 @@
       </c>
       <c r="D450" t="inlineStr">
         <is>
-          <t xml:space="preserve">H6</t>
+          <t xml:space="preserve">H4</t>
         </is>
       </c>
       <c r="E450" t="inlineStr">
@@ -37217,7 +37207,7 @@
       </c>
       <c r="S450" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d4t1e-5</t>
+          <t xml:space="preserve">v-mv5d4t1e-3</t>
         </is>
       </c>
     </row>
@@ -37239,7 +37229,7 @@
       </c>
       <c r="D451" t="inlineStr">
         <is>
-          <t xml:space="preserve">H7</t>
+          <t xml:space="preserve">H5</t>
         </is>
       </c>
       <c r="E451" t="inlineStr">
@@ -37304,7 +37294,7 @@
       </c>
       <c r="S451" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d4t1e-6</t>
+          <t xml:space="preserve">v-mv5d4t1e-4</t>
         </is>
       </c>
     </row>
@@ -37326,7 +37316,7 @@
       </c>
       <c r="D452" t="inlineStr">
         <is>
-          <t xml:space="preserve">H8</t>
+          <t xml:space="preserve">H6</t>
         </is>
       </c>
       <c r="E452" t="inlineStr">
@@ -37391,7 +37381,7 @@
       </c>
       <c r="S452" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d4t1e-7</t>
+          <t xml:space="preserve">v-mv5d4t1e-5</t>
         </is>
       </c>
     </row>
@@ -37413,7 +37403,7 @@
       </c>
       <c r="D453" t="inlineStr">
         <is>
-          <t xml:space="preserve">H9</t>
+          <t xml:space="preserve">H7</t>
         </is>
       </c>
       <c r="E453" t="inlineStr">
@@ -37478,7 +37468,7 @@
       </c>
       <c r="S453" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d4t1e-8</t>
+          <t xml:space="preserve">v-mv5d4t1e-6</t>
         </is>
       </c>
     </row>
@@ -37500,22 +37490,22 @@
       </c>
       <c r="D454" t="inlineStr">
         <is>
-          <t xml:space="preserve">I1</t>
+          <t xml:space="preserve">H8</t>
         </is>
       </c>
       <c r="E454" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F454" t="inlineStr">
         <is>
-          <t xml:space="preserve">p13</t>
+          <t xml:space="preserve">p+23</t>
         </is>
       </c>
       <c r="G454" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H454" t="inlineStr">
@@ -37530,7 +37520,7 @@
       </c>
       <c r="K454" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L454" t="inlineStr">
@@ -37540,12 +37530,12 @@
       </c>
       <c r="M454" t="inlineStr">
         <is>
-          <t xml:space="preserve">CR</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N454" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O454" t="inlineStr">
@@ -37553,6 +37543,11 @@
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
+      <c r="Q454" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mCherr</t>
+        </is>
+      </c>
       <c r="R454" t="inlineStr">
         <is>
           <t xml:space="preserve">stored</t>
@@ -37560,7 +37555,7 @@
       </c>
       <c r="S454" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d5bk8-0</t>
+          <t xml:space="preserve">v-mv5d4t1e-7</t>
         </is>
       </c>
     </row>
@@ -37582,22 +37577,22 @@
       </c>
       <c r="D455" t="inlineStr">
         <is>
-          <t xml:space="preserve">I2</t>
+          <t xml:space="preserve">H9</t>
         </is>
       </c>
       <c r="E455" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F455" t="inlineStr">
         <is>
-          <t xml:space="preserve">p13</t>
+          <t xml:space="preserve">p+23</t>
         </is>
       </c>
       <c r="G455" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H455" t="inlineStr">
@@ -37612,7 +37607,7 @@
       </c>
       <c r="K455" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L455" t="inlineStr">
@@ -37622,12 +37617,12 @@
       </c>
       <c r="M455" t="inlineStr">
         <is>
-          <t xml:space="preserve">CR</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N455" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O455" t="inlineStr">
@@ -37635,6 +37630,11 @@
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
+      <c r="Q455" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mCherr</t>
+        </is>
+      </c>
       <c r="R455" t="inlineStr">
         <is>
           <t xml:space="preserve">stored</t>
@@ -37642,7 +37642,7 @@
       </c>
       <c r="S455" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d5bk8-1</t>
+          <t xml:space="preserve">v-mv5d4t1e-8</t>
         </is>
       </c>
     </row>
@@ -37664,7 +37664,7 @@
       </c>
       <c r="D456" t="inlineStr">
         <is>
-          <t xml:space="preserve">I3</t>
+          <t xml:space="preserve">I1</t>
         </is>
       </c>
       <c r="E456" t="inlineStr">
@@ -37724,7 +37724,7 @@
       </c>
       <c r="S456" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d5bk8-2</t>
+          <t xml:space="preserve">v-mv5d5bk8-0</t>
         </is>
       </c>
     </row>
@@ -37746,7 +37746,7 @@
       </c>
       <c r="D457" t="inlineStr">
         <is>
-          <t xml:space="preserve">I4</t>
+          <t xml:space="preserve">I2</t>
         </is>
       </c>
       <c r="E457" t="inlineStr">
@@ -37806,7 +37806,7 @@
       </c>
       <c r="S457" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d5bk8-3</t>
+          <t xml:space="preserve">v-mv5d5bk8-1</t>
         </is>
       </c>
     </row>
@@ -37828,7 +37828,7 @@
       </c>
       <c r="D458" t="inlineStr">
         <is>
-          <t xml:space="preserve">I5</t>
+          <t xml:space="preserve">I3</t>
         </is>
       </c>
       <c r="E458" t="inlineStr">
@@ -37888,7 +37888,7 @@
       </c>
       <c r="S458" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d5bk8-4</t>
+          <t xml:space="preserve">v-mv5d5bk8-2</t>
         </is>
       </c>
     </row>
@@ -37910,7 +37910,7 @@
       </c>
       <c r="D459" t="inlineStr">
         <is>
-          <t xml:space="preserve">I6</t>
+          <t xml:space="preserve">I4</t>
         </is>
       </c>
       <c r="E459" t="inlineStr">
@@ -37970,7 +37970,7 @@
       </c>
       <c r="S459" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d5bk8-5</t>
+          <t xml:space="preserve">v-mv5d5bk8-3</t>
         </is>
       </c>
     </row>
@@ -37992,7 +37992,7 @@
       </c>
       <c r="D460" t="inlineStr">
         <is>
-          <t xml:space="preserve">I7</t>
+          <t xml:space="preserve">I5</t>
         </is>
       </c>
       <c r="E460" t="inlineStr">
@@ -38052,7 +38052,7 @@
       </c>
       <c r="S460" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d5bk8-6</t>
+          <t xml:space="preserve">v-mv5d5bk8-4</t>
         </is>
       </c>
     </row>
@@ -38074,7 +38074,7 @@
       </c>
       <c r="D461" t="inlineStr">
         <is>
-          <t xml:space="preserve">I8</t>
+          <t xml:space="preserve">I6</t>
         </is>
       </c>
       <c r="E461" t="inlineStr">
@@ -38134,7 +38134,7 @@
       </c>
       <c r="S461" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d5bk8-7</t>
+          <t xml:space="preserve">v-mv5d5bk8-5</t>
         </is>
       </c>
     </row>
@@ -38156,7 +38156,7 @@
       </c>
       <c r="D462" t="inlineStr">
         <is>
-          <t xml:space="preserve">I9</t>
+          <t xml:space="preserve">I7</t>
         </is>
       </c>
       <c r="E462" t="inlineStr">
@@ -38216,7 +38216,7 @@
       </c>
       <c r="S462" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mv5d5bk8-8</t>
+          <t xml:space="preserve">v-mv5d5bk8-6</t>
         </is>
       </c>
     </row>
@@ -38228,27 +38228,27 @@
       </c>
       <c r="B463" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C463" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D463" t="inlineStr">
         <is>
-          <t xml:space="preserve">A1</t>
+          <t xml:space="preserve">I8</t>
         </is>
       </c>
       <c r="E463" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="F463" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p13</t>
         </is>
       </c>
       <c r="G463" t="inlineStr">
@@ -38258,17 +38258,17 @@
       </c>
       <c r="H463" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="I463" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="K463" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L463" t="inlineStr">
@@ -38278,7 +38278,7 @@
       </c>
       <c r="M463" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N463" t="inlineStr">
@@ -38298,7 +38298,7 @@
       </c>
       <c r="S463" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-0</t>
+          <t xml:space="preserve">v-mv5d5bk8-7</t>
         </is>
       </c>
     </row>
@@ -38310,27 +38310,27 @@
       </c>
       <c r="B464" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rack 2</t>
+          <t xml:space="preserve">Rack 1</t>
         </is>
       </c>
       <c r="C464" t="inlineStr">
         <is>
-          <t xml:space="preserve">Common Box #1</t>
+          <t xml:space="preserve">Umut Cell Box -5-</t>
         </is>
       </c>
       <c r="D464" t="inlineStr">
         <is>
-          <t xml:space="preserve">A2</t>
+          <t xml:space="preserve">I9</t>
         </is>
       </c>
       <c r="E464" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="F464" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p13</t>
         </is>
       </c>
       <c r="G464" t="inlineStr">
@@ -38340,17 +38340,17 @@
       </c>
       <c r="H464" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="I464" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-01</t>
+          <t xml:space="preserve">2026-10-12</t>
         </is>
       </c>
       <c r="K464" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L464" t="inlineStr">
@@ -38360,7 +38360,7 @@
       </c>
       <c r="M464" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N464" t="inlineStr">
@@ -38380,7 +38380,7 @@
       </c>
       <c r="S464" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-1</t>
+          <t xml:space="preserve">v-mv5d5bk8-8</t>
         </is>
       </c>
     </row>
@@ -38402,7 +38402,7 @@
       </c>
       <c r="D465" t="inlineStr">
         <is>
-          <t xml:space="preserve">A3</t>
+          <t xml:space="preserve">A1</t>
         </is>
       </c>
       <c r="E465" t="inlineStr">
@@ -38462,7 +38462,7 @@
       </c>
       <c r="S465" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-2</t>
+          <t xml:space="preserve">v-mupot2zh-0</t>
         </is>
       </c>
     </row>
@@ -38484,7 +38484,7 @@
       </c>
       <c r="D466" t="inlineStr">
         <is>
-          <t xml:space="preserve">A4</t>
+          <t xml:space="preserve">A2</t>
         </is>
       </c>
       <c r="E466" t="inlineStr">
@@ -38544,7 +38544,7 @@
       </c>
       <c r="S466" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-3</t>
+          <t xml:space="preserve">v-mupot2zh-1</t>
         </is>
       </c>
     </row>
@@ -38566,7 +38566,7 @@
       </c>
       <c r="D467" t="inlineStr">
         <is>
-          <t xml:space="preserve">A5</t>
+          <t xml:space="preserve">A3</t>
         </is>
       </c>
       <c r="E467" t="inlineStr">
@@ -38626,7 +38626,7 @@
       </c>
       <c r="S467" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mupot2zh-4</t>
+          <t xml:space="preserve">v-mupot2zh-2</t>
         </is>
       </c>
     </row>
@@ -38648,17 +38648,17 @@
       </c>
       <c r="D468" t="inlineStr">
         <is>
-          <t xml:space="preserve">B1</t>
+          <t xml:space="preserve">A4</t>
         </is>
       </c>
       <c r="E468" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX gP2</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="F468" t="inlineStr">
         <is>
-          <t xml:space="preserve">26</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G468" t="inlineStr">
@@ -38668,17 +38668,17 @@
       </c>
       <c r="H468" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-16</t>
+          <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
       <c r="I468" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-16</t>
+          <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
       <c r="K468" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L468" t="inlineStr">
@@ -38688,17 +38688,17 @@
       </c>
       <c r="M468" t="inlineStr">
         <is>
-          <t xml:space="preserve">CR</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N468" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">No Casp</t>
         </is>
       </c>
       <c r="O468" t="inlineStr">
         <is>
-          <t xml:space="preserve">gP2</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R468" t="inlineStr">
@@ -38708,7 +38708,7 @@
       </c>
       <c r="S468" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mvaskevu-2</t>
+          <t xml:space="preserve">v-mupot2zh-3</t>
         </is>
       </c>
     </row>
@@ -38730,17 +38730,17 @@
       </c>
       <c r="D469" t="inlineStr">
         <is>
-          <t xml:space="preserve">B2</t>
+          <t xml:space="preserve">A5</t>
         </is>
       </c>
       <c r="E469" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX gP2</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="F469" t="inlineStr">
         <is>
-          <t xml:space="preserve">26</t>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G469" t="inlineStr">
@@ -38750,17 +38750,17 @@
       </c>
       <c r="H469" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-16</t>
+          <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
       <c r="I469" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-16</t>
+          <t xml:space="preserve">2026-10-01</t>
         </is>
       </c>
       <c r="K469" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L469" t="inlineStr">
@@ -38770,17 +38770,17 @@
       </c>
       <c r="M469" t="inlineStr">
         <is>
-          <t xml:space="preserve">CR</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N469" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">No Casp</t>
         </is>
       </c>
       <c r="O469" t="inlineStr">
         <is>
-          <t xml:space="preserve">gP2</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R469" t="inlineStr">
@@ -38790,7 +38790,7 @@
       </c>
       <c r="S469" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mvaskevu-3</t>
+          <t xml:space="preserve">v-mupot2zh-4</t>
         </is>
       </c>
     </row>
@@ -38812,12 +38812,12 @@
       </c>
       <c r="D470" t="inlineStr">
         <is>
-          <t xml:space="preserve">B3</t>
+          <t xml:space="preserve">B1</t>
         </is>
       </c>
       <c r="E470" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX gP4</t>
+          <t xml:space="preserve">LUCX gP2</t>
         </is>
       </c>
       <c r="F470" t="inlineStr">
@@ -38862,7 +38862,7 @@
       </c>
       <c r="O470" t="inlineStr">
         <is>
-          <t xml:space="preserve">gP4</t>
+          <t xml:space="preserve">gP2</t>
         </is>
       </c>
       <c r="R470" t="inlineStr">
@@ -38872,7 +38872,7 @@
       </c>
       <c r="S470" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mvaskevu-4</t>
+          <t xml:space="preserve">v-mvaskevu-2</t>
         </is>
       </c>
     </row>
@@ -38894,213 +38894,243 @@
       </c>
       <c r="D471" t="inlineStr">
         <is>
+          <t xml:space="preserve">B2</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LUCX gP2</t>
+        </is>
+      </c>
+      <c r="F471" t="inlineStr">
+        <is>
+          <t xml:space="preserve">26</t>
+        </is>
+      </c>
+      <c r="G471" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H471" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-16</t>
+        </is>
+      </c>
+      <c r="I471" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-16</t>
+        </is>
+      </c>
+      <c r="K471" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LuCap35CR</t>
+        </is>
+      </c>
+      <c r="L471" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M471" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CR</t>
+        </is>
+      </c>
+      <c r="N471" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASPEX</t>
+        </is>
+      </c>
+      <c r="O471" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gP2</t>
+        </is>
+      </c>
+      <c r="R471" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S471" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mvaskevu-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B3</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LUCX gP4</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr">
+        <is>
+          <t xml:space="preserve">26</t>
+        </is>
+      </c>
+      <c r="G472" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H472" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-16</t>
+        </is>
+      </c>
+      <c r="I472" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-10-16</t>
+        </is>
+      </c>
+      <c r="K472" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LuCap35CR</t>
+        </is>
+      </c>
+      <c r="L472" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M472" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CR</t>
+        </is>
+      </c>
+      <c r="N472" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CASPEX</t>
+        </is>
+      </c>
+      <c r="O472" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gP4</t>
+        </is>
+      </c>
+      <c r="R472" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stored</t>
+        </is>
+      </c>
+      <c r="S472" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mvaskevu-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Freezer 1</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rack 2</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Common Box #1</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
           <t xml:space="preserve">B4</t>
         </is>
       </c>
-      <c r="E471" t="inlineStr">
+      <c r="E473" t="inlineStr">
         <is>
           <t xml:space="preserve">LUCX gP4</t>
         </is>
       </c>
-      <c r="F471" t="inlineStr">
+      <c r="F473" t="inlineStr">
         <is>
           <t xml:space="preserve">26</t>
         </is>
       </c>
-      <c r="G471" t="inlineStr">
+      <c r="G473" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H471" t="inlineStr">
+      <c r="H473" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-16</t>
         </is>
       </c>
-      <c r="I471" t="inlineStr">
+      <c r="I473" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-16</t>
         </is>
       </c>
-      <c r="K471" t="inlineStr">
+      <c r="K473" t="inlineStr">
         <is>
           <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
-      <c r="L471" t="inlineStr">
+      <c r="L473" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
         </is>
       </c>
-      <c r="M471" t="inlineStr">
+      <c r="M473" t="inlineStr">
         <is>
           <t xml:space="preserve">CR</t>
         </is>
       </c>
-      <c r="N471" t="inlineStr">
+      <c r="N473" t="inlineStr">
         <is>
           <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
-      <c r="O471" t="inlineStr">
+      <c r="O473" t="inlineStr">
         <is>
           <t xml:space="preserve">gP4</t>
         </is>
       </c>
-      <c r="R471" t="inlineStr">
+      <c r="R473" t="inlineStr">
         <is>
           <t xml:space="preserve">stored</t>
         </is>
       </c>
-      <c r="S471" t="inlineStr">
+      <c r="S473" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mvaskevu-5</t>
-        </is>
-      </c>
-    </row>
-    <row r="472">
-      <c r="E472" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LNCX</t>
-        </is>
-      </c>
-      <c r="F472" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p+21</t>
-        </is>
-      </c>
-      <c r="G472" t="inlineStr">
-        <is>
-          <t xml:space="preserve">relative</t>
-        </is>
-      </c>
-      <c r="H472" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-05-15</t>
-        </is>
-      </c>
-      <c r="I472" t="inlineStr">
-        <is>
-          <t xml:space="preserve">15-05-26</t>
-        </is>
-      </c>
-      <c r="K472" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="L472" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M472" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Par</t>
-        </is>
-      </c>
-      <c r="N472" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CASPEX</t>
-        </is>
-      </c>
-      <c r="O472" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="R472" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S472" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-199</t>
-        </is>
-      </c>
-    </row>
-    <row r="473">
-      <c r="E473" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LUCX</t>
-        </is>
-      </c>
-      <c r="F473" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p19</t>
-        </is>
-      </c>
-      <c r="G473" t="inlineStr">
-        <is>
-          <t xml:space="preserve">absolute</t>
-        </is>
-      </c>
-      <c r="H473" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2026-07-31</t>
-        </is>
-      </c>
-      <c r="I473" t="inlineStr">
-        <is>
-          <t xml:space="preserve">31-07-26</t>
-        </is>
-      </c>
-      <c r="K473" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR</t>
-        </is>
-      </c>
-      <c r="L473" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="M473" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CR</t>
-        </is>
-      </c>
-      <c r="N473" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CASPEX</t>
-        </is>
-      </c>
-      <c r="O473" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No guide/sh</t>
-        </is>
-      </c>
-      <c r="P473" t="inlineStr">
-        <is>
-          <t xml:space="preserve">to-do</t>
-        </is>
-      </c>
-      <c r="Q473" t="inlineStr">
-        <is>
-          <t xml:space="preserve">to-do box / thaw</t>
-        </is>
-      </c>
-      <c r="R473" t="inlineStr">
-        <is>
-          <t xml:space="preserve">withdrawn</t>
-        </is>
-      </c>
-      <c r="S473" t="inlineStr">
-        <is>
-          <t xml:space="preserve">v-233</t>
         </is>
       </c>
     </row>
     <row r="474">
       <c r="E474" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B KO g3</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F474" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+13</t>
+          <t xml:space="preserve">p+21</t>
         </is>
       </c>
       <c r="G474" t="inlineStr">
@@ -39110,22 +39140,22 @@
       </c>
       <c r="H474" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-07-20</t>
+          <t xml:space="preserve">2026-05-15</t>
         </is>
       </c>
       <c r="I474" t="inlineStr">
         <is>
-          <t xml:space="preserve">20-07-26</t>
+          <t xml:space="preserve">15-05-26</t>
         </is>
       </c>
       <c r="K474" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L474" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M474" t="inlineStr">
@@ -39135,12 +39165,12 @@
       </c>
       <c r="N474" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O474" t="inlineStr">
         <is>
-          <t xml:space="preserve">g3</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R474" t="inlineStr">
@@ -39150,19 +39180,19 @@
       </c>
       <c r="S474" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-262</t>
+          <t xml:space="preserve">v-199</t>
         </is>
       </c>
     </row>
     <row r="475">
       <c r="E475" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATP7B GFP</t>
+          <t xml:space="preserve">LUCX</t>
         </is>
       </c>
       <c r="F475" t="inlineStr">
         <is>
-          <t xml:space="preserve">p53</t>
+          <t xml:space="preserve">p19</t>
         </is>
       </c>
       <c r="G475" t="inlineStr">
@@ -39172,17 +39202,17 @@
       </c>
       <c r="H475" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-06-26</t>
+          <t xml:space="preserve">2026-07-31</t>
         </is>
       </c>
       <c r="I475" t="inlineStr">
         <is>
-          <t xml:space="preserve">26-06-26</t>
+          <t xml:space="preserve">31-07-26</t>
         </is>
       </c>
       <c r="K475" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L475" t="inlineStr">
@@ -39192,12 +39222,12 @@
       </c>
       <c r="M475" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N475" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O475" t="inlineStr">
@@ -39205,6 +39235,16 @@
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
+      <c r="P475" t="inlineStr">
+        <is>
+          <t xml:space="preserve">to-do</t>
+        </is>
+      </c>
+      <c r="Q475" t="inlineStr">
+        <is>
+          <t xml:space="preserve">to-do box / thaw</t>
+        </is>
+      </c>
       <c r="R475" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
@@ -39212,44 +39252,44 @@
       </c>
       <c r="S475" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-277</t>
+          <t xml:space="preserve">v-233</t>
         </is>
       </c>
     </row>
     <row r="476">
       <c r="E476" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">HEK ATP7B KO g3</t>
         </is>
       </c>
       <c r="F476" t="inlineStr">
         <is>
-          <t xml:space="preserve">p?</t>
+          <t xml:space="preserve">p+13</t>
         </is>
       </c>
       <c r="G476" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H476" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-06-30</t>
+          <t xml:space="preserve">2026-07-20</t>
         </is>
       </c>
       <c r="I476" t="inlineStr">
         <is>
-          <t xml:space="preserve">30-06-25</t>
+          <t xml:space="preserve">20-07-26</t>
         </is>
       </c>
       <c r="K476" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L476" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M476" t="inlineStr">
@@ -39264,7 +39304,7 @@
       </c>
       <c r="O476" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">g3</t>
         </is>
       </c>
       <c r="R476" t="inlineStr">
@@ -39274,19 +39314,19 @@
       </c>
       <c r="S476" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-295</t>
+          <t xml:space="preserve">v-262</t>
         </is>
       </c>
     </row>
     <row r="477">
       <c r="E477" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">HEK ATP7B GFP</t>
         </is>
       </c>
       <c r="F477" t="inlineStr">
         <is>
-          <t xml:space="preserve">p11</t>
+          <t xml:space="preserve">p53</t>
         </is>
       </c>
       <c r="G477" t="inlineStr">
@@ -39296,17 +39336,17 @@
       </c>
       <c r="H477" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-06-12</t>
+          <t xml:space="preserve">2026-06-26</t>
         </is>
       </c>
       <c r="I477" t="inlineStr">
         <is>
-          <t xml:space="preserve">12/6/2026</t>
+          <t xml:space="preserve">26-06-26</t>
         </is>
       </c>
       <c r="K477" t="inlineStr">
         <is>
-          <t xml:space="preserve">LuCap35CR</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L477" t="inlineStr">
@@ -39316,7 +39356,7 @@
       </c>
       <c r="M477" t="inlineStr">
         <is>
-          <t xml:space="preserve">CR</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N477" t="inlineStr">
@@ -39336,19 +39376,19 @@
       </c>
       <c r="S477" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-311</t>
+          <t xml:space="preserve">v-277</t>
         </is>
       </c>
     </row>
     <row r="478">
       <c r="E478" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap ER</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="F478" t="inlineStr">
         <is>
-          <t xml:space="preserve">p</t>
+          <t xml:space="preserve">p?</t>
         </is>
       </c>
       <c r="G478" t="inlineStr">
@@ -39358,17 +39398,17 @@
       </c>
       <c r="H478" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-07-31</t>
+          <t xml:space="preserve">2025-06-30</t>
         </is>
       </c>
       <c r="I478" t="inlineStr">
         <is>
-          <t xml:space="preserve">31-07-25</t>
+          <t xml:space="preserve">30-06-25</t>
         </is>
       </c>
       <c r="K478" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="L478" t="inlineStr">
@@ -39378,7 +39418,7 @@
       </c>
       <c r="M478" t="inlineStr">
         <is>
-          <t xml:space="preserve">EnzaR</t>
+          <t xml:space="preserve">Par</t>
         </is>
       </c>
       <c r="N478" t="inlineStr">
@@ -39398,39 +39438,39 @@
       </c>
       <c r="S478" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-32</t>
+          <t xml:space="preserve">v-295</t>
         </is>
       </c>
     </row>
     <row r="479">
       <c r="E479" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="F479" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+17</t>
+          <t xml:space="preserve">p11</t>
         </is>
       </c>
       <c r="G479" t="inlineStr">
         <is>
-          <t xml:space="preserve">relative</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H479" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-03-30</t>
+          <t xml:space="preserve">2026-06-12</t>
         </is>
       </c>
       <c r="I479" t="inlineStr">
         <is>
-          <t xml:space="preserve">30-03-26</t>
+          <t xml:space="preserve">12/6/2026</t>
         </is>
       </c>
       <c r="K479" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="L479" t="inlineStr">
@@ -39440,12 +39480,12 @@
       </c>
       <c r="M479" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">CR</t>
         </is>
       </c>
       <c r="N479" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">No Casp</t>
         </is>
       </c>
       <c r="O479" t="inlineStr">
@@ -39460,34 +39500,34 @@
       </c>
       <c r="S479" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-320</t>
+          <t xml:space="preserve">v-311</t>
         </is>
       </c>
     </row>
     <row r="480">
       <c r="E480" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada</t>
+          <t xml:space="preserve">LnCap ER</t>
         </is>
       </c>
       <c r="F480" t="inlineStr">
         <is>
-          <t xml:space="preserve">p+14</t>
+          <t xml:space="preserve">p</t>
         </is>
       </c>
       <c r="G480" t="inlineStr">
         <is>
-          <t xml:space="preserve">relative</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H480" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-03-23</t>
+          <t xml:space="preserve">2025-07-31</t>
         </is>
       </c>
       <c r="I480" t="inlineStr">
         <is>
-          <t xml:space="preserve">23-03-26</t>
+          <t xml:space="preserve">31-07-25</t>
         </is>
       </c>
       <c r="K480" t="inlineStr">
@@ -39502,7 +39542,7 @@
       </c>
       <c r="M480" t="inlineStr">
         <is>
-          <t xml:space="preserve">Par</t>
+          <t xml:space="preserve">EnzaR</t>
         </is>
       </c>
       <c r="N480" t="inlineStr">
@@ -39522,39 +39562,39 @@
       </c>
       <c r="S480" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-321</t>
+          <t xml:space="preserve">v-32</t>
         </is>
       </c>
     </row>
     <row r="481">
       <c r="E481" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LNCX</t>
         </is>
       </c>
       <c r="F481" t="inlineStr">
         <is>
-          <t xml:space="preserve">p16</t>
+          <t xml:space="preserve">p+17</t>
         </is>
       </c>
       <c r="G481" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H481" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-11-06</t>
+          <t xml:space="preserve">2026-03-30</t>
         </is>
       </c>
       <c r="I481" t="inlineStr">
         <is>
-          <t xml:space="preserve">6/11/2025</t>
+          <t xml:space="preserve">30-03-26</t>
         </is>
       </c>
       <c r="K481" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L481" t="inlineStr">
@@ -39569,7 +39609,7 @@
       </c>
       <c r="N481" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O481" t="inlineStr">
@@ -39584,39 +39624,39 @@
       </c>
       <c r="S481" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-338</t>
+          <t xml:space="preserve">v-320</t>
         </is>
       </c>
     </row>
     <row r="482">
       <c r="E482" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap Canada</t>
         </is>
       </c>
       <c r="F482" t="inlineStr">
         <is>
-          <t xml:space="preserve">p15</t>
+          <t xml:space="preserve">p+14</t>
         </is>
       </c>
       <c r="G482" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">relative</t>
         </is>
       </c>
       <c r="H482" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-08-10</t>
+          <t xml:space="preserve">2026-03-23</t>
         </is>
       </c>
       <c r="I482" t="inlineStr">
         <is>
-          <t xml:space="preserve">10/8/2026</t>
+          <t xml:space="preserve">23-03-26</t>
         </is>
       </c>
       <c r="K482" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="L482" t="inlineStr">
@@ -39646,19 +39686,19 @@
       </c>
       <c r="S482" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-354</t>
+          <t xml:space="preserve">v-321</t>
         </is>
       </c>
     </row>
     <row r="483">
       <c r="E483" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="F483" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p16</t>
         </is>
       </c>
       <c r="G483" t="inlineStr">
@@ -39668,12 +39708,12 @@
       </c>
       <c r="H483" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2025-11-06</t>
         </is>
       </c>
       <c r="I483" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">6/11/2025</t>
         </is>
       </c>
       <c r="K483" t="inlineStr">
@@ -39698,7 +39738,7 @@
       </c>
       <c r="O483" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R483" t="inlineStr">
@@ -39708,19 +39748,19 @@
       </c>
       <c r="S483" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdx0po-0</t>
+          <t xml:space="preserve">v-338</t>
         </is>
       </c>
     </row>
     <row r="484">
       <c r="E484" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="F484" t="inlineStr">
         <is>
-          <t xml:space="preserve">p21</t>
+          <t xml:space="preserve">p15</t>
         </is>
       </c>
       <c r="G484" t="inlineStr">
@@ -39730,22 +39770,22 @@
       </c>
       <c r="H484" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">2026-08-10</t>
         </is>
       </c>
       <c r="I484" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-07</t>
+          <t xml:space="preserve">10/8/2026</t>
         </is>
       </c>
       <c r="K484" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L484" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M484" t="inlineStr">
@@ -39770,14 +39810,14 @@
       </c>
       <c r="S484" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdxsum-0</t>
+          <t xml:space="preserve">v-354</t>
         </is>
       </c>
     </row>
     <row r="485">
       <c r="E485" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">HEK gNT</t>
         </is>
       </c>
       <c r="F485" t="inlineStr">
@@ -39807,7 +39847,7 @@
       </c>
       <c r="L485" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M485" t="inlineStr">
@@ -39822,7 +39862,7 @@
       </c>
       <c r="O485" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R485" t="inlineStr">
@@ -39832,14 +39872,14 @@
       </c>
       <c r="S485" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-0</t>
+          <t xml:space="preserve">v-mtrdx0po-0</t>
         </is>
       </c>
     </row>
     <row r="486">
       <c r="E486" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="F486" t="inlineStr">
@@ -39869,7 +39909,7 @@
       </c>
       <c r="L486" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M486" t="inlineStr">
@@ -39894,19 +39934,19 @@
       </c>
       <c r="S486" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdyhss-1</t>
+          <t xml:space="preserve">v-mtrdxsum-0</t>
         </is>
       </c>
     </row>
     <row r="487">
       <c r="E487" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="F487" t="inlineStr">
         <is>
-          <t xml:space="preserve">p28</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G487" t="inlineStr">
@@ -39931,7 +39971,7 @@
       </c>
       <c r="L487" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M487" t="inlineStr">
@@ -39956,19 +39996,19 @@
       </c>
       <c r="S487" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdz1vx-0</t>
+          <t xml:space="preserve">v-mtrdyhss-0</t>
         </is>
       </c>
     </row>
     <row r="488">
       <c r="E488" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="F488" t="inlineStr">
         <is>
-          <t xml:space="preserve">p17</t>
+          <t xml:space="preserve">p21</t>
         </is>
       </c>
       <c r="G488" t="inlineStr">
@@ -39988,12 +40028,12 @@
       </c>
       <c r="K488" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L488" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M488" t="inlineStr">
@@ -40008,7 +40048,7 @@
       </c>
       <c r="O488" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
       <c r="R488" t="inlineStr">
@@ -40018,19 +40058,19 @@
       </c>
       <c r="S488" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtrdzpx7-0</t>
+          <t xml:space="preserve">v-mtrdyhss-1</t>
         </is>
       </c>
     </row>
     <row r="489">
       <c r="E489" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="F489" t="inlineStr">
         <is>
-          <t xml:space="preserve">p18</t>
+          <t xml:space="preserve">p28</t>
         </is>
       </c>
       <c r="G489" t="inlineStr">
@@ -40050,12 +40090,12 @@
       </c>
       <c r="K489" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="L489" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M489" t="inlineStr">
@@ -40080,14 +40120,14 @@
       </c>
       <c r="S489" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0daw-0</t>
+          <t xml:space="preserve">v-mtrdz1vx-0</t>
         </is>
       </c>
     </row>
     <row r="490">
       <c r="E490" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
+          <t xml:space="preserve">Huh7 gNT</t>
         </is>
       </c>
       <c r="F490" t="inlineStr">
@@ -40117,7 +40157,7 @@
       </c>
       <c r="L490" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M490" t="inlineStr">
@@ -40132,7 +40172,7 @@
       </c>
       <c r="O490" t="inlineStr">
         <is>
-          <t xml:space="preserve">No guide/sh</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="R490" t="inlineStr">
@@ -40142,14 +40182,14 @@
       </c>
       <c r="S490" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre0w3q-0</t>
+          <t xml:space="preserve">v-mtrdzpx7-0</t>
         </is>
       </c>
     </row>
     <row r="491">
       <c r="E491" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="F491" t="inlineStr">
@@ -40179,7 +40219,7 @@
       </c>
       <c r="L491" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="M491" t="inlineStr">
@@ -40204,19 +40244,19 @@
       </c>
       <c r="S491" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtre1ko0-0</t>
+          <t xml:space="preserve">v-mtre0daw-0</t>
         </is>
       </c>
     </row>
     <row r="492">
       <c r="E492" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hek caspex</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="F492" t="inlineStr">
         <is>
-          <t xml:space="preserve">p6</t>
+          <t xml:space="preserve">p17</t>
         </is>
       </c>
       <c r="G492" t="inlineStr">
@@ -40226,22 +40266,22 @@
       </c>
       <c r="H492" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I492" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="K492" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L492" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="M492" t="inlineStr">
@@ -40251,7 +40291,7 @@
       </c>
       <c r="N492" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">No Casp</t>
         </is>
       </c>
       <c r="O492" t="inlineStr">
@@ -40266,29 +40306,39 @@
       </c>
       <c r="S492" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtski3re-0</t>
+          <t xml:space="preserve">v-mtre0w3q-0</t>
         </is>
       </c>
     </row>
     <row r="493">
       <c r="E493" t="inlineStr">
         <is>
-          <t xml:space="preserve">klm ox</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+        </is>
+      </c>
+      <c r="F493" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p18</t>
         </is>
       </c>
       <c r="G493" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H493" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
         </is>
       </c>
       <c r="I493" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-08</t>
+          <t xml:space="preserve">2026-09-07</t>
+        </is>
+      </c>
+      <c r="K493" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="L493" t="inlineStr">
@@ -40318,19 +40368,24 @@
       </c>
       <c r="S493" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt0h140-0</t>
+          <t xml:space="preserve">v-mtre1ko0-0</t>
         </is>
       </c>
     </row>
     <row r="494">
       <c r="E494" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">Hek caspex</t>
+        </is>
+      </c>
+      <c r="F494" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p6</t>
         </is>
       </c>
       <c r="G494" t="inlineStr">
         <is>
-          <t xml:space="preserve">unknown</t>
+          <t xml:space="preserve">absolute</t>
         </is>
       </c>
       <c r="H494" t="inlineStr">
@@ -40343,6 +40398,11 @@
           <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
+      <c r="K494" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
       <c r="L494" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -40355,7 +40415,7 @@
       </c>
       <c r="N494" t="inlineStr">
         <is>
-          <t xml:space="preserve">No Casp</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="O494" t="inlineStr">
@@ -40370,14 +40430,14 @@
       </c>
       <c r="S494" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-0</t>
+          <t xml:space="preserve">v-mtski3re-0</t>
         </is>
       </c>
     </row>
     <row r="495">
       <c r="E495" t="inlineStr">
         <is>
-          <t xml:space="preserve">jkl</t>
+          <t xml:space="preserve">klm ox</t>
         </is>
       </c>
       <c r="G495" t="inlineStr">
@@ -40397,7 +40457,7 @@
       </c>
       <c r="L495" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="M495" t="inlineStr">
@@ -40422,7 +40482,7 @@
       </c>
       <c r="S495" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-1</t>
+          <t xml:space="preserve">v-mtt0h140-0</t>
         </is>
       </c>
     </row>
@@ -40474,14 +40534,14 @@
       </c>
       <c r="S496" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt3mo6u-2</t>
+          <t xml:space="preserve">v-mtt3mo6u-0</t>
         </is>
       </c>
     </row>
     <row r="497">
       <c r="E497" t="inlineStr">
         <is>
-          <t xml:space="preserve">khk</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="G497" t="inlineStr">
@@ -40526,14 +40586,14 @@
       </c>
       <c r="S497" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtt5ckqo-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-1</t>
         </is>
       </c>
     </row>
     <row r="498">
       <c r="E498" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">jkl</t>
         </is>
       </c>
       <c r="G498" t="inlineStr">
@@ -40543,12 +40603,12 @@
       </c>
       <c r="H498" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I498" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="L498" t="inlineStr">
@@ -40578,14 +40638,14 @@
       </c>
       <c r="S498" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmw7m-0</t>
+          <t xml:space="preserve">v-mtt3mo6u-2</t>
         </is>
       </c>
     </row>
     <row r="499">
       <c r="E499" t="inlineStr">
         <is>
-          <t xml:space="preserve">kkk</t>
+          <t xml:space="preserve">khk</t>
         </is>
       </c>
       <c r="G499" t="inlineStr">
@@ -40595,12 +40655,12 @@
       </c>
       <c r="H499" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="I499" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-09</t>
+          <t xml:space="preserve">2026-09-08</t>
         </is>
       </c>
       <c r="L499" t="inlineStr">
@@ -40630,7 +40690,7 @@
       </c>
       <c r="S499" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmmypa-0</t>
+          <t xml:space="preserve">v-mtt5ckqo-0</t>
         </is>
       </c>
     </row>
@@ -40682,14 +40742,14 @@
       </c>
       <c r="S500" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mttmn045-0</t>
+          <t xml:space="preserve">v-mttmmw7m-0</t>
         </is>
       </c>
     </row>
     <row r="501">
       <c r="E501" t="inlineStr">
         <is>
-          <t xml:space="preserve">deneme</t>
+          <t xml:space="preserve">kkk</t>
         </is>
       </c>
       <c r="G501" t="inlineStr">
@@ -40707,11 +40767,6 @@
           <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
-      <c r="K501" t="inlineStr">
-        <is>
-          <t xml:space="preserve">deneme</t>
-        </is>
-      </c>
       <c r="L501" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
@@ -40739,44 +40794,34 @@
       </c>
       <c r="S501" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mtu5lgdc-0</t>
+          <t xml:space="preserve">v-mttmmypa-0</t>
         </is>
       </c>
     </row>
     <row r="502">
       <c r="E502" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
-        </is>
-      </c>
-      <c r="F502" t="inlineStr">
-        <is>
-          <t xml:space="preserve">p19</t>
+          <t xml:space="preserve">kkk</t>
         </is>
       </c>
       <c r="G502" t="inlineStr">
         <is>
-          <t xml:space="preserve">absolute</t>
+          <t xml:space="preserve">unknown</t>
         </is>
       </c>
       <c r="H502" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-17</t>
+          <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
       <c r="I502" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-09-17</t>
-        </is>
-      </c>
-      <c r="K502" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">2026-09-09</t>
         </is>
       </c>
       <c r="L502" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="M502" t="inlineStr">
@@ -40801,67 +40846,186 @@
       </c>
       <c r="S502" t="inlineStr">
         <is>
-          <t xml:space="preserve">v-mu5anec8-0</t>
+          <t xml:space="preserve">v-mttmn045-0</t>
         </is>
       </c>
     </row>
     <row r="503">
       <c r="E503" t="inlineStr">
         <is>
+          <t xml:space="preserve">deneme</t>
+        </is>
+      </c>
+      <c r="G503" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unknown</t>
+        </is>
+      </c>
+      <c r="H503" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="I503" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-09</t>
+        </is>
+      </c>
+      <c r="K503" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deneme</t>
+        </is>
+      </c>
+      <c r="L503" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="M503" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N503" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O503" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R503" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S503" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mtu5lgdc-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="E504" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
+        </is>
+      </c>
+      <c r="F504" t="inlineStr">
+        <is>
+          <t xml:space="preserve">p19</t>
+        </is>
+      </c>
+      <c r="G504" t="inlineStr">
+        <is>
+          <t xml:space="preserve">absolute</t>
+        </is>
+      </c>
+      <c r="H504" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-17</t>
+        </is>
+      </c>
+      <c r="I504" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-09-17</t>
+        </is>
+      </c>
+      <c r="K504" t="inlineStr">
+        <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="F503" t="inlineStr">
+      <c r="L504" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FLAG</t>
+        </is>
+      </c>
+      <c r="M504" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Par</t>
+        </is>
+      </c>
+      <c r="N504" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No Casp</t>
+        </is>
+      </c>
+      <c r="O504" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No guide/sh</t>
+        </is>
+      </c>
+      <c r="R504" t="inlineStr">
+        <is>
+          <t xml:space="preserve">withdrawn</t>
+        </is>
+      </c>
+      <c r="S504" t="inlineStr">
+        <is>
+          <t xml:space="preserve">v-mu5anec8-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="E505" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Huh7</t>
+        </is>
+      </c>
+      <c r="F505" t="inlineStr">
         <is>
           <t xml:space="preserve">18</t>
         </is>
       </c>
-      <c r="G503" t="inlineStr">
+      <c r="G505" t="inlineStr">
         <is>
           <t xml:space="preserve">absolute</t>
         </is>
       </c>
-      <c r="H503" t="inlineStr">
+      <c r="H505" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
-      <c r="I503" t="inlineStr">
+      <c r="I505" t="inlineStr">
         <is>
           <t xml:space="preserve">2026-10-09</t>
         </is>
       </c>
-      <c r="K503" t="inlineStr">
+      <c r="K505" t="inlineStr">
         <is>
           <t xml:space="preserve">Huh7</t>
         </is>
       </c>
-      <c r="L503" t="inlineStr">
+      <c r="L505" t="inlineStr">
         <is>
           <t xml:space="preserve">WT</t>
         </is>
       </c>
-      <c r="M503" t="inlineStr">
+      <c r="M505" t="inlineStr">
         <is>
           <t xml:space="preserve">Par</t>
         </is>
       </c>
-      <c r="N503" t="inlineStr">
+      <c r="N505" t="inlineStr">
         <is>
           <t xml:space="preserve">No Casp</t>
         </is>
       </c>
-      <c r="O503" t="inlineStr">
+      <c r="O505" t="inlineStr">
         <is>
           <t xml:space="preserve">No guide/sh</t>
         </is>
       </c>
-      <c r="R503" t="inlineStr">
+      <c r="R505" t="inlineStr">
         <is>
           <t xml:space="preserve">withdrawn</t>
         </is>
       </c>
-      <c r="S503" t="inlineStr">
+      <c r="S505" t="inlineStr">
         <is>
           <t xml:space="preserve">v-mv4yequa-5</t>
         </is>
@@ -41705,22 +41869,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCX gP2</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LuCap35CR</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gP2</t>
+          <t xml:space="preserve">LNC478 #2</t>
         </is>
       </c>
       <c r="E28">
@@ -41736,38 +41885,38 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK 3xFLAG</t>
+          <t xml:space="preserve">LUCX gP2</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">LuCap35CR</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">FLAG</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gP2</t>
         </is>
       </c>
       <c r="E29">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F29">
+        <v>0</v>
+      </c>
+      <c r="G29">
         <v>2</v>
-      </c>
-      <c r="G29">
-        <v>3</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK TOX4 KO g2</t>
+          <t xml:space="preserve">HEK 3xFLAG</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -41777,33 +41926,33 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E30">
         <v>3</v>
       </c>
       <c r="F30">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G30">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 TOX4 KO</t>
+          <t xml:space="preserve">HEK TOX4 KO g2</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7</t>
+          <t xml:space="preserve">HEK293T</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -41813,7 +41962,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E31">
@@ -41829,7 +41978,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 gNT</t>
+          <t xml:space="preserve">Huh7 TOX4 KO</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -41839,19 +41988,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E32">
         <v>3</v>
       </c>
       <c r="F32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G32">
         <v>2</v>
@@ -41860,12 +42009,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-I no sort</t>
+          <t xml:space="preserve">Huh7 gNT</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -41875,23 +42024,23 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E33">
         <v>3</v>
       </c>
       <c r="F33">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G33">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-K no sort</t>
+          <t xml:space="preserve">LCC-I no sort</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -41922,7 +42071,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-R no sort</t>
+          <t xml:space="preserve">LCC-K no sort</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -41953,7 +42102,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gC1</t>
+          <t xml:space="preserve">LCC-R no sort</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E36">
@@ -41963,13 +42127,13 @@
         <v>0</v>
       </c>
       <c r="G36">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gC2</t>
+          <t xml:space="preserve">LNCX gC1</t>
         </is>
       </c>
       <c r="E37">
@@ -41985,22 +42149,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gC3</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gC3</t>
+          <t xml:space="preserve">LNCX gC2</t>
         </is>
       </c>
       <c r="E38">
@@ -42016,7 +42165,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gC4</t>
+          <t xml:space="preserve">LNCX gC3</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gC3</t>
         </is>
       </c>
       <c r="E39">
@@ -42032,22 +42196,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNCX gP3</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LnCap</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gP3</t>
+          <t xml:space="preserve">LNCX gC4</t>
         </is>
       </c>
       <c r="E40">
@@ -42063,7 +42212,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap Canada CASPEX (no sort)</t>
+          <t xml:space="preserve">LNCX gP3</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -42073,12 +42222,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">gP3</t>
         </is>
       </c>
       <c r="E41">
@@ -42088,32 +42237,32 @@
         <v>0</v>
       </c>
       <c r="G41">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145 TOX4 KO g2.2</t>
+          <t xml:space="preserve">LnCap Canada CASPEX (no sort)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Du145</t>
+          <t xml:space="preserve">LnCap</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2.2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E42">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F42">
         <v>0</v>
@@ -42125,7 +42274,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuDtxR</t>
+          <t xml:space="preserve">Du145 TOX4 KO g2.2</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -42135,12 +42284,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2.2</t>
         </is>
       </c>
       <c r="E43">
@@ -42156,7 +42305,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR ATF3 KO</t>
+          <t xml:space="preserve">DuDtxR</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -42166,7 +42315,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -42187,7 +42336,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR ATP7B KO</t>
+          <t xml:space="preserve">DuPar50CR ATF3 KO</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -42218,7 +42367,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR MTF1 KO</t>
+          <t xml:space="preserve">DuPar50CR ATP7B KO</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -42249,7 +42398,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR NT KO</t>
+          <t xml:space="preserve">DuPar50CR MTF1 KO</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -42280,7 +42429,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR TOX4 KO g1.2</t>
+          <t xml:space="preserve">DuPar50CR NT KO</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -42290,12 +42439,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1.2</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E48">
@@ -42311,7 +42460,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">DuPar50CR TOX4 KO g2.2</t>
+          <t xml:space="preserve">DuPar50CR TOX4 KO g1.2</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -42326,7 +42475,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2.2</t>
+          <t xml:space="preserve">g1.2</t>
         </is>
       </c>
       <c r="E49">
@@ -42342,29 +42491,29 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 KO rep2</t>
+          <t xml:space="preserve">DuPar50CR TOX4 KO g2.2</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK293T</t>
+          <t xml:space="preserve">Du145</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2.2</t>
         </is>
       </c>
       <c r="E50">
         <v>2</v>
       </c>
       <c r="F50">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G50">
         <v>1</v>
@@ -42373,7 +42522,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK ATF3 OX rep3</t>
+          <t xml:space="preserve">HEK ATF3 KO rep2</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -42383,7 +42532,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -42404,7 +42553,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CASPEX Single</t>
+          <t xml:space="preserve">HEK ATF3 OX rep3</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -42414,7 +42563,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t xml:space="preserve">CASPEX</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -42426,7 +42575,7 @@
         <v>2</v>
       </c>
       <c r="F52">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G52">
         <v>1</v>
@@ -42435,7 +42584,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX</t>
+          <t xml:space="preserve">HEK CASPEX Single</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -42445,12 +42594,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">CASPEX</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E53">
@@ -42466,7 +42615,22 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK CuAdapt CuCl2 100</t>
+          <t xml:space="preserve">HEK CBX3 KO g1 ATP7B OX</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OX</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E54">
@@ -42482,22 +42646,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK E2F1 sh1</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HEK293T</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WT</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">HEK CuAdapt CuCl2 100</t>
         </is>
       </c>
       <c r="E55">
@@ -42513,7 +42662,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK E2F1 sh2</t>
+          <t xml:space="preserve">HEK E2F1 sh1</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -42544,7 +42693,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK FOXA1 KO g1</t>
+          <t xml:space="preserve">HEK E2F1 sh2</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -42554,12 +42703,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">WT</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E57">
@@ -42575,7 +42724,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK FOXA1 KO g2</t>
+          <t xml:space="preserve">HEK FOXA1 KO g1</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -42590,7 +42739,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E58">
@@ -42606,7 +42755,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK HOXB6 OX</t>
+          <t xml:space="preserve">HEK FOXA1 KO g2</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -42621,7 +42770,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E59">
@@ -42637,7 +42786,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g1</t>
+          <t xml:space="preserve">HEK HOXB6 OX</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -42647,12 +42796,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t xml:space="preserve">g1</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E60">
@@ -42662,13 +42811,13 @@
         <v>0</v>
       </c>
       <c r="G60">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK POU3F3 KO g2</t>
+          <t xml:space="preserve">HEK POU3F3 KO g1</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -42683,7 +42832,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t xml:space="preserve">g2</t>
+          <t xml:space="preserve">g1</t>
         </is>
       </c>
       <c r="E61">
@@ -42693,13 +42842,13 @@
         <v>0</v>
       </c>
       <c r="G61">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK STAT1 KO g2</t>
+          <t xml:space="preserve">HEK POU3F3 KO g2</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -42730,7 +42879,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK gNT(20)</t>
+          <t xml:space="preserve">HEK STAT1 KO g2</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -42740,12 +42889,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t xml:space="preserve">gNT</t>
+          <t xml:space="preserve">g2</t>
         </is>
       </c>
       <c r="E63">
@@ -42755,13 +42904,28 @@
         <v>0</v>
       </c>
       <c r="G63">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">HEK pCDH-YY1 OX-2</t>
+          <t xml:space="preserve">HEK gNT(20)</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HEK293T</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gNT</t>
         </is>
       </c>
       <c r="E64">
@@ -42771,44 +42935,29 @@
         <v>0</v>
       </c>
       <c r="G64">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 3xFLAG</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Huh7</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FLAG</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t xml:space="preserve">-</t>
+          <t xml:space="preserve">HEK pCDH-YY1 OX-2</t>
         </is>
       </c>
       <c r="E65">
         <v>2</v>
       </c>
       <c r="F65">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G65">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
+          <t xml:space="preserve">Huh7 3xFLAG</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -42818,7 +42967,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">FLAG</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -42830,16 +42979,16 @@
         <v>2</v>
       </c>
       <c r="F66">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G66">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
+          <t xml:space="preserve">Huh7 ATF3 KO rep3</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -42849,7 +42998,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t xml:space="preserve">OX</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -42870,7 +43019,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Huh7 ATP7B KO #24</t>
+          <t xml:space="preserve">Huh7 ATF3 OX rep3</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -42880,7 +43029,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t xml:space="preserve">KO</t>
+          <t xml:space="preserve">OX</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -42892,7 +43041,7 @@
         <v>2</v>
       </c>
       <c r="F68">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G68">
         <v>1</v>
@@ -42901,17 +43050,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-V</t>
+          <t xml:space="preserve">Huh7 ATP7B KO #24</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t xml:space="preserve">LnCap</t>
+          <t xml:space="preserve">Huh7</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t xml:space="preserve">WT</t>
+          <t xml:space="preserve">KO</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -42926,13 +43075,13 @@
         <v>0</v>
       </c>
       <c r="G69">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t xml:space="preserve">LCC-V 99.17%</t>
+          <t xml:space="preserve">LCC-V</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -42963,7 +43112,22 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t xml:space="preserve">LNC478 #2</t>
+          <t xml:space="preserve">LCC-V 99.17%</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LnCap</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WT</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E71">
@@ -42973,7 +43137,7 @@
         <v>0</v>
       </c>
       <c r="G71">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="72">
@@ -48962,10 +49126,10 @@
         <v>81</v>
       </c>
       <c r="I18">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="J18">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19">

</xml_diff>